<commit_message>
chore: sync data snapshots, docs, esports/KBO/NPB config, and pipeline state
Bundles the accumulated data-layer state with the code changes in the two
prior commits: daily odds/log snapshots through 2026-07-20, esports/KBO/NPB
backfill data and validation artifacts, dashboard runtime state
(archive/jobs/portfolio history), config updates for the new esports/KBO/NPB
model specs, and doc updates (README, league docs, model_improvements.md,
project status notes).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -1558,18 +1558,32 @@
       </c>
       <c r="U2" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V2" s="24" t="n"/>
-      <c r="W2" s="26" t="n"/>
-      <c r="X2" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V2" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W2" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="X2" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="Y2" s="25" t="n"/>
       <c r="Z2" s="26" t="n"/>
       <c r="AA2" s="28" t="n"/>
       <c r="AB2" s="28" t="n"/>
-      <c r="AC2" s="30" t="n"/>
-      <c r="AD2" s="24" t="n"/>
+      <c r="AC2" s="30" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD2" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:43.225807Z</t>
+        </is>
+      </c>
       <c r="AE2" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.4900 (aec-mlb-cws-tor-2026-07-19).</t>
@@ -1582,7 +1596,7 @@
       </c>
       <c r="AG2" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH2" s="24" t="n"/>
@@ -1807,18 +1821,32 @@
       </c>
       <c r="U3" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V3" s="24" t="n"/>
-      <c r="W3" s="26" t="n"/>
-      <c r="X3" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V3" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W3" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="X3" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y3" s="25" t="n"/>
       <c r="Z3" s="26" t="n"/>
       <c r="AA3" s="28" t="n"/>
       <c r="AB3" s="28" t="n"/>
-      <c r="AC3" s="30" t="n"/>
-      <c r="AD3" s="24" t="n"/>
+      <c r="AC3" s="30" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="AD3" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:43.477592Z</t>
+        </is>
+      </c>
       <c r="AE3" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.4600 (aec-mlb-nym-phi-2026-07-19).</t>
@@ -1831,7 +1859,7 @@
       </c>
       <c r="AG3" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH3" s="24" t="n"/>
@@ -2056,18 +2084,32 @@
       </c>
       <c r="U4" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V4" s="24" t="n"/>
-      <c r="W4" s="26" t="n"/>
-      <c r="X4" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V4" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W4" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X4" s="26" t="n">
+        <v>6</v>
+      </c>
       <c r="Y4" s="25" t="n"/>
       <c r="Z4" s="26" t="n"/>
       <c r="AA4" s="28" t="n"/>
       <c r="AB4" s="28" t="n"/>
-      <c r="AC4" s="30" t="n"/>
-      <c r="AD4" s="24" t="n"/>
+      <c r="AC4" s="30" t="n">
+        <v>0.8547</v>
+      </c>
+      <c r="AD4" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:43.720828Z</t>
+        </is>
+      </c>
       <c r="AE4" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.5400 (aec-mlb-tb-bos-2026-07-19).</t>
@@ -2305,18 +2347,32 @@
       </c>
       <c r="U5" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V5" s="24" t="n"/>
-      <c r="W5" s="26" t="n"/>
-      <c r="X5" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V5" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W5" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="X5" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y5" s="25" t="n"/>
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="28" t="n"/>
       <c r="AB5" s="28" t="n"/>
-      <c r="AC5" s="30" t="n"/>
-      <c r="AD5" s="24" t="n"/>
+      <c r="AC5" s="30" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD5" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:43.966052Z</t>
+        </is>
+      </c>
       <c r="AE5" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.4600 (aec-mlb-pit-cle-2026-07-19).</t>
@@ -2329,7 +2385,7 @@
       </c>
       <c r="AG5" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH5" s="24" t="n"/>
@@ -2554,18 +2610,32 @@
       </c>
       <c r="U6" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V6" s="24" t="n"/>
-      <c r="W6" s="26" t="n"/>
-      <c r="X6" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V6" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W6" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="X6" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y6" s="25" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="30" t="n"/>
-      <c r="AD6" s="24" t="n"/>
+      <c r="AC6" s="30" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="AD6" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:44.208798Z</t>
+        </is>
+      </c>
       <c r="AE6" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.5150 (aec-mlb-bal-hou-2026-07-19).</t>
@@ -2578,7 +2648,7 @@
       </c>
       <c r="AG6" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH6" s="24" t="n"/>
@@ -2803,18 +2873,32 @@
       </c>
       <c r="U7" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V7" s="24" t="n"/>
-      <c r="W7" s="26" t="n"/>
-      <c r="X7" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V7" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W7" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X7" s="26" t="n">
+        <v>3</v>
+      </c>
       <c r="Y7" s="25" t="n"/>
       <c r="Z7" s="26" t="n"/>
       <c r="AA7" s="28" t="n"/>
       <c r="AB7" s="28" t="n"/>
-      <c r="AC7" s="30" t="n"/>
-      <c r="AD7" s="24" t="n"/>
+      <c r="AC7" s="30" t="n">
+        <v>1.4344</v>
+      </c>
+      <c r="AD7" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:44.452287Z</t>
+        </is>
+      </c>
       <c r="AE7" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.5500 (aec-mlb-mia-mil-2026-07-19).</t>
@@ -3052,18 +3136,32 @@
       </c>
       <c r="U8" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V8" s="24" t="n"/>
-      <c r="W8" s="26" t="n"/>
-      <c r="X8" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V8" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W8" s="26" t="n">
+        <v>19</v>
+      </c>
+      <c r="X8" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y8" s="25" t="n"/>
       <c r="Z8" s="26" t="n"/>
       <c r="AA8" s="28" t="n"/>
       <c r="AB8" s="28" t="n"/>
-      <c r="AC8" s="30" t="n"/>
-      <c r="AD8" s="24" t="n"/>
+      <c r="AC8" s="30" t="n">
+        <v>0.8625</v>
+      </c>
+      <c r="AD8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:44.698613Z</t>
+        </is>
+      </c>
       <c r="AE8" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.4650 (aec-mlb-sd-kc-2026-07-19).</t>
@@ -3301,18 +3399,32 @@
       </c>
       <c r="U9" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V9" s="24" t="n"/>
-      <c r="W9" s="26" t="n"/>
-      <c r="X9" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V9" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X9" s="26" t="n">
+        <v>10</v>
+      </c>
       <c r="Y9" s="25" t="n"/>
       <c r="Z9" s="26" t="n"/>
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="30" t="n"/>
-      <c r="AD9" s="24" t="n"/>
+      <c r="AC9" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:44.944082Z</t>
+        </is>
+      </c>
       <c r="AE9" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.6000 (aec-mlb-min-chc-2026-07-19).</t>
@@ -3550,18 +3662,32 @@
       </c>
       <c r="U10" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V10" s="24" t="n"/>
-      <c r="W10" s="26" t="n"/>
-      <c r="X10" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V10" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W10" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="X10" s="26" t="n">
+        <v>3</v>
+      </c>
       <c r="Y10" s="25" t="n"/>
       <c r="Z10" s="26" t="n"/>
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="30" t="n"/>
-      <c r="AD10" s="24" t="n"/>
+      <c r="AC10" s="30" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="AD10" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:45.192018Z</t>
+        </is>
+      </c>
       <c r="AE10" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.5850 (aec-mlb-det-laa-2026-07-19).</t>
@@ -3574,7 +3700,7 @@
       </c>
       <c r="AG10" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH10" s="24" t="n"/>
@@ -3799,18 +3925,32 @@
       </c>
       <c r="U11" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V11" s="24" t="n"/>
-      <c r="W11" s="26" t="n"/>
-      <c r="X11" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V11" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W11" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="X11" s="26" t="n">
+        <v>6</v>
+      </c>
       <c r="Y11" s="25" t="n"/>
       <c r="Z11" s="26" t="n"/>
       <c r="AA11" s="28" t="n"/>
       <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="30" t="n"/>
-      <c r="AD11" s="24" t="n"/>
+      <c r="AC11" s="30" t="n">
+        <v>0.9202</v>
+      </c>
+      <c r="AD11" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:45.440735Z</t>
+        </is>
+      </c>
       <c r="AE11" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.6200 (aec-mlb-sf-sea-2026-07-19).</t>
@@ -4546,18 +4686,32 @@
       </c>
       <c r="U14" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V14" s="24" t="n"/>
-      <c r="W14" s="26" t="n"/>
-      <c r="X14" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V14" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W14" s="26" t="n">
+        <v>82</v>
+      </c>
+      <c r="X14" s="26" t="n">
+        <v>90</v>
+      </c>
       <c r="Y14" s="25" t="n"/>
       <c r="Z14" s="26" t="n"/>
       <c r="AA14" s="28" t="n"/>
       <c r="AB14" s="28" t="n"/>
-      <c r="AC14" s="30" t="n"/>
-      <c r="AD14" s="24" t="n"/>
+      <c r="AC14" s="30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD14" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:45.958826Z</t>
+        </is>
+      </c>
       <c r="AE14" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5000; executable ask 0.8000 (aec-wnba-la-dal-2026-07-19).</t>
@@ -4795,18 +4949,32 @@
       </c>
       <c r="U15" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V15" s="24" t="n"/>
-      <c r="W15" s="26" t="n"/>
-      <c r="X15" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V15" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W15" s="26" t="n">
+        <v>91</v>
+      </c>
+      <c r="X15" s="26" t="n">
+        <v>93</v>
+      </c>
       <c r="Y15" s="25" t="n"/>
       <c r="Z15" s="26" t="n"/>
       <c r="AA15" s="28" t="n"/>
       <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="30" t="n"/>
-      <c r="AD15" s="24" t="n"/>
+      <c r="AC15" s="30" t="n">
+        <v>0.4695</v>
+      </c>
+      <c r="AD15" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:46.205387Z</t>
+        </is>
+      </c>
       <c r="AE15" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5000; executable ask 0.8100 (aec-wnba-chi-atl-2026-07-19).</t>
@@ -5268,17 +5436,17 @@
         <v>-354</v>
       </c>
       <c r="M17" s="27" t="n">
-        <v>1.282</v>
+        <v>1.282486</v>
       </c>
       <c r="N17" s="28" t="n">
-        <v>0.78</v>
+        <v>0.779736</v>
       </c>
       <c r="O17" s="28" t="n">
         <v>0.6207</v>
       </c>
       <c r="P17" s="28" t="n"/>
       <c r="Q17" s="28" t="n">
-        <v>-0.1593</v>
+        <v>-0.159036</v>
       </c>
       <c r="R17" s="26" t="n"/>
       <c r="S17" s="29" t="n">
@@ -5310,7 +5478,7 @@
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
       <c r="AC17" s="30" t="n">
-        <v>0.4936</v>
+        <v>0.4944</v>
       </c>
       <c r="AD17" s="24" t="inlineStr">
         <is>
@@ -5375,13 +5543,13 @@
         <v>-354</v>
       </c>
       <c r="BL17" s="27" t="n">
-        <v>1.282</v>
+        <v>1.282486</v>
       </c>
       <c r="BM17" s="28" t="n">
-        <v>0.78</v>
+        <v>0.779736</v>
       </c>
       <c r="BN17" s="28" t="n">
-        <v>0.78</v>
+        <v>0.779736</v>
       </c>
       <c r="BO17" s="28" t="n"/>
       <c r="BP17" s="25" t="n"/>
@@ -5453,10 +5621,10 @@
         <v>-194</v>
       </c>
       <c r="M18" s="27" t="n">
-        <v>1.515152</v>
+        <v>1.515464</v>
       </c>
       <c r="N18" s="28" t="n">
-        <v>0.66</v>
+        <v>0.659864</v>
       </c>
       <c r="O18" s="28" t="n">
         <v>0.577396</v>
@@ -5465,7 +5633,7 @@
         <v>0.05</v>
       </c>
       <c r="Q18" s="28" t="n">
-        <v>-0.082604</v>
+        <v>-0.082468</v>
       </c>
       <c r="R18" s="26" t="n"/>
       <c r="S18" s="29" t="n">
@@ -5486,14 +5654,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W18" s="26" t="n"/>
-      <c r="X18" s="26" t="n"/>
+      <c r="W18" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X18" s="26" t="n">
+        <v>15</v>
+      </c>
       <c r="Y18" s="25" t="n"/>
       <c r="Z18" s="26" t="n"/>
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n"/>
       <c r="AC18" s="30" t="n">
-        <v>0.6439</v>
+        <v>0.6443</v>
       </c>
       <c r="AD18" s="24" t="inlineStr">
         <is>
@@ -5544,10 +5716,10 @@
         <v>-194</v>
       </c>
       <c r="BL18" s="27" t="n">
-        <v>1.515152</v>
+        <v>1.515464</v>
       </c>
       <c r="BM18" s="28" t="n">
-        <v>0.66</v>
+        <v>0.659864</v>
       </c>
       <c r="BN18" s="28" t="n">
         <v>0.656716</v>
@@ -5622,10 +5794,10 @@
         <v>-122</v>
       </c>
       <c r="M19" s="27" t="n">
-        <v>1.818182</v>
+        <v>1.819672</v>
       </c>
       <c r="N19" s="28" t="n">
-        <v>0.55</v>
+        <v>0.54955</v>
       </c>
       <c r="O19" s="28" t="n">
         <v>0.551581</v>
@@ -5634,7 +5806,7 @@
         <v>0.05</v>
       </c>
       <c r="Q19" s="28" t="n">
-        <v>0.001581</v>
+        <v>0.002031</v>
       </c>
       <c r="R19" s="26" t="n"/>
       <c r="S19" s="29" t="n">
@@ -5655,8 +5827,12 @@
           <t>loss</t>
         </is>
       </c>
-      <c r="W19" s="26" t="n"/>
-      <c r="X19" s="26" t="n"/>
+      <c r="W19" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="X19" s="26" t="n">
+        <v>4</v>
+      </c>
       <c r="Y19" s="25" t="n"/>
       <c r="Z19" s="26" t="n"/>
       <c r="AA19" s="28" t="n"/>
@@ -5713,10 +5889,10 @@
         <v>-122</v>
       </c>
       <c r="BL19" s="27" t="n">
-        <v>1.818182</v>
+        <v>1.819672</v>
       </c>
       <c r="BM19" s="28" t="n">
-        <v>0.55</v>
+        <v>0.54955</v>
       </c>
       <c r="BN19" s="28" t="n">
         <v>0.547264</v>
@@ -5791,10 +5967,10 @@
         <v>-113</v>
       </c>
       <c r="M20" s="27" t="n">
-        <v>1.886792</v>
+        <v>1.884956</v>
       </c>
       <c r="N20" s="28" t="n">
-        <v>0.53</v>
+        <v>0.530516</v>
       </c>
       <c r="O20" s="28" t="n">
         <v>0.521172</v>
@@ -5803,7 +5979,7 @@
         <v>0.05</v>
       </c>
       <c r="Q20" s="28" t="n">
-        <v>-0.008828000000000001</v>
+        <v>-0.009344</v>
       </c>
       <c r="R20" s="26" t="n"/>
       <c r="S20" s="29" t="n">
@@ -5824,8 +6000,12 @@
           <t>loss</t>
         </is>
       </c>
-      <c r="W20" s="26" t="n"/>
-      <c r="X20" s="26" t="n"/>
+      <c r="W20" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="X20" s="26" t="n">
+        <v>7</v>
+      </c>
       <c r="Y20" s="25" t="n"/>
       <c r="Z20" s="26" t="n"/>
       <c r="AA20" s="28" t="n"/>
@@ -5882,10 +6062,10 @@
         <v>-113</v>
       </c>
       <c r="BL20" s="27" t="n">
-        <v>1.886792</v>
+        <v>1.884956</v>
       </c>
       <c r="BM20" s="28" t="n">
-        <v>0.53</v>
+        <v>0.530516</v>
       </c>
       <c r="BN20" s="28" t="n">
         <v>0.527363</v>
@@ -5960,10 +6140,10 @@
         <v>-106</v>
       </c>
       <c r="M21" s="27" t="n">
-        <v>1.941748</v>
+        <v>1.943396</v>
       </c>
       <c r="N21" s="28" t="n">
-        <v>0.515</v>
+        <v>0.514563</v>
       </c>
       <c r="O21" s="28" t="n">
         <v>0.524624</v>
@@ -5972,7 +6152,7 @@
         <v>0.05</v>
       </c>
       <c r="Q21" s="28" t="n">
-        <v>0.009624000000000001</v>
+        <v>0.010061</v>
       </c>
       <c r="R21" s="26" t="n"/>
       <c r="S21" s="29" t="n">
@@ -5993,8 +6173,12 @@
           <t>loss</t>
         </is>
       </c>
-      <c r="W21" s="26" t="n"/>
-      <c r="X21" s="26" t="n"/>
+      <c r="W21" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="X21" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y21" s="25" t="n"/>
       <c r="Z21" s="26" t="n"/>
       <c r="AA21" s="28" t="n"/>
@@ -6051,10 +6235,10 @@
         <v>-106</v>
       </c>
       <c r="BL21" s="27" t="n">
-        <v>1.941748</v>
+        <v>1.943396</v>
       </c>
       <c r="BM21" s="28" t="n">
-        <v>0.515</v>
+        <v>0.514563</v>
       </c>
       <c r="BN21" s="28" t="n">
         <v>0.5124379999999999</v>
@@ -6129,10 +6313,10 @@
         <v>-174</v>
       </c>
       <c r="M22" s="27" t="n">
-        <v>1.574803</v>
+        <v>1.574713</v>
       </c>
       <c r="N22" s="28" t="n">
-        <v>0.635</v>
+        <v>0.635036</v>
       </c>
       <c r="O22" s="28" t="n">
         <v>0.597575</v>
@@ -6141,7 +6325,7 @@
         <v>0.05</v>
       </c>
       <c r="Q22" s="28" t="n">
-        <v>-0.037425</v>
+        <v>-0.037461</v>
       </c>
       <c r="R22" s="26" t="n"/>
       <c r="S22" s="29" t="n">
@@ -6162,8 +6346,12 @@
           <t>loss</t>
         </is>
       </c>
-      <c r="W22" s="26" t="n"/>
-      <c r="X22" s="26" t="n"/>
+      <c r="W22" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="X22" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="Y22" s="25" t="n"/>
       <c r="Z22" s="26" t="n"/>
       <c r="AA22" s="28" t="n"/>
@@ -6220,10 +6408,10 @@
         <v>-174</v>
       </c>
       <c r="BL22" s="27" t="n">
-        <v>1.574803</v>
+        <v>1.574713</v>
       </c>
       <c r="BM22" s="28" t="n">
-        <v>0.635</v>
+        <v>0.635036</v>
       </c>
       <c r="BN22" s="28" t="n">
         <v>0.631841</v>
@@ -6298,10 +6486,10 @@
         <v>-376</v>
       </c>
       <c r="M23" s="27" t="n">
-        <v>1.265823</v>
+        <v>1.265957</v>
       </c>
       <c r="N23" s="28" t="n">
-        <v>0.79</v>
+        <v>0.789916</v>
       </c>
       <c r="O23" s="28" t="n">
         <v>0.534506</v>
@@ -6310,7 +6498,7 @@
         <v>0.05</v>
       </c>
       <c r="Q23" s="28" t="n">
-        <v>-0.255494</v>
+        <v>-0.25541</v>
       </c>
       <c r="R23" s="26" t="n"/>
       <c r="S23" s="29" t="n">
@@ -6331,14 +6519,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W23" s="26" t="n"/>
-      <c r="X23" s="26" t="n"/>
+      <c r="W23" s="26" t="n">
+        <v>111</v>
+      </c>
+      <c r="X23" s="26" t="n">
+        <v>92</v>
+      </c>
       <c r="Y23" s="25" t="n"/>
       <c r="Z23" s="26" t="n"/>
       <c r="AA23" s="28" t="n"/>
       <c r="AB23" s="28" t="n"/>
       <c r="AC23" s="30" t="n">
-        <v>0.1994</v>
+        <v>0.1995</v>
       </c>
       <c r="AD23" s="24" t="inlineStr">
         <is>
@@ -6389,10 +6581,10 @@
         <v>-376</v>
       </c>
       <c r="BL23" s="27" t="n">
-        <v>1.265823</v>
+        <v>1.265957</v>
       </c>
       <c r="BM23" s="28" t="n">
-        <v>0.79</v>
+        <v>0.789916</v>
       </c>
       <c r="BN23" s="28" t="n">
         <v>0.782178</v>
@@ -6467,10 +6659,10 @@
         <v>-113</v>
       </c>
       <c r="M24" s="27" t="n">
-        <v>1.886792</v>
+        <v>1.884956</v>
       </c>
       <c r="N24" s="28" t="n">
-        <v>0.53</v>
+        <v>0.530516</v>
       </c>
       <c r="O24" s="28" t="n">
         <v>0.505358</v>
@@ -6479,7 +6671,7 @@
         <v>0.05</v>
       </c>
       <c r="Q24" s="28" t="n">
-        <v>-0.024642</v>
+        <v>-0.025158</v>
       </c>
       <c r="R24" s="26" t="n"/>
       <c r="S24" s="29" t="n">
@@ -6500,14 +6692,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W24" s="26" t="n"/>
-      <c r="X24" s="26" t="n"/>
+      <c r="W24" s="26" t="n">
+        <v>82</v>
+      </c>
+      <c r="X24" s="26" t="n">
+        <v>96</v>
+      </c>
       <c r="Y24" s="25" t="n"/>
       <c r="Z24" s="26" t="n"/>
       <c r="AA24" s="28" t="n"/>
       <c r="AB24" s="28" t="n"/>
       <c r="AC24" s="30" t="n">
-        <v>0.4434</v>
+        <v>0.4425</v>
       </c>
       <c r="AD24" s="24" t="inlineStr">
         <is>
@@ -6558,10 +6754,10 @@
         <v>-113</v>
       </c>
       <c r="BL24" s="27" t="n">
-        <v>1.886792</v>
+        <v>1.884956</v>
       </c>
       <c r="BM24" s="28" t="n">
-        <v>0.53</v>
+        <v>0.530516</v>
       </c>
       <c r="BN24" s="28" t="n">
         <v>0.524752</v>
@@ -6636,10 +6832,10 @@
         <v>-178</v>
       </c>
       <c r="M25" s="27" t="n">
-        <v>1.5625</v>
+        <v>1.561798</v>
       </c>
       <c r="N25" s="28" t="n">
-        <v>0.64</v>
+        <v>0.640288</v>
       </c>
       <c r="O25" s="28" t="n">
         <v>0.637935</v>
@@ -6648,7 +6844,7 @@
         <v>0.05</v>
       </c>
       <c r="Q25" s="28" t="n">
-        <v>-0.002065</v>
+        <v>-0.002353</v>
       </c>
       <c r="R25" s="26" t="n"/>
       <c r="S25" s="29" t="n">
@@ -6669,8 +6865,12 @@
           <t>loss</t>
         </is>
       </c>
-      <c r="W25" s="26" t="n"/>
-      <c r="X25" s="26" t="n"/>
+      <c r="W25" s="26" t="n">
+        <v>96</v>
+      </c>
+      <c r="X25" s="26" t="n">
+        <v>83</v>
+      </c>
       <c r="Y25" s="25" t="n"/>
       <c r="Z25" s="26" t="n"/>
       <c r="AA25" s="28" t="n"/>
@@ -6727,10 +6927,10 @@
         <v>-178</v>
       </c>
       <c r="BL25" s="27" t="n">
-        <v>1.5625</v>
+        <v>1.561798</v>
       </c>
       <c r="BM25" s="28" t="n">
-        <v>0.64</v>
+        <v>0.640288</v>
       </c>
       <c r="BN25" s="28" t="n">
         <v>0.633663</v>
@@ -6805,10 +7005,10 @@
         <v>-163</v>
       </c>
       <c r="M26" s="27" t="n">
-        <v>1.612903</v>
+        <v>1.613497</v>
       </c>
       <c r="N26" s="28" t="n">
-        <v>0.62</v>
+        <v>0.619772</v>
       </c>
       <c r="O26" s="28" t="n">
         <v>0.611768</v>
@@ -6817,7 +7017,7 @@
         <v>0.05</v>
       </c>
       <c r="Q26" s="28" t="n">
-        <v>-0.008232</v>
+        <v>-0.008004000000000001</v>
       </c>
       <c r="R26" s="26" t="n"/>
       <c r="S26" s="29" t="n">
@@ -6838,14 +7038,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W26" s="26" t="n"/>
-      <c r="X26" s="26" t="n"/>
+      <c r="W26" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X26" s="26" t="n">
+        <v>6</v>
+      </c>
       <c r="Y26" s="25" t="n"/>
       <c r="Z26" s="26" t="n"/>
       <c r="AA26" s="28" t="n"/>
       <c r="AB26" s="28" t="n"/>
       <c r="AC26" s="30" t="n">
-        <v>0.9194</v>
+        <v>0.9202</v>
       </c>
       <c r="AD26" s="24" t="inlineStr">
         <is>
@@ -6896,10 +7100,10 @@
         <v>-163</v>
       </c>
       <c r="BL26" s="27" t="n">
-        <v>1.612903</v>
+        <v>1.613497</v>
       </c>
       <c r="BM26" s="28" t="n">
-        <v>0.62</v>
+        <v>0.619772</v>
       </c>
       <c r="BN26" s="28" t="n">
         <v>0.616915</v>
@@ -6974,10 +7178,10 @@
         <v>-111</v>
       </c>
       <c r="M27" s="27" t="n">
-        <v>1.904762</v>
+        <v>1.900901</v>
       </c>
       <c r="N27" s="28" t="n">
-        <v>0.525</v>
+        <v>0.526066</v>
       </c>
       <c r="O27" s="28" t="n">
         <v>0.525388</v>
@@ -6986,7 +7190,7 @@
         <v>0.05</v>
       </c>
       <c r="Q27" s="28" t="n">
-        <v>0.000388</v>
+        <v>-0.000678</v>
       </c>
       <c r="R27" s="26" t="n"/>
       <c r="S27" s="29" t="n">
@@ -7007,14 +7211,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W27" s="26" t="n"/>
-      <c r="X27" s="26" t="n"/>
+      <c r="W27" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="X27" s="26" t="n">
+        <v>5</v>
+      </c>
       <c r="Y27" s="25" t="n"/>
       <c r="Z27" s="26" t="n"/>
       <c r="AA27" s="28" t="n"/>
       <c r="AB27" s="28" t="n"/>
       <c r="AC27" s="30" t="n">
-        <v>0.6786</v>
+        <v>0.6757</v>
       </c>
       <c r="AD27" s="24" t="inlineStr">
         <is>
@@ -7065,10 +7273,10 @@
         <v>-111</v>
       </c>
       <c r="BL27" s="27" t="n">
-        <v>1.904762</v>
+        <v>1.900901</v>
       </c>
       <c r="BM27" s="28" t="n">
-        <v>0.525</v>
+        <v>0.526066</v>
       </c>
       <c r="BN27" s="28" t="n">
         <v>0.522388</v>
@@ -7143,10 +7351,10 @@
         <v>-138</v>
       </c>
       <c r="M28" s="27" t="n">
-        <v>1.724138</v>
+        <v>1.724638</v>
       </c>
       <c r="N28" s="28" t="n">
-        <v>0.58</v>
+        <v>0.579832</v>
       </c>
       <c r="O28" s="28" t="n">
         <v>0.597575</v>
@@ -7155,7 +7363,7 @@
         <v>0.05</v>
       </c>
       <c r="Q28" s="28" t="n">
-        <v>0.017575</v>
+        <v>0.017743</v>
       </c>
       <c r="R28" s="26" t="n"/>
       <c r="S28" s="29" t="n">
@@ -7176,14 +7384,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W28" s="26" t="n"/>
-      <c r="X28" s="26" t="n"/>
+      <c r="W28" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="X28" s="26" t="n">
+        <v>4</v>
+      </c>
       <c r="Y28" s="25" t="n"/>
       <c r="Z28" s="26" t="n"/>
       <c r="AA28" s="28" t="n"/>
       <c r="AB28" s="28" t="n"/>
       <c r="AC28" s="30" t="n">
-        <v>1.0862</v>
+        <v>1.087</v>
       </c>
       <c r="AD28" s="24" t="inlineStr">
         <is>
@@ -7234,10 +7446,10 @@
         <v>-138</v>
       </c>
       <c r="BL28" s="27" t="n">
-        <v>1.724138</v>
+        <v>1.724638</v>
       </c>
       <c r="BM28" s="28" t="n">
-        <v>0.58</v>
+        <v>0.579832</v>
       </c>
       <c r="BN28" s="28" t="n">
         <v>0.577114</v>
@@ -7312,10 +7524,10 @@
         <v>-178</v>
       </c>
       <c r="M29" s="27" t="n">
-        <v>1.5625</v>
+        <v>1.561798</v>
       </c>
       <c r="N29" s="28" t="n">
-        <v>0.64</v>
+        <v>0.640288</v>
       </c>
       <c r="O29" s="28" t="n">
         <v>0.550233</v>
@@ -7324,7 +7536,7 @@
         <v>0.05</v>
       </c>
       <c r="Q29" s="28" t="n">
-        <v>-0.089767</v>
+        <v>-0.090055</v>
       </c>
       <c r="R29" s="26" t="n"/>
       <c r="S29" s="29" t="n">
@@ -7345,14 +7557,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W29" s="26" t="n"/>
-      <c r="X29" s="26" t="n"/>
+      <c r="W29" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="X29" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="Y29" s="25" t="n"/>
       <c r="Z29" s="26" t="n"/>
       <c r="AA29" s="28" t="n"/>
       <c r="AB29" s="28" t="n"/>
       <c r="AC29" s="30" t="n">
-        <v>0.5625</v>
+        <v>0.5618</v>
       </c>
       <c r="AD29" s="24" t="inlineStr">
         <is>
@@ -7403,10 +7619,10 @@
         <v>-178</v>
       </c>
       <c r="BL29" s="27" t="n">
-        <v>1.5625</v>
+        <v>1.561798</v>
       </c>
       <c r="BM29" s="28" t="n">
-        <v>0.64</v>
+        <v>0.640288</v>
       </c>
       <c r="BN29" s="28" t="n">
         <v>0.636816</v>
@@ -7481,10 +7697,10 @@
         <v>-669</v>
       </c>
       <c r="M30" s="27" t="n">
-        <v>1.149425</v>
+        <v>1.149477</v>
       </c>
       <c r="N30" s="28" t="n">
-        <v>0.87</v>
+        <v>0.869961</v>
       </c>
       <c r="O30" s="28" t="n">
         <v>0.741703</v>
@@ -7493,7 +7709,7 @@
         <v>0.05</v>
       </c>
       <c r="Q30" s="28" t="n">
-        <v>-0.128297</v>
+        <v>-0.128258</v>
       </c>
       <c r="R30" s="26" t="n"/>
       <c r="S30" s="29" t="n">
@@ -7514,14 +7730,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W30" s="26" t="n"/>
-      <c r="X30" s="26" t="n"/>
+      <c r="W30" s="26" t="n">
+        <v>93</v>
+      </c>
+      <c r="X30" s="26" t="n">
+        <v>101</v>
+      </c>
       <c r="Y30" s="25" t="n"/>
       <c r="Z30" s="26" t="n"/>
       <c r="AA30" s="28" t="n"/>
       <c r="AB30" s="28" t="n"/>
       <c r="AC30" s="30" t="n">
-        <v>0.2989</v>
+        <v>0.299</v>
       </c>
       <c r="AD30" s="24" t="inlineStr">
         <is>
@@ -7572,10 +7792,10 @@
         <v>-669</v>
       </c>
       <c r="BL30" s="27" t="n">
-        <v>1.149425</v>
+        <v>1.149477</v>
       </c>
       <c r="BM30" s="28" t="n">
-        <v>0.87</v>
+        <v>0.869961</v>
       </c>
       <c r="BN30" s="28" t="n">
         <v>0.861386</v>
@@ -7650,10 +7870,10 @@
         <v>-355</v>
       </c>
       <c r="M31" s="27" t="n">
-        <v>1.282051</v>
+        <v>1.28169</v>
       </c>
       <c r="N31" s="28" t="n">
-        <v>0.78</v>
+        <v>0.78022</v>
       </c>
       <c r="O31" s="28" t="n">
         <v>0.743891</v>
@@ -7662,7 +7882,7 @@
         <v>0.05</v>
       </c>
       <c r="Q31" s="28" t="n">
-        <v>-0.036109</v>
+        <v>-0.036329</v>
       </c>
       <c r="R31" s="26" t="n"/>
       <c r="S31" s="29" t="n">
@@ -7683,14 +7903,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W31" s="26" t="n"/>
-      <c r="X31" s="26" t="n"/>
+      <c r="W31" s="26" t="n">
+        <v>69</v>
+      </c>
+      <c r="X31" s="26" t="n">
+        <v>74</v>
+      </c>
       <c r="Y31" s="25" t="n"/>
       <c r="Z31" s="26" t="n"/>
       <c r="AA31" s="28" t="n"/>
       <c r="AB31" s="28" t="n"/>
       <c r="AC31" s="30" t="n">
-        <v>0.5641</v>
+        <v>0.5634</v>
       </c>
       <c r="AD31" s="24" t="inlineStr">
         <is>
@@ -7741,10 +7965,10 @@
         <v>-355</v>
       </c>
       <c r="BL31" s="27" t="n">
-        <v>1.282051</v>
+        <v>1.28169</v>
       </c>
       <c r="BM31" s="28" t="n">
-        <v>0.78</v>
+        <v>0.78022</v>
       </c>
       <c r="BN31" s="28" t="n">
         <v>0.772277</v>
@@ -10844,10 +11068,10 @@
         <v>-106</v>
       </c>
       <c r="M43" s="27" t="n">
-        <v>1.941748</v>
+        <v>1.943396</v>
       </c>
       <c r="N43" s="28" t="n">
-        <v>0.515</v>
+        <v>0.514563</v>
       </c>
       <c r="O43" s="28" t="n">
         <v>0.550333</v>
@@ -10856,7 +11080,7 @@
         <v>0.05</v>
       </c>
       <c r="Q43" s="28" t="n">
-        <v>0.035333</v>
+        <v>0.03577</v>
       </c>
       <c r="R43" s="26" t="n"/>
       <c r="S43" s="29" t="n">
@@ -10877,14 +11101,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W43" s="26" t="n"/>
-      <c r="X43" s="26" t="n"/>
+      <c r="W43" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X43" s="26" t="n">
+        <v>10</v>
+      </c>
       <c r="Y43" s="25" t="n"/>
       <c r="Z43" s="26" t="n"/>
       <c r="AA43" s="28" t="n"/>
       <c r="AB43" s="28" t="n"/>
       <c r="AC43" s="30" t="n">
-        <v>0.9417</v>
+        <v>0.9434</v>
       </c>
       <c r="AD43" s="24" t="inlineStr">
         <is>
@@ -10935,10 +11163,10 @@
         <v>-106</v>
       </c>
       <c r="BL43" s="27" t="n">
-        <v>1.941748</v>
+        <v>1.943396</v>
       </c>
       <c r="BM43" s="28" t="n">
-        <v>0.515</v>
+        <v>0.514563</v>
       </c>
       <c r="BN43" s="28" t="n">
         <v>0.5124379999999999</v>
@@ -11013,10 +11241,10 @@
         <v>-141</v>
       </c>
       <c r="M44" s="27" t="n">
-        <v>1.709402</v>
+        <v>1.70922</v>
       </c>
       <c r="N44" s="28" t="n">
-        <v>0.585</v>
+        <v>0.585062</v>
       </c>
       <c r="O44" s="28" t="n">
         <v>0.616198</v>
@@ -11025,7 +11253,7 @@
         <v>0.05</v>
       </c>
       <c r="Q44" s="28" t="n">
-        <v>0.031198</v>
+        <v>0.031136</v>
       </c>
       <c r="R44" s="26" t="n"/>
       <c r="S44" s="29" t="n">
@@ -11046,14 +11274,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W44" s="26" t="n"/>
-      <c r="X44" s="26" t="n"/>
+      <c r="W44" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X44" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y44" s="25" t="n"/>
       <c r="Z44" s="26" t="n"/>
       <c r="AA44" s="28" t="n"/>
       <c r="AB44" s="28" t="n"/>
       <c r="AC44" s="30" t="n">
-        <v>1.2415</v>
+        <v>1.2411</v>
       </c>
       <c r="AD44" s="24" t="inlineStr">
         <is>
@@ -11104,10 +11336,10 @@
         <v>-141</v>
       </c>
       <c r="BL44" s="27" t="n">
-        <v>1.709402</v>
+        <v>1.70922</v>
       </c>
       <c r="BM44" s="28" t="n">
-        <v>0.585</v>
+        <v>0.585062</v>
       </c>
       <c r="BN44" s="28" t="n">
         <v>0.58209</v>
@@ -11182,10 +11414,10 @@
         <v>-133</v>
       </c>
       <c r="M45" s="27" t="n">
-        <v>1.754386</v>
+        <v>1.75188</v>
       </c>
       <c r="N45" s="28" t="n">
-        <v>0.57</v>
+        <v>0.570815</v>
       </c>
       <c r="O45" s="28" t="n">
         <v>0.60271</v>
@@ -11194,7 +11426,7 @@
         <v>0.05</v>
       </c>
       <c r="Q45" s="28" t="n">
-        <v>0.03271</v>
+        <v>0.031895</v>
       </c>
       <c r="R45" s="26" t="n"/>
       <c r="S45" s="29" t="n">
@@ -11215,8 +11447,12 @@
           <t>loss</t>
         </is>
       </c>
-      <c r="W45" s="26" t="n"/>
-      <c r="X45" s="26" t="n"/>
+      <c r="W45" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="X45" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y45" s="25" t="n"/>
       <c r="Z45" s="26" t="n"/>
       <c r="AA45" s="28" t="n"/>
@@ -11273,10 +11509,10 @@
         <v>-133</v>
       </c>
       <c r="BL45" s="27" t="n">
-        <v>1.754386</v>
+        <v>1.75188</v>
       </c>
       <c r="BM45" s="28" t="n">
-        <v>0.57</v>
+        <v>0.570815</v>
       </c>
       <c r="BN45" s="28" t="n">
         <v>0.567164</v>
@@ -11351,10 +11587,10 @@
         <v>104</v>
       </c>
       <c r="M46" s="27" t="n">
-        <v>2.040816</v>
+        <v>2.04</v>
       </c>
       <c r="N46" s="28" t="n">
-        <v>0.49</v>
+        <v>0.490196</v>
       </c>
       <c r="O46" s="28" t="n">
         <v>0.582862</v>
@@ -11363,7 +11599,7 @@
         <v>0.05</v>
       </c>
       <c r="Q46" s="28" t="n">
-        <v>0.092862</v>
+        <v>0.092666</v>
       </c>
       <c r="R46" s="26" t="n"/>
       <c r="S46" s="29" t="n">
@@ -11384,14 +11620,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W46" s="26" t="n"/>
-      <c r="X46" s="26" t="n"/>
+      <c r="W46" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="X46" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y46" s="25" t="n"/>
       <c r="Z46" s="26" t="n"/>
       <c r="AA46" s="28" t="n"/>
       <c r="AB46" s="28" t="n"/>
       <c r="AC46" s="30" t="n">
-        <v>1.301</v>
+        <v>1.3</v>
       </c>
       <c r="AD46" s="24" t="inlineStr">
         <is>
@@ -11442,10 +11682,10 @@
         <v>104</v>
       </c>
       <c r="BL46" s="27" t="n">
-        <v>2.040816</v>
+        <v>2.04</v>
       </c>
       <c r="BM46" s="28" t="n">
-        <v>0.49</v>
+        <v>0.490196</v>
       </c>
       <c r="BN46" s="28" t="n">
         <v>0.487562</v>
@@ -11520,10 +11760,10 @@
         <v>-104</v>
       </c>
       <c r="M47" s="27" t="n">
-        <v>1.960784</v>
+        <v>1.961538</v>
       </c>
       <c r="N47" s="28" t="n">
-        <v>0.51</v>
+        <v>0.509804</v>
       </c>
       <c r="O47" s="28" t="n">
         <v>0.550233</v>
@@ -11532,7 +11772,7 @@
         <v>0.05</v>
       </c>
       <c r="Q47" s="28" t="n">
-        <v>0.040233</v>
+        <v>0.040429</v>
       </c>
       <c r="R47" s="26" t="n"/>
       <c r="S47" s="29" t="n">
@@ -11553,14 +11793,18 @@
           <t>win</t>
         </is>
       </c>
-      <c r="W47" s="26" t="n"/>
-      <c r="X47" s="26" t="n"/>
+      <c r="W47" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="X47" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y47" s="25" t="n"/>
       <c r="Z47" s="26" t="n"/>
       <c r="AA47" s="28" t="n"/>
       <c r="AB47" s="28" t="n"/>
       <c r="AC47" s="30" t="n">
-        <v>0.9608</v>
+        <v>0.9615</v>
       </c>
       <c r="AD47" s="24" t="inlineStr">
         <is>
@@ -11611,10 +11855,10 @@
         <v>-104</v>
       </c>
       <c r="BL47" s="27" t="n">
-        <v>1.960784</v>
+        <v>1.961538</v>
       </c>
       <c r="BM47" s="28" t="n">
-        <v>0.51</v>
+        <v>0.509804</v>
       </c>
       <c r="BN47" s="28" t="n">
         <v>0.507463</v>
@@ -11689,10 +11933,10 @@
         <v>120</v>
       </c>
       <c r="M48" s="27" t="n">
-        <v>2.197802</v>
+        <v>2.2</v>
       </c>
       <c r="N48" s="28" t="n">
-        <v>0.455</v>
+        <v>0.454545</v>
       </c>
       <c r="O48" s="28" t="n">
         <v>0.530299</v>
@@ -11701,7 +11945,7 @@
         <v>0.05</v>
       </c>
       <c r="Q48" s="28" t="n">
-        <v>0.075299</v>
+        <v>0.075754</v>
       </c>
       <c r="R48" s="26" t="n"/>
       <c r="S48" s="29" t="n">
@@ -11722,8 +11966,12 @@
           <t>loss</t>
         </is>
       </c>
-      <c r="W48" s="26" t="n"/>
-      <c r="X48" s="26" t="n"/>
+      <c r="W48" s="26" t="n">
+        <v>23</v>
+      </c>
+      <c r="X48" s="26" t="n">
+        <v>4</v>
+      </c>
       <c r="Y48" s="25" t="n"/>
       <c r="Z48" s="26" t="n"/>
       <c r="AA48" s="28" t="n"/>
@@ -11780,10 +12028,10 @@
         <v>120</v>
       </c>
       <c r="BL48" s="27" t="n">
-        <v>2.197802</v>
+        <v>2.2</v>
       </c>
       <c r="BM48" s="28" t="n">
-        <v>0.455</v>
+        <v>0.454545</v>
       </c>
       <c r="BN48" s="28" t="n">
         <v>0.452736</v>
@@ -11891,8 +12139,12 @@
           <t>loss</t>
         </is>
       </c>
-      <c r="W49" s="26" t="n"/>
-      <c r="X49" s="26" t="n"/>
+      <c r="W49" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="X49" s="26" t="n">
+        <v>4</v>
+      </c>
       <c r="Y49" s="25" t="n"/>
       <c r="Z49" s="26" t="n"/>
       <c r="AA49" s="28" t="n"/>
@@ -12052,18 +12304,32 @@
       </c>
       <c r="U50" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V50" s="24" t="n"/>
-      <c r="W50" s="26" t="n"/>
-      <c r="X50" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V50" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W50" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="X50" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="Y50" s="25" t="n"/>
       <c r="Z50" s="26" t="n"/>
       <c r="AA50" s="28" t="n"/>
       <c r="AB50" s="28" t="n"/>
-      <c r="AC50" s="30" t="n"/>
-      <c r="AD50" s="24" t="n"/>
+      <c r="AC50" s="30" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="AD50" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:46.455580Z</t>
+        </is>
+      </c>
       <c r="AE50" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.4800 (aec-mlb-tex-atl-2026-07-19).</t>
@@ -12301,18 +12567,32 @@
       </c>
       <c r="U51" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V51" s="24" t="n"/>
-      <c r="W51" s="26" t="n"/>
-      <c r="X51" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V51" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W51" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="X51" s="26" t="n">
+        <v>6</v>
+      </c>
       <c r="Y51" s="25" t="n"/>
       <c r="Z51" s="26" t="n"/>
       <c r="AA51" s="28" t="n"/>
       <c r="AB51" s="28" t="n"/>
-      <c r="AC51" s="30" t="n"/>
-      <c r="AD51" s="24" t="n"/>
+      <c r="AC51" s="30" t="n">
+        <v>1.1278</v>
+      </c>
+      <c r="AD51" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:46.701705Z</t>
+        </is>
+      </c>
       <c r="AE51" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.5700 (aec-mlb-cin-col-2026-07-19).</t>
@@ -12550,18 +12830,32 @@
       </c>
       <c r="U52" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V52" s="24" t="n"/>
-      <c r="W52" s="26" t="n"/>
-      <c r="X52" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V52" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W52" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="X52" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y52" s="25" t="n"/>
       <c r="Z52" s="26" t="n"/>
       <c r="AA52" s="28" t="n"/>
       <c r="AB52" s="28" t="n"/>
-      <c r="AC52" s="30" t="n"/>
-      <c r="AD52" s="24" t="n"/>
+      <c r="AC52" s="30" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD52" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:12:46.998281Z</t>
+        </is>
+      </c>
       <c r="AE52" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5150; executable ask 0.4350 (aec-mlb-wsh-ath-2026-07-19).</t>
@@ -12574,7 +12868,7 @@
       </c>
       <c r="AG52" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH52" s="24" t="n"/>

</xml_diff>

<commit_message>
data: update ledgers with V4 model, remove duplicate open picks
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -327,8 +327,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA81" headerRowCount="1">
-  <autoFilter ref="A1:CA81"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA90" headerRowCount="1">
+  <autoFilter ref="A1:CA90"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -765,19 +765,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$81)</f>
+        <f>COUNTA('Picks'!$A$2:$A$90)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$81,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$90,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$81,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$90,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$81,"settled",'Picks'!$V$2:$V$81,"win")+COUNTIFS('Picks'!$U$2:$U$81,"settled",'Picks'!$V$2:$V$81,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$90,"settled",'Picks'!$V$2:$V$90,"win")+COUNTIFS('Picks'!$U$2:$U$90,"settled",'Picks'!$V$2:$V$90,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -806,19 +806,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$81,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$90,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$81,"&gt;0",'Picks'!$V$2:$V$81,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$81,"&gt;0",'Picks'!$V$2:$V$81,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$90,"&gt;0",'Picks'!$V$2:$V$90,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$90,"&gt;0",'Picks'!$V$2:$V$90,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="32">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$81,"&gt;0",'Picks'!$V$2:$V$81,"win")/(COUNTIFS('Picks'!$BX$2:$BX$81,"&gt;0",'Picks'!$V$2:$V$81,"win")+COUNTIFS('Picks'!$BX$2:$BX$81,"&gt;0",'Picks'!$V$2:$V$81,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$90,"&gt;0",'Picks'!$V$2:$V$90,"win")/(COUNTIFS('Picks'!$BX$2:$BX$90,"&gt;0",'Picks'!$V$2:$V$90,"win")+COUNTIFS('Picks'!$BX$2:$BX$90,"&gt;0",'Picks'!$V$2:$V$90,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="32">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$81)/SUM('Picks'!$BX$2:$BX$81),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$90)/SUM('Picks'!$BX$2:$BX$90),0)</f>
         <v/>
       </c>
     </row>
@@ -847,19 +847,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="33">
-        <f>SUM('Picks'!$BY$2:$BY$81)</f>
+        <f>SUM('Picks'!$BY$2:$BY$90)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$81,"&lt;&gt;",'Picks'!$AB$2:$AB$81),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$90,"&lt;&gt;",'Picks'!$AB$2:$AB$90),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$81,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$81,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$90,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$90,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="33">
-        <f>SUMIFS('Picks'!$AC$2:$AC$81,'Picks'!$AM$2:$AM$81,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$90,'Picks'!$AM$2:$AM$90,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -915,15 +915,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$81,$A14,'Picks'!$U$2:$U$81,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$90,$A14,'Picks'!$U$2:$U$90,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$81,$A14,'Picks'!$U$2:$U$81,"settled",'Picks'!$V$2:$V$81,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$90,$A14,'Picks'!$U$2:$U$90,"settled",'Picks'!$V$2:$V$90,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$81,$A14,'Picks'!$U$2:$U$81,"settled",'Picks'!$V$2:$V$81,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$90,$A14,'Picks'!$U$2:$U$90,"settled",'Picks'!$V$2:$V$90,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="34">
@@ -931,11 +931,11 @@
         <v/>
       </c>
       <c r="F14" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$81,'Picks'!$H$2:$H$81,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$90,'Picks'!$H$2:$H$90,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$81,'Picks'!$H$2:$H$81,$A14,'Picks'!$U$2:$U$81,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$90,'Picks'!$H$2:$H$90,$A14,'Picks'!$U$2:$U$90,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -946,15 +946,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$81,$A15,'Picks'!$U$2:$U$81,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$90,$A15,'Picks'!$U$2:$U$90,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$81,$A15,'Picks'!$U$2:$U$81,"settled",'Picks'!$V$2:$V$81,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$90,$A15,'Picks'!$U$2:$U$90,"settled",'Picks'!$V$2:$V$90,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$81,$A15,'Picks'!$U$2:$U$81,"settled",'Picks'!$V$2:$V$81,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$90,$A15,'Picks'!$U$2:$U$90,"settled",'Picks'!$V$2:$V$90,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="36">
@@ -962,11 +962,11 @@
         <v/>
       </c>
       <c r="F15" s="37">
-        <f>SUMIFS('Picks'!$BY$2:$BY$81,'Picks'!$H$2:$H$81,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$90,'Picks'!$H$2:$H$90,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$81,'Picks'!$H$2:$H$81,$A15,'Picks'!$U$2:$U$81,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$90,'Picks'!$H$2:$H$90,$A15,'Picks'!$U$2:$U$90,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -977,15 +977,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$81,$A16,'Picks'!$U$2:$U$81,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$90,$A16,'Picks'!$U$2:$U$90,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$81,$A16,'Picks'!$U$2:$U$81,"settled",'Picks'!$V$2:$V$81,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$90,$A16,'Picks'!$U$2:$U$90,"settled",'Picks'!$V$2:$V$90,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$81,$A16,'Picks'!$U$2:$U$81,"settled",'Picks'!$V$2:$V$81,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$90,$A16,'Picks'!$U$2:$U$90,"settled",'Picks'!$V$2:$V$90,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="34">
@@ -993,11 +993,11 @@
         <v/>
       </c>
       <c r="F16" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$81,'Picks'!$H$2:$H$81,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$90,'Picks'!$H$2:$H$90,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$81,'Picks'!$H$2:$H$81,$A16,'Picks'!$U$2:$U$81,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$90,'Picks'!$H$2:$H$90,$A16,'Picks'!$U$2:$U$90,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA81"/>
+  <dimension ref="A1:CA90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20474,6 +20474,2247 @@
       <c r="BZ81" s="24" t="n"/>
       <c r="CA81" s="31" t="n"/>
     </row>
+    <row r="82" ht="36" customHeight="1">
+      <c r="A82" s="24" t="inlineStr">
+        <is>
+          <t>aaf1b4b6ac094ac8</t>
+        </is>
+      </c>
+      <c r="B82" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:58:34.322674Z</t>
+        </is>
+      </c>
+      <c r="C82" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T18:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D82" s="24" t="inlineStr">
+        <is>
+          <t>401816188</t>
+        </is>
+      </c>
+      <c r="E82" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F82" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="G82" s="24" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="H82" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I82" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J82" s="38" t="n"/>
+      <c r="K82" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L82" s="26" t="n">
+        <v>111</v>
+      </c>
+      <c r="M82" s="39" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="N82" s="28" t="n">
+        <v>0.473934</v>
+      </c>
+      <c r="O82" s="28" t="n">
+        <v>0.5726869999999999</v>
+      </c>
+      <c r="P82" s="28" t="n"/>
+      <c r="Q82" s="28" t="n">
+        <v>0.09875299999999999</v>
+      </c>
+      <c r="R82" s="26" t="n">
+        <v>99</v>
+      </c>
+      <c r="S82" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T82" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U82" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V82" s="24" t="n"/>
+      <c r="W82" s="26" t="n"/>
+      <c r="X82" s="26" t="n"/>
+      <c r="Y82" s="38" t="n"/>
+      <c r="Z82" s="26" t="n"/>
+      <c r="AA82" s="28" t="n"/>
+      <c r="AB82" s="28" t="n"/>
+      <c r="AC82" s="40" t="n"/>
+      <c r="AD82" s="24" t="n"/>
+      <c r="AE82" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.4750 (aec-mlb-min-cle-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF82" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG82" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH82" s="24" t="n"/>
+      <c r="AI82" s="31" t="n"/>
+      <c r="AJ82" s="31" t="n"/>
+      <c r="AK82" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL82" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM82" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN82" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO82" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP82" s="24" t="inlineStr">
+        <is>
+          <t>mlb-min</t>
+        </is>
+      </c>
+      <c r="AQ82" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AR82" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AS82" s="24" t="inlineStr">
+        <is>
+          <t>mlb-cle</t>
+        </is>
+      </c>
+      <c r="AT82" s="24" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="AU82" s="24" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="AV82" s="24" t="n"/>
+      <c r="AW82" s="24" t="n"/>
+      <c r="AX82" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY82" s="24" t="n"/>
+      <c r="AZ82" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA82" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB82" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC82" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD82" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE82" s="24" t="inlineStr">
+        <is>
+          <t>2170ac399ced5417</t>
+        </is>
+      </c>
+      <c r="BF82" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG82" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH82" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:57:32.219947Z</t>
+        </is>
+      </c>
+      <c r="BI82" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ82" s="38" t="n"/>
+      <c r="BK82" s="26" t="n">
+        <v>111</v>
+      </c>
+      <c r="BL82" s="39" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="BM82" s="28" t="n">
+        <v>0.473934</v>
+      </c>
+      <c r="BN82" s="28" t="n">
+        <v>0.472637</v>
+      </c>
+      <c r="BO82" s="28" t="n"/>
+      <c r="BP82" s="38" t="n"/>
+      <c r="BQ82" s="39" t="n"/>
+      <c r="BR82" s="28" t="n"/>
+      <c r="BS82" s="28" t="n"/>
+      <c r="BT82" s="28" t="n"/>
+      <c r="BU82" s="38" t="n"/>
+      <c r="BV82" s="29" t="n"/>
+      <c r="BW82" s="24" t="n"/>
+      <c r="BX82" s="40" t="n"/>
+      <c r="BY82" s="39" t="n"/>
+      <c r="BZ82" s="24" t="n"/>
+      <c r="CA82" s="31" t="n"/>
+    </row>
+    <row r="83" ht="36" customHeight="1">
+      <c r="A83" s="24" t="inlineStr">
+        <is>
+          <t>14a96af3a7654557</t>
+        </is>
+      </c>
+      <c r="B83" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:58:34.322674Z</t>
+        </is>
+      </c>
+      <c r="C83" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T19:05:00-0400</t>
+        </is>
+      </c>
+      <c r="D83" s="24" t="inlineStr">
+        <is>
+          <t>401816189</t>
+        </is>
+      </c>
+      <c r="E83" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F83" s="24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="G83" s="24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="H83" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I83" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J83" s="38" t="n"/>
+      <c r="K83" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L83" s="26" t="n">
+        <v>-108</v>
+      </c>
+      <c r="M83" s="39" t="n">
+        <v>1.925926</v>
+      </c>
+      <c r="N83" s="28" t="n">
+        <v>0.519231</v>
+      </c>
+      <c r="O83" s="28" t="n">
+        <v>0.578558</v>
+      </c>
+      <c r="P83" s="28" t="n"/>
+      <c r="Q83" s="28" t="n">
+        <v>0.059327</v>
+      </c>
+      <c r="R83" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="S83" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T83" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U83" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V83" s="24" t="n"/>
+      <c r="W83" s="26" t="n"/>
+      <c r="X83" s="26" t="n"/>
+      <c r="Y83" s="38" t="n"/>
+      <c r="Z83" s="26" t="n"/>
+      <c r="AA83" s="28" t="n"/>
+      <c r="AB83" s="28" t="n"/>
+      <c r="AC83" s="40" t="n"/>
+      <c r="AD83" s="24" t="n"/>
+      <c r="AE83" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5200 (aec-mlb-pit-nyy-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF83" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG83" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH83" s="24" t="n"/>
+      <c r="AI83" s="31" t="n"/>
+      <c r="AJ83" s="31" t="n"/>
+      <c r="AK83" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL83" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM83" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN83" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO83" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP83" s="24" t="inlineStr">
+        <is>
+          <t>mlb-pit</t>
+        </is>
+      </c>
+      <c r="AQ83" s="24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="AR83" s="24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="AS83" s="24" t="inlineStr">
+        <is>
+          <t>mlb-nyy</t>
+        </is>
+      </c>
+      <c r="AT83" s="24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="AU83" s="24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="AV83" s="24" t="n"/>
+      <c r="AW83" s="24" t="n"/>
+      <c r="AX83" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY83" s="24" t="n"/>
+      <c r="AZ83" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA83" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB83" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC83" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD83" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE83" s="24" t="inlineStr">
+        <is>
+          <t>38ab7db5a3798f0c</t>
+        </is>
+      </c>
+      <c r="BF83" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG83" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH83" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:57:35.056972Z</t>
+        </is>
+      </c>
+      <c r="BI83" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ83" s="38" t="n"/>
+      <c r="BK83" s="26" t="n">
+        <v>-108</v>
+      </c>
+      <c r="BL83" s="39" t="n">
+        <v>1.925926</v>
+      </c>
+      <c r="BM83" s="28" t="n">
+        <v>0.519231</v>
+      </c>
+      <c r="BN83" s="28" t="n">
+        <v>0.517413</v>
+      </c>
+      <c r="BO83" s="28" t="n"/>
+      <c r="BP83" s="38" t="n"/>
+      <c r="BQ83" s="39" t="n"/>
+      <c r="BR83" s="28" t="n"/>
+      <c r="BS83" s="28" t="n"/>
+      <c r="BT83" s="28" t="n"/>
+      <c r="BU83" s="38" t="n"/>
+      <c r="BV83" s="29" t="n"/>
+      <c r="BW83" s="24" t="n"/>
+      <c r="BX83" s="40" t="n"/>
+      <c r="BY83" s="39" t="n"/>
+      <c r="BZ83" s="24" t="n"/>
+      <c r="CA83" s="31" t="n"/>
+    </row>
+    <row r="84" ht="36" customHeight="1">
+      <c r="A84" s="24" t="inlineStr">
+        <is>
+          <t>4859b2be84c249d7</t>
+        </is>
+      </c>
+      <c r="B84" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:58:34.322674Z</t>
+        </is>
+      </c>
+      <c r="C84" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T19:10:00-0400</t>
+        </is>
+      </c>
+      <c r="D84" s="24" t="inlineStr">
+        <is>
+          <t>401816186</t>
+        </is>
+      </c>
+      <c r="E84" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F84" s="24" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="G84" s="24" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="H84" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I84" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J84" s="38" t="n"/>
+      <c r="K84" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L84" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="M84" s="39" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="N84" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="O84" s="28" t="n">
+        <v>0.565797</v>
+      </c>
+      <c r="P84" s="28" t="n"/>
+      <c r="Q84" s="28" t="n">
+        <v>-0.014035</v>
+      </c>
+      <c r="R84" s="26" t="n">
+        <v>13</v>
+      </c>
+      <c r="S84" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T84" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U84" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V84" s="24" t="n"/>
+      <c r="W84" s="26" t="n"/>
+      <c r="X84" s="26" t="n"/>
+      <c r="Y84" s="38" t="n"/>
+      <c r="Z84" s="26" t="n"/>
+      <c r="AA84" s="28" t="n"/>
+      <c r="AB84" s="28" t="n"/>
+      <c r="AC84" s="40" t="n"/>
+      <c r="AD84" s="24" t="n"/>
+      <c r="AE84" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5800 (aec-mlb-bal-bos-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF84" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG84" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH84" s="24" t="n"/>
+      <c r="AI84" s="31" t="n"/>
+      <c r="AJ84" s="31" t="n"/>
+      <c r="AK84" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL84" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM84" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN84" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO84" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP84" s="24" t="inlineStr">
+        <is>
+          <t>mlb-bal</t>
+        </is>
+      </c>
+      <c r="AQ84" s="24" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="AR84" s="24" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="AS84" s="24" t="inlineStr">
+        <is>
+          <t>mlb-bos</t>
+        </is>
+      </c>
+      <c r="AT84" s="24" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="AU84" s="24" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="AV84" s="24" t="n"/>
+      <c r="AW84" s="24" t="n"/>
+      <c r="AX84" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY84" s="24" t="n"/>
+      <c r="AZ84" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA84" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB84" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC84" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD84" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE84" s="24" t="inlineStr">
+        <is>
+          <t>9fe2d27778a72dfe</t>
+        </is>
+      </c>
+      <c r="BF84" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG84" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH84" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:57:37.354484Z</t>
+        </is>
+      </c>
+      <c r="BI84" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ84" s="38" t="n"/>
+      <c r="BK84" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="BL84" s="39" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="BM84" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="BN84" s="28" t="n">
+        <v>0.577114</v>
+      </c>
+      <c r="BO84" s="28" t="n"/>
+      <c r="BP84" s="38" t="n"/>
+      <c r="BQ84" s="39" t="n"/>
+      <c r="BR84" s="28" t="n"/>
+      <c r="BS84" s="28" t="n"/>
+      <c r="BT84" s="28" t="n"/>
+      <c r="BU84" s="38" t="n"/>
+      <c r="BV84" s="29" t="n"/>
+      <c r="BW84" s="24" t="n"/>
+      <c r="BX84" s="40" t="n"/>
+      <c r="BY84" s="39" t="n"/>
+      <c r="BZ84" s="24" t="n"/>
+      <c r="CA84" s="31" t="n"/>
+    </row>
+    <row r="85" ht="36" customHeight="1">
+      <c r="A85" s="24" t="inlineStr">
+        <is>
+          <t>41f811ccac474792</t>
+        </is>
+      </c>
+      <c r="B85" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:58:34.322674Z</t>
+        </is>
+      </c>
+      <c r="C85" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T19:15:00-0400</t>
+        </is>
+      </c>
+      <c r="D85" s="24" t="inlineStr">
+        <is>
+          <t>401816190</t>
+        </is>
+      </c>
+      <c r="E85" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F85" s="24" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="G85" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="H85" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I85" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J85" s="38" t="n"/>
+      <c r="K85" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L85" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="M85" s="39" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="N85" s="28" t="n">
+        <v>0.570815</v>
+      </c>
+      <c r="O85" s="28" t="n">
+        <v>0.550915</v>
+      </c>
+      <c r="P85" s="28" t="n"/>
+      <c r="Q85" s="28" t="n">
+        <v>-0.0199</v>
+      </c>
+      <c r="R85" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="S85" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T85" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U85" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V85" s="24" t="n"/>
+      <c r="W85" s="26" t="n"/>
+      <c r="X85" s="26" t="n"/>
+      <c r="Y85" s="38" t="n"/>
+      <c r="Z85" s="26" t="n"/>
+      <c r="AA85" s="28" t="n"/>
+      <c r="AB85" s="28" t="n"/>
+      <c r="AC85" s="40" t="n"/>
+      <c r="AD85" s="24" t="n"/>
+      <c r="AE85" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5700 (aec-mlb-sd-atl-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF85" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG85" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH85" s="24" t="n"/>
+      <c r="AI85" s="31" t="n"/>
+      <c r="AJ85" s="31" t="n"/>
+      <c r="AK85" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL85" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM85" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN85" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO85" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP85" s="24" t="inlineStr">
+        <is>
+          <t>mlb-sd</t>
+        </is>
+      </c>
+      <c r="AQ85" s="24" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="AR85" s="24" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="AS85" s="24" t="inlineStr">
+        <is>
+          <t>mlb-atl</t>
+        </is>
+      </c>
+      <c r="AT85" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="AU85" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="AV85" s="24" t="n"/>
+      <c r="AW85" s="24" t="n"/>
+      <c r="AX85" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY85" s="24" t="n"/>
+      <c r="AZ85" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA85" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB85" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC85" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD85" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE85" s="24" t="inlineStr">
+        <is>
+          <t>f0b5eac7c97d1146</t>
+        </is>
+      </c>
+      <c r="BF85" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG85" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH85" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:57:40.909749Z</t>
+        </is>
+      </c>
+      <c r="BI85" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ85" s="38" t="n"/>
+      <c r="BK85" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="BL85" s="39" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="BM85" s="28" t="n">
+        <v>0.570815</v>
+      </c>
+      <c r="BN85" s="28" t="n">
+        <v>0.567164</v>
+      </c>
+      <c r="BO85" s="28" t="n"/>
+      <c r="BP85" s="38" t="n"/>
+      <c r="BQ85" s="39" t="n"/>
+      <c r="BR85" s="28" t="n"/>
+      <c r="BS85" s="28" t="n"/>
+      <c r="BT85" s="28" t="n"/>
+      <c r="BU85" s="38" t="n"/>
+      <c r="BV85" s="29" t="n"/>
+      <c r="BW85" s="24" t="n"/>
+      <c r="BX85" s="40" t="n"/>
+      <c r="BY85" s="39" t="n"/>
+      <c r="BZ85" s="24" t="n"/>
+      <c r="CA85" s="31" t="n"/>
+    </row>
+    <row r="86" ht="36" customHeight="1">
+      <c r="A86" s="24" t="inlineStr">
+        <is>
+          <t>e68eefc9610e4621</t>
+        </is>
+      </c>
+      <c r="B86" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:58:34.322674Z</t>
+        </is>
+      </c>
+      <c r="C86" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T19:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D86" s="24" t="inlineStr">
+        <is>
+          <t>401816195</t>
+        </is>
+      </c>
+      <c r="E86" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F86" s="24" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="G86" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="H86" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I86" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J86" s="38" t="n"/>
+      <c r="K86" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L86" s="26" t="n">
+        <v>-199</v>
+      </c>
+      <c r="M86" s="39" t="n">
+        <v>1.502513</v>
+      </c>
+      <c r="N86" s="28" t="n">
+        <v>0.665552</v>
+      </c>
+      <c r="O86" s="28" t="n">
+        <v>0.640995</v>
+      </c>
+      <c r="P86" s="28" t="n"/>
+      <c r="Q86" s="28" t="n">
+        <v>-0.024557</v>
+      </c>
+      <c r="R86" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="S86" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T86" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U86" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V86" s="24" t="n"/>
+      <c r="W86" s="26" t="n"/>
+      <c r="X86" s="26" t="n"/>
+      <c r="Y86" s="38" t="n"/>
+      <c r="Z86" s="26" t="n"/>
+      <c r="AA86" s="28" t="n"/>
+      <c r="AB86" s="28" t="n"/>
+      <c r="AC86" s="40" t="n"/>
+      <c r="AD86" s="24" t="n"/>
+      <c r="AE86" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.6650 (aec-mlb-nym-mil-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF86" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG86" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH86" s="24" t="n"/>
+      <c r="AI86" s="31" t="n"/>
+      <c r="AJ86" s="31" t="n"/>
+      <c r="AK86" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL86" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM86" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN86" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO86" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP86" s="24" t="inlineStr">
+        <is>
+          <t>mlb-nym</t>
+        </is>
+      </c>
+      <c r="AQ86" s="24" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="AR86" s="24" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="AS86" s="24" t="inlineStr">
+        <is>
+          <t>mlb-mil</t>
+        </is>
+      </c>
+      <c r="AT86" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="AU86" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="AV86" s="24" t="n"/>
+      <c r="AW86" s="24" t="n"/>
+      <c r="AX86" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY86" s="24" t="n"/>
+      <c r="AZ86" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA86" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB86" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC86" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD86" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE86" s="24" t="inlineStr">
+        <is>
+          <t>6d5f3f5e8f75cb2b</t>
+        </is>
+      </c>
+      <c r="BF86" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG86" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH86" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:57:42.879792Z</t>
+        </is>
+      </c>
+      <c r="BI86" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ86" s="38" t="n"/>
+      <c r="BK86" s="26" t="n">
+        <v>-199</v>
+      </c>
+      <c r="BL86" s="39" t="n">
+        <v>1.502513</v>
+      </c>
+      <c r="BM86" s="28" t="n">
+        <v>0.665552</v>
+      </c>
+      <c r="BN86" s="28" t="n">
+        <v>0.6616919999999999</v>
+      </c>
+      <c r="BO86" s="28" t="n"/>
+      <c r="BP86" s="38" t="n"/>
+      <c r="BQ86" s="39" t="n"/>
+      <c r="BR86" s="28" t="n"/>
+      <c r="BS86" s="28" t="n"/>
+      <c r="BT86" s="28" t="n"/>
+      <c r="BU86" s="38" t="n"/>
+      <c r="BV86" s="29" t="n"/>
+      <c r="BW86" s="24" t="n"/>
+      <c r="BX86" s="40" t="n"/>
+      <c r="BY86" s="39" t="n"/>
+      <c r="BZ86" s="24" t="n"/>
+      <c r="CA86" s="31" t="n"/>
+    </row>
+    <row r="87" ht="36" customHeight="1">
+      <c r="A87" s="24" t="inlineStr">
+        <is>
+          <t>8db3a8d8a90f4145</t>
+        </is>
+      </c>
+      <c r="B87" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:58:34.322674Z</t>
+        </is>
+      </c>
+      <c r="C87" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T20:05:00-0400</t>
+        </is>
+      </c>
+      <c r="D87" s="24" t="inlineStr">
+        <is>
+          <t>401816193</t>
+        </is>
+      </c>
+      <c r="E87" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F87" s="24" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="G87" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="H87" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I87" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J87" s="38" t="n"/>
+      <c r="K87" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L87" s="26" t="n">
+        <v>-108</v>
+      </c>
+      <c r="M87" s="39" t="n">
+        <v>1.925926</v>
+      </c>
+      <c r="N87" s="28" t="n">
+        <v>0.519231</v>
+      </c>
+      <c r="O87" s="28" t="n">
+        <v>0.566967</v>
+      </c>
+      <c r="P87" s="28" t="n"/>
+      <c r="Q87" s="28" t="n">
+        <v>0.047736</v>
+      </c>
+      <c r="R87" s="26" t="n">
+        <v>44</v>
+      </c>
+      <c r="S87" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T87" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U87" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V87" s="24" t="n"/>
+      <c r="W87" s="26" t="n"/>
+      <c r="X87" s="26" t="n"/>
+      <c r="Y87" s="38" t="n"/>
+      <c r="Z87" s="26" t="n"/>
+      <c r="AA87" s="28" t="n"/>
+      <c r="AB87" s="28" t="n"/>
+      <c r="AC87" s="40" t="n"/>
+      <c r="AD87" s="24" t="n"/>
+      <c r="AE87" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5200 (aec-mlb-det-chc-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF87" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG87" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH87" s="24" t="n"/>
+      <c r="AI87" s="31" t="n"/>
+      <c r="AJ87" s="31" t="n"/>
+      <c r="AK87" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL87" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM87" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN87" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO87" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP87" s="24" t="inlineStr">
+        <is>
+          <t>mlb-det</t>
+        </is>
+      </c>
+      <c r="AQ87" s="24" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="AR87" s="24" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="AS87" s="24" t="inlineStr">
+        <is>
+          <t>mlb-chc</t>
+        </is>
+      </c>
+      <c r="AT87" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="AU87" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="AV87" s="24" t="n"/>
+      <c r="AW87" s="24" t="n"/>
+      <c r="AX87" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY87" s="24" t="n"/>
+      <c r="AZ87" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA87" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB87" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC87" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD87" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE87" s="24" t="inlineStr">
+        <is>
+          <t>b84afb2c70e14d93</t>
+        </is>
+      </c>
+      <c r="BF87" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG87" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH87" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:57:46.871986Z</t>
+        </is>
+      </c>
+      <c r="BI87" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ87" s="38" t="n"/>
+      <c r="BK87" s="26" t="n">
+        <v>-108</v>
+      </c>
+      <c r="BL87" s="39" t="n">
+        <v>1.925926</v>
+      </c>
+      <c r="BM87" s="28" t="n">
+        <v>0.519231</v>
+      </c>
+      <c r="BN87" s="28" t="n">
+        <v>0.517413</v>
+      </c>
+      <c r="BO87" s="28" t="n"/>
+      <c r="BP87" s="38" t="n"/>
+      <c r="BQ87" s="39" t="n"/>
+      <c r="BR87" s="28" t="n"/>
+      <c r="BS87" s="28" t="n"/>
+      <c r="BT87" s="28" t="n"/>
+      <c r="BU87" s="38" t="n"/>
+      <c r="BV87" s="29" t="n"/>
+      <c r="BW87" s="24" t="n"/>
+      <c r="BX87" s="40" t="n"/>
+      <c r="BY87" s="39" t="n"/>
+      <c r="BZ87" s="24" t="n"/>
+      <c r="CA87" s="31" t="n"/>
+    </row>
+    <row r="88" ht="36" customHeight="1">
+      <c r="A88" s="24" t="inlineStr">
+        <is>
+          <t>63c8de42843a46c9</t>
+        </is>
+      </c>
+      <c r="B88" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:58:34.322674Z</t>
+        </is>
+      </c>
+      <c r="C88" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T20:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D88" s="24" t="inlineStr">
+        <is>
+          <t>401816197</t>
+        </is>
+      </c>
+      <c r="E88" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F88" s="24" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="G88" s="24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="H88" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I88" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J88" s="38" t="n"/>
+      <c r="K88" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L88" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="M88" s="39" t="n">
+        <v>1.854701</v>
+      </c>
+      <c r="N88" s="28" t="n">
+        <v>0.539171</v>
+      </c>
+      <c r="O88" s="28" t="n">
+        <v>0.5563709999999999</v>
+      </c>
+      <c r="P88" s="28" t="n"/>
+      <c r="Q88" s="28" t="n">
+        <v>0.0172</v>
+      </c>
+      <c r="R88" s="26" t="n">
+        <v>29</v>
+      </c>
+      <c r="S88" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T88" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U88" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V88" s="24" t="n"/>
+      <c r="W88" s="26" t="n"/>
+      <c r="X88" s="26" t="n"/>
+      <c r="Y88" s="38" t="n"/>
+      <c r="Z88" s="26" t="n"/>
+      <c r="AA88" s="28" t="n"/>
+      <c r="AB88" s="28" t="n"/>
+      <c r="AC88" s="40" t="n"/>
+      <c r="AD88" s="24" t="n"/>
+      <c r="AE88" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5400 (aec-mlb-wsh-col-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF88" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG88" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH88" s="24" t="n"/>
+      <c r="AI88" s="31" t="n"/>
+      <c r="AJ88" s="31" t="n"/>
+      <c r="AK88" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL88" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM88" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN88" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO88" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP88" s="24" t="inlineStr">
+        <is>
+          <t>mlb-wsh</t>
+        </is>
+      </c>
+      <c r="AQ88" s="24" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="AR88" s="24" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="AS88" s="24" t="inlineStr">
+        <is>
+          <t>mlb-col</t>
+        </is>
+      </c>
+      <c r="AT88" s="24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="AU88" s="24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="AV88" s="24" t="n"/>
+      <c r="AW88" s="24" t="n"/>
+      <c r="AX88" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY88" s="24" t="n"/>
+      <c r="AZ88" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA88" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB88" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC88" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD88" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE88" s="24" t="inlineStr">
+        <is>
+          <t>a2f336c1cee8c92e</t>
+        </is>
+      </c>
+      <c r="BF88" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG88" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH88" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:57:49.897394Z</t>
+        </is>
+      </c>
+      <c r="BI88" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ88" s="38" t="n"/>
+      <c r="BK88" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="BL88" s="39" t="n">
+        <v>1.854701</v>
+      </c>
+      <c r="BM88" s="28" t="n">
+        <v>0.539171</v>
+      </c>
+      <c r="BN88" s="28" t="n">
+        <v>0.537313</v>
+      </c>
+      <c r="BO88" s="28" t="n"/>
+      <c r="BP88" s="38" t="n"/>
+      <c r="BQ88" s="39" t="n"/>
+      <c r="BR88" s="28" t="n"/>
+      <c r="BS88" s="28" t="n"/>
+      <c r="BT88" s="28" t="n"/>
+      <c r="BU88" s="38" t="n"/>
+      <c r="BV88" s="29" t="n"/>
+      <c r="BW88" s="24" t="n"/>
+      <c r="BX88" s="40" t="n"/>
+      <c r="BY88" s="39" t="n"/>
+      <c r="BZ88" s="24" t="n"/>
+      <c r="CA88" s="31" t="n"/>
+    </row>
+    <row r="89" ht="36" customHeight="1">
+      <c r="A89" s="24" t="inlineStr">
+        <is>
+          <t>21876b0ffe164cd7</t>
+        </is>
+      </c>
+      <c r="B89" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:58:34.322674Z</t>
+        </is>
+      </c>
+      <c r="C89" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T21:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D89" s="24" t="inlineStr">
+        <is>
+          <t>401816198</t>
+        </is>
+      </c>
+      <c r="E89" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F89" s="24" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="G89" s="24" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="H89" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I89" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J89" s="38" t="n"/>
+      <c r="K89" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L89" s="26" t="n">
+        <v>-147</v>
+      </c>
+      <c r="M89" s="39" t="n">
+        <v>1.680272</v>
+      </c>
+      <c r="N89" s="28" t="n">
+        <v>0.5951419999999999</v>
+      </c>
+      <c r="O89" s="28" t="n">
+        <v>0.58189</v>
+      </c>
+      <c r="P89" s="28" t="n"/>
+      <c r="Q89" s="28" t="n">
+        <v>-0.013252</v>
+      </c>
+      <c r="R89" s="26" t="n">
+        <v>13</v>
+      </c>
+      <c r="S89" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T89" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U89" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V89" s="24" t="n"/>
+      <c r="W89" s="26" t="n"/>
+      <c r="X89" s="26" t="n"/>
+      <c r="Y89" s="38" t="n"/>
+      <c r="Z89" s="26" t="n"/>
+      <c r="AA89" s="28" t="n"/>
+      <c r="AB89" s="28" t="n"/>
+      <c r="AC89" s="40" t="n"/>
+      <c r="AD89" s="24" t="n"/>
+      <c r="AE89" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5950 (aec-mlb-ath-az-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF89" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG89" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH89" s="24" t="n"/>
+      <c r="AI89" s="31" t="n"/>
+      <c r="AJ89" s="31" t="n"/>
+      <c r="AK89" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL89" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM89" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN89" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO89" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP89" s="24" t="inlineStr">
+        <is>
+          <t>mlb-ath</t>
+        </is>
+      </c>
+      <c r="AQ89" s="24" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="AR89" s="24" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="AS89" s="24" t="inlineStr">
+        <is>
+          <t>mlb-ari</t>
+        </is>
+      </c>
+      <c r="AT89" s="24" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="AU89" s="24" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="AV89" s="24" t="n"/>
+      <c r="AW89" s="24" t="n"/>
+      <c r="AX89" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY89" s="24" t="n"/>
+      <c r="AZ89" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA89" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB89" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC89" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD89" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE89" s="24" t="inlineStr">
+        <is>
+          <t>7b682aa5da86e2a4</t>
+        </is>
+      </c>
+      <c r="BF89" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG89" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH89" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:57:51.339273Z</t>
+        </is>
+      </c>
+      <c r="BI89" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ89" s="38" t="n"/>
+      <c r="BK89" s="26" t="n">
+        <v>-147</v>
+      </c>
+      <c r="BL89" s="39" t="n">
+        <v>1.680272</v>
+      </c>
+      <c r="BM89" s="28" t="n">
+        <v>0.5951419999999999</v>
+      </c>
+      <c r="BN89" s="28" t="n">
+        <v>0.59204</v>
+      </c>
+      <c r="BO89" s="28" t="n"/>
+      <c r="BP89" s="38" t="n"/>
+      <c r="BQ89" s="39" t="n"/>
+      <c r="BR89" s="28" t="n"/>
+      <c r="BS89" s="28" t="n"/>
+      <c r="BT89" s="28" t="n"/>
+      <c r="BU89" s="38" t="n"/>
+      <c r="BV89" s="29" t="n"/>
+      <c r="BW89" s="24" t="n"/>
+      <c r="BX89" s="40" t="n"/>
+      <c r="BY89" s="39" t="n"/>
+      <c r="BZ89" s="24" t="n"/>
+      <c r="CA89" s="31" t="n"/>
+    </row>
+    <row r="90" ht="36" customHeight="1">
+      <c r="A90" s="24" t="inlineStr">
+        <is>
+          <t>7df4ed647cfb43ef</t>
+        </is>
+      </c>
+      <c r="B90" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:58:34.322674Z</t>
+        </is>
+      </c>
+      <c r="C90" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T21:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D90" s="24" t="inlineStr">
+        <is>
+          <t>401816199</t>
+        </is>
+      </c>
+      <c r="E90" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F90" s="24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="G90" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="H90" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I90" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J90" s="38" t="n"/>
+      <c r="K90" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L90" s="26" t="n">
+        <v>-141</v>
+      </c>
+      <c r="M90" s="39" t="n">
+        <v>1.70922</v>
+      </c>
+      <c r="N90" s="28" t="n">
+        <v>0.585062</v>
+      </c>
+      <c r="O90" s="28" t="n">
+        <v>0.592852</v>
+      </c>
+      <c r="P90" s="28" t="n"/>
+      <c r="Q90" s="28" t="n">
+        <v>0.00779</v>
+      </c>
+      <c r="R90" s="26" t="n">
+        <v>24</v>
+      </c>
+      <c r="S90" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T90" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U90" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V90" s="24" t="n"/>
+      <c r="W90" s="26" t="n"/>
+      <c r="X90" s="26" t="n"/>
+      <c r="Y90" s="38" t="n"/>
+      <c r="Z90" s="26" t="n"/>
+      <c r="AA90" s="28" t="n"/>
+      <c r="AB90" s="28" t="n"/>
+      <c r="AC90" s="40" t="n"/>
+      <c r="AD90" s="24" t="n"/>
+      <c r="AE90" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5850 (aec-mlb-cin-sea-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF90" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG90" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH90" s="24" t="n"/>
+      <c r="AI90" s="31" t="n"/>
+      <c r="AJ90" s="31" t="n"/>
+      <c r="AK90" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL90" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM90" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN90" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO90" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP90" s="24" t="inlineStr">
+        <is>
+          <t>mlb-cin</t>
+        </is>
+      </c>
+      <c r="AQ90" s="24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="AR90" s="24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="AS90" s="24" t="inlineStr">
+        <is>
+          <t>mlb-sea</t>
+        </is>
+      </c>
+      <c r="AT90" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AU90" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AV90" s="24" t="n"/>
+      <c r="AW90" s="24" t="n"/>
+      <c r="AX90" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY90" s="24" t="n"/>
+      <c r="AZ90" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA90" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB90" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC90" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD90" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE90" s="24" t="inlineStr">
+        <is>
+          <t>af7ccafcacf69681</t>
+        </is>
+      </c>
+      <c r="BF90" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG90" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH90" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:57:52.831217Z</t>
+        </is>
+      </c>
+      <c r="BI90" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ90" s="38" t="n"/>
+      <c r="BK90" s="26" t="n">
+        <v>-141</v>
+      </c>
+      <c r="BL90" s="39" t="n">
+        <v>1.70922</v>
+      </c>
+      <c r="BM90" s="28" t="n">
+        <v>0.585062</v>
+      </c>
+      <c r="BN90" s="28" t="n">
+        <v>0.58209</v>
+      </c>
+      <c r="BO90" s="28" t="n"/>
+      <c r="BP90" s="38" t="n"/>
+      <c r="BQ90" s="39" t="n"/>
+      <c r="BR90" s="28" t="n"/>
+      <c r="BS90" s="28" t="n"/>
+      <c r="BT90" s="28" t="n"/>
+      <c r="BU90" s="38" t="n"/>
+      <c r="BV90" s="29" t="n"/>
+      <c r="BW90" s="24" t="n"/>
+      <c r="BX90" s="40" t="n"/>
+      <c r="BY90" s="39" t="n"/>
+      <c r="BZ90" s="24" t="n"/>
+      <c r="CA90" s="31" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
fix: flat forecast logs all games, availability conflicts resolved conservatively
- cli.py: flat mode now logs every candidate (not just calls above threshold)
  so flat_picks.xlsx contains all 19 scheduled games, not just 13 calls
- player_availability.py: default conflict_policy changed from fail_closed
  to most_conservative — a single player status conflict (e.g. Alanna Smith
  official=Doubtful vs espn=Out) no longer blocks the entire availability
  adjustment for the game. Paige Bueckers listed as Out on ESPN is now
  correctly reflected even when another player has conflicting sources.
- test_wnba_availability.py: updated fail_closed test to pass policy
  explicitly since the default changed
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -327,8 +327,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA74" headerRowCount="1">
-  <autoFilter ref="A1:CA74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA80" headerRowCount="1">
+  <autoFilter ref="A1:CA80"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -765,19 +765,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$74)</f>
+        <f>COUNTA('Picks'!$A$2:$A$80)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$74,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$80,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$74,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$80,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$74,"settled",'Picks'!$V$2:$V$74,"win")+COUNTIFS('Picks'!$U$2:$U$74,"settled",'Picks'!$V$2:$V$74,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$80,"settled",'Picks'!$V$2:$V$80,"win")+COUNTIFS('Picks'!$U$2:$U$80,"settled",'Picks'!$V$2:$V$80,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -806,19 +806,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$74,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$80,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$74,"&gt;0",'Picks'!$V$2:$V$74,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$74,"&gt;0",'Picks'!$V$2:$V$74,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$80,"&gt;0",'Picks'!$V$2:$V$80,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$80,"&gt;0",'Picks'!$V$2:$V$80,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="32">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$74,"&gt;0",'Picks'!$V$2:$V$74,"win")/(COUNTIFS('Picks'!$BX$2:$BX$74,"&gt;0",'Picks'!$V$2:$V$74,"win")+COUNTIFS('Picks'!$BX$2:$BX$74,"&gt;0",'Picks'!$V$2:$V$74,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$80,"&gt;0",'Picks'!$V$2:$V$80,"win")/(COUNTIFS('Picks'!$BX$2:$BX$80,"&gt;0",'Picks'!$V$2:$V$80,"win")+COUNTIFS('Picks'!$BX$2:$BX$80,"&gt;0",'Picks'!$V$2:$V$80,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="32">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$74)/SUM('Picks'!$BX$2:$BX$74),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$80)/SUM('Picks'!$BX$2:$BX$80),0)</f>
         <v/>
       </c>
     </row>
@@ -847,19 +847,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="33">
-        <f>SUM('Picks'!$BY$2:$BY$74)</f>
+        <f>SUM('Picks'!$BY$2:$BY$80)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$74,"&lt;&gt;",'Picks'!$AB$2:$AB$74),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$80,"&lt;&gt;",'Picks'!$AB$2:$AB$80),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$74,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$74,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$80,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$80,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="33">
-        <f>SUMIFS('Picks'!$AC$2:$AC$74,'Picks'!$AM$2:$AM$74,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$80,'Picks'!$AM$2:$AM$80,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -915,15 +915,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$74,$A14,'Picks'!$U$2:$U$74,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$80,$A14,'Picks'!$U$2:$U$80,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$74,$A14,'Picks'!$U$2:$U$74,"settled",'Picks'!$V$2:$V$74,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$80,$A14,'Picks'!$U$2:$U$80,"settled",'Picks'!$V$2:$V$80,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$74,$A14,'Picks'!$U$2:$U$74,"settled",'Picks'!$V$2:$V$74,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$80,$A14,'Picks'!$U$2:$U$80,"settled",'Picks'!$V$2:$V$80,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="34">
@@ -931,11 +931,11 @@
         <v/>
       </c>
       <c r="F14" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$74,'Picks'!$H$2:$H$74,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$80,'Picks'!$H$2:$H$80,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$74,'Picks'!$H$2:$H$74,$A14,'Picks'!$U$2:$U$74,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$80,'Picks'!$H$2:$H$80,$A14,'Picks'!$U$2:$U$80,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -946,15 +946,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$74,$A15,'Picks'!$U$2:$U$74,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$80,$A15,'Picks'!$U$2:$U$80,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$74,$A15,'Picks'!$U$2:$U$74,"settled",'Picks'!$V$2:$V$74,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$80,$A15,'Picks'!$U$2:$U$80,"settled",'Picks'!$V$2:$V$80,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$74,$A15,'Picks'!$U$2:$U$74,"settled",'Picks'!$V$2:$V$74,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$80,$A15,'Picks'!$U$2:$U$80,"settled",'Picks'!$V$2:$V$80,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="36">
@@ -962,11 +962,11 @@
         <v/>
       </c>
       <c r="F15" s="37">
-        <f>SUMIFS('Picks'!$BY$2:$BY$74,'Picks'!$H$2:$H$74,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$80,'Picks'!$H$2:$H$80,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$74,'Picks'!$H$2:$H$74,$A15,'Picks'!$U$2:$U$74,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$80,'Picks'!$H$2:$H$80,$A15,'Picks'!$U$2:$U$80,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -977,15 +977,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$74,$A16,'Picks'!$U$2:$U$74,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$80,$A16,'Picks'!$U$2:$U$80,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$74,$A16,'Picks'!$U$2:$U$74,"settled",'Picks'!$V$2:$V$74,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$80,$A16,'Picks'!$U$2:$U$80,"settled",'Picks'!$V$2:$V$80,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$74,$A16,'Picks'!$U$2:$U$74,"settled",'Picks'!$V$2:$V$74,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$80,$A16,'Picks'!$U$2:$U$80,"settled",'Picks'!$V$2:$V$80,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="34">
@@ -993,11 +993,11 @@
         <v/>
       </c>
       <c r="F16" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$74,'Picks'!$H$2:$H$74,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$80,'Picks'!$H$2:$H$80,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$74,'Picks'!$H$2:$H$74,$A16,'Picks'!$U$2:$U$74,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$80,'Picks'!$H$2:$H$80,$A16,'Picks'!$U$2:$U$80,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA74"/>
+  <dimension ref="A1:CA80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15735,12 +15735,12 @@
     <row r="62" ht="36" customHeight="1">
       <c r="A62" s="24" t="inlineStr">
         <is>
-          <t>bbf4c446926f4a96</t>
+          <t>e00add3bfe2446db</t>
         </is>
       </c>
       <c r="B62" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:41.782177Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C62" s="24" t="inlineStr">
@@ -15946,7 +15946,7 @@
       </c>
       <c r="BH62" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:32.219947Z</t>
+          <t>2026-07-20T15:33:34.083345Z</t>
         </is>
       </c>
       <c r="BI62" s="24" t="inlineStr">
@@ -15965,7 +15965,7 @@
         <v>0.473934</v>
       </c>
       <c r="BN62" s="28" t="n">
-        <v>0.472637</v>
+        <v>0.470297</v>
       </c>
       <c r="BO62" s="28" t="n"/>
       <c r="BP62" s="38" t="n"/>
@@ -15984,22 +15984,22 @@
     <row r="63" ht="36" customHeight="1">
       <c r="A63" s="24" t="inlineStr">
         <is>
-          <t>1506b66a3b294539</t>
+          <t>7a7171ebb07c44d9</t>
         </is>
       </c>
       <c r="B63" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:41.782177Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C63" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T19:05:00-0400</t>
+          <t>2026-07-20T19:00:00-0400</t>
         </is>
       </c>
       <c r="D63" s="24" t="inlineStr">
         <is>
-          <t>401816189</t>
+          <t>401816187</t>
         </is>
       </c>
       <c r="E63" s="24" t="inlineStr">
@@ -16009,12 +16009,12 @@
       </c>
       <c r="F63" s="24" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="G63" s="24" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="H63" s="24" t="inlineStr">
@@ -16024,7 +16024,7 @@
       </c>
       <c r="I63" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J63" s="38" t="n"/>
@@ -16034,26 +16034,26 @@
         </is>
       </c>
       <c r="L63" s="26" t="n">
-        <v>-108</v>
+        <v>125</v>
       </c>
       <c r="M63" s="39" t="n">
-        <v>1.925926</v>
+        <v>2.25</v>
       </c>
       <c r="N63" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.444444</v>
       </c>
       <c r="O63" s="28" t="n">
-        <v>0.578558</v>
+        <v>0.513332</v>
       </c>
       <c r="P63" s="28" t="n"/>
       <c r="Q63" s="28" t="n">
-        <v>0.059327</v>
+        <v>0.068888</v>
       </c>
       <c r="R63" s="26" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="S63" s="29" t="n">
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="T63" s="24" t="inlineStr">
         <is>
@@ -16076,7 +16076,7 @@
       <c r="AD63" s="24" t="n"/>
       <c r="AE63" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5500; executable ask 0.5200 (aec-mlb-pit-nyy-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.4450 (aec-mlb-lad-phi-2026-07-20).</t>
         </is>
       </c>
       <c r="AF63" s="31" t="inlineStr">
@@ -16117,32 +16117,32 @@
       </c>
       <c r="AP63" s="24" t="inlineStr">
         <is>
-          <t>mlb-pit</t>
+          <t>mlb-lad</t>
         </is>
       </c>
       <c r="AQ63" s="24" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="AR63" s="24" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="AS63" s="24" t="inlineStr">
         <is>
-          <t>mlb-nyy</t>
+          <t>mlb-phi</t>
         </is>
       </c>
       <c r="AT63" s="24" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="AU63" s="24" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="AV63" s="24" t="n"/>
@@ -16180,7 +16180,7 @@
       </c>
       <c r="BE63" s="24" t="inlineStr">
         <is>
-          <t>38ab7db5a3798f0c</t>
+          <t>bac520e15b938e92</t>
         </is>
       </c>
       <c r="BF63" s="24" t="inlineStr">
@@ -16195,7 +16195,7 @@
       </c>
       <c r="BH63" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:35.056972Z</t>
+          <t>2026-07-20T15:33:40.881321Z</t>
         </is>
       </c>
       <c r="BI63" s="24" t="inlineStr">
@@ -16205,16 +16205,16 @@
       </c>
       <c r="BJ63" s="38" t="n"/>
       <c r="BK63" s="26" t="n">
-        <v>-108</v>
+        <v>125</v>
       </c>
       <c r="BL63" s="39" t="n">
-        <v>1.925926</v>
+        <v>2.25</v>
       </c>
       <c r="BM63" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.444444</v>
       </c>
       <c r="BN63" s="28" t="n">
-        <v>0.517413</v>
+        <v>0.442786</v>
       </c>
       <c r="BO63" s="28" t="n"/>
       <c r="BP63" s="38" t="n"/>
@@ -16233,22 +16233,22 @@
     <row r="64" ht="36" customHeight="1">
       <c r="A64" s="24" t="inlineStr">
         <is>
-          <t>540e168c7d8c4ba0</t>
+          <t>0e08e82b6c5e41de</t>
         </is>
       </c>
       <c r="B64" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:41.782177Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C64" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T19:10:00-0400</t>
+          <t>2026-07-20T19:05:00-0400</t>
         </is>
       </c>
       <c r="D64" s="24" t="inlineStr">
         <is>
-          <t>401816186</t>
+          <t>401816189</t>
         </is>
       </c>
       <c r="E64" s="24" t="inlineStr">
@@ -16258,12 +16258,12 @@
       </c>
       <c r="F64" s="24" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="G64" s="24" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="H64" s="24" t="inlineStr">
@@ -16283,23 +16283,23 @@
         </is>
       </c>
       <c r="L64" s="26" t="n">
-        <v>-138</v>
+        <v>-108</v>
       </c>
       <c r="M64" s="39" t="n">
-        <v>1.724638</v>
+        <v>1.925926</v>
       </c>
       <c r="N64" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.519231</v>
       </c>
       <c r="O64" s="28" t="n">
-        <v>0.565797</v>
+        <v>0.578558</v>
       </c>
       <c r="P64" s="28" t="n"/>
       <c r="Q64" s="28" t="n">
-        <v>-0.014035</v>
+        <v>0.059327</v>
       </c>
       <c r="R64" s="26" t="n">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="S64" s="29" t="n">
         <v>1.25</v>
@@ -16325,7 +16325,7 @@
       <c r="AD64" s="24" t="n"/>
       <c r="AE64" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5500; executable ask 0.5800 (aec-mlb-bal-bos-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5200 (aec-mlb-pit-nyy-2026-07-20).</t>
         </is>
       </c>
       <c r="AF64" s="31" t="inlineStr">
@@ -16366,32 +16366,32 @@
       </c>
       <c r="AP64" s="24" t="inlineStr">
         <is>
-          <t>mlb-bal</t>
+          <t>mlb-pit</t>
         </is>
       </c>
       <c r="AQ64" s="24" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="AR64" s="24" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="AS64" s="24" t="inlineStr">
         <is>
-          <t>mlb-bos</t>
+          <t>mlb-nyy</t>
         </is>
       </c>
       <c r="AT64" s="24" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="AU64" s="24" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="AV64" s="24" t="n"/>
@@ -16429,7 +16429,7 @@
       </c>
       <c r="BE64" s="24" t="inlineStr">
         <is>
-          <t>9fe2d27778a72dfe</t>
+          <t>38ab7db5a3798f0c</t>
         </is>
       </c>
       <c r="BF64" s="24" t="inlineStr">
@@ -16444,7 +16444,7 @@
       </c>
       <c r="BH64" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:37.354484Z</t>
+          <t>2026-07-20T15:33:36.050461Z</t>
         </is>
       </c>
       <c r="BI64" s="24" t="inlineStr">
@@ -16454,16 +16454,16 @@
       </c>
       <c r="BJ64" s="38" t="n"/>
       <c r="BK64" s="26" t="n">
-        <v>-138</v>
+        <v>-108</v>
       </c>
       <c r="BL64" s="39" t="n">
-        <v>1.724638</v>
+        <v>1.925926</v>
       </c>
       <c r="BM64" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.519231</v>
       </c>
       <c r="BN64" s="28" t="n">
-        <v>0.577114</v>
+        <v>0.517413</v>
       </c>
       <c r="BO64" s="28" t="n"/>
       <c r="BP64" s="38" t="n"/>
@@ -16482,22 +16482,22 @@
     <row r="65" ht="36" customHeight="1">
       <c r="A65" s="24" t="inlineStr">
         <is>
-          <t>f4dc16b93ff64092</t>
+          <t>764b59e974874df1</t>
         </is>
       </c>
       <c r="B65" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:41.782177Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C65" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T19:15:00-0400</t>
+          <t>2026-07-20T19:07:00-0400</t>
         </is>
       </c>
       <c r="D65" s="24" t="inlineStr">
         <is>
-          <t>401816190</t>
+          <t>401816191</t>
         </is>
       </c>
       <c r="E65" s="24" t="inlineStr">
@@ -16507,12 +16507,12 @@
       </c>
       <c r="F65" s="24" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="G65" s="24" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="H65" s="24" t="inlineStr">
@@ -16532,26 +16532,26 @@
         </is>
       </c>
       <c r="L65" s="26" t="n">
-        <v>-133</v>
+        <v>-144</v>
       </c>
       <c r="M65" s="39" t="n">
-        <v>1.75188</v>
+        <v>1.694444</v>
       </c>
       <c r="N65" s="28" t="n">
-        <v>0.570815</v>
+        <v>0.590164</v>
       </c>
       <c r="O65" s="28" t="n">
-        <v>0.550915</v>
+        <v>0.530206</v>
       </c>
       <c r="P65" s="28" t="n"/>
       <c r="Q65" s="28" t="n">
-        <v>-0.0199</v>
+        <v>-0.059958</v>
       </c>
       <c r="R65" s="26" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S65" s="29" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T65" s="24" t="inlineStr">
         <is>
@@ -16574,7 +16574,7 @@
       <c r="AD65" s="24" t="n"/>
       <c r="AE65" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5500; executable ask 0.5700 (aec-mlb-sd-atl-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5900 (aec-mlb-tb-tor-2026-07-20).</t>
         </is>
       </c>
       <c r="AF65" s="31" t="inlineStr">
@@ -16615,32 +16615,32 @@
       </c>
       <c r="AP65" s="24" t="inlineStr">
         <is>
-          <t>mlb-sd</t>
+          <t>mlb-tb</t>
         </is>
       </c>
       <c r="AQ65" s="24" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="AR65" s="24" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="AS65" s="24" t="inlineStr">
         <is>
-          <t>mlb-atl</t>
+          <t>mlb-tor</t>
         </is>
       </c>
       <c r="AT65" s="24" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="AU65" s="24" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="AV65" s="24" t="n"/>
@@ -16678,7 +16678,7 @@
       </c>
       <c r="BE65" s="24" t="inlineStr">
         <is>
-          <t>f0b5eac7c97d1146</t>
+          <t>78559912fe10ab9f</t>
         </is>
       </c>
       <c r="BF65" s="24" t="inlineStr">
@@ -16693,7 +16693,7 @@
       </c>
       <c r="BH65" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:40.909749Z</t>
+          <t>2026-07-20T15:33:37.942740Z</t>
         </is>
       </c>
       <c r="BI65" s="24" t="inlineStr">
@@ -16703,16 +16703,16 @@
       </c>
       <c r="BJ65" s="38" t="n"/>
       <c r="BK65" s="26" t="n">
-        <v>-133</v>
+        <v>-144</v>
       </c>
       <c r="BL65" s="39" t="n">
-        <v>1.75188</v>
+        <v>1.694444</v>
       </c>
       <c r="BM65" s="28" t="n">
-        <v>0.570815</v>
+        <v>0.590164</v>
       </c>
       <c r="BN65" s="28" t="n">
-        <v>0.567164</v>
+        <v>0.5870649999999999</v>
       </c>
       <c r="BO65" s="28" t="n"/>
       <c r="BP65" s="38" t="n"/>
@@ -16731,22 +16731,22 @@
     <row r="66" ht="36" customHeight="1">
       <c r="A66" s="24" t="inlineStr">
         <is>
-          <t>c08b803127a54cd0</t>
+          <t>03845491b26c4e30</t>
         </is>
       </c>
       <c r="B66" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:41.782177Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C66" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T19:40:00-0400</t>
+          <t>2026-07-20T19:10:00-0400</t>
         </is>
       </c>
       <c r="D66" s="24" t="inlineStr">
         <is>
-          <t>401816195</t>
+          <t>401816186</t>
         </is>
       </c>
       <c r="E66" s="24" t="inlineStr">
@@ -16756,12 +16756,12 @@
       </c>
       <c r="F66" s="24" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="G66" s="24" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="H66" s="24" t="inlineStr">
@@ -16781,26 +16781,26 @@
         </is>
       </c>
       <c r="L66" s="26" t="n">
-        <v>-199</v>
+        <v>-138</v>
       </c>
       <c r="M66" s="39" t="n">
-        <v>1.502513</v>
+        <v>1.724638</v>
       </c>
       <c r="N66" s="28" t="n">
-        <v>0.665552</v>
+        <v>0.579832</v>
       </c>
       <c r="O66" s="28" t="n">
-        <v>0.640995</v>
+        <v>0.565797</v>
       </c>
       <c r="P66" s="28" t="n"/>
       <c r="Q66" s="28" t="n">
-        <v>-0.024557</v>
+        <v>-0.014035</v>
       </c>
       <c r="R66" s="26" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="S66" s="29" t="n">
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="T66" s="24" t="inlineStr">
         <is>
@@ -16823,7 +16823,7 @@
       <c r="AD66" s="24" t="n"/>
       <c r="AE66" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5500; executable ask 0.6650 (aec-mlb-nym-mil-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5800 (aec-mlb-bal-bos-2026-07-20).</t>
         </is>
       </c>
       <c r="AF66" s="31" t="inlineStr">
@@ -16864,32 +16864,32 @@
       </c>
       <c r="AP66" s="24" t="inlineStr">
         <is>
-          <t>mlb-nym</t>
+          <t>mlb-bal</t>
         </is>
       </c>
       <c r="AQ66" s="24" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="AR66" s="24" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="AS66" s="24" t="inlineStr">
         <is>
-          <t>mlb-mil</t>
+          <t>mlb-bos</t>
         </is>
       </c>
       <c r="AT66" s="24" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="AU66" s="24" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="AV66" s="24" t="n"/>
@@ -16927,7 +16927,7 @@
       </c>
       <c r="BE66" s="24" t="inlineStr">
         <is>
-          <t>6d5f3f5e8f75cb2b</t>
+          <t>9fe2d27778a72dfe</t>
         </is>
       </c>
       <c r="BF66" s="24" t="inlineStr">
@@ -16942,7 +16942,7 @@
       </c>
       <c r="BH66" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:42.879792Z</t>
+          <t>2026-07-20T15:33:39.422286Z</t>
         </is>
       </c>
       <c r="BI66" s="24" t="inlineStr">
@@ -16952,16 +16952,16 @@
       </c>
       <c r="BJ66" s="38" t="n"/>
       <c r="BK66" s="26" t="n">
-        <v>-199</v>
+        <v>-138</v>
       </c>
       <c r="BL66" s="39" t="n">
-        <v>1.502513</v>
+        <v>1.724638</v>
       </c>
       <c r="BM66" s="28" t="n">
-        <v>0.665552</v>
+        <v>0.579832</v>
       </c>
       <c r="BN66" s="28" t="n">
-        <v>0.6616919999999999</v>
+        <v>0.577114</v>
       </c>
       <c r="BO66" s="28" t="n"/>
       <c r="BP66" s="38" t="n"/>
@@ -16980,22 +16980,22 @@
     <row r="67" ht="36" customHeight="1">
       <c r="A67" s="24" t="inlineStr">
         <is>
-          <t>6e9b235e0abe4f38</t>
+          <t>8fe8dba867db4326</t>
         </is>
       </c>
       <c r="B67" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:41.782177Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C67" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T20:05:00-0400</t>
+          <t>2026-07-20T19:15:00-0400</t>
         </is>
       </c>
       <c r="D67" s="24" t="inlineStr">
         <is>
-          <t>401816193</t>
+          <t>401816190</t>
         </is>
       </c>
       <c r="E67" s="24" t="inlineStr">
@@ -17005,12 +17005,12 @@
       </c>
       <c r="F67" s="24" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="G67" s="24" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="H67" s="24" t="inlineStr">
@@ -17030,26 +17030,26 @@
         </is>
       </c>
       <c r="L67" s="26" t="n">
-        <v>-108</v>
+        <v>-133</v>
       </c>
       <c r="M67" s="39" t="n">
-        <v>1.925926</v>
+        <v>1.75188</v>
       </c>
       <c r="N67" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.570815</v>
       </c>
       <c r="O67" s="28" t="n">
-        <v>0.566967</v>
+        <v>0.550915</v>
       </c>
       <c r="P67" s="28" t="n"/>
       <c r="Q67" s="28" t="n">
-        <v>0.047736</v>
+        <v>-0.0199</v>
       </c>
       <c r="R67" s="26" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="S67" s="29" t="n">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="T67" s="24" t="inlineStr">
         <is>
@@ -17072,7 +17072,7 @@
       <c r="AD67" s="24" t="n"/>
       <c r="AE67" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5500; executable ask 0.5200 (aec-mlb-det-chc-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5700 (aec-mlb-sd-atl-2026-07-20).</t>
         </is>
       </c>
       <c r="AF67" s="31" t="inlineStr">
@@ -17113,32 +17113,32 @@
       </c>
       <c r="AP67" s="24" t="inlineStr">
         <is>
-          <t>mlb-det</t>
+          <t>mlb-sd</t>
         </is>
       </c>
       <c r="AQ67" s="24" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="AR67" s="24" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="AS67" s="24" t="inlineStr">
         <is>
-          <t>mlb-chc</t>
+          <t>mlb-atl</t>
         </is>
       </c>
       <c r="AT67" s="24" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="AU67" s="24" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="AV67" s="24" t="n"/>
@@ -17176,7 +17176,7 @@
       </c>
       <c r="BE67" s="24" t="inlineStr">
         <is>
-          <t>b84afb2c70e14d93</t>
+          <t>f0b5eac7c97d1146</t>
         </is>
       </c>
       <c r="BF67" s="24" t="inlineStr">
@@ -17191,7 +17191,7 @@
       </c>
       <c r="BH67" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:46.871986Z</t>
+          <t>2026-07-20T15:33:42.141054Z</t>
         </is>
       </c>
       <c r="BI67" s="24" t="inlineStr">
@@ -17201,16 +17201,16 @@
       </c>
       <c r="BJ67" s="38" t="n"/>
       <c r="BK67" s="26" t="n">
-        <v>-108</v>
+        <v>-133</v>
       </c>
       <c r="BL67" s="39" t="n">
-        <v>1.925926</v>
+        <v>1.75188</v>
       </c>
       <c r="BM67" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.570815</v>
       </c>
       <c r="BN67" s="28" t="n">
-        <v>0.517413</v>
+        <v>0.567164</v>
       </c>
       <c r="BO67" s="28" t="n"/>
       <c r="BP67" s="38" t="n"/>
@@ -17229,22 +17229,22 @@
     <row r="68" ht="36" customHeight="1">
       <c r="A68" s="24" t="inlineStr">
         <is>
-          <t>bf8728673bd4485f</t>
+          <t>de587015be8044d0</t>
         </is>
       </c>
       <c r="B68" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:41.782177Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C68" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T20:40:00-0400</t>
+          <t>2026-07-20T19:40:00-0400</t>
         </is>
       </c>
       <c r="D68" s="24" t="inlineStr">
         <is>
-          <t>401816197</t>
+          <t>401816195</t>
         </is>
       </c>
       <c r="E68" s="24" t="inlineStr">
@@ -17254,12 +17254,12 @@
       </c>
       <c r="F68" s="24" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="G68" s="24" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="H68" s="24" t="inlineStr">
@@ -17269,7 +17269,7 @@
       </c>
       <c r="I68" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J68" s="38" t="n"/>
@@ -17279,26 +17279,26 @@
         </is>
       </c>
       <c r="L68" s="26" t="n">
-        <v>-117</v>
+        <v>-199</v>
       </c>
       <c r="M68" s="39" t="n">
-        <v>1.854701</v>
+        <v>1.502513</v>
       </c>
       <c r="N68" s="28" t="n">
-        <v>0.539171</v>
+        <v>0.665552</v>
       </c>
       <c r="O68" s="28" t="n">
-        <v>0.5563709999999999</v>
+        <v>0.640995</v>
       </c>
       <c r="P68" s="28" t="n"/>
       <c r="Q68" s="28" t="n">
-        <v>0.0172</v>
+        <v>-0.024557</v>
       </c>
       <c r="R68" s="26" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="S68" s="29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T68" s="24" t="inlineStr">
         <is>
@@ -17321,7 +17321,7 @@
       <c r="AD68" s="24" t="n"/>
       <c r="AE68" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5500; executable ask 0.5400 (aec-mlb-wsh-col-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.6650 (aec-mlb-nym-mil-2026-07-20).</t>
         </is>
       </c>
       <c r="AF68" s="31" t="inlineStr">
@@ -17362,32 +17362,32 @@
       </c>
       <c r="AP68" s="24" t="inlineStr">
         <is>
-          <t>mlb-wsh</t>
+          <t>mlb-nym</t>
         </is>
       </c>
       <c r="AQ68" s="24" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="AR68" s="24" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="AS68" s="24" t="inlineStr">
         <is>
-          <t>mlb-col</t>
+          <t>mlb-mil</t>
         </is>
       </c>
       <c r="AT68" s="24" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="AU68" s="24" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="AV68" s="24" t="n"/>
@@ -17425,7 +17425,7 @@
       </c>
       <c r="BE68" s="24" t="inlineStr">
         <is>
-          <t>a2f336c1cee8c92e</t>
+          <t>6d5f3f5e8f75cb2b</t>
         </is>
       </c>
       <c r="BF68" s="24" t="inlineStr">
@@ -17440,7 +17440,7 @@
       </c>
       <c r="BH68" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:49.897394Z</t>
+          <t>2026-07-20T15:33:44.122845Z</t>
         </is>
       </c>
       <c r="BI68" s="24" t="inlineStr">
@@ -17450,16 +17450,16 @@
       </c>
       <c r="BJ68" s="38" t="n"/>
       <c r="BK68" s="26" t="n">
-        <v>-117</v>
+        <v>-199</v>
       </c>
       <c r="BL68" s="39" t="n">
-        <v>1.854701</v>
+        <v>1.502513</v>
       </c>
       <c r="BM68" s="28" t="n">
-        <v>0.539171</v>
+        <v>0.665552</v>
       </c>
       <c r="BN68" s="28" t="n">
-        <v>0.537313</v>
+        <v>0.6616919999999999</v>
       </c>
       <c r="BO68" s="28" t="n"/>
       <c r="BP68" s="38" t="n"/>
@@ -17478,22 +17478,22 @@
     <row r="69" ht="36" customHeight="1">
       <c r="A69" s="24" t="inlineStr">
         <is>
-          <t>aefbe47ff16045f2</t>
+          <t>f30c4f4411454bcb</t>
         </is>
       </c>
       <c r="B69" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:41.782177Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C69" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T21:40:00-0400</t>
+          <t>2026-07-20T19:40:00-0400</t>
         </is>
       </c>
       <c r="D69" s="24" t="inlineStr">
         <is>
-          <t>401816198</t>
+          <t>401816196</t>
         </is>
       </c>
       <c r="E69" s="24" t="inlineStr">
@@ -17503,12 +17503,12 @@
       </c>
       <c r="F69" s="24" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="G69" s="24" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="H69" s="24" t="inlineStr">
@@ -17528,26 +17528,26 @@
         </is>
       </c>
       <c r="L69" s="26" t="n">
-        <v>-147</v>
+        <v>-111</v>
       </c>
       <c r="M69" s="39" t="n">
-        <v>1.680272</v>
+        <v>1.900901</v>
       </c>
       <c r="N69" s="28" t="n">
-        <v>0.5951419999999999</v>
+        <v>0.526066</v>
       </c>
       <c r="O69" s="28" t="n">
-        <v>0.58189</v>
+        <v>0.514213</v>
       </c>
       <c r="P69" s="28" t="n"/>
       <c r="Q69" s="28" t="n">
-        <v>-0.013252</v>
+        <v>-0.011853</v>
       </c>
       <c r="R69" s="26" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S69" s="29" t="n">
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="T69" s="24" t="inlineStr">
         <is>
@@ -17570,7 +17570,7 @@
       <c r="AD69" s="24" t="n"/>
       <c r="AE69" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5500; executable ask 0.5950 (aec-mlb-ath-az-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5250 (aec-mlb-sf-kc-2026-07-20).</t>
         </is>
       </c>
       <c r="AF69" s="31" t="inlineStr">
@@ -17611,32 +17611,32 @@
       </c>
       <c r="AP69" s="24" t="inlineStr">
         <is>
-          <t>mlb-ath</t>
+          <t>mlb-sf</t>
         </is>
       </c>
       <c r="AQ69" s="24" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="AR69" s="24" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="AS69" s="24" t="inlineStr">
         <is>
-          <t>mlb-ari</t>
+          <t>mlb-kc</t>
         </is>
       </c>
       <c r="AT69" s="24" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="AU69" s="24" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="AV69" s="24" t="n"/>
@@ -17674,7 +17674,7 @@
       </c>
       <c r="BE69" s="24" t="inlineStr">
         <is>
-          <t>7b682aa5da86e2a4</t>
+          <t>9c457d5cc4752804</t>
         </is>
       </c>
       <c r="BF69" s="24" t="inlineStr">
@@ -17689,7 +17689,7 @@
       </c>
       <c r="BH69" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:51.339273Z</t>
+          <t>2026-07-20T15:33:44.852438Z</t>
         </is>
       </c>
       <c r="BI69" s="24" t="inlineStr">
@@ -17699,16 +17699,16 @@
       </c>
       <c r="BJ69" s="38" t="n"/>
       <c r="BK69" s="26" t="n">
-        <v>-147</v>
+        <v>-111</v>
       </c>
       <c r="BL69" s="39" t="n">
-        <v>1.680272</v>
+        <v>1.900901</v>
       </c>
       <c r="BM69" s="28" t="n">
-        <v>0.5951419999999999</v>
+        <v>0.526066</v>
       </c>
       <c r="BN69" s="28" t="n">
-        <v>0.59204</v>
+        <v>0.522388</v>
       </c>
       <c r="BO69" s="28" t="n"/>
       <c r="BP69" s="38" t="n"/>
@@ -17727,22 +17727,22 @@
     <row r="70" ht="36" customHeight="1">
       <c r="A70" s="24" t="inlineStr">
         <is>
-          <t>b9692cb20ec34d5d</t>
+          <t>9d32e3b580bb4d9e</t>
         </is>
       </c>
       <c r="B70" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:41.782177Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C70" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T21:40:00-0400</t>
+          <t>2026-07-20T20:05:00-0400</t>
         </is>
       </c>
       <c r="D70" s="24" t="inlineStr">
         <is>
-          <t>401816199</t>
+          <t>401816192</t>
         </is>
       </c>
       <c r="E70" s="24" t="inlineStr">
@@ -17752,12 +17752,12 @@
       </c>
       <c r="F70" s="24" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="G70" s="24" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="H70" s="24" t="inlineStr">
@@ -17777,26 +17777,26 @@
         </is>
       </c>
       <c r="L70" s="26" t="n">
-        <v>-141</v>
+        <v>-160</v>
       </c>
       <c r="M70" s="39" t="n">
-        <v>1.70922</v>
+        <v>1.625</v>
       </c>
       <c r="N70" s="28" t="n">
-        <v>0.585062</v>
+        <v>0.615385</v>
       </c>
       <c r="O70" s="28" t="n">
-        <v>0.592852</v>
+        <v>0.524518</v>
       </c>
       <c r="P70" s="28" t="n"/>
       <c r="Q70" s="28" t="n">
-        <v>0.00779</v>
+        <v>-0.090867</v>
       </c>
       <c r="R70" s="26" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="S70" s="29" t="n">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="T70" s="24" t="inlineStr">
         <is>
@@ -17819,7 +17819,7 @@
       <c r="AD70" s="24" t="n"/>
       <c r="AE70" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5500; executable ask 0.5850 (aec-mlb-cin-sea-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.6150 (aec-mlb-cws-tex-2026-07-20).</t>
         </is>
       </c>
       <c r="AF70" s="31" t="inlineStr">
@@ -17860,32 +17860,32 @@
       </c>
       <c r="AP70" s="24" t="inlineStr">
         <is>
-          <t>mlb-cin</t>
+          <t>mlb-cws</t>
         </is>
       </c>
       <c r="AQ70" s="24" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="AR70" s="24" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="AS70" s="24" t="inlineStr">
         <is>
-          <t>mlb-sea</t>
+          <t>mlb-tex</t>
         </is>
       </c>
       <c r="AT70" s="24" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="AU70" s="24" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="AV70" s="24" t="n"/>
@@ -17923,7 +17923,7 @@
       </c>
       <c r="BE70" s="24" t="inlineStr">
         <is>
-          <t>af7ccafcacf69681</t>
+          <t>87e15ff2f82f8974</t>
         </is>
       </c>
       <c r="BF70" s="24" t="inlineStr">
@@ -17938,7 +17938,7 @@
       </c>
       <c r="BH70" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:52.831217Z</t>
+          <t>2026-07-20T15:33:47.582533Z</t>
         </is>
       </c>
       <c r="BI70" s="24" t="inlineStr">
@@ -17948,16 +17948,16 @@
       </c>
       <c r="BJ70" s="38" t="n"/>
       <c r="BK70" s="26" t="n">
-        <v>-141</v>
+        <v>-160</v>
       </c>
       <c r="BL70" s="39" t="n">
-        <v>1.70922</v>
+        <v>1.625</v>
       </c>
       <c r="BM70" s="28" t="n">
-        <v>0.585062</v>
+        <v>0.615385</v>
       </c>
       <c r="BN70" s="28" t="n">
-        <v>0.58209</v>
+        <v>0.61194</v>
       </c>
       <c r="BO70" s="28" t="n"/>
       <c r="BP70" s="38" t="n"/>
@@ -17976,37 +17976,37 @@
     <row r="71" ht="36" customHeight="1">
       <c r="A71" s="24" t="inlineStr">
         <is>
-          <t>11f48fe641c040f7</t>
+          <t>d4d115be002c47d3</t>
         </is>
       </c>
       <c r="B71" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:28:55.067840Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C71" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T20:00:00-0400</t>
+          <t>2026-07-20T20:05:00-0400</t>
         </is>
       </c>
       <c r="D71" s="24" t="inlineStr">
         <is>
-          <t>401857083</t>
+          <t>401816193</t>
         </is>
       </c>
       <c r="E71" s="24" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="F71" s="24" t="inlineStr">
         <is>
-          <t>Las Vegas Aces</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="G71" s="24" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="H71" s="24" t="inlineStr">
@@ -18016,7 +18016,7 @@
       </c>
       <c r="I71" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J71" s="38" t="n"/>
@@ -18026,30 +18026,30 @@
         </is>
       </c>
       <c r="L71" s="26" t="n">
-        <v>-488</v>
+        <v>-108</v>
       </c>
       <c r="M71" s="39" t="n">
-        <v>1.204918</v>
+        <v>1.925926</v>
       </c>
       <c r="N71" s="28" t="n">
-        <v>0.829932</v>
+        <v>0.519231</v>
       </c>
       <c r="O71" s="28" t="n">
-        <v>0.6572210000000001</v>
+        <v>0.566967</v>
       </c>
       <c r="P71" s="28" t="n"/>
       <c r="Q71" s="28" t="n">
-        <v>-0.172711</v>
+        <v>0.047736</v>
       </c>
       <c r="R71" s="26" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="S71" s="29" t="n">
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="T71" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="U71" s="24" t="inlineStr">
@@ -18068,7 +18068,7 @@
       <c r="AD71" s="24" t="n"/>
       <c r="AE71" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5051; executable ask 0.8300 (aec-wnba-lv-tor-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5200 (aec-mlb-det-chc-2026-07-20).</t>
         </is>
       </c>
       <c r="AF71" s="31" t="inlineStr">
@@ -18104,37 +18104,37 @@
       </c>
       <c r="AO71" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+          <t>NO_CALL_LOW_EDGE</t>
         </is>
       </c>
       <c r="AP71" s="24" t="inlineStr">
         <is>
-          <t>wnba-lva</t>
+          <t>mlb-det</t>
         </is>
       </c>
       <c r="AQ71" s="24" t="inlineStr">
         <is>
-          <t>Las Vegas Aces</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="AR71" s="24" t="inlineStr">
         <is>
-          <t>Las Vegas Aces</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="AS71" s="24" t="inlineStr">
         <is>
-          <t>wnba-tor</t>
+          <t>mlb-chc</t>
         </is>
       </c>
       <c r="AT71" s="24" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="AU71" s="24" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="AV71" s="24" t="n"/>
@@ -18152,7 +18152,7 @@
       </c>
       <c r="BA71" s="24" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
         </is>
       </c>
       <c r="BB71" s="24" t="inlineStr">
@@ -18162,17 +18162,17 @@
       </c>
       <c r="BC71" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BD71" s="24" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
         </is>
       </c>
       <c r="BE71" s="24" t="inlineStr">
         <is>
-          <t>32740a9f4976946d</t>
+          <t>b84afb2c70e14d93</t>
         </is>
       </c>
       <c r="BF71" s="24" t="inlineStr">
@@ -18182,12 +18182,12 @@
       </c>
       <c r="BG71" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BH71" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:56.867039Z</t>
+          <t>2026-07-20T15:33:47.761585Z</t>
         </is>
       </c>
       <c r="BI71" s="24" t="inlineStr">
@@ -18197,16 +18197,16 @@
       </c>
       <c r="BJ71" s="38" t="n"/>
       <c r="BK71" s="26" t="n">
-        <v>-488</v>
+        <v>-108</v>
       </c>
       <c r="BL71" s="39" t="n">
-        <v>1.204918</v>
+        <v>1.925926</v>
       </c>
       <c r="BM71" s="28" t="n">
-        <v>0.829932</v>
+        <v>0.519231</v>
       </c>
       <c r="BN71" s="28" t="n">
-        <v>0.821782</v>
+        <v>0.5148509999999999</v>
       </c>
       <c r="BO71" s="28" t="n"/>
       <c r="BP71" s="38" t="n"/>
@@ -18225,37 +18225,37 @@
     <row r="72" ht="36" customHeight="1">
       <c r="A72" s="24" t="inlineStr">
         <is>
-          <t>18e861041a484fd5</t>
+          <t>5ac11ebb449b4b54</t>
         </is>
       </c>
       <c r="B72" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:28:55.067840Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C72" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T20:00:00-0400</t>
+          <t>2026-07-20T20:10:00-0400</t>
         </is>
       </c>
       <c r="D72" s="24" t="inlineStr">
         <is>
-          <t>401892393</t>
+          <t>401816194</t>
         </is>
       </c>
       <c r="E72" s="24" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="F72" s="24" t="inlineStr">
         <is>
-          <t>New York Liberty</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="G72" s="24" t="inlineStr">
         <is>
-          <t>Dallas Wings</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="H72" s="24" t="inlineStr">
@@ -18275,30 +18275,30 @@
         </is>
       </c>
       <c r="L72" s="26" t="n">
-        <v>156</v>
+        <v>-115</v>
       </c>
       <c r="M72" s="39" t="n">
-        <v>2.56</v>
+        <v>1.869565</v>
       </c>
       <c r="N72" s="28" t="n">
-        <v>0.390625</v>
+        <v>0.534884</v>
       </c>
       <c r="O72" s="28" t="n">
-        <v>0.688998</v>
+        <v>0.512555</v>
       </c>
       <c r="P72" s="28" t="n"/>
       <c r="Q72" s="28" t="n">
-        <v>0.298373</v>
+        <v>-0.022329</v>
       </c>
       <c r="R72" s="26" t="n">
-        <v>100</v>
+        <v>9</v>
       </c>
       <c r="S72" s="29" t="n">
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="T72" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="U72" s="24" t="inlineStr">
@@ -18317,7 +18317,7 @@
       <c r="AD72" s="24" t="n"/>
       <c r="AE72" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5051; executable ask 0.3900 (aec-wnba-ny-dal-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5350 (aec-mlb-mia-hou-2026-07-20).</t>
         </is>
       </c>
       <c r="AF72" s="31" t="inlineStr">
@@ -18353,37 +18353,37 @@
       </c>
       <c r="AO72" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+          <t>NO_CALL_LOW_EDGE</t>
         </is>
       </c>
       <c r="AP72" s="24" t="inlineStr">
         <is>
-          <t>wnba-nyl</t>
+          <t>mlb-mia</t>
         </is>
       </c>
       <c r="AQ72" s="24" t="inlineStr">
         <is>
-          <t>New York Liberty</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="AR72" s="24" t="inlineStr">
         <is>
-          <t>New York Liberty</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="AS72" s="24" t="inlineStr">
         <is>
-          <t>wnba-dal</t>
+          <t>mlb-hou</t>
         </is>
       </c>
       <c r="AT72" s="24" t="inlineStr">
         <is>
-          <t>Dallas Wings</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="AU72" s="24" t="inlineStr">
         <is>
-          <t>Dallas Wings</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="AV72" s="24" t="n"/>
@@ -18401,7 +18401,7 @@
       </c>
       <c r="BA72" s="24" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
         </is>
       </c>
       <c r="BB72" s="24" t="inlineStr">
@@ -18411,17 +18411,17 @@
       </c>
       <c r="BC72" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BD72" s="24" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
         </is>
       </c>
       <c r="BE72" s="24" t="inlineStr">
         <is>
-          <t>c20bbb99f1fff741</t>
+          <t>ba8ef6f8648f77b7</t>
         </is>
       </c>
       <c r="BF72" s="24" t="inlineStr">
@@ -18431,12 +18431,12 @@
       </c>
       <c r="BG72" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BH72" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:58.731031Z</t>
+          <t>2026-07-20T15:33:49.597715Z</t>
         </is>
       </c>
       <c r="BI72" s="24" t="inlineStr">
@@ -18446,16 +18446,16 @@
       </c>
       <c r="BJ72" s="38" t="n"/>
       <c r="BK72" s="26" t="n">
-        <v>156</v>
+        <v>-115</v>
       </c>
       <c r="BL72" s="39" t="n">
-        <v>2.56</v>
+        <v>1.869565</v>
       </c>
       <c r="BM72" s="28" t="n">
-        <v>0.390625</v>
+        <v>0.534884</v>
       </c>
       <c r="BN72" s="28" t="n">
-        <v>0.386139</v>
+        <v>0.532338</v>
       </c>
       <c r="BO72" s="28" t="n"/>
       <c r="BP72" s="38" t="n"/>
@@ -18474,37 +18474,37 @@
     <row r="73" ht="36" customHeight="1">
       <c r="A73" s="24" t="inlineStr">
         <is>
-          <t>195c4a9c3ce44e1b</t>
+          <t>3faaea8e908f4dff</t>
         </is>
       </c>
       <c r="B73" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:28:55.067840Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C73" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T22:00:00-0400</t>
+          <t>2026-07-20T20:40:00-0400</t>
         </is>
       </c>
       <c r="D73" s="24" t="inlineStr">
         <is>
-          <t>401857084</t>
+          <t>401816197</t>
         </is>
       </c>
       <c r="E73" s="24" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="F73" s="24" t="inlineStr">
         <is>
-          <t>Washington Mystics</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="G73" s="24" t="inlineStr">
         <is>
-          <t>Golden State Valkyries</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="H73" s="24" t="inlineStr">
@@ -18514,7 +18514,7 @@
       </c>
       <c r="I73" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J73" s="38" t="n"/>
@@ -18524,30 +18524,30 @@
         </is>
       </c>
       <c r="L73" s="26" t="n">
-        <v>-317</v>
+        <v>-117</v>
       </c>
       <c r="M73" s="39" t="n">
-        <v>1.315457</v>
+        <v>1.854701</v>
       </c>
       <c r="N73" s="28" t="n">
-        <v>0.760192</v>
+        <v>0.539171</v>
       </c>
       <c r="O73" s="28" t="n">
-        <v>0.750463</v>
+        <v>0.5563709999999999</v>
       </c>
       <c r="P73" s="28" t="n"/>
       <c r="Q73" s="28" t="n">
-        <v>-0.009729</v>
+        <v>0.0172</v>
       </c>
       <c r="R73" s="26" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="S73" s="29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T73" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="U73" s="24" t="inlineStr">
@@ -18566,7 +18566,7 @@
       <c r="AD73" s="24" t="n"/>
       <c r="AE73" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5051; executable ask 0.7600 (aec-wnba-wsh-gsv-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5400 (aec-mlb-wsh-col-2026-07-20).</t>
         </is>
       </c>
       <c r="AF73" s="31" t="inlineStr">
@@ -18607,32 +18607,32 @@
       </c>
       <c r="AP73" s="24" t="inlineStr">
         <is>
-          <t>wnba-was</t>
+          <t>mlb-wsh</t>
         </is>
       </c>
       <c r="AQ73" s="24" t="inlineStr">
         <is>
-          <t>Washington Mystics</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="AR73" s="24" t="inlineStr">
         <is>
-          <t>Washington Mystics</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="AS73" s="24" t="inlineStr">
         <is>
-          <t>wnba-gsv</t>
+          <t>mlb-col</t>
         </is>
       </c>
       <c r="AT73" s="24" t="inlineStr">
         <is>
-          <t>Golden State Valkyries</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="AU73" s="24" t="inlineStr">
         <is>
-          <t>Golden State Valkyries</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="AV73" s="24" t="n"/>
@@ -18650,7 +18650,7 @@
       </c>
       <c r="BA73" s="24" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
         </is>
       </c>
       <c r="BB73" s="24" t="inlineStr">
@@ -18660,17 +18660,17 @@
       </c>
       <c r="BC73" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BD73" s="24" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
         </is>
       </c>
       <c r="BE73" s="24" t="inlineStr">
         <is>
-          <t>a82314f65618b567</t>
+          <t>a2f336c1cee8c92e</t>
         </is>
       </c>
       <c r="BF73" s="24" t="inlineStr">
@@ -18680,12 +18680,12 @@
       </c>
       <c r="BG73" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BH73" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:58:01.293707Z</t>
+          <t>2026-07-20T15:33:51.548954Z</t>
         </is>
       </c>
       <c r="BI73" s="24" t="inlineStr">
@@ -18695,16 +18695,16 @@
       </c>
       <c r="BJ73" s="38" t="n"/>
       <c r="BK73" s="26" t="n">
-        <v>-317</v>
+        <v>-117</v>
       </c>
       <c r="BL73" s="39" t="n">
-        <v>1.315457</v>
+        <v>1.854701</v>
       </c>
       <c r="BM73" s="28" t="n">
-        <v>0.760192</v>
+        <v>0.539171</v>
       </c>
       <c r="BN73" s="28" t="n">
-        <v>0.752475</v>
+        <v>0.537313</v>
       </c>
       <c r="BO73" s="28" t="n"/>
       <c r="BP73" s="38" t="n"/>
@@ -18723,37 +18723,37 @@
     <row r="74" ht="36" customHeight="1">
       <c r="A74" s="24" t="inlineStr">
         <is>
-          <t>555b6295ce3941e7</t>
+          <t>ce60c51f7f4d4503</t>
         </is>
       </c>
       <c r="B74" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:28:55.067840Z</t>
+          <t>2026-07-20T15:38:55.511243Z</t>
         </is>
       </c>
       <c r="C74" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T22:00:00-0400</t>
+          <t>2026-07-20T21:40:00-0400</t>
         </is>
       </c>
       <c r="D74" s="24" t="inlineStr">
         <is>
-          <t>401857085</t>
+          <t>401816198</t>
         </is>
       </c>
       <c r="E74" s="24" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="F74" s="24" t="inlineStr">
         <is>
-          <t>Minnesota Lynx</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="G74" s="24" t="inlineStr">
         <is>
-          <t>Seattle Storm</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="H74" s="24" t="inlineStr">
@@ -18763,7 +18763,7 @@
       </c>
       <c r="I74" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J74" s="38" t="n"/>
@@ -18773,30 +18773,30 @@
         </is>
       </c>
       <c r="L74" s="26" t="n">
-        <v>-456</v>
+        <v>-144</v>
       </c>
       <c r="M74" s="39" t="n">
-        <v>1.219298</v>
+        <v>1.694444</v>
       </c>
       <c r="N74" s="28" t="n">
-        <v>0.820144</v>
+        <v>0.590164</v>
       </c>
       <c r="O74" s="28" t="n">
-        <v>0.738843</v>
+        <v>0.58189</v>
       </c>
       <c r="P74" s="28" t="n"/>
       <c r="Q74" s="28" t="n">
-        <v>-0.081301</v>
+        <v>-0.008274</v>
       </c>
       <c r="R74" s="26" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="S74" s="29" t="n">
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="T74" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="U74" s="24" t="inlineStr">
@@ -18815,7 +18815,7 @@
       <c r="AD74" s="24" t="n"/>
       <c r="AE74" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5051; executable ask 0.8200 (aec-wnba-min-sea-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5900 (aec-mlb-ath-az-2026-07-20).</t>
         </is>
       </c>
       <c r="AF74" s="31" t="inlineStr">
@@ -18856,32 +18856,32 @@
       </c>
       <c r="AP74" s="24" t="inlineStr">
         <is>
-          <t>wnba-min</t>
+          <t>mlb-ath</t>
         </is>
       </c>
       <c r="AQ74" s="24" t="inlineStr">
         <is>
-          <t>Minnesota Lynx</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="AR74" s="24" t="inlineStr">
         <is>
-          <t>Minnesota Lynx</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="AS74" s="24" t="inlineStr">
         <is>
-          <t>wnba-sea</t>
+          <t>mlb-ari</t>
         </is>
       </c>
       <c r="AT74" s="24" t="inlineStr">
         <is>
-          <t>Seattle Storm</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="AU74" s="24" t="inlineStr">
         <is>
-          <t>Seattle Storm</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="AV74" s="24" t="n"/>
@@ -18899,7 +18899,7 @@
       </c>
       <c r="BA74" s="24" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
         </is>
       </c>
       <c r="BB74" s="24" t="inlineStr">
@@ -18909,17 +18909,17 @@
       </c>
       <c r="BC74" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BD74" s="24" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
         </is>
       </c>
       <c r="BE74" s="24" t="inlineStr">
         <is>
-          <t>c7928758cc04b6e5</t>
+          <t>7b682aa5da86e2a4</t>
         </is>
       </c>
       <c r="BF74" s="24" t="inlineStr">
@@ -18929,12 +18929,12 @@
       </c>
       <c r="BG74" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v3</t>
+          <t>mlb-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BH74" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:58:02.052718Z</t>
+          <t>2026-07-20T15:33:52.295961Z</t>
         </is>
       </c>
       <c r="BI74" s="24" t="inlineStr">
@@ -18944,16 +18944,16 @@
       </c>
       <c r="BJ74" s="38" t="n"/>
       <c r="BK74" s="26" t="n">
-        <v>-456</v>
+        <v>-144</v>
       </c>
       <c r="BL74" s="39" t="n">
-        <v>1.219298</v>
+        <v>1.694444</v>
       </c>
       <c r="BM74" s="28" t="n">
-        <v>0.820144</v>
+        <v>0.590164</v>
       </c>
       <c r="BN74" s="28" t="n">
-        <v>0.811881</v>
+        <v>0.5870649999999999</v>
       </c>
       <c r="BO74" s="28" t="n"/>
       <c r="BP74" s="38" t="n"/>
@@ -18969,6 +18969,1500 @@
       <c r="BZ74" s="24" t="n"/>
       <c r="CA74" s="31" t="n"/>
     </row>
+    <row r="75" ht="36" customHeight="1">
+      <c r="A75" s="24" t="inlineStr">
+        <is>
+          <t>adfd7bf912a84989</t>
+        </is>
+      </c>
+      <c r="B75" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:38:55.511243Z</t>
+        </is>
+      </c>
+      <c r="C75" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T21:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D75" s="24" t="inlineStr">
+        <is>
+          <t>401816199</t>
+        </is>
+      </c>
+      <c r="E75" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F75" s="24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="G75" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="H75" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I75" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J75" s="38" t="n"/>
+      <c r="K75" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L75" s="26" t="n">
+        <v>-141</v>
+      </c>
+      <c r="M75" s="39" t="n">
+        <v>1.70922</v>
+      </c>
+      <c r="N75" s="28" t="n">
+        <v>0.585062</v>
+      </c>
+      <c r="O75" s="28" t="n">
+        <v>0.592852</v>
+      </c>
+      <c r="P75" s="28" t="n"/>
+      <c r="Q75" s="28" t="n">
+        <v>0.00779</v>
+      </c>
+      <c r="R75" s="26" t="n">
+        <v>24</v>
+      </c>
+      <c r="S75" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T75" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U75" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V75" s="24" t="n"/>
+      <c r="W75" s="26" t="n"/>
+      <c r="X75" s="26" t="n"/>
+      <c r="Y75" s="38" t="n"/>
+      <c r="Z75" s="26" t="n"/>
+      <c r="AA75" s="28" t="n"/>
+      <c r="AB75" s="28" t="n"/>
+      <c r="AC75" s="40" t="n"/>
+      <c r="AD75" s="24" t="n"/>
+      <c r="AE75" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5850 (aec-mlb-cin-sea-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF75" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG75" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH75" s="24" t="n"/>
+      <c r="AI75" s="31" t="n"/>
+      <c r="AJ75" s="31" t="n"/>
+      <c r="AK75" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL75" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM75" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN75" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO75" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP75" s="24" t="inlineStr">
+        <is>
+          <t>mlb-cin</t>
+        </is>
+      </c>
+      <c r="AQ75" s="24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="AR75" s="24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="AS75" s="24" t="inlineStr">
+        <is>
+          <t>mlb-sea</t>
+        </is>
+      </c>
+      <c r="AT75" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AU75" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AV75" s="24" t="n"/>
+      <c r="AW75" s="24" t="n"/>
+      <c r="AX75" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY75" s="24" t="n"/>
+      <c r="AZ75" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA75" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB75" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC75" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD75" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE75" s="24" t="inlineStr">
+        <is>
+          <t>af7ccafcacf69681</t>
+        </is>
+      </c>
+      <c r="BF75" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG75" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH75" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:33:53.701471Z</t>
+        </is>
+      </c>
+      <c r="BI75" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ75" s="38" t="n"/>
+      <c r="BK75" s="26" t="n">
+        <v>-141</v>
+      </c>
+      <c r="BL75" s="39" t="n">
+        <v>1.70922</v>
+      </c>
+      <c r="BM75" s="28" t="n">
+        <v>0.585062</v>
+      </c>
+      <c r="BN75" s="28" t="n">
+        <v>0.58209</v>
+      </c>
+      <c r="BO75" s="28" t="n"/>
+      <c r="BP75" s="38" t="n"/>
+      <c r="BQ75" s="39" t="n"/>
+      <c r="BR75" s="28" t="n"/>
+      <c r="BS75" s="28" t="n"/>
+      <c r="BT75" s="28" t="n"/>
+      <c r="BU75" s="38" t="n"/>
+      <c r="BV75" s="29" t="n"/>
+      <c r="BW75" s="24" t="n"/>
+      <c r="BX75" s="40" t="n"/>
+      <c r="BY75" s="39" t="n"/>
+      <c r="BZ75" s="24" t="n"/>
+      <c r="CA75" s="31" t="n"/>
+    </row>
+    <row r="76" ht="36" customHeight="1">
+      <c r="A76" s="24" t="inlineStr">
+        <is>
+          <t>e912f9cec2ac4e02</t>
+        </is>
+      </c>
+      <c r="B76" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:38:55.511243Z</t>
+        </is>
+      </c>
+      <c r="C76" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T22:00:00-0400</t>
+        </is>
+      </c>
+      <c r="D76" s="24" t="inlineStr">
+        <is>
+          <t>401816200</t>
+        </is>
+      </c>
+      <c r="E76" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F76" s="24" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="G76" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="H76" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I76" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J76" s="38" t="n"/>
+      <c r="K76" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L76" s="26" t="n">
+        <v>102</v>
+      </c>
+      <c r="M76" s="39" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="N76" s="28" t="n">
+        <v>0.49505</v>
+      </c>
+      <c r="O76" s="28" t="n">
+        <v>0.52919</v>
+      </c>
+      <c r="P76" s="28" t="n"/>
+      <c r="Q76" s="28" t="n">
+        <v>0.03414</v>
+      </c>
+      <c r="R76" s="26" t="n">
+        <v>37</v>
+      </c>
+      <c r="S76" s="29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T76" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U76" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V76" s="24" t="n"/>
+      <c r="W76" s="26" t="n"/>
+      <c r="X76" s="26" t="n"/>
+      <c r="Y76" s="38" t="n"/>
+      <c r="Z76" s="26" t="n"/>
+      <c r="AA76" s="28" t="n"/>
+      <c r="AB76" s="28" t="n"/>
+      <c r="AC76" s="40" t="n"/>
+      <c r="AD76" s="24" t="n"/>
+      <c r="AE76" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.4950 (aec-mlb-stl-laa-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF76" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG76" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH76" s="24" t="n"/>
+      <c r="AI76" s="31" t="n"/>
+      <c r="AJ76" s="31" t="n"/>
+      <c r="AK76" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL76" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM76" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN76" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO76" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP76" s="24" t="inlineStr">
+        <is>
+          <t>mlb-stl</t>
+        </is>
+      </c>
+      <c r="AQ76" s="24" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="AR76" s="24" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="AS76" s="24" t="inlineStr">
+        <is>
+          <t>mlb-laa</t>
+        </is>
+      </c>
+      <c r="AT76" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="AU76" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="AV76" s="24" t="n"/>
+      <c r="AW76" s="24" t="n"/>
+      <c r="AX76" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY76" s="24" t="n"/>
+      <c r="AZ76" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA76" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BB76" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC76" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD76" s="24" t="inlineStr">
+        <is>
+          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+        </is>
+      </c>
+      <c r="BE76" s="24" t="inlineStr">
+        <is>
+          <t>e8de503e18ea775f</t>
+        </is>
+      </c>
+      <c r="BF76" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG76" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH76" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:33:54.984623Z</t>
+        </is>
+      </c>
+      <c r="BI76" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ76" s="38" t="n"/>
+      <c r="BK76" s="26" t="n">
+        <v>102</v>
+      </c>
+      <c r="BL76" s="39" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="BM76" s="28" t="n">
+        <v>0.49505</v>
+      </c>
+      <c r="BN76" s="28" t="n">
+        <v>0.492537</v>
+      </c>
+      <c r="BO76" s="28" t="n"/>
+      <c r="BP76" s="38" t="n"/>
+      <c r="BQ76" s="39" t="n"/>
+      <c r="BR76" s="28" t="n"/>
+      <c r="BS76" s="28" t="n"/>
+      <c r="BT76" s="28" t="n"/>
+      <c r="BU76" s="38" t="n"/>
+      <c r="BV76" s="29" t="n"/>
+      <c r="BW76" s="24" t="n"/>
+      <c r="BX76" s="40" t="n"/>
+      <c r="BY76" s="39" t="n"/>
+      <c r="BZ76" s="24" t="n"/>
+      <c r="CA76" s="31" t="n"/>
+    </row>
+    <row r="77" ht="36" customHeight="1">
+      <c r="A77" s="24" t="inlineStr">
+        <is>
+          <t>e9767a845c794040</t>
+        </is>
+      </c>
+      <c r="B77" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:39:03.207125Z</t>
+        </is>
+      </c>
+      <c r="C77" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T20:00:00-0400</t>
+        </is>
+      </c>
+      <c r="D77" s="24" t="inlineStr">
+        <is>
+          <t>401857083</t>
+        </is>
+      </c>
+      <c r="E77" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F77" s="24" t="inlineStr">
+        <is>
+          <t>Las Vegas Aces</t>
+        </is>
+      </c>
+      <c r="G77" s="24" t="inlineStr">
+        <is>
+          <t>Toronto Tempo</t>
+        </is>
+      </c>
+      <c r="H77" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I77" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J77" s="38" t="n"/>
+      <c r="K77" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L77" s="26" t="n">
+        <v>-488</v>
+      </c>
+      <c r="M77" s="39" t="n">
+        <v>1.204918</v>
+      </c>
+      <c r="N77" s="28" t="n">
+        <v>0.829932</v>
+      </c>
+      <c r="O77" s="28" t="n">
+        <v>0.6572210000000001</v>
+      </c>
+      <c r="P77" s="28" t="n"/>
+      <c r="Q77" s="28" t="n">
+        <v>-0.172711</v>
+      </c>
+      <c r="R77" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S77" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T77" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U77" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V77" s="24" t="n"/>
+      <c r="W77" s="26" t="n"/>
+      <c r="X77" s="26" t="n"/>
+      <c r="Y77" s="38" t="n"/>
+      <c r="Z77" s="26" t="n"/>
+      <c r="AA77" s="28" t="n"/>
+      <c r="AB77" s="28" t="n"/>
+      <c r="AC77" s="40" t="n"/>
+      <c r="AD77" s="24" t="n"/>
+      <c r="AE77" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5051; executable ask 0.8300 (aec-wnba-lv-tor-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF77" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG77" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH77" s="24" t="n"/>
+      <c r="AI77" s="31" t="n"/>
+      <c r="AJ77" s="31" t="n"/>
+      <c r="AK77" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL77" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM77" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN77" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO77" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP77" s="24" t="inlineStr">
+        <is>
+          <t>wnba-lva</t>
+        </is>
+      </c>
+      <c r="AQ77" s="24" t="inlineStr">
+        <is>
+          <t>Las Vegas Aces</t>
+        </is>
+      </c>
+      <c r="AR77" s="24" t="inlineStr">
+        <is>
+          <t>Las Vegas Aces</t>
+        </is>
+      </c>
+      <c r="AS77" s="24" t="inlineStr">
+        <is>
+          <t>wnba-tor</t>
+        </is>
+      </c>
+      <c r="AT77" s="24" t="inlineStr">
+        <is>
+          <t>Toronto Tempo</t>
+        </is>
+      </c>
+      <c r="AU77" s="24" t="inlineStr">
+        <is>
+          <t>Toronto Tempo</t>
+        </is>
+      </c>
+      <c r="AV77" s="24" t="n"/>
+      <c r="AW77" s="24" t="n"/>
+      <c r="AX77" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY77" s="24" t="n"/>
+      <c r="AZ77" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA77" s="24" t="inlineStr">
+        <is>
+          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+        </is>
+      </c>
+      <c r="BB77" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC77" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD77" s="24" t="inlineStr">
+        <is>
+          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+        </is>
+      </c>
+      <c r="BE77" s="24" t="inlineStr">
+        <is>
+          <t>32740a9f4976946d</t>
+        </is>
+      </c>
+      <c r="BF77" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG77" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH77" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:33:56.676680Z</t>
+        </is>
+      </c>
+      <c r="BI77" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ77" s="38" t="n"/>
+      <c r="BK77" s="26" t="n">
+        <v>-488</v>
+      </c>
+      <c r="BL77" s="39" t="n">
+        <v>1.204918</v>
+      </c>
+      <c r="BM77" s="28" t="n">
+        <v>0.829932</v>
+      </c>
+      <c r="BN77" s="28" t="n">
+        <v>0.821782</v>
+      </c>
+      <c r="BO77" s="28" t="n"/>
+      <c r="BP77" s="38" t="n"/>
+      <c r="BQ77" s="39" t="n"/>
+      <c r="BR77" s="28" t="n"/>
+      <c r="BS77" s="28" t="n"/>
+      <c r="BT77" s="28" t="n"/>
+      <c r="BU77" s="38" t="n"/>
+      <c r="BV77" s="29" t="n"/>
+      <c r="BW77" s="24" t="n"/>
+      <c r="BX77" s="40" t="n"/>
+      <c r="BY77" s="39" t="n"/>
+      <c r="BZ77" s="24" t="n"/>
+      <c r="CA77" s="31" t="n"/>
+    </row>
+    <row r="78" ht="36" customHeight="1">
+      <c r="A78" s="24" t="inlineStr">
+        <is>
+          <t>8e2265c74515471f</t>
+        </is>
+      </c>
+      <c r="B78" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:39:03.207125Z</t>
+        </is>
+      </c>
+      <c r="C78" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T20:00:00-0400</t>
+        </is>
+      </c>
+      <c r="D78" s="24" t="inlineStr">
+        <is>
+          <t>401892393</t>
+        </is>
+      </c>
+      <c r="E78" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F78" s="24" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="G78" s="24" t="inlineStr">
+        <is>
+          <t>Dallas Wings</t>
+        </is>
+      </c>
+      <c r="H78" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I78" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J78" s="38" t="n"/>
+      <c r="K78" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L78" s="26" t="n">
+        <v>156</v>
+      </c>
+      <c r="M78" s="39" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="N78" s="28" t="n">
+        <v>0.390625</v>
+      </c>
+      <c r="O78" s="28" t="n">
+        <v>0.688998</v>
+      </c>
+      <c r="P78" s="28" t="n"/>
+      <c r="Q78" s="28" t="n">
+        <v>0.298373</v>
+      </c>
+      <c r="R78" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S78" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T78" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U78" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V78" s="24" t="n"/>
+      <c r="W78" s="26" t="n"/>
+      <c r="X78" s="26" t="n"/>
+      <c r="Y78" s="38" t="n"/>
+      <c r="Z78" s="26" t="n"/>
+      <c r="AA78" s="28" t="n"/>
+      <c r="AB78" s="28" t="n"/>
+      <c r="AC78" s="40" t="n"/>
+      <c r="AD78" s="24" t="n"/>
+      <c r="AE78" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5051; executable ask 0.3900 (aec-wnba-ny-dal-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF78" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG78" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH78" s="24" t="n"/>
+      <c r="AI78" s="31" t="n"/>
+      <c r="AJ78" s="31" t="n"/>
+      <c r="AK78" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL78" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM78" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN78" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO78" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP78" s="24" t="inlineStr">
+        <is>
+          <t>wnba-nyl</t>
+        </is>
+      </c>
+      <c r="AQ78" s="24" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="AR78" s="24" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="AS78" s="24" t="inlineStr">
+        <is>
+          <t>wnba-dal</t>
+        </is>
+      </c>
+      <c r="AT78" s="24" t="inlineStr">
+        <is>
+          <t>Dallas Wings</t>
+        </is>
+      </c>
+      <c r="AU78" s="24" t="inlineStr">
+        <is>
+          <t>Dallas Wings</t>
+        </is>
+      </c>
+      <c r="AV78" s="24" t="n"/>
+      <c r="AW78" s="24" t="n"/>
+      <c r="AX78" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY78" s="24" t="n"/>
+      <c r="AZ78" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA78" s="24" t="inlineStr">
+        <is>
+          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+        </is>
+      </c>
+      <c r="BB78" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC78" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD78" s="24" t="inlineStr">
+        <is>
+          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+        </is>
+      </c>
+      <c r="BE78" s="24" t="inlineStr">
+        <is>
+          <t>c20bbb99f1fff741</t>
+        </is>
+      </c>
+      <c r="BF78" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG78" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH78" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:33:58.690931Z</t>
+        </is>
+      </c>
+      <c r="BI78" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ78" s="38" t="n"/>
+      <c r="BK78" s="26" t="n">
+        <v>156</v>
+      </c>
+      <c r="BL78" s="39" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="BM78" s="28" t="n">
+        <v>0.390625</v>
+      </c>
+      <c r="BN78" s="28" t="n">
+        <v>0.386139</v>
+      </c>
+      <c r="BO78" s="28" t="n"/>
+      <c r="BP78" s="38" t="n"/>
+      <c r="BQ78" s="39" t="n"/>
+      <c r="BR78" s="28" t="n"/>
+      <c r="BS78" s="28" t="n"/>
+      <c r="BT78" s="28" t="n"/>
+      <c r="BU78" s="38" t="n"/>
+      <c r="BV78" s="29" t="n"/>
+      <c r="BW78" s="24" t="n"/>
+      <c r="BX78" s="40" t="n"/>
+      <c r="BY78" s="39" t="n"/>
+      <c r="BZ78" s="24" t="n"/>
+      <c r="CA78" s="31" t="n"/>
+    </row>
+    <row r="79" ht="36" customHeight="1">
+      <c r="A79" s="24" t="inlineStr">
+        <is>
+          <t>a4f324e828eb4cee</t>
+        </is>
+      </c>
+      <c r="B79" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:39:03.207125Z</t>
+        </is>
+      </c>
+      <c r="C79" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T22:00:00-0400</t>
+        </is>
+      </c>
+      <c r="D79" s="24" t="inlineStr">
+        <is>
+          <t>401857084</t>
+        </is>
+      </c>
+      <c r="E79" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F79" s="24" t="inlineStr">
+        <is>
+          <t>Washington Mystics</t>
+        </is>
+      </c>
+      <c r="G79" s="24" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries</t>
+        </is>
+      </c>
+      <c r="H79" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I79" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J79" s="38" t="n"/>
+      <c r="K79" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L79" s="26" t="n">
+        <v>-317</v>
+      </c>
+      <c r="M79" s="39" t="n">
+        <v>1.315457</v>
+      </c>
+      <c r="N79" s="28" t="n">
+        <v>0.760192</v>
+      </c>
+      <c r="O79" s="28" t="n">
+        <v>0.750463</v>
+      </c>
+      <c r="P79" s="28" t="n"/>
+      <c r="Q79" s="28" t="n">
+        <v>-0.009729</v>
+      </c>
+      <c r="R79" s="26" t="n">
+        <v>15</v>
+      </c>
+      <c r="S79" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T79" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U79" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V79" s="24" t="n"/>
+      <c r="W79" s="26" t="n"/>
+      <c r="X79" s="26" t="n"/>
+      <c r="Y79" s="38" t="n"/>
+      <c r="Z79" s="26" t="n"/>
+      <c r="AA79" s="28" t="n"/>
+      <c r="AB79" s="28" t="n"/>
+      <c r="AC79" s="40" t="n"/>
+      <c r="AD79" s="24" t="n"/>
+      <c r="AE79" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5051; executable ask 0.7600 (aec-wnba-wsh-gsv-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF79" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG79" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH79" s="24" t="n"/>
+      <c r="AI79" s="31" t="n"/>
+      <c r="AJ79" s="31" t="n"/>
+      <c r="AK79" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL79" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM79" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN79" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO79" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP79" s="24" t="inlineStr">
+        <is>
+          <t>wnba-was</t>
+        </is>
+      </c>
+      <c r="AQ79" s="24" t="inlineStr">
+        <is>
+          <t>Washington Mystics</t>
+        </is>
+      </c>
+      <c r="AR79" s="24" t="inlineStr">
+        <is>
+          <t>Washington Mystics</t>
+        </is>
+      </c>
+      <c r="AS79" s="24" t="inlineStr">
+        <is>
+          <t>wnba-gsv</t>
+        </is>
+      </c>
+      <c r="AT79" s="24" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries</t>
+        </is>
+      </c>
+      <c r="AU79" s="24" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries</t>
+        </is>
+      </c>
+      <c r="AV79" s="24" t="n"/>
+      <c r="AW79" s="24" t="n"/>
+      <c r="AX79" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY79" s="24" t="n"/>
+      <c r="AZ79" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA79" s="24" t="inlineStr">
+        <is>
+          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+        </is>
+      </c>
+      <c r="BB79" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC79" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD79" s="24" t="inlineStr">
+        <is>
+          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+        </is>
+      </c>
+      <c r="BE79" s="24" t="inlineStr">
+        <is>
+          <t>a82314f65618b567</t>
+        </is>
+      </c>
+      <c r="BF79" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG79" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH79" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:34:00.890171Z</t>
+        </is>
+      </c>
+      <c r="BI79" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ79" s="38" t="n"/>
+      <c r="BK79" s="26" t="n">
+        <v>-317</v>
+      </c>
+      <c r="BL79" s="39" t="n">
+        <v>1.315457</v>
+      </c>
+      <c r="BM79" s="28" t="n">
+        <v>0.760192</v>
+      </c>
+      <c r="BN79" s="28" t="n">
+        <v>0.752475</v>
+      </c>
+      <c r="BO79" s="28" t="n"/>
+      <c r="BP79" s="38" t="n"/>
+      <c r="BQ79" s="39" t="n"/>
+      <c r="BR79" s="28" t="n"/>
+      <c r="BS79" s="28" t="n"/>
+      <c r="BT79" s="28" t="n"/>
+      <c r="BU79" s="38" t="n"/>
+      <c r="BV79" s="29" t="n"/>
+      <c r="BW79" s="24" t="n"/>
+      <c r="BX79" s="40" t="n"/>
+      <c r="BY79" s="39" t="n"/>
+      <c r="BZ79" s="24" t="n"/>
+      <c r="CA79" s="31" t="n"/>
+    </row>
+    <row r="80" ht="36" customHeight="1">
+      <c r="A80" s="24" t="inlineStr">
+        <is>
+          <t>e010b6ed614649a7</t>
+        </is>
+      </c>
+      <c r="B80" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:39:03.207125Z</t>
+        </is>
+      </c>
+      <c r="C80" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T22:00:00-0400</t>
+        </is>
+      </c>
+      <c r="D80" s="24" t="inlineStr">
+        <is>
+          <t>401857085</t>
+        </is>
+      </c>
+      <c r="E80" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F80" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="G80" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Storm</t>
+        </is>
+      </c>
+      <c r="H80" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I80" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J80" s="38" t="n"/>
+      <c r="K80" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L80" s="26" t="n">
+        <v>-456</v>
+      </c>
+      <c r="M80" s="39" t="n">
+        <v>1.219298</v>
+      </c>
+      <c r="N80" s="28" t="n">
+        <v>0.820144</v>
+      </c>
+      <c r="O80" s="28" t="n">
+        <v>0.738843</v>
+      </c>
+      <c r="P80" s="28" t="n"/>
+      <c r="Q80" s="28" t="n">
+        <v>-0.081301</v>
+      </c>
+      <c r="R80" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S80" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T80" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U80" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V80" s="24" t="n"/>
+      <c r="W80" s="26" t="n"/>
+      <c r="X80" s="26" t="n"/>
+      <c r="Y80" s="38" t="n"/>
+      <c r="Z80" s="26" t="n"/>
+      <c r="AA80" s="28" t="n"/>
+      <c r="AB80" s="28" t="n"/>
+      <c r="AC80" s="40" t="n"/>
+      <c r="AD80" s="24" t="n"/>
+      <c r="AE80" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5051; executable ask 0.8200 (aec-wnba-min-sea-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF80" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG80" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH80" s="24" t="n"/>
+      <c r="AI80" s="31" t="n"/>
+      <c r="AJ80" s="31" t="n"/>
+      <c r="AK80" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL80" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM80" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN80" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO80" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP80" s="24" t="inlineStr">
+        <is>
+          <t>wnba-min</t>
+        </is>
+      </c>
+      <c r="AQ80" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="AR80" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="AS80" s="24" t="inlineStr">
+        <is>
+          <t>wnba-sea</t>
+        </is>
+      </c>
+      <c r="AT80" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Storm</t>
+        </is>
+      </c>
+      <c r="AU80" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Storm</t>
+        </is>
+      </c>
+      <c r="AV80" s="24" t="n"/>
+      <c r="AW80" s="24" t="n"/>
+      <c r="AX80" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY80" s="24" t="n"/>
+      <c r="AZ80" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA80" s="24" t="inlineStr">
+        <is>
+          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+        </is>
+      </c>
+      <c r="BB80" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC80" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD80" s="24" t="inlineStr">
+        <is>
+          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+        </is>
+      </c>
+      <c r="BE80" s="24" t="inlineStr">
+        <is>
+          <t>c7928758cc04b6e5</t>
+        </is>
+      </c>
+      <c r="BF80" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG80" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH80" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T15:34:01.619683Z</t>
+        </is>
+      </c>
+      <c r="BI80" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ80" s="38" t="n"/>
+      <c r="BK80" s="26" t="n">
+        <v>-456</v>
+      </c>
+      <c r="BL80" s="39" t="n">
+        <v>1.219298</v>
+      </c>
+      <c r="BM80" s="28" t="n">
+        <v>0.820144</v>
+      </c>
+      <c r="BN80" s="28" t="n">
+        <v>0.811881</v>
+      </c>
+      <c r="BO80" s="28" t="n"/>
+      <c r="BP80" s="38" t="n"/>
+      <c r="BQ80" s="39" t="n"/>
+      <c r="BR80" s="28" t="n"/>
+      <c r="BS80" s="28" t="n"/>
+      <c r="BT80" s="28" t="n"/>
+      <c r="BU80" s="38" t="n"/>
+      <c r="BV80" s="29" t="n"/>
+      <c r="BW80" s="24" t="n"/>
+      <c r="BX80" s="40" t="n"/>
+      <c r="BY80" s="39" t="n"/>
+      <c r="BZ80" s="24" t="n"/>
+      <c r="CA80" s="31" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
fix: esports selection can be home or away, --all includes esports
- _log_esports_forecast: selection now reflects which Polymarket
  contract side we're picking. home_team/away_team follow contract's
  teams ordering; selection='home' or 'away' accordingly.
- Example: INTZ e-Sports @ 7REX, pick=away (7REX is away side)
- forecast --all / flat-forecast --all now includes lol/cs2 titles
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -20435,12 +20435,12 @@
     <row r="81" ht="36" customHeight="1">
       <c r="A81" s="24" t="inlineStr">
         <is>
-          <t>1a48e42752fa4d4d</t>
+          <t>9a9d4b57a88e423c</t>
         </is>
       </c>
       <c r="B81" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:23.198474Z</t>
+          <t>2026-07-20T16:47:44.302889Z</t>
         </is>
       </c>
       <c r="C81" s="24" t="inlineStr">
@@ -20646,7 +20646,7 @@
       </c>
       <c r="BH81" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:23.198474Z</t>
+          <t>2026-07-20T16:47:44.302889Z</t>
         </is>
       </c>
       <c r="BI81" s="24" t="inlineStr">
@@ -20682,12 +20682,12 @@
     <row r="82" ht="36" customHeight="1">
       <c r="A82" s="24" t="inlineStr">
         <is>
-          <t>c8a2ce99ec2b4bb4</t>
+          <t>3317c6b205ce46df</t>
         </is>
       </c>
       <c r="B82" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:23.412348Z</t>
+          <t>2026-07-20T16:47:44.584921Z</t>
         </is>
       </c>
       <c r="C82" s="24" t="inlineStr">
@@ -20707,14 +20707,14 @@
       </c>
       <c r="F82" s="24" t="inlineStr">
         <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="G82" s="24" t="inlineStr">
+        <is>
           <t>INTZ e-Sports</t>
         </is>
       </c>
-      <c r="G82" s="24" t="inlineStr">
-        <is>
-          <t>7REX</t>
-        </is>
-      </c>
       <c r="H82" s="24" t="inlineStr">
         <is>
           <t>moneyline</t>
@@ -20722,7 +20722,7 @@
       </c>
       <c r="I82" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J82" s="25" t="n"/>
@@ -20815,32 +20815,32 @@
       </c>
       <c r="AP82" s="24" t="inlineStr">
         <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="AQ82" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="AR82" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="AS82" s="24" t="inlineStr">
+        <is>
           <t>INTZ e-Sports</t>
         </is>
       </c>
-      <c r="AQ82" s="24" t="inlineStr">
+      <c r="AT82" s="24" t="inlineStr">
         <is>
           <t>INTZ e-Sports</t>
         </is>
       </c>
-      <c r="AR82" s="24" t="inlineStr">
+      <c r="AU82" s="24" t="inlineStr">
         <is>
           <t>INTZ e-Sports</t>
-        </is>
-      </c>
-      <c r="AS82" s="24" t="inlineStr">
-        <is>
-          <t>7REX</t>
-        </is>
-      </c>
-      <c r="AT82" s="24" t="inlineStr">
-        <is>
-          <t>7REX</t>
-        </is>
-      </c>
-      <c r="AU82" s="24" t="inlineStr">
-        <is>
-          <t>7REX</t>
         </is>
       </c>
       <c r="AV82" s="24" t="n"/>
@@ -20893,7 +20893,7 @@
       </c>
       <c r="BH82" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:23.412348Z</t>
+          <t>2026-07-20T16:47:44.584921Z</t>
         </is>
       </c>
       <c r="BI82" s="24" t="inlineStr">
@@ -20929,12 +20929,12 @@
     <row r="83" ht="36" customHeight="1">
       <c r="A83" s="24" t="inlineStr">
         <is>
-          <t>59e23c595c724c2d</t>
+          <t>e255a57d46ac4478</t>
         </is>
       </c>
       <c r="B83" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:23.600706Z</t>
+          <t>2026-07-20T16:47:44.797663Z</t>
         </is>
       </c>
       <c r="C83" s="24" t="inlineStr">
@@ -20954,14 +20954,14 @@
       </c>
       <c r="F83" s="24" t="inlineStr">
         <is>
+          <t>RMD Gaming</t>
+        </is>
+      </c>
+      <c r="G83" s="24" t="inlineStr">
+        <is>
           <t>Team Solid</t>
         </is>
       </c>
-      <c r="G83" s="24" t="inlineStr">
-        <is>
-          <t>RMD Gaming</t>
-        </is>
-      </c>
       <c r="H83" s="24" t="inlineStr">
         <is>
           <t>moneyline</t>
@@ -20969,7 +20969,7 @@
       </c>
       <c r="I83" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J83" s="25" t="n"/>
@@ -21062,32 +21062,32 @@
       </c>
       <c r="AP83" s="24" t="inlineStr">
         <is>
+          <t>RMD Gaming</t>
+        </is>
+      </c>
+      <c r="AQ83" s="24" t="inlineStr">
+        <is>
+          <t>RMD Gaming</t>
+        </is>
+      </c>
+      <c r="AR83" s="24" t="inlineStr">
+        <is>
+          <t>RMD Gaming</t>
+        </is>
+      </c>
+      <c r="AS83" s="24" t="inlineStr">
+        <is>
           <t>Team Solid</t>
         </is>
       </c>
-      <c r="AQ83" s="24" t="inlineStr">
+      <c r="AT83" s="24" t="inlineStr">
         <is>
           <t>Team Solid</t>
         </is>
       </c>
-      <c r="AR83" s="24" t="inlineStr">
+      <c r="AU83" s="24" t="inlineStr">
         <is>
           <t>Team Solid</t>
-        </is>
-      </c>
-      <c r="AS83" s="24" t="inlineStr">
-        <is>
-          <t>RMD Gaming</t>
-        </is>
-      </c>
-      <c r="AT83" s="24" t="inlineStr">
-        <is>
-          <t>RMD Gaming</t>
-        </is>
-      </c>
-      <c r="AU83" s="24" t="inlineStr">
-        <is>
-          <t>RMD Gaming</t>
         </is>
       </c>
       <c r="AV83" s="24" t="n"/>
@@ -21140,7 +21140,7 @@
       </c>
       <c r="BH83" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:23.600706Z</t>
+          <t>2026-07-20T16:47:44.797663Z</t>
         </is>
       </c>
       <c r="BI83" s="24" t="inlineStr">
@@ -21176,12 +21176,12 @@
     <row r="84" ht="36" customHeight="1">
       <c r="A84" s="24" t="inlineStr">
         <is>
-          <t>13b3d8aeb7054f14</t>
+          <t>5eb5e85b3a8f4197</t>
         </is>
       </c>
       <c r="B84" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:29.969000Z</t>
+          <t>2026-07-20T16:47:49.894690Z</t>
         </is>
       </c>
       <c r="C84" s="24" t="inlineStr">
@@ -21387,7 +21387,7 @@
       </c>
       <c r="BH84" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:29.969000Z</t>
+          <t>2026-07-20T16:47:49.894690Z</t>
         </is>
       </c>
       <c r="BI84" s="24" t="inlineStr">
@@ -21423,12 +21423,12 @@
     <row r="85" ht="36" customHeight="1">
       <c r="A85" s="24" t="inlineStr">
         <is>
-          <t>b56aaa797c2a4200</t>
+          <t>081d51f5bea5463a</t>
         </is>
       </c>
       <c r="B85" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:30.199856Z</t>
+          <t>2026-07-20T16:47:50.137639Z</t>
         </is>
       </c>
       <c r="C85" s="24" t="inlineStr">
@@ -21634,7 +21634,7 @@
       </c>
       <c r="BH85" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:43:30.199856Z</t>
+          <t>2026-07-20T16:47:50.137639Z</t>
         </is>
       </c>
       <c r="BI85" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Dota2 + LOL v3 tiered-elo models
- Dota2: K=32 th=0.18 (14,509 matches, 1,809 teams)
- LOL: K=32 th=0.20 (11,916 matches, 675 teams)
- Updated model.yaml to v3 for both
- Reran all Dota2 (9 picks) and LOL (33 picks) with v3 predictions
- CS2/LOL/Dota2 all on v3 tiered-elo now
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -1805,11 +1805,11 @@
         <v>0.65035</v>
       </c>
       <c r="O4" t="n">
-        <v>0.567916</v>
+        <v>0.537085</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>-0.08243399999999999</v>
+        <v>-0.113265</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="BA4" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB4" t="inlineStr">
@@ -2053,11 +2053,11 @@
         <v>0.640288</v>
       </c>
       <c r="O5" t="n">
-        <v>0.57491</v>
+        <v>0.471633</v>
       </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>-0.06537800000000001</v>
+        <v>-0.168655</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="BA5" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB5" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>-0.180511</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>dota2-neutral-series-elo-v2</t>
+          <t>dota2-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -3795,11 +3795,11 @@
         <v>0.420168</v>
       </c>
       <c r="O12" t="n">
-        <v>0.583304</v>
+        <v>0.5</v>
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>0.163136</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
         <v>100</v>
@@ -3809,7 +3809,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>dota2-neutral-series-elo-v2</t>
+          <t>dota2-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -4043,11 +4043,11 @@
         <v>0.4</v>
       </c>
       <c r="O13" t="n">
-        <v>0.625394</v>
+        <v>0.5</v>
       </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>0.225394</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
         <v>100</v>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>dota2-neutral-series-elo-v2</t>
+          <t>dota2-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>0.119772</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
         <v>100</v>
@@ -4305,7 +4305,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>dota2-neutral-series-elo-v2</t>
+          <t>dota2-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>-0.169967</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -4553,7 +4553,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>dota2-neutral-series-elo-v2</t>
+          <t>dota2-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -7267,11 +7267,11 @@
         <v>0.539171</v>
       </c>
       <c r="O26" t="n">
-        <v>0.625647</v>
+        <v>0.700126</v>
       </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="n">
-        <v>0.086476</v>
+        <v>0.160955</v>
       </c>
       <c r="R26" t="n">
         <v>63</v>
@@ -7281,7 +7281,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="BA26" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB26" t="inlineStr">
@@ -7515,11 +7515,11 @@
         <v>0.619772</v>
       </c>
       <c r="O27" t="n">
-        <v>0.651459</v>
+        <v>0.769629</v>
       </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="n">
-        <v>0.031687</v>
+        <v>0.149857</v>
       </c>
       <c r="R27" t="n">
         <v>36</v>
@@ -7529,7 +7529,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="BA27" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB27" t="inlineStr">
@@ -7763,11 +7763,11 @@
         <v>0.6997</v>
       </c>
       <c r="O28" t="n">
-        <v>0.6156779999999999</v>
+        <v>0.651112</v>
       </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="n">
-        <v>-0.084022</v>
+        <v>-0.048588</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
@@ -7777,7 +7777,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="BA28" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB28" t="inlineStr">
@@ -8011,11 +8011,11 @@
         <v>0.309598</v>
       </c>
       <c r="O29" t="n">
-        <v>0.549502</v>
+        <v>0.600415</v>
       </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="n">
-        <v>0.239904</v>
+        <v>0.290817</v>
       </c>
       <c r="R29" t="n">
         <v>100</v>
@@ -8025,7 +8025,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="BA29" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB29" t="inlineStr">
@@ -8259,11 +8259,11 @@
         <v>0.420168</v>
       </c>
       <c r="O30" t="n">
-        <v>0.589489</v>
+        <v>0.589971</v>
       </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="n">
-        <v>0.169321</v>
+        <v>0.169803</v>
       </c>
       <c r="R30" t="n">
         <v>100</v>
@@ -8273,7 +8273,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -8376,7 +8376,7 @@
       </c>
       <c r="BA30" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB30" t="inlineStr">
@@ -8507,11 +8507,11 @@
         <v>0.6</v>
       </c>
       <c r="O31" t="n">
-        <v>0.689025</v>
+        <v>0.662969</v>
       </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="n">
-        <v>0.08902500000000001</v>
+        <v>0.062969</v>
       </c>
       <c r="R31" t="n">
         <v>65</v>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="BA31" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB31" t="inlineStr">
@@ -8755,11 +8755,11 @@
         <v>0.54955</v>
       </c>
       <c r="O32" t="n">
-        <v>0.501696</v>
+        <v>0.556402</v>
       </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="n">
-        <v>-0.047854</v>
+        <v>0.006852</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -8769,7 +8769,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -8872,7 +8872,7 @@
       </c>
       <c r="BA32" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB32" t="inlineStr">
@@ -9003,11 +9003,11 @@
         <v>0.669967</v>
       </c>
       <c r="O33" t="n">
-        <v>0.612384</v>
+        <v>0.7733100000000001</v>
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="n">
-        <v>-0.057583</v>
+        <v>0.103343</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -9017,7 +9017,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v2</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -9120,7 +9120,7 @@
       </c>
       <c r="BA33" t="inlineStr">
         <is>
-          <t>daa3fc90ca4593e2a301d3702bff6f84e813dc20ca7f7c0733d1637d80aeadf8</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB33" t="inlineStr">
@@ -10023,11 +10023,11 @@
         <v>0.579832</v>
       </c>
       <c r="O37" t="n">
-        <v>0.577373</v>
+        <v>0.5</v>
       </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="n">
-        <v>-0.002627</v>
+        <v>0</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -10037,7 +10037,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>dota2-neutral-series-elo-v1</t>
+          <t>dota2-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -13429,11 +13429,11 @@
         <v>0.6997</v>
       </c>
       <c r="O50" t="n">
-        <v>0.704201</v>
+        <v>0.6887720000000001</v>
       </c>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="n">
-        <v>0.004201</v>
+        <v>-0.010928</v>
       </c>
       <c r="R50" t="n">
         <v>4</v>
@@ -13443,7 +13443,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -13560,7 +13560,7 @@
       </c>
       <c r="BA50" t="inlineStr">
         <is>
-          <t>82612f1b27d5065af8d70fd6669509ff00dc1c7e3a91bb423192bf3b0a9736ce</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB50" t="inlineStr">
@@ -13691,11 +13691,11 @@
         <v>0.659864</v>
       </c>
       <c r="O51" t="n">
-        <v>0.603723</v>
+        <v>0.5767600000000001</v>
       </c>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="n">
-        <v>-0.056277</v>
+        <v>-0.083104</v>
       </c>
       <c r="R51" t="n">
         <v>0</v>
@@ -13705,7 +13705,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -13822,7 +13822,7 @@
       </c>
       <c r="BA51" t="inlineStr">
         <is>
-          <t>82612f1b27d5065af8d70fd6669509ff00dc1c7e3a91bb423192bf3b0a9736ce</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB51" t="inlineStr">
@@ -13953,11 +13953,11 @@
         <v>0.320513</v>
       </c>
       <c r="O52" t="n">
-        <v>0.59232</v>
+        <v>0.563621</v>
       </c>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="n">
-        <v>0.27232</v>
+        <v>0.243108</v>
       </c>
       <c r="R52" t="n">
         <v>100</v>
@@ -13967,7 +13967,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -14084,7 +14084,7 @@
       </c>
       <c r="BA52" t="inlineStr">
         <is>
-          <t>82612f1b27d5065af8d70fd6669509ff00dc1c7e3a91bb423192bf3b0a9736ce</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB52" t="inlineStr">
@@ -14215,11 +14215,11 @@
         <v>0.669967</v>
       </c>
       <c r="O53" t="n">
-        <v>0.731785</v>
+        <v>0.753541</v>
       </c>
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="n">
-        <v>0.061785</v>
+        <v>0.083574</v>
       </c>
       <c r="R53" t="n">
         <v>61</v>
@@ -14229,7 +14229,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -14346,7 +14346,7 @@
       </c>
       <c r="BA53" t="inlineStr">
         <is>
-          <t>82612f1b27d5065af8d70fd6669509ff00dc1c7e3a91bb423192bf3b0a9736ce</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB53" t="inlineStr">
@@ -14477,11 +14477,11 @@
         <v>0.659864</v>
       </c>
       <c r="O54" t="n">
-        <v>0.748054</v>
+        <v>0.8542149999999999</v>
       </c>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="n">
-        <v>0.08805399999999999</v>
+        <v>0.194351</v>
       </c>
       <c r="R54" t="n">
         <v>88</v>
@@ -14491,7 +14491,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="BA54" t="inlineStr">
         <is>
-          <t>82612f1b27d5065af8d70fd6669509ff00dc1c7e3a91bb423192bf3b0a9736ce</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB54" t="inlineStr">
@@ -14739,11 +14739,11 @@
         <v>0.469484</v>
       </c>
       <c r="O55" t="n">
-        <v>0.503502</v>
+        <v>0.5</v>
       </c>
       <c r="P55" t="inlineStr"/>
       <c r="Q55" t="n">
-        <v>0.033502</v>
+        <v>0</v>
       </c>
       <c r="R55" t="n">
         <v>33</v>
@@ -14753,7 +14753,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -15001,11 +15001,11 @@
         <v>0.65035</v>
       </c>
       <c r="O56" t="n">
-        <v>0.650024</v>
+        <v>0.616388</v>
       </c>
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="n">
-        <v>2.4e-05</v>
+        <v>-0.033962</v>
       </c>
       <c r="R56" t="n">
         <v>0</v>
@@ -15015,7 +15015,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="BA56" t="inlineStr">
         <is>
-          <t>82612f1b27d5065af8d70fd6669509ff00dc1c7e3a91bb423192bf3b0a9736ce</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB56" t="inlineStr">
@@ -15263,11 +15263,11 @@
         <v>0.590164</v>
       </c>
       <c r="O57" t="n">
-        <v>0.650242</v>
+        <v>0.615103</v>
       </c>
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="n">
-        <v>0.060242</v>
+        <v>0.024939</v>
       </c>
       <c r="R57" t="n">
         <v>60</v>
@@ -15277,7 +15277,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -15394,7 +15394,7 @@
       </c>
       <c r="BA57" t="inlineStr">
         <is>
-          <t>82612f1b27d5065af8d70fd6669509ff00dc1c7e3a91bb423192bf3b0a9736ce</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB57" t="inlineStr">
@@ -15525,11 +15525,11 @@
         <v>0.340136</v>
       </c>
       <c r="O58" t="n">
-        <v>0.75</v>
+        <v>0.958215</v>
       </c>
       <c r="P58" t="inlineStr"/>
       <c r="Q58" t="n">
-        <v>0.41</v>
+        <v>0.618079</v>
       </c>
       <c r="R58" t="n">
         <v>100</v>
@@ -15539,7 +15539,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -15656,7 +15656,7 @@
       </c>
       <c r="BA58" t="inlineStr">
         <is>
-          <t>82612f1b27d5065af8d70fd6669509ff00dc1c7e3a91bb423192bf3b0a9736ce</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB58" t="inlineStr">
@@ -15787,11 +15787,11 @@
         <v>0.409836</v>
       </c>
       <c r="O59" t="n">
-        <v>0.7499980000000001</v>
+        <v>0.933732</v>
       </c>
       <c r="P59" t="inlineStr"/>
       <c r="Q59" t="n">
-        <v>0.339998</v>
+        <v>0.523896</v>
       </c>
       <c r="R59" t="n">
         <v>100</v>
@@ -15801,7 +15801,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>lol-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -15918,7 +15918,7 @@
       </c>
       <c r="BA59" t="inlineStr">
         <is>
-          <t>82612f1b27d5065af8d70fd6669509ff00dc1c7e3a91bb423192bf3b0a9736ce</t>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
         </is>
       </c>
       <c r="BB59" t="inlineStr">

</xml_diff>

<commit_message>
Valorant v3 tiered-elo. All 4 esports now on v3
CS2: K=96 th=0.20 | Dota2: K=32 th=0.18 | LOL: K=32 th=0.20 | Valorant: K=32 th=0.20
All use dual-threshold: flat=0.0 (research), main=gated (edge>=0.02 + confidence)
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -3055,7 +3055,7 @@
       </c>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>-0.070815</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>valorant-neutral-series-elo-v2</t>
+          <t>valorant-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>-0.059471</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>valorant-neutral-series-elo-v2</t>
+          <t>valorant-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -9255,7 +9255,7 @@
       </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="n">
-        <v>-0.17</v>
+        <v>0</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -9265,7 +9265,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>valorant-neutral-series-elo-v1</t>
+          <t>valorant-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="n">
-        <v>-0.19</v>
+        <v>0</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -9513,7 +9513,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>valorant-neutral-series-elo-v1</t>
+          <t>valorant-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -9765,7 +9765,7 @@
       </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="n">
-        <v>-0.09</v>
+        <v>0</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -9775,7 +9775,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>valorant-neutral-series-elo-v1</t>
+          <t>valorant-tiered-elo-v3</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">

</xml_diff>

<commit_message>
Finalize: per-sport gates, v3 esports, MLB+LOL gate=0.00, all ledgers synced
Flat: 105 settled, -0.84U (research, call all)
Main: 91 settled, +5.99U (edge-gated, +6.83U vs flat)
MLB: 70p +6.23U | LOL: 17p +0.50U | CS2: 2p -0.50U
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CB126" headerRowCount="1">
-  <autoFilter ref="A1:CB126"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CB137" headerRowCount="1">
+  <autoFilter ref="A1:CB137"/>
   <tableColumns count="80">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -739,19 +739,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$126)</f>
+        <f>COUNTA('Picks'!$A$2:$A$137)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$126,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$137,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$126,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$137,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$126,"settled",'Picks'!$V$2:$V$126,"win")+COUNTIFS('Picks'!$U$2:$U$126,"settled",'Picks'!$V$2:$V$126,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$137,"settled",'Picks'!$V$2:$V$137,"win")+COUNTIFS('Picks'!$U$2:$U$137,"settled",'Picks'!$V$2:$V$137,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -779,19 +779,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$126,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$137,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$126,"&gt;0",'Picks'!$V$2:$V$126,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$126,"&gt;0",'Picks'!$V$2:$V$126,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$137,"&gt;0",'Picks'!$V$2:$V$137,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$137,"&gt;0",'Picks'!$V$2:$V$137,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$126,"&gt;0",'Picks'!$V$2:$V$126,"win")/(COUNTIFS('Picks'!$BX$2:$BX$126,"&gt;0",'Picks'!$V$2:$V$126,"win")+COUNTIFS('Picks'!$BX$2:$BX$126,"&gt;0",'Picks'!$V$2:$V$126,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$137,"&gt;0",'Picks'!$V$2:$V$137,"win")/(COUNTIFS('Picks'!$BX$2:$BX$137,"&gt;0",'Picks'!$V$2:$V$137,"win")+COUNTIFS('Picks'!$BX$2:$BX$137,"&gt;0",'Picks'!$V$2:$V$137,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$126)/SUM('Picks'!$BX$2:$BX$126),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$137)/SUM('Picks'!$BX$2:$BX$137),0)</f>
         <v/>
       </c>
     </row>
@@ -819,19 +819,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$126)</f>
+        <f>SUM('Picks'!$BY$2:$BY$137)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$126,"&lt;&gt;",'Picks'!$AB$2:$AB$126),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$137,"&lt;&gt;",'Picks'!$AB$2:$AB$137),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$126,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$126,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$137,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$137,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$126,'Picks'!$AM$2:$AM$126,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$137,'Picks'!$AM$2:$AM$137,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -886,15 +886,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$126,$A14,'Picks'!$U$2:$U$126,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$137,$A14,'Picks'!$U$2:$U$137,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$126,$A14,'Picks'!$U$2:$U$126,"settled",'Picks'!$V$2:$V$126,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$137,$A14,'Picks'!$U$2:$U$137,"settled",'Picks'!$V$2:$V$137,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$126,$A14,'Picks'!$U$2:$U$126,"settled",'Picks'!$V$2:$V$126,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$137,$A14,'Picks'!$U$2:$U$137,"settled",'Picks'!$V$2:$V$137,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -902,11 +902,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$126,'Picks'!$H$2:$H$126,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$137,'Picks'!$H$2:$H$137,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$126,'Picks'!$H$2:$H$126,$A14,'Picks'!$U$2:$U$126,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$137,'Picks'!$H$2:$H$137,$A14,'Picks'!$U$2:$U$137,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -917,15 +917,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$126,$A15,'Picks'!$U$2:$U$126,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$137,$A15,'Picks'!$U$2:$U$137,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$126,$A15,'Picks'!$U$2:$U$126,"settled",'Picks'!$V$2:$V$126,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$137,$A15,'Picks'!$U$2:$U$137,"settled",'Picks'!$V$2:$V$137,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$126,$A15,'Picks'!$U$2:$U$126,"settled",'Picks'!$V$2:$V$126,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$137,$A15,'Picks'!$U$2:$U$137,"settled",'Picks'!$V$2:$V$137,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -933,11 +933,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$126,'Picks'!$H$2:$H$126,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$137,'Picks'!$H$2:$H$137,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$126,'Picks'!$H$2:$H$126,$A15,'Picks'!$U$2:$U$126,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$137,'Picks'!$H$2:$H$137,$A15,'Picks'!$U$2:$U$137,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -948,15 +948,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$126,$A16,'Picks'!$U$2:$U$126,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$137,$A16,'Picks'!$U$2:$U$137,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$126,$A16,'Picks'!$U$2:$U$126,"settled",'Picks'!$V$2:$V$126,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$137,$A16,'Picks'!$U$2:$U$137,"settled",'Picks'!$V$2:$V$137,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$126,$A16,'Picks'!$U$2:$U$126,"settled",'Picks'!$V$2:$V$126,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$137,$A16,'Picks'!$U$2:$U$137,"settled",'Picks'!$V$2:$V$137,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -964,11 +964,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$126,'Picks'!$H$2:$H$126,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$137,'Picks'!$H$2:$H$137,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$126,'Picks'!$H$2:$H$126,$A16,'Picks'!$U$2:$U$126,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$137,'Picks'!$H$2:$H$137,$A16,'Picks'!$U$2:$U$137,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CB126"/>
+  <dimension ref="A1:CB137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -33748,6 +33748,2734 @@
       <c r="CA126" s="31" t="n"/>
       <c r="CB126" s="24" t="n"/>
     </row>
+    <row r="127" ht="36" customHeight="1">
+      <c r="A127" s="24" t="inlineStr">
+        <is>
+          <t>d487a54363744159</t>
+        </is>
+      </c>
+      <c r="B127" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C127" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T09:00:00Z</t>
+        </is>
+      </c>
+      <c r="D127" s="24" t="inlineStr">
+        <is>
+          <t>55954</t>
+        </is>
+      </c>
+      <c r="E127" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F127" s="24" t="inlineStr">
+        <is>
+          <t>EDward Gaming</t>
+        </is>
+      </c>
+      <c r="G127" s="24" t="inlineStr">
+        <is>
+          <t>LGD Gaming</t>
+        </is>
+      </c>
+      <c r="H127" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I127" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J127" s="25" t="n"/>
+      <c r="K127" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L127" s="26" t="n">
+        <v>-122</v>
+      </c>
+      <c r="M127" s="27" t="n">
+        <v>1.819672</v>
+      </c>
+      <c r="N127" s="28" t="n">
+        <v>0.54955</v>
+      </c>
+      <c r="O127" s="28" t="n">
+        <v>0.528201</v>
+      </c>
+      <c r="P127" s="28" t="n"/>
+      <c r="Q127" s="28" t="n">
+        <v>-0.021349</v>
+      </c>
+      <c r="R127" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="S127" s="29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T127" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U127" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V127" s="24" t="n"/>
+      <c r="W127" s="26" t="n"/>
+      <c r="X127" s="26" t="n"/>
+      <c r="Y127" s="25" t="n"/>
+      <c r="Z127" s="26" t="n"/>
+      <c r="AA127" s="28" t="n"/>
+      <c r="AB127" s="28" t="n"/>
+      <c r="AC127" s="30" t="n"/>
+      <c r="AD127" s="24" t="n"/>
+      <c r="AE127" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5500 (market_slug=aec-lol-lgd-edg-2026-07-22).</t>
+        </is>
+      </c>
+      <c r="AF127" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG127" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH127" s="24" t="n"/>
+      <c r="AI127" s="31" t="n"/>
+      <c r="AJ127" s="31" t="n"/>
+      <c r="AK127" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL127" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM127" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN127" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO127" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP127" s="24" t="inlineStr">
+        <is>
+          <t>EDward Gaming</t>
+        </is>
+      </c>
+      <c r="AQ127" s="24" t="inlineStr">
+        <is>
+          <t>EDward Gaming</t>
+        </is>
+      </c>
+      <c r="AR127" s="24" t="inlineStr">
+        <is>
+          <t>EDward Gaming</t>
+        </is>
+      </c>
+      <c r="AS127" s="24" t="inlineStr">
+        <is>
+          <t>LGD Gaming</t>
+        </is>
+      </c>
+      <c r="AT127" s="24" t="inlineStr">
+        <is>
+          <t>LGD Gaming</t>
+        </is>
+      </c>
+      <c r="AU127" s="24" t="inlineStr">
+        <is>
+          <t>LGD Gaming</t>
+        </is>
+      </c>
+      <c r="AV127" s="24" t="n"/>
+      <c r="AW127" s="24" t="n"/>
+      <c r="AX127" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY127" s="24" t="n"/>
+      <c r="AZ127" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA127" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB127" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC127" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD127" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE127" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF127" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG127" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH127" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:02.737464Z</t>
+        </is>
+      </c>
+      <c r="BI127" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ127" s="25" t="n"/>
+      <c r="BK127" s="26" t="n">
+        <v>-122</v>
+      </c>
+      <c r="BL127" s="27" t="n">
+        <v>1.819672</v>
+      </c>
+      <c r="BM127" s="28" t="n">
+        <v>0.54955</v>
+      </c>
+      <c r="BN127" s="28" t="n"/>
+      <c r="BO127" s="28" t="n"/>
+      <c r="BP127" s="25" t="n"/>
+      <c r="BQ127" s="27" t="n"/>
+      <c r="BR127" s="28" t="n"/>
+      <c r="BS127" s="28" t="n"/>
+      <c r="BT127" s="28" t="n"/>
+      <c r="BU127" s="25" t="n"/>
+      <c r="BV127" s="29" t="n"/>
+      <c r="BW127" s="24" t="n"/>
+      <c r="BX127" s="30" t="n"/>
+      <c r="BY127" s="27" t="n"/>
+      <c r="BZ127" s="24" t="n"/>
+      <c r="CA127" s="31" t="n"/>
+      <c r="CB127" s="24" t="n"/>
+    </row>
+    <row r="128" ht="36" customHeight="1">
+      <c r="A128" s="24" t="inlineStr">
+        <is>
+          <t>53088914289f4187</t>
+        </is>
+      </c>
+      <c r="B128" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C128" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T11:00:00Z</t>
+        </is>
+      </c>
+      <c r="D128" s="24" t="inlineStr">
+        <is>
+          <t>55996</t>
+        </is>
+      </c>
+      <c r="E128" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F128" s="24" t="inlineStr">
+        <is>
+          <t>Team WE</t>
+        </is>
+      </c>
+      <c r="G128" s="24" t="inlineStr">
+        <is>
+          <t>Top Esports</t>
+        </is>
+      </c>
+      <c r="H128" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I128" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J128" s="25" t="n"/>
+      <c r="K128" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L128" s="26" t="n">
+        <v>-223</v>
+      </c>
+      <c r="M128" s="27" t="n">
+        <v>1.44843</v>
+      </c>
+      <c r="N128" s="28" t="n">
+        <v>0.690402</v>
+      </c>
+      <c r="O128" s="28" t="n">
+        <v>0.636655</v>
+      </c>
+      <c r="P128" s="28" t="n"/>
+      <c r="Q128" s="28" t="n">
+        <v>-0.053747</v>
+      </c>
+      <c r="R128" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S128" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T128" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U128" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V128" s="24" t="n"/>
+      <c r="W128" s="26" t="n"/>
+      <c r="X128" s="26" t="n"/>
+      <c r="Y128" s="25" t="n"/>
+      <c r="Z128" s="26" t="n"/>
+      <c r="AA128" s="28" t="n"/>
+      <c r="AB128" s="28" t="n"/>
+      <c r="AC128" s="30" t="n"/>
+      <c r="AD128" s="24" t="n"/>
+      <c r="AE128" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6900 (market_slug=aec-lol-tes-we-2026-07-22).</t>
+        </is>
+      </c>
+      <c r="AF128" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG128" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH128" s="24" t="n"/>
+      <c r="AI128" s="31" t="n"/>
+      <c r="AJ128" s="31" t="n"/>
+      <c r="AK128" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL128" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM128" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN128" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO128" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP128" s="24" t="inlineStr">
+        <is>
+          <t>Team WE</t>
+        </is>
+      </c>
+      <c r="AQ128" s="24" t="inlineStr">
+        <is>
+          <t>Team WE</t>
+        </is>
+      </c>
+      <c r="AR128" s="24" t="inlineStr">
+        <is>
+          <t>Team WE</t>
+        </is>
+      </c>
+      <c r="AS128" s="24" t="inlineStr">
+        <is>
+          <t>Top Esports</t>
+        </is>
+      </c>
+      <c r="AT128" s="24" t="inlineStr">
+        <is>
+          <t>Top Esports</t>
+        </is>
+      </c>
+      <c r="AU128" s="24" t="inlineStr">
+        <is>
+          <t>Top Esports</t>
+        </is>
+      </c>
+      <c r="AV128" s="24" t="n"/>
+      <c r="AW128" s="24" t="n"/>
+      <c r="AX128" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY128" s="24" t="n"/>
+      <c r="AZ128" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA128" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB128" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC128" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD128" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE128" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF128" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG128" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH128" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:03.510789Z</t>
+        </is>
+      </c>
+      <c r="BI128" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ128" s="25" t="n"/>
+      <c r="BK128" s="26" t="n">
+        <v>-223</v>
+      </c>
+      <c r="BL128" s="27" t="n">
+        <v>1.44843</v>
+      </c>
+      <c r="BM128" s="28" t="n">
+        <v>0.690402</v>
+      </c>
+      <c r="BN128" s="28" t="n"/>
+      <c r="BO128" s="28" t="n"/>
+      <c r="BP128" s="25" t="n"/>
+      <c r="BQ128" s="27" t="n"/>
+      <c r="BR128" s="28" t="n"/>
+      <c r="BS128" s="28" t="n"/>
+      <c r="BT128" s="28" t="n"/>
+      <c r="BU128" s="25" t="n"/>
+      <c r="BV128" s="29" t="n"/>
+      <c r="BW128" s="24" t="n"/>
+      <c r="BX128" s="30" t="n"/>
+      <c r="BY128" s="27" t="n"/>
+      <c r="BZ128" s="24" t="n"/>
+      <c r="CA128" s="31" t="n"/>
+      <c r="CB128" s="24" t="n"/>
+    </row>
+    <row r="129" ht="36" customHeight="1">
+      <c r="A129" s="24" t="inlineStr">
+        <is>
+          <t>71faf50807664dea</t>
+        </is>
+      </c>
+      <c r="B129" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C129" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T17:00:00Z</t>
+        </is>
+      </c>
+      <c r="D129" s="24" t="inlineStr">
+        <is>
+          <t>56126</t>
+        </is>
+      </c>
+      <c r="E129" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F129" s="24" t="inlineStr">
+        <is>
+          <t>GMBLERS ESPORTS</t>
+        </is>
+      </c>
+      <c r="G129" s="24" t="inlineStr">
+        <is>
+          <t>HMBLE</t>
+        </is>
+      </c>
+      <c r="H129" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I129" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J129" s="25" t="n"/>
+      <c r="K129" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L129" s="26" t="n">
+        <v>-233</v>
+      </c>
+      <c r="M129" s="27" t="n">
+        <v>1.429185</v>
+      </c>
+      <c r="N129" s="28" t="n">
+        <v>0.6997</v>
+      </c>
+      <c r="O129" s="28" t="n">
+        <v>0.575556</v>
+      </c>
+      <c r="P129" s="28" t="n"/>
+      <c r="Q129" s="28" t="n">
+        <v>-0.124144</v>
+      </c>
+      <c r="R129" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S129" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T129" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U129" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V129" s="24" t="n"/>
+      <c r="W129" s="26" t="n"/>
+      <c r="X129" s="26" t="n"/>
+      <c r="Y129" s="25" t="n"/>
+      <c r="Z129" s="26" t="n"/>
+      <c r="AA129" s="28" t="n"/>
+      <c r="AB129" s="28" t="n"/>
+      <c r="AC129" s="30" t="n"/>
+      <c r="AD129" s="24" t="n"/>
+      <c r="AE129" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.7000 (market_slug=aec-lol-hmble-gmb-2026-07-22).</t>
+        </is>
+      </c>
+      <c r="AF129" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG129" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH129" s="24" t="n"/>
+      <c r="AI129" s="31" t="n"/>
+      <c r="AJ129" s="31" t="n"/>
+      <c r="AK129" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL129" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM129" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN129" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO129" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP129" s="24" t="inlineStr">
+        <is>
+          <t>GMBLERS ESPORTS</t>
+        </is>
+      </c>
+      <c r="AQ129" s="24" t="inlineStr">
+        <is>
+          <t>GMBLERS ESPORTS</t>
+        </is>
+      </c>
+      <c r="AR129" s="24" t="inlineStr">
+        <is>
+          <t>GMBLERS ESPORTS</t>
+        </is>
+      </c>
+      <c r="AS129" s="24" t="inlineStr">
+        <is>
+          <t>HMBLE</t>
+        </is>
+      </c>
+      <c r="AT129" s="24" t="inlineStr">
+        <is>
+          <t>HMBLE</t>
+        </is>
+      </c>
+      <c r="AU129" s="24" t="inlineStr">
+        <is>
+          <t>HMBLE</t>
+        </is>
+      </c>
+      <c r="AV129" s="24" t="n"/>
+      <c r="AW129" s="24" t="n"/>
+      <c r="AX129" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY129" s="24" t="n"/>
+      <c r="AZ129" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA129" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB129" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC129" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD129" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE129" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF129" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG129" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH129" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:10.295865Z</t>
+        </is>
+      </c>
+      <c r="BI129" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ129" s="25" t="n"/>
+      <c r="BK129" s="26" t="n">
+        <v>-233</v>
+      </c>
+      <c r="BL129" s="27" t="n">
+        <v>1.429185</v>
+      </c>
+      <c r="BM129" s="28" t="n">
+        <v>0.6997</v>
+      </c>
+      <c r="BN129" s="28" t="n"/>
+      <c r="BO129" s="28" t="n"/>
+      <c r="BP129" s="25" t="n"/>
+      <c r="BQ129" s="27" t="n"/>
+      <c r="BR129" s="28" t="n"/>
+      <c r="BS129" s="28" t="n"/>
+      <c r="BT129" s="28" t="n"/>
+      <c r="BU129" s="25" t="n"/>
+      <c r="BV129" s="29" t="n"/>
+      <c r="BW129" s="24" t="n"/>
+      <c r="BX129" s="30" t="n"/>
+      <c r="BY129" s="27" t="n"/>
+      <c r="BZ129" s="24" t="n"/>
+      <c r="CA129" s="31" t="n"/>
+      <c r="CB129" s="24" t="n"/>
+    </row>
+    <row r="130" ht="36" customHeight="1">
+      <c r="A130" s="24" t="inlineStr">
+        <is>
+          <t>f003875538a34221</t>
+        </is>
+      </c>
+      <c r="B130" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C130" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T17:00:00Z</t>
+        </is>
+      </c>
+      <c r="D130" s="24" t="inlineStr">
+        <is>
+          <t>58172</t>
+        </is>
+      </c>
+      <c r="E130" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F130" s="24" t="inlineStr">
+        <is>
+          <t>Unicorns Of Love Sexy Edition</t>
+        </is>
+      </c>
+      <c r="G130" s="24" t="inlineStr">
+        <is>
+          <t>Kaufland Hangry Knights</t>
+        </is>
+      </c>
+      <c r="H130" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I130" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J130" s="25" t="n"/>
+      <c r="K130" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L130" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="M130" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="N130" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="O130" s="28" t="n">
+        <v>0.634815</v>
+      </c>
+      <c r="P130" s="28" t="n"/>
+      <c r="Q130" s="28" t="n">
+        <v>0.015043</v>
+      </c>
+      <c r="R130" s="26" t="n">
+        <v>28</v>
+      </c>
+      <c r="S130" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T130" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U130" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V130" s="24" t="n"/>
+      <c r="W130" s="26" t="n"/>
+      <c r="X130" s="26" t="n"/>
+      <c r="Y130" s="25" t="n"/>
+      <c r="Z130" s="26" t="n"/>
+      <c r="AA130" s="28" t="n"/>
+      <c r="AB130" s="28" t="n"/>
+      <c r="AC130" s="30" t="n"/>
+      <c r="AD130" s="24" t="n"/>
+      <c r="AE130" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-lol-khk-use-2026-07-22).</t>
+        </is>
+      </c>
+      <c r="AF130" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG130" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH130" s="24" t="n"/>
+      <c r="AI130" s="31" t="n"/>
+      <c r="AJ130" s="31" t="n"/>
+      <c r="AK130" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL130" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM130" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN130" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO130" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP130" s="24" t="inlineStr">
+        <is>
+          <t>Unicorns Of Love Sexy Edition</t>
+        </is>
+      </c>
+      <c r="AQ130" s="24" t="inlineStr">
+        <is>
+          <t>Unicorns Of Love Sexy Edition</t>
+        </is>
+      </c>
+      <c r="AR130" s="24" t="inlineStr">
+        <is>
+          <t>Unicorns Of Love Sexy Edition</t>
+        </is>
+      </c>
+      <c r="AS130" s="24" t="inlineStr">
+        <is>
+          <t>Kaufland Hangry Knights</t>
+        </is>
+      </c>
+      <c r="AT130" s="24" t="inlineStr">
+        <is>
+          <t>Kaufland Hangry Knights</t>
+        </is>
+      </c>
+      <c r="AU130" s="24" t="inlineStr">
+        <is>
+          <t>Kaufland Hangry Knights</t>
+        </is>
+      </c>
+      <c r="AV130" s="24" t="n"/>
+      <c r="AW130" s="24" t="n"/>
+      <c r="AX130" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY130" s="24" t="n"/>
+      <c r="AZ130" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA130" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB130" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC130" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD130" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE130" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF130" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG130" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH130" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:11.065754Z</t>
+        </is>
+      </c>
+      <c r="BI130" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ130" s="25" t="n"/>
+      <c r="BK130" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="BL130" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="BM130" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="BN130" s="28" t="n"/>
+      <c r="BO130" s="28" t="n"/>
+      <c r="BP130" s="25" t="n"/>
+      <c r="BQ130" s="27" t="n"/>
+      <c r="BR130" s="28" t="n"/>
+      <c r="BS130" s="28" t="n"/>
+      <c r="BT130" s="28" t="n"/>
+      <c r="BU130" s="25" t="n"/>
+      <c r="BV130" s="29" t="n"/>
+      <c r="BW130" s="24" t="n"/>
+      <c r="BX130" s="30" t="n"/>
+      <c r="BY130" s="27" t="n"/>
+      <c r="BZ130" s="24" t="n"/>
+      <c r="CA130" s="31" t="n"/>
+      <c r="CB130" s="24" t="n"/>
+    </row>
+    <row r="131" ht="36" customHeight="1">
+      <c r="A131" s="24" t="inlineStr">
+        <is>
+          <t>b3933a7255314a9c</t>
+        </is>
+      </c>
+      <c r="B131" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C131" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T17:30:00Z</t>
+        </is>
+      </c>
+      <c r="D131" s="24" t="inlineStr">
+        <is>
+          <t>56127</t>
+        </is>
+      </c>
+      <c r="E131" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F131" s="24" t="inlineStr">
+        <is>
+          <t>UCAM Esports Club</t>
+        </is>
+      </c>
+      <c r="G131" s="24" t="inlineStr">
+        <is>
+          <t>Barça eSports</t>
+        </is>
+      </c>
+      <c r="H131" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I131" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J131" s="25" t="n"/>
+      <c r="K131" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L131" s="26" t="n">
+        <v>-150</v>
+      </c>
+      <c r="M131" s="27" t="n">
+        <v>1.666667</v>
+      </c>
+      <c r="N131" s="28" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="O131" s="28" t="n">
+        <v>0.581485</v>
+      </c>
+      <c r="P131" s="28" t="n"/>
+      <c r="Q131" s="28" t="n">
+        <v>-0.018515</v>
+      </c>
+      <c r="R131" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="S131" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T131" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U131" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V131" s="24" t="n"/>
+      <c r="W131" s="26" t="n"/>
+      <c r="X131" s="26" t="n"/>
+      <c r="Y131" s="25" t="n"/>
+      <c r="Z131" s="26" t="n"/>
+      <c r="AA131" s="28" t="n"/>
+      <c r="AB131" s="28" t="n"/>
+      <c r="AC131" s="30" t="n"/>
+      <c r="AD131" s="24" t="n"/>
+      <c r="AE131" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6000 (market_slug=aec-lol-bar-ucam-2026-07-22).</t>
+        </is>
+      </c>
+      <c r="AF131" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG131" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH131" s="24" t="n"/>
+      <c r="AI131" s="31" t="n"/>
+      <c r="AJ131" s="31" t="n"/>
+      <c r="AK131" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL131" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM131" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN131" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO131" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP131" s="24" t="inlineStr">
+        <is>
+          <t>UCAM Esports Club</t>
+        </is>
+      </c>
+      <c r="AQ131" s="24" t="inlineStr">
+        <is>
+          <t>UCAM Esports Club</t>
+        </is>
+      </c>
+      <c r="AR131" s="24" t="inlineStr">
+        <is>
+          <t>UCAM Esports Club</t>
+        </is>
+      </c>
+      <c r="AS131" s="24" t="inlineStr">
+        <is>
+          <t>Barça eSports</t>
+        </is>
+      </c>
+      <c r="AT131" s="24" t="inlineStr">
+        <is>
+          <t>Barça eSports</t>
+        </is>
+      </c>
+      <c r="AU131" s="24" t="inlineStr">
+        <is>
+          <t>Barça eSports</t>
+        </is>
+      </c>
+      <c r="AV131" s="24" t="n"/>
+      <c r="AW131" s="24" t="n"/>
+      <c r="AX131" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY131" s="24" t="n"/>
+      <c r="AZ131" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA131" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB131" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC131" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD131" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE131" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF131" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG131" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH131" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:11.800383Z</t>
+        </is>
+      </c>
+      <c r="BI131" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ131" s="25" t="n"/>
+      <c r="BK131" s="26" t="n">
+        <v>-150</v>
+      </c>
+      <c r="BL131" s="27" t="n">
+        <v>1.666667</v>
+      </c>
+      <c r="BM131" s="28" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BN131" s="28" t="n"/>
+      <c r="BO131" s="28" t="n"/>
+      <c r="BP131" s="25" t="n"/>
+      <c r="BQ131" s="27" t="n"/>
+      <c r="BR131" s="28" t="n"/>
+      <c r="BS131" s="28" t="n"/>
+      <c r="BT131" s="28" t="n"/>
+      <c r="BU131" s="25" t="n"/>
+      <c r="BV131" s="29" t="n"/>
+      <c r="BW131" s="24" t="n"/>
+      <c r="BX131" s="30" t="n"/>
+      <c r="BY131" s="27" t="n"/>
+      <c r="BZ131" s="24" t="n"/>
+      <c r="CA131" s="31" t="n"/>
+      <c r="CB131" s="24" t="n"/>
+    </row>
+    <row r="132" ht="36" customHeight="1">
+      <c r="A132" s="24" t="inlineStr">
+        <is>
+          <t>69fb3791da444f92</t>
+        </is>
+      </c>
+      <c r="B132" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C132" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="D132" s="24" t="inlineStr">
+        <is>
+          <t>56129</t>
+        </is>
+      </c>
+      <c r="E132" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F132" s="24" t="inlineStr">
+        <is>
+          <t>EKO Esports</t>
+        </is>
+      </c>
+      <c r="G132" s="24" t="inlineStr">
+        <is>
+          <t>TITANS</t>
+        </is>
+      </c>
+      <c r="H132" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I132" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J132" s="25" t="n"/>
+      <c r="K132" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L132" s="26" t="n">
+        <v>133</v>
+      </c>
+      <c r="M132" s="27" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="N132" s="28" t="n">
+        <v>0.429185</v>
+      </c>
+      <c r="O132" s="28" t="n">
+        <v>0.514184</v>
+      </c>
+      <c r="P132" s="28" t="n"/>
+      <c r="Q132" s="28" t="n">
+        <v>0.08499900000000001</v>
+      </c>
+      <c r="R132" s="26" t="n">
+        <v>62</v>
+      </c>
+      <c r="S132" s="29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T132" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U132" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V132" s="24" t="n"/>
+      <c r="W132" s="26" t="n"/>
+      <c r="X132" s="26" t="n"/>
+      <c r="Y132" s="25" t="n"/>
+      <c r="Z132" s="26" t="n"/>
+      <c r="AA132" s="28" t="n"/>
+      <c r="AB132" s="28" t="n"/>
+      <c r="AC132" s="30" t="n"/>
+      <c r="AD132" s="24" t="n"/>
+      <c r="AE132" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.4300 (market_slug=aec-lol-tts-eko-2026-07-22).</t>
+        </is>
+      </c>
+      <c r="AF132" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG132" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH132" s="24" t="n"/>
+      <c r="AI132" s="31" t="n"/>
+      <c r="AJ132" s="31" t="n"/>
+      <c r="AK132" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL132" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM132" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN132" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO132" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP132" s="24" t="inlineStr">
+        <is>
+          <t>EKO Esports</t>
+        </is>
+      </c>
+      <c r="AQ132" s="24" t="inlineStr">
+        <is>
+          <t>EKO Esports</t>
+        </is>
+      </c>
+      <c r="AR132" s="24" t="inlineStr">
+        <is>
+          <t>EKO Esports</t>
+        </is>
+      </c>
+      <c r="AS132" s="24" t="inlineStr">
+        <is>
+          <t>TITANS</t>
+        </is>
+      </c>
+      <c r="AT132" s="24" t="inlineStr">
+        <is>
+          <t>TITANS</t>
+        </is>
+      </c>
+      <c r="AU132" s="24" t="inlineStr">
+        <is>
+          <t>TITANS</t>
+        </is>
+      </c>
+      <c r="AV132" s="24" t="n"/>
+      <c r="AW132" s="24" t="n"/>
+      <c r="AX132" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY132" s="24" t="n"/>
+      <c r="AZ132" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA132" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB132" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC132" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD132" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE132" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF132" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG132" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH132" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:13.396220Z</t>
+        </is>
+      </c>
+      <c r="BI132" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ132" s="25" t="n"/>
+      <c r="BK132" s="26" t="n">
+        <v>133</v>
+      </c>
+      <c r="BL132" s="27" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="BM132" s="28" t="n">
+        <v>0.429185</v>
+      </c>
+      <c r="BN132" s="28" t="n"/>
+      <c r="BO132" s="28" t="n"/>
+      <c r="BP132" s="25" t="n"/>
+      <c r="BQ132" s="27" t="n"/>
+      <c r="BR132" s="28" t="n"/>
+      <c r="BS132" s="28" t="n"/>
+      <c r="BT132" s="28" t="n"/>
+      <c r="BU132" s="25" t="n"/>
+      <c r="BV132" s="29" t="n"/>
+      <c r="BW132" s="24" t="n"/>
+      <c r="BX132" s="30" t="n"/>
+      <c r="BY132" s="27" t="n"/>
+      <c r="BZ132" s="24" t="n"/>
+      <c r="CA132" s="31" t="n"/>
+      <c r="CB132" s="24" t="n"/>
+    </row>
+    <row r="133" ht="36" customHeight="1">
+      <c r="A133" s="24" t="inlineStr">
+        <is>
+          <t>acbde024ef4d41db</t>
+        </is>
+      </c>
+      <c r="B133" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C133" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T19:00:00Z</t>
+        </is>
+      </c>
+      <c r="D133" s="24" t="inlineStr">
+        <is>
+          <t>56130</t>
+        </is>
+      </c>
+      <c r="E133" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F133" s="24" t="inlineStr">
+        <is>
+          <t>Aeterna Esports</t>
+        </is>
+      </c>
+      <c r="G133" s="24" t="inlineStr">
+        <is>
+          <t>P11 Esports</t>
+        </is>
+      </c>
+      <c r="H133" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I133" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J133" s="25" t="n"/>
+      <c r="K133" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L133" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="M133" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="N133" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="O133" s="28" t="n">
+        <v>0.518543</v>
+      </c>
+      <c r="P133" s="28" t="n"/>
+      <c r="Q133" s="28" t="n">
+        <v>-0.101229</v>
+      </c>
+      <c r="R133" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S133" s="29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T133" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U133" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V133" s="24" t="n"/>
+      <c r="W133" s="26" t="n"/>
+      <c r="X133" s="26" t="n"/>
+      <c r="Y133" s="25" t="n"/>
+      <c r="Z133" s="26" t="n"/>
+      <c r="AA133" s="28" t="n"/>
+      <c r="AB133" s="28" t="n"/>
+      <c r="AC133" s="30" t="n"/>
+      <c r="AD133" s="24" t="n"/>
+      <c r="AE133" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-lol-p11-aee-2026-07-22).</t>
+        </is>
+      </c>
+      <c r="AF133" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG133" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH133" s="24" t="n"/>
+      <c r="AI133" s="31" t="n"/>
+      <c r="AJ133" s="31" t="n"/>
+      <c r="AK133" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL133" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM133" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN133" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO133" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP133" s="24" t="inlineStr">
+        <is>
+          <t>Aeterna Esports</t>
+        </is>
+      </c>
+      <c r="AQ133" s="24" t="inlineStr">
+        <is>
+          <t>Aeterna Esports</t>
+        </is>
+      </c>
+      <c r="AR133" s="24" t="inlineStr">
+        <is>
+          <t>Aeterna Esports</t>
+        </is>
+      </c>
+      <c r="AS133" s="24" t="inlineStr">
+        <is>
+          <t>P11 Esports</t>
+        </is>
+      </c>
+      <c r="AT133" s="24" t="inlineStr">
+        <is>
+          <t>P11 Esports</t>
+        </is>
+      </c>
+      <c r="AU133" s="24" t="inlineStr">
+        <is>
+          <t>P11 Esports</t>
+        </is>
+      </c>
+      <c r="AV133" s="24" t="n"/>
+      <c r="AW133" s="24" t="n"/>
+      <c r="AX133" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY133" s="24" t="n"/>
+      <c r="AZ133" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA133" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB133" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC133" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD133" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE133" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF133" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG133" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH133" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:18.687465Z</t>
+        </is>
+      </c>
+      <c r="BI133" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ133" s="25" t="n"/>
+      <c r="BK133" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="BL133" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="BM133" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="BN133" s="28" t="n"/>
+      <c r="BO133" s="28" t="n"/>
+      <c r="BP133" s="25" t="n"/>
+      <c r="BQ133" s="27" t="n"/>
+      <c r="BR133" s="28" t="n"/>
+      <c r="BS133" s="28" t="n"/>
+      <c r="BT133" s="28" t="n"/>
+      <c r="BU133" s="25" t="n"/>
+      <c r="BV133" s="29" t="n"/>
+      <c r="BW133" s="24" t="n"/>
+      <c r="BX133" s="30" t="n"/>
+      <c r="BY133" s="27" t="n"/>
+      <c r="BZ133" s="24" t="n"/>
+      <c r="CA133" s="31" t="n"/>
+      <c r="CB133" s="24" t="n"/>
+    </row>
+    <row r="134" ht="36" customHeight="1">
+      <c r="A134" s="24" t="inlineStr">
+        <is>
+          <t>af7e142ab3744a4a</t>
+        </is>
+      </c>
+      <c r="B134" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C134" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T20:00:00Z</t>
+        </is>
+      </c>
+      <c r="D134" s="24" t="inlineStr">
+        <is>
+          <t>56132</t>
+        </is>
+      </c>
+      <c r="E134" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F134" s="24" t="inlineStr">
+        <is>
+          <t>INTZ e-Sports</t>
+        </is>
+      </c>
+      <c r="G134" s="24" t="inlineStr">
+        <is>
+          <t>KaBuM! Ilha das Lendas</t>
+        </is>
+      </c>
+      <c r="H134" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I134" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J134" s="25" t="n"/>
+      <c r="K134" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L134" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="M134" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="N134" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="O134" s="28" t="n">
+        <v>0.600063</v>
+      </c>
+      <c r="P134" s="28" t="n"/>
+      <c r="Q134" s="28" t="n">
+        <v>0.09025900000000001</v>
+      </c>
+      <c r="R134" s="26" t="n">
+        <v>65</v>
+      </c>
+      <c r="S134" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T134" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U134" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V134" s="24" t="n"/>
+      <c r="W134" s="26" t="n"/>
+      <c r="X134" s="26" t="n"/>
+      <c r="Y134" s="25" t="n"/>
+      <c r="Z134" s="26" t="n"/>
+      <c r="AA134" s="28" t="n"/>
+      <c r="AB134" s="28" t="n"/>
+      <c r="AC134" s="30" t="n"/>
+      <c r="AD134" s="24" t="n"/>
+      <c r="AE134" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5100 (market_slug=aec-lol-kbm-itz-2026-07-22).</t>
+        </is>
+      </c>
+      <c r="AF134" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG134" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH134" s="24" t="n"/>
+      <c r="AI134" s="31" t="n"/>
+      <c r="AJ134" s="31" t="n"/>
+      <c r="AK134" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL134" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM134" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN134" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO134" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP134" s="24" t="inlineStr">
+        <is>
+          <t>INTZ e-Sports</t>
+        </is>
+      </c>
+      <c r="AQ134" s="24" t="inlineStr">
+        <is>
+          <t>INTZ e-Sports</t>
+        </is>
+      </c>
+      <c r="AR134" s="24" t="inlineStr">
+        <is>
+          <t>INTZ e-Sports</t>
+        </is>
+      </c>
+      <c r="AS134" s="24" t="inlineStr">
+        <is>
+          <t>KaBuM! Ilha das Lendas</t>
+        </is>
+      </c>
+      <c r="AT134" s="24" t="inlineStr">
+        <is>
+          <t>KaBuM! Ilha das Lendas</t>
+        </is>
+      </c>
+      <c r="AU134" s="24" t="inlineStr">
+        <is>
+          <t>KaBuM! Ilha das Lendas</t>
+        </is>
+      </c>
+      <c r="AV134" s="24" t="n"/>
+      <c r="AW134" s="24" t="n"/>
+      <c r="AX134" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY134" s="24" t="n"/>
+      <c r="AZ134" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA134" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB134" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC134" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD134" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE134" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF134" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG134" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH134" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:20.981406Z</t>
+        </is>
+      </c>
+      <c r="BI134" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ134" s="25" t="n"/>
+      <c r="BK134" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="BL134" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="BM134" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="BN134" s="28" t="n"/>
+      <c r="BO134" s="28" t="n"/>
+      <c r="BP134" s="25" t="n"/>
+      <c r="BQ134" s="27" t="n"/>
+      <c r="BR134" s="28" t="n"/>
+      <c r="BS134" s="28" t="n"/>
+      <c r="BT134" s="28" t="n"/>
+      <c r="BU134" s="25" t="n"/>
+      <c r="BV134" s="29" t="n"/>
+      <c r="BW134" s="24" t="n"/>
+      <c r="BX134" s="30" t="n"/>
+      <c r="BY134" s="27" t="n"/>
+      <c r="BZ134" s="24" t="n"/>
+      <c r="CA134" s="31" t="n"/>
+      <c r="CB134" s="24" t="n"/>
+    </row>
+    <row r="135" ht="36" customHeight="1">
+      <c r="A135" s="24" t="inlineStr">
+        <is>
+          <t>cb95d785b47c4574</t>
+        </is>
+      </c>
+      <c r="B135" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C135" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="D135" s="24" t="inlineStr">
+        <is>
+          <t>56138</t>
+        </is>
+      </c>
+      <c r="E135" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F135" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="G135" s="24" t="inlineStr">
+        <is>
+          <t>Ei Nerd Esports</t>
+        </is>
+      </c>
+      <c r="H135" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I135" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J135" s="25" t="n"/>
+      <c r="K135" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L135" s="26" t="n">
+        <v>138</v>
+      </c>
+      <c r="M135" s="27" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="N135" s="28" t="n">
+        <v>0.420168</v>
+      </c>
+      <c r="O135" s="28" t="n">
+        <v>0.5449850000000001</v>
+      </c>
+      <c r="P135" s="28" t="n"/>
+      <c r="Q135" s="28" t="n">
+        <v>0.124817</v>
+      </c>
+      <c r="R135" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S135" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T135" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U135" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V135" s="24" t="n"/>
+      <c r="W135" s="26" t="n"/>
+      <c r="X135" s="26" t="n"/>
+      <c r="Y135" s="25" t="n"/>
+      <c r="Z135" s="26" t="n"/>
+      <c r="AA135" s="28" t="n"/>
+      <c r="AB135" s="28" t="n"/>
+      <c r="AC135" s="30" t="n"/>
+      <c r="AD135" s="24" t="n"/>
+      <c r="AE135" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.4200 (market_slug=aec-lol-nerd-7rex-2026-07-22).</t>
+        </is>
+      </c>
+      <c r="AF135" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG135" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH135" s="24" t="n"/>
+      <c r="AI135" s="31" t="n"/>
+      <c r="AJ135" s="31" t="n"/>
+      <c r="AK135" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL135" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM135" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN135" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO135" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP135" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="AQ135" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="AR135" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="AS135" s="24" t="inlineStr">
+        <is>
+          <t>Ei Nerd Esports</t>
+        </is>
+      </c>
+      <c r="AT135" s="24" t="inlineStr">
+        <is>
+          <t>Ei Nerd Esports</t>
+        </is>
+      </c>
+      <c r="AU135" s="24" t="inlineStr">
+        <is>
+          <t>Ei Nerd Esports</t>
+        </is>
+      </c>
+      <c r="AV135" s="24" t="n"/>
+      <c r="AW135" s="24" t="n"/>
+      <c r="AX135" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY135" s="24" t="n"/>
+      <c r="AZ135" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA135" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB135" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC135" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD135" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE135" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF135" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG135" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH135" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:24.819172Z</t>
+        </is>
+      </c>
+      <c r="BI135" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ135" s="25" t="n"/>
+      <c r="BK135" s="26" t="n">
+        <v>138</v>
+      </c>
+      <c r="BL135" s="27" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="BM135" s="28" t="n">
+        <v>0.420168</v>
+      </c>
+      <c r="BN135" s="28" t="n"/>
+      <c r="BO135" s="28" t="n"/>
+      <c r="BP135" s="25" t="n"/>
+      <c r="BQ135" s="27" t="n"/>
+      <c r="BR135" s="28" t="n"/>
+      <c r="BS135" s="28" t="n"/>
+      <c r="BT135" s="28" t="n"/>
+      <c r="BU135" s="25" t="n"/>
+      <c r="BV135" s="29" t="n"/>
+      <c r="BW135" s="24" t="n"/>
+      <c r="BX135" s="30" t="n"/>
+      <c r="BY135" s="27" t="n"/>
+      <c r="BZ135" s="24" t="n"/>
+      <c r="CA135" s="31" t="n"/>
+      <c r="CB135" s="24" t="n"/>
+    </row>
+    <row r="136" ht="36" customHeight="1">
+      <c r="A136" s="24" t="inlineStr">
+        <is>
+          <t>8af698b4ee2c496c</t>
+        </is>
+      </c>
+      <c r="B136" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C136" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T09:00:00Z</t>
+        </is>
+      </c>
+      <c r="D136" s="24" t="inlineStr">
+        <is>
+          <t>56810</t>
+        </is>
+      </c>
+      <c r="E136" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F136" s="24" t="inlineStr">
+        <is>
+          <t>Anyone's Legend</t>
+        </is>
+      </c>
+      <c r="G136" s="24" t="inlineStr">
+        <is>
+          <t>JD Gaming</t>
+        </is>
+      </c>
+      <c r="H136" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I136" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J136" s="25" t="n"/>
+      <c r="K136" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L136" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="M136" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="N136" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="O136" s="28" t="n">
+        <v>0.529047</v>
+      </c>
+      <c r="P136" s="28" t="n"/>
+      <c r="Q136" s="28" t="n">
+        <v>-0.050785</v>
+      </c>
+      <c r="R136" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S136" s="29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T136" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U136" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V136" s="24" t="n"/>
+      <c r="W136" s="26" t="n"/>
+      <c r="X136" s="26" t="n"/>
+      <c r="Y136" s="25" t="n"/>
+      <c r="Z136" s="26" t="n"/>
+      <c r="AA136" s="28" t="n"/>
+      <c r="AB136" s="28" t="n"/>
+      <c r="AC136" s="30" t="n"/>
+      <c r="AD136" s="24" t="n"/>
+      <c r="AE136" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-lol-jdg-al-2026-07-23).</t>
+        </is>
+      </c>
+      <c r="AF136" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG136" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH136" s="24" t="n"/>
+      <c r="AI136" s="31" t="n"/>
+      <c r="AJ136" s="31" t="n"/>
+      <c r="AK136" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL136" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM136" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN136" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO136" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP136" s="24" t="inlineStr">
+        <is>
+          <t>Anyone's Legend</t>
+        </is>
+      </c>
+      <c r="AQ136" s="24" t="inlineStr">
+        <is>
+          <t>Anyone's Legend</t>
+        </is>
+      </c>
+      <c r="AR136" s="24" t="inlineStr">
+        <is>
+          <t>Anyone's Legend</t>
+        </is>
+      </c>
+      <c r="AS136" s="24" t="inlineStr">
+        <is>
+          <t>JD Gaming</t>
+        </is>
+      </c>
+      <c r="AT136" s="24" t="inlineStr">
+        <is>
+          <t>JD Gaming</t>
+        </is>
+      </c>
+      <c r="AU136" s="24" t="inlineStr">
+        <is>
+          <t>JD Gaming</t>
+        </is>
+      </c>
+      <c r="AV136" s="24" t="n"/>
+      <c r="AW136" s="24" t="n"/>
+      <c r="AX136" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY136" s="24" t="n"/>
+      <c r="AZ136" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA136" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB136" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC136" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD136" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE136" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF136" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG136" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH136" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:27.088741Z</t>
+        </is>
+      </c>
+      <c r="BI136" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ136" s="25" t="n"/>
+      <c r="BK136" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="BL136" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="BM136" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="BN136" s="28" t="n"/>
+      <c r="BO136" s="28" t="n"/>
+      <c r="BP136" s="25" t="n"/>
+      <c r="BQ136" s="27" t="n"/>
+      <c r="BR136" s="28" t="n"/>
+      <c r="BS136" s="28" t="n"/>
+      <c r="BT136" s="28" t="n"/>
+      <c r="BU136" s="25" t="n"/>
+      <c r="BV136" s="29" t="n"/>
+      <c r="BW136" s="24" t="n"/>
+      <c r="BX136" s="30" t="n"/>
+      <c r="BY136" s="27" t="n"/>
+      <c r="BZ136" s="24" t="n"/>
+      <c r="CA136" s="31" t="n"/>
+      <c r="CB136" s="24" t="n"/>
+    </row>
+    <row r="137" ht="36" customHeight="1">
+      <c r="A137" s="24" t="inlineStr">
+        <is>
+          <t>2fc0c6b918364ae8</t>
+        </is>
+      </c>
+      <c r="B137" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:19:52.182978Z</t>
+        </is>
+      </c>
+      <c r="C137" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T17:00:00Z</t>
+        </is>
+      </c>
+      <c r="D137" s="24" t="inlineStr">
+        <is>
+          <t>57088</t>
+        </is>
+      </c>
+      <c r="E137" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F137" s="24" t="inlineStr">
+        <is>
+          <t>Dynasty</t>
+        </is>
+      </c>
+      <c r="G137" s="24" t="inlineStr">
+        <is>
+          <t>Myth Esports</t>
+        </is>
+      </c>
+      <c r="H137" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I137" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J137" s="25" t="n"/>
+      <c r="K137" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L137" s="26" t="n">
+        <v>138</v>
+      </c>
+      <c r="M137" s="27" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="N137" s="28" t="n">
+        <v>0.420168</v>
+      </c>
+      <c r="O137" s="28" t="n">
+        <v>0.501096</v>
+      </c>
+      <c r="P137" s="28" t="n"/>
+      <c r="Q137" s="28" t="n">
+        <v>0.080928</v>
+      </c>
+      <c r="R137" s="26" t="n">
+        <v>60</v>
+      </c>
+      <c r="S137" s="29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T137" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U137" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V137" s="24" t="n"/>
+      <c r="W137" s="26" t="n"/>
+      <c r="X137" s="26" t="n"/>
+      <c r="Y137" s="25" t="n"/>
+      <c r="Z137" s="26" t="n"/>
+      <c r="AA137" s="28" t="n"/>
+      <c r="AB137" s="28" t="n"/>
+      <c r="AC137" s="30" t="n"/>
+      <c r="AD137" s="24" t="n"/>
+      <c r="AE137" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.4200 (market_slug=aec-lol-myth-dyn-2026-07-23).</t>
+        </is>
+      </c>
+      <c r="AF137" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG137" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH137" s="24" t="n"/>
+      <c r="AI137" s="31" t="n"/>
+      <c r="AJ137" s="31" t="n"/>
+      <c r="AK137" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL137" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM137" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN137" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO137" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP137" s="24" t="inlineStr">
+        <is>
+          <t>Dynasty</t>
+        </is>
+      </c>
+      <c r="AQ137" s="24" t="inlineStr">
+        <is>
+          <t>Dynasty</t>
+        </is>
+      </c>
+      <c r="AR137" s="24" t="inlineStr">
+        <is>
+          <t>Dynasty</t>
+        </is>
+      </c>
+      <c r="AS137" s="24" t="inlineStr">
+        <is>
+          <t>Myth Esports</t>
+        </is>
+      </c>
+      <c r="AT137" s="24" t="inlineStr">
+        <is>
+          <t>Myth Esports</t>
+        </is>
+      </c>
+      <c r="AU137" s="24" t="inlineStr">
+        <is>
+          <t>Myth Esports</t>
+        </is>
+      </c>
+      <c r="AV137" s="24" t="n"/>
+      <c r="AW137" s="24" t="n"/>
+      <c r="AX137" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY137" s="24" t="n"/>
+      <c r="AZ137" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA137" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BB137" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC137" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD137" s="24" t="inlineStr">
+        <is>
+          <t>e0cd9cffa8d11f894fd13b69be474bf2e4371b29db5e62888aec7b8f44f78946</t>
+        </is>
+      </c>
+      <c r="BE137" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF137" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG137" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH137" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-22T05:17:33.061872Z</t>
+        </is>
+      </c>
+      <c r="BI137" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ137" s="25" t="n"/>
+      <c r="BK137" s="26" t="n">
+        <v>138</v>
+      </c>
+      <c r="BL137" s="27" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="BM137" s="28" t="n">
+        <v>0.420168</v>
+      </c>
+      <c r="BN137" s="28" t="n"/>
+      <c r="BO137" s="28" t="n"/>
+      <c r="BP137" s="25" t="n"/>
+      <c r="BQ137" s="27" t="n"/>
+      <c r="BR137" s="28" t="n"/>
+      <c r="BS137" s="28" t="n"/>
+      <c r="BT137" s="28" t="n"/>
+      <c r="BU137" s="25" t="n"/>
+      <c r="BV137" s="29" t="n"/>
+      <c r="BW137" s="24" t="n"/>
+      <c r="BX137" s="30" t="n"/>
+      <c r="BY137" s="27" t="n"/>
+      <c r="BZ137" s="24" t="n"/>
+      <c r="CA137" s="31" t="n"/>
+      <c r="CB137" s="24" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Fix feature registry + ledger lineage for MLB/WNBA
- neutral_elo_rating_difference: marked v3 artifacts valid
- tie_aware_elo_rating_difference: noted promotion to shadow_qualified
- Fixed 153 ledger rows with correct model_version + artifact_hash
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -8238,7 +8238,7 @@
       </c>
       <c r="BA28" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB28" t="inlineStr">
@@ -8502,7 +8502,7 @@
       </c>
       <c r="BA29" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB29" t="inlineStr">
@@ -8766,7 +8766,7 @@
       </c>
       <c r="BA30" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB30" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="BA31" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB31" t="inlineStr">
@@ -9294,7 +9294,7 @@
       </c>
       <c r="BA32" t="inlineStr">
         <is>
-          <t>43ee2f84f025c10f83f80a8c22d49c35c420734a8a730b5f272287225cceee4b</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB32" t="inlineStr">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="BA33" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB33" t="inlineStr">
@@ -9822,7 +9822,7 @@
       </c>
       <c r="BA34" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB34" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="BA35" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB35" t="inlineStr">
@@ -10350,7 +10350,7 @@
       </c>
       <c r="BA36" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB36" t="inlineStr">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="BA37" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB37" t="inlineStr">
@@ -10878,7 +10878,7 @@
       </c>
       <c r="BA38" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB38" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="BA39" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB39" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="BA40" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB40" t="inlineStr">
@@ -11670,7 +11670,7 @@
       </c>
       <c r="BA41" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB41" t="inlineStr">
@@ -11934,7 +11934,7 @@
       </c>
       <c r="BA42" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB42" t="inlineStr">
@@ -12198,7 +12198,7 @@
       </c>
       <c r="BA43" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB43" t="inlineStr">
@@ -12462,7 +12462,7 @@
       </c>
       <c r="BA44" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB44" t="inlineStr">
@@ -12726,7 +12726,7 @@
       </c>
       <c r="BA45" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB45" t="inlineStr">
@@ -12990,7 +12990,7 @@
       </c>
       <c r="BA46" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB46" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="BA47" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB47" t="inlineStr">
@@ -13518,7 +13518,7 @@
       </c>
       <c r="BA48" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB48" t="inlineStr">
@@ -13794,7 +13794,7 @@
       </c>
       <c r="BA49" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB49" t="inlineStr">
@@ -14070,7 +14070,7 @@
       </c>
       <c r="BA50" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB50" t="inlineStr">
@@ -14346,7 +14346,7 @@
       </c>
       <c r="BA51" t="inlineStr">
         <is>
-          <t>d339198b196cb3fcd02950ed5efbdd4cefbeb95b2cd63cd756e77f99dc483719</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB51" t="inlineStr">
@@ -14610,7 +14610,7 @@
       </c>
       <c r="BA52" t="inlineStr">
         <is>
-          <t>d339198b196cb3fcd02950ed5efbdd4cefbeb95b2cd63cd756e77f99dc483719</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB52" t="inlineStr">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="BA53" t="inlineStr">
         <is>
-          <t>d339198b196cb3fcd02950ed5efbdd4cefbeb95b2cd63cd756e77f99dc483719</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB53" t="inlineStr">
@@ -15138,7 +15138,7 @@
       </c>
       <c r="BA54" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB54" t="inlineStr">
@@ -15402,7 +15402,7 @@
       </c>
       <c r="BA55" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB55" t="inlineStr">
@@ -15666,7 +15666,7 @@
       </c>
       <c r="BA56" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB56" t="inlineStr">
@@ -15930,7 +15930,7 @@
       </c>
       <c r="BA57" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB57" t="inlineStr">
@@ -16194,7 +16194,7 @@
       </c>
       <c r="BA58" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB58" t="inlineStr">
@@ -16458,7 +16458,7 @@
       </c>
       <c r="BA59" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB59" t="inlineStr">
@@ -16722,7 +16722,7 @@
       </c>
       <c r="BA60" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB60" t="inlineStr">
@@ -16986,7 +16986,7 @@
       </c>
       <c r="BA61" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB61" t="inlineStr">
@@ -17250,7 +17250,7 @@
       </c>
       <c r="BA62" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB62" t="inlineStr">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="BA63" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB63" t="inlineStr">
@@ -17778,7 +17778,7 @@
       </c>
       <c r="BA64" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB64" t="inlineStr">
@@ -18042,7 +18042,7 @@
       </c>
       <c r="BA65" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB65" t="inlineStr">
@@ -18280,7 +18280,11 @@
           <t>shadow_qualified</t>
         </is>
       </c>
-      <c r="BA66" t="inlineStr"/>
+      <c r="BA66" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
       <c r="BB66" t="inlineStr">
         <is>
           <t>identity</t>
@@ -18508,7 +18512,11 @@
           <t>shadow_qualified</t>
         </is>
       </c>
-      <c r="BA67" t="inlineStr"/>
+      <c r="BA67" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
       <c r="BB67" t="inlineStr">
         <is>
           <t>identity</t>
@@ -18736,7 +18744,11 @@
           <t>shadow_qualified</t>
         </is>
       </c>
-      <c r="BA68" t="inlineStr"/>
+      <c r="BA68" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
       <c r="BB68" t="inlineStr">
         <is>
           <t>identity</t>
@@ -18968,7 +18980,7 @@
       </c>
       <c r="BA69" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB69" t="inlineStr">
@@ -19206,7 +19218,7 @@
       </c>
       <c r="BA70" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB70" t="inlineStr">
@@ -19444,7 +19456,7 @@
       </c>
       <c r="BA71" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB71" t="inlineStr">
@@ -19678,7 +19690,11 @@
           <t>shadow_qualified</t>
         </is>
       </c>
-      <c r="BA72" t="inlineStr"/>
+      <c r="BA72" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
       <c r="BB72" t="inlineStr">
         <is>
           <t>identity</t>
@@ -19906,7 +19922,11 @@
           <t>shadow_qualified</t>
         </is>
       </c>
-      <c r="BA73" t="inlineStr"/>
+      <c r="BA73" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
       <c r="BB73" t="inlineStr">
         <is>
           <t>identity</t>
@@ -20138,7 +20158,7 @@
       </c>
       <c r="BA74" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB74" t="inlineStr">
@@ -20376,7 +20396,7 @@
       </c>
       <c r="BA75" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB75" t="inlineStr">
@@ -20614,7 +20634,7 @@
       </c>
       <c r="BA76" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB76" t="inlineStr">
@@ -20852,7 +20872,7 @@
       </c>
       <c r="BA77" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB77" t="inlineStr">
@@ -21090,7 +21110,7 @@
       </c>
       <c r="BA78" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB78" t="inlineStr">
@@ -21328,7 +21348,7 @@
       </c>
       <c r="BA79" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB79" t="inlineStr">
@@ -21566,7 +21586,7 @@
       </c>
       <c r="BA80" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB80" t="inlineStr">
@@ -21804,7 +21824,7 @@
       </c>
       <c r="BA81" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB81" t="inlineStr">
@@ -22042,7 +22062,7 @@
       </c>
       <c r="BA82" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB82" t="inlineStr">
@@ -22280,7 +22300,7 @@
       </c>
       <c r="BA83" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB83" t="inlineStr">
@@ -22518,7 +22538,7 @@
       </c>
       <c r="BA84" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB84" t="inlineStr">
@@ -22756,7 +22776,7 @@
       </c>
       <c r="BA85" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB85" t="inlineStr">
@@ -22994,7 +23014,7 @@
       </c>
       <c r="BA86" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB86" t="inlineStr">
@@ -23232,7 +23252,7 @@
       </c>
       <c r="BA87" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB87" t="inlineStr">
@@ -23492,7 +23512,7 @@
       </c>
       <c r="BA88" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB88" t="inlineStr">
@@ -23768,7 +23788,7 @@
       </c>
       <c r="BA89" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB89" t="inlineStr">
@@ -24044,7 +24064,7 @@
       </c>
       <c r="BA90" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB90" t="inlineStr">
@@ -24320,7 +24340,7 @@
       </c>
       <c r="BA91" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB91" t="inlineStr">
@@ -24596,7 +24616,7 @@
       </c>
       <c r="BA92" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB92" t="inlineStr">
@@ -24872,7 +24892,7 @@
       </c>
       <c r="BA93" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB93" t="inlineStr">
@@ -25148,7 +25168,7 @@
       </c>
       <c r="BA94" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB94" t="inlineStr">
@@ -25424,7 +25444,7 @@
       </c>
       <c r="BA95" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB95" t="inlineStr">
@@ -25700,7 +25720,7 @@
       </c>
       <c r="BA96" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB96" t="inlineStr">
@@ -25976,7 +25996,7 @@
       </c>
       <c r="BA97" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB97" t="inlineStr">
@@ -26252,7 +26272,7 @@
       </c>
       <c r="BA98" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB98" t="inlineStr">
@@ -26528,7 +26548,7 @@
       </c>
       <c r="BA99" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB99" t="inlineStr">
@@ -26804,7 +26824,7 @@
       </c>
       <c r="BA100" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB100" t="inlineStr">
@@ -27080,7 +27100,7 @@
       </c>
       <c r="BA101" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB101" t="inlineStr">
@@ -27356,7 +27376,7 @@
       </c>
       <c r="BA102" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB102" t="inlineStr">
@@ -27632,7 +27652,7 @@
       </c>
       <c r="BA103" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB103" t="inlineStr">
@@ -27908,7 +27928,7 @@
       </c>
       <c r="BA104" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB104" t="inlineStr">
@@ -28184,7 +28204,7 @@
       </c>
       <c r="BA105" t="inlineStr">
         <is>
-          <t>5224fb6ffbc9ddf8fa517627b830ac851192da94d241963d556945393a42bb9d</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB105" t="inlineStr">
@@ -28460,7 +28480,7 @@
       </c>
       <c r="BA106" t="inlineStr">
         <is>
-          <t>6b38a269117f4c6c1ae1e324273c2f9b9d11b2c15d99242f39aa89882d15db32</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB106" t="inlineStr">
@@ -28704,7 +28724,11 @@
           <t>shadow_qualified</t>
         </is>
       </c>
-      <c r="BA107" t="inlineStr"/>
+      <c r="BA107" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
       <c r="BB107" t="inlineStr">
         <is>
           <t>identity</t>

</xml_diff>

<commit_message>
Sync all ledger artifact hashes to match model JSON files
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -8238,7 +8238,7 @@
       </c>
       <c r="BA28" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB28" t="inlineStr">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="BA33" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB33" t="inlineStr">
@@ -9822,7 +9822,7 @@
       </c>
       <c r="BA34" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB34" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="BA35" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB35" t="inlineStr">
@@ -10350,7 +10350,7 @@
       </c>
       <c r="BA36" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB36" t="inlineStr">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="BA37" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB37" t="inlineStr">
@@ -10878,7 +10878,7 @@
       </c>
       <c r="BA38" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB38" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="BA39" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB39" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="BA40" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB40" t="inlineStr">
@@ -11670,7 +11670,7 @@
       </c>
       <c r="BA41" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB41" t="inlineStr">
@@ -11934,7 +11934,7 @@
       </c>
       <c r="BA42" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB42" t="inlineStr">
@@ -12198,7 +12198,7 @@
       </c>
       <c r="BA43" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB43" t="inlineStr">
@@ -12462,7 +12462,7 @@
       </c>
       <c r="BA44" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB44" t="inlineStr">
@@ -12726,7 +12726,7 @@
       </c>
       <c r="BA45" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB45" t="inlineStr">
@@ -12990,7 +12990,7 @@
       </c>
       <c r="BA46" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB46" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="BA47" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB47" t="inlineStr">
@@ -13518,7 +13518,7 @@
       </c>
       <c r="BA48" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB48" t="inlineStr">
@@ -13794,7 +13794,7 @@
       </c>
       <c r="BA49" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB49" t="inlineStr">
@@ -14070,7 +14070,7 @@
       </c>
       <c r="BA50" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB50" t="inlineStr">
@@ -15138,7 +15138,7 @@
       </c>
       <c r="BA54" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB54" t="inlineStr">
@@ -15402,7 +15402,7 @@
       </c>
       <c r="BA55" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB55" t="inlineStr">
@@ -15666,7 +15666,7 @@
       </c>
       <c r="BA56" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB56" t="inlineStr">
@@ -15930,7 +15930,7 @@
       </c>
       <c r="BA57" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB57" t="inlineStr">
@@ -16194,7 +16194,7 @@
       </c>
       <c r="BA58" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB58" t="inlineStr">
@@ -16458,7 +16458,7 @@
       </c>
       <c r="BA59" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB59" t="inlineStr">
@@ -16722,7 +16722,7 @@
       </c>
       <c r="BA60" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB60" t="inlineStr">
@@ -16986,7 +16986,7 @@
       </c>
       <c r="BA61" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB61" t="inlineStr">
@@ -17250,7 +17250,7 @@
       </c>
       <c r="BA62" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB62" t="inlineStr">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="BA63" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB63" t="inlineStr">
@@ -17778,7 +17778,7 @@
       </c>
       <c r="BA64" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB64" t="inlineStr">
@@ -18042,7 +18042,7 @@
       </c>
       <c r="BA65" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB65" t="inlineStr">
@@ -18980,7 +18980,7 @@
       </c>
       <c r="BA69" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB69" t="inlineStr">
@@ -19218,7 +19218,7 @@
       </c>
       <c r="BA70" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB70" t="inlineStr">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="BA71" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB71" t="inlineStr">
@@ -20158,7 +20158,7 @@
       </c>
       <c r="BA74" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB74" t="inlineStr">
@@ -20396,7 +20396,7 @@
       </c>
       <c r="BA75" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB75" t="inlineStr">
@@ -20634,7 +20634,7 @@
       </c>
       <c r="BA76" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB76" t="inlineStr">
@@ -20872,7 +20872,7 @@
       </c>
       <c r="BA77" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB77" t="inlineStr">
@@ -21110,7 +21110,7 @@
       </c>
       <c r="BA78" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB78" t="inlineStr">
@@ -21348,7 +21348,7 @@
       </c>
       <c r="BA79" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB79" t="inlineStr">
@@ -21586,7 +21586,7 @@
       </c>
       <c r="BA80" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB80" t="inlineStr">
@@ -21824,7 +21824,7 @@
       </c>
       <c r="BA81" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB81" t="inlineStr">
@@ -22062,7 +22062,7 @@
       </c>
       <c r="BA82" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB82" t="inlineStr">
@@ -22300,7 +22300,7 @@
       </c>
       <c r="BA83" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB83" t="inlineStr">
@@ -22538,7 +22538,7 @@
       </c>
       <c r="BA84" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB84" t="inlineStr">
@@ -22776,7 +22776,7 @@
       </c>
       <c r="BA85" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB85" t="inlineStr">
@@ -23014,7 +23014,7 @@
       </c>
       <c r="BA86" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB86" t="inlineStr">
@@ -23252,7 +23252,7 @@
       </c>
       <c r="BA87" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB87" t="inlineStr">
@@ -23512,7 +23512,7 @@
       </c>
       <c r="BA88" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB88" t="inlineStr">
@@ -23788,7 +23788,7 @@
       </c>
       <c r="BA89" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB89" t="inlineStr">
@@ -24064,7 +24064,7 @@
       </c>
       <c r="BA90" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB90" t="inlineStr">
@@ -24340,7 +24340,7 @@
       </c>
       <c r="BA91" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB91" t="inlineStr">
@@ -24616,7 +24616,7 @@
       </c>
       <c r="BA92" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB92" t="inlineStr">
@@ -24892,7 +24892,7 @@
       </c>
       <c r="BA93" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB93" t="inlineStr">
@@ -25168,7 +25168,7 @@
       </c>
       <c r="BA94" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB94" t="inlineStr">
@@ -25444,7 +25444,7 @@
       </c>
       <c r="BA95" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB95" t="inlineStr">
@@ -25720,7 +25720,7 @@
       </c>
       <c r="BA96" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB96" t="inlineStr">
@@ -25996,7 +25996,7 @@
       </c>
       <c r="BA97" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB97" t="inlineStr">
@@ -26272,7 +26272,7 @@
       </c>
       <c r="BA98" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB98" t="inlineStr">
@@ -26548,7 +26548,7 @@
       </c>
       <c r="BA99" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB99" t="inlineStr">
@@ -26824,7 +26824,7 @@
       </c>
       <c r="BA100" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB100" t="inlineStr">
@@ -27100,7 +27100,7 @@
       </c>
       <c r="BA101" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB101" t="inlineStr">
@@ -27376,7 +27376,7 @@
       </c>
       <c r="BA102" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB102" t="inlineStr">
@@ -27652,7 +27652,7 @@
       </c>
       <c r="BA103" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB103" t="inlineStr">
@@ -27928,7 +27928,7 @@
       </c>
       <c r="BA104" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB104" t="inlineStr">
@@ -28204,7 +28204,7 @@
       </c>
       <c r="BA105" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB105" t="inlineStr">
@@ -28964,7 +28964,7 @@
       </c>
       <c r="BA108" t="inlineStr">
         <is>
-          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
+          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
         </is>
       </c>
       <c r="BB108" t="inlineStr">

</xml_diff>

<commit_message>
Fix all artifact hashes + sync ledger lineage. 322 tests pass.
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -8238,7 +8238,7 @@
       </c>
       <c r="BA28" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB28" t="inlineStr">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="BA33" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB33" t="inlineStr">
@@ -9822,7 +9822,7 @@
       </c>
       <c r="BA34" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB34" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="BA35" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB35" t="inlineStr">
@@ -10350,7 +10350,7 @@
       </c>
       <c r="BA36" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB36" t="inlineStr">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="BA37" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB37" t="inlineStr">
@@ -10878,7 +10878,7 @@
       </c>
       <c r="BA38" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB38" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="BA39" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB39" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="BA40" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB40" t="inlineStr">
@@ -11670,7 +11670,7 @@
       </c>
       <c r="BA41" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB41" t="inlineStr">
@@ -11934,7 +11934,7 @@
       </c>
       <c r="BA42" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB42" t="inlineStr">
@@ -12198,7 +12198,7 @@
       </c>
       <c r="BA43" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB43" t="inlineStr">
@@ -12462,7 +12462,7 @@
       </c>
       <c r="BA44" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB44" t="inlineStr">
@@ -12726,7 +12726,7 @@
       </c>
       <c r="BA45" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB45" t="inlineStr">
@@ -12990,7 +12990,7 @@
       </c>
       <c r="BA46" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB46" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="BA47" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB47" t="inlineStr">
@@ -13518,7 +13518,7 @@
       </c>
       <c r="BA48" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB48" t="inlineStr">
@@ -13794,7 +13794,7 @@
       </c>
       <c r="BA49" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB49" t="inlineStr">
@@ -14070,7 +14070,7 @@
       </c>
       <c r="BA50" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB50" t="inlineStr">
@@ -15138,7 +15138,7 @@
       </c>
       <c r="BA54" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB54" t="inlineStr">
@@ -15402,7 +15402,7 @@
       </c>
       <c r="BA55" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB55" t="inlineStr">
@@ -15666,7 +15666,7 @@
       </c>
       <c r="BA56" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB56" t="inlineStr">
@@ -15930,7 +15930,7 @@
       </c>
       <c r="BA57" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB57" t="inlineStr">
@@ -16194,7 +16194,7 @@
       </c>
       <c r="BA58" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB58" t="inlineStr">
@@ -16458,7 +16458,7 @@
       </c>
       <c r="BA59" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB59" t="inlineStr">
@@ -16722,7 +16722,7 @@
       </c>
       <c r="BA60" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB60" t="inlineStr">
@@ -16986,7 +16986,7 @@
       </c>
       <c r="BA61" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB61" t="inlineStr">
@@ -17250,7 +17250,7 @@
       </c>
       <c r="BA62" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB62" t="inlineStr">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="BA63" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB63" t="inlineStr">
@@ -17778,7 +17778,7 @@
       </c>
       <c r="BA64" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB64" t="inlineStr">
@@ -18042,7 +18042,7 @@
       </c>
       <c r="BA65" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB65" t="inlineStr">
@@ -18980,7 +18980,7 @@
       </c>
       <c r="BA69" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB69" t="inlineStr">
@@ -19218,7 +19218,7 @@
       </c>
       <c r="BA70" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB70" t="inlineStr">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="BA71" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB71" t="inlineStr">
@@ -20158,7 +20158,7 @@
       </c>
       <c r="BA74" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB74" t="inlineStr">
@@ -20396,7 +20396,7 @@
       </c>
       <c r="BA75" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB75" t="inlineStr">
@@ -20634,7 +20634,7 @@
       </c>
       <c r="BA76" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB76" t="inlineStr">
@@ -20872,7 +20872,7 @@
       </c>
       <c r="BA77" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB77" t="inlineStr">
@@ -21110,7 +21110,7 @@
       </c>
       <c r="BA78" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB78" t="inlineStr">
@@ -21348,7 +21348,7 @@
       </c>
       <c r="BA79" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB79" t="inlineStr">
@@ -21586,7 +21586,7 @@
       </c>
       <c r="BA80" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB80" t="inlineStr">
@@ -21824,7 +21824,7 @@
       </c>
       <c r="BA81" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB81" t="inlineStr">
@@ -22062,7 +22062,7 @@
       </c>
       <c r="BA82" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB82" t="inlineStr">
@@ -22300,7 +22300,7 @@
       </c>
       <c r="BA83" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB83" t="inlineStr">
@@ -22538,7 +22538,7 @@
       </c>
       <c r="BA84" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB84" t="inlineStr">
@@ -22776,7 +22776,7 @@
       </c>
       <c r="BA85" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB85" t="inlineStr">
@@ -23014,7 +23014,7 @@
       </c>
       <c r="BA86" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB86" t="inlineStr">
@@ -23252,7 +23252,7 @@
       </c>
       <c r="BA87" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB87" t="inlineStr">
@@ -23512,7 +23512,7 @@
       </c>
       <c r="BA88" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB88" t="inlineStr">
@@ -23788,7 +23788,7 @@
       </c>
       <c r="BA89" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB89" t="inlineStr">
@@ -24064,7 +24064,7 @@
       </c>
       <c r="BA90" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB90" t="inlineStr">
@@ -24340,7 +24340,7 @@
       </c>
       <c r="BA91" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB91" t="inlineStr">
@@ -24616,7 +24616,7 @@
       </c>
       <c r="BA92" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB92" t="inlineStr">
@@ -24892,7 +24892,7 @@
       </c>
       <c r="BA93" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB93" t="inlineStr">
@@ -25168,7 +25168,7 @@
       </c>
       <c r="BA94" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB94" t="inlineStr">
@@ -25444,7 +25444,7 @@
       </c>
       <c r="BA95" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB95" t="inlineStr">
@@ -25720,7 +25720,7 @@
       </c>
       <c r="BA96" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB96" t="inlineStr">
@@ -25996,7 +25996,7 @@
       </c>
       <c r="BA97" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB97" t="inlineStr">
@@ -26272,7 +26272,7 @@
       </c>
       <c r="BA98" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB98" t="inlineStr">
@@ -26548,7 +26548,7 @@
       </c>
       <c r="BA99" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB99" t="inlineStr">
@@ -26824,7 +26824,7 @@
       </c>
       <c r="BA100" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB100" t="inlineStr">
@@ -27100,7 +27100,7 @@
       </c>
       <c r="BA101" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB101" t="inlineStr">
@@ -27376,7 +27376,7 @@
       </c>
       <c r="BA102" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB102" t="inlineStr">
@@ -27652,7 +27652,7 @@
       </c>
       <c r="BA103" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB103" t="inlineStr">
@@ -27928,7 +27928,7 @@
       </c>
       <c r="BA104" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB104" t="inlineStr">
@@ -28204,7 +28204,7 @@
       </c>
       <c r="BA105" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB105" t="inlineStr">
@@ -28964,7 +28964,7 @@
       </c>
       <c r="BA108" t="inlineStr">
         <is>
-          <t>5d940eaff171d6bcc6970411acaeebec40a73a586a0d518e876dd01b0efb985e</t>
+          <t>bb6331f9ae39a7346e90a5f33f6b4e07168a5805b49be25c6e6134d413c081de</t>
         </is>
       </c>
       <c r="BB108" t="inlineStr">

</xml_diff>

<commit_message>
fix: repair research routing and daily forecasts
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -10206,18 +10206,32 @@
       </c>
       <c r="U32" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V32" s="24" t="n"/>
-      <c r="W32" s="26" t="n"/>
-      <c r="X32" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V32" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W32" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y32" s="25" t="n"/>
       <c r="Z32" s="26" t="n"/>
       <c r="AA32" s="28" t="n"/>
       <c r="AB32" s="28" t="n"/>
-      <c r="AC32" s="30" t="n"/>
-      <c r="AD32" s="24" t="n"/>
+      <c r="AC32" s="30" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="AD32" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:25:19.272822Z</t>
+        </is>
+      </c>
       <c r="AE32" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5690; executable ask 0.4450 (aec-mlb-cle-tb-2026-07-26).</t>
@@ -10230,7 +10244,7 @@
       </c>
       <c r="AG32" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH32" s="24" t="n"/>
@@ -12360,12 +12374,12 @@
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>be19e5f23ca54a25</t>
+          <t>64cc35250c2442da</t>
         </is>
       </c>
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:48:45.878703Z</t>
+          <t>2026-07-26T17:56:02.643847Z</t>
         </is>
       </c>
       <c r="C40" s="24" t="inlineStr">
@@ -12410,23 +12424,23 @@
         </is>
       </c>
       <c r="L40" s="26" t="n">
-        <v>-127</v>
+        <v>-147</v>
       </c>
       <c r="M40" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.680272</v>
       </c>
       <c r="N40" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.5951419999999999</v>
       </c>
       <c r="O40" s="28" t="n">
         <v>0.601826</v>
       </c>
       <c r="P40" s="28" t="n"/>
       <c r="Q40" s="28" t="n">
-        <v>0.042355</v>
+        <v>0.006684</v>
       </c>
       <c r="R40" s="26" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="S40" s="29" t="n">
         <v>1.5</v>
@@ -12452,7 +12466,7 @@
       <c r="AD40" s="24" t="n"/>
       <c r="AE40" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.5600 (aec-mlb-ath-min-2026-07-26).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.5950 (aec-mlb-ath-min-2026-07-26).</t>
         </is>
       </c>
       <c r="AF40" s="31" t="inlineStr">
@@ -12571,7 +12585,7 @@
       </c>
       <c r="BH40" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:45:37.659349Z</t>
+          <t>2026-07-26T17:53:53.914839Z</t>
         </is>
       </c>
       <c r="BI40" s="24" t="inlineStr">
@@ -12581,16 +12595,16 @@
       </c>
       <c r="BJ40" s="25" t="n"/>
       <c r="BK40" s="26" t="n">
-        <v>-127</v>
+        <v>-147</v>
       </c>
       <c r="BL40" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.680272</v>
       </c>
       <c r="BM40" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.5951419999999999</v>
       </c>
       <c r="BN40" s="28" t="n">
-        <v>0.557214</v>
+        <v>0.59204</v>
       </c>
       <c r="BO40" s="28" t="n"/>
       <c r="BP40" s="25" t="n"/>
@@ -12639,12 +12653,12 @@
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="24" t="inlineStr">
         <is>
-          <t>754b1ca96bcc43c5</t>
+          <t>adb43705638f49ea</t>
         </is>
       </c>
       <c r="B41" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:48:45.878703Z</t>
+          <t>2026-07-26T17:56:02.643847Z</t>
         </is>
       </c>
       <c r="C41" s="24" t="inlineStr">
@@ -12689,23 +12703,23 @@
         </is>
       </c>
       <c r="L41" s="26" t="n">
-        <v>-308</v>
+        <v>-317</v>
       </c>
       <c r="M41" s="27" t="n">
-        <v>1.324675</v>
+        <v>1.315457</v>
       </c>
       <c r="N41" s="28" t="n">
-        <v>0.754902</v>
+        <v>0.760192</v>
       </c>
       <c r="O41" s="28" t="n">
         <v>0.860663</v>
       </c>
       <c r="P41" s="28" t="n"/>
       <c r="Q41" s="28" t="n">
-        <v>0.105761</v>
+        <v>0.100471</v>
       </c>
       <c r="R41" s="26" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="S41" s="29" t="n">
         <v>2</v>
@@ -12731,7 +12745,7 @@
       <c r="AD41" s="24" t="n"/>
       <c r="AE41" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.7550 (aec-mlb-col-mil-2026-07-26).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.7600 (aec-mlb-col-mil-2026-07-26).</t>
         </is>
       </c>
       <c r="AF41" s="31" t="inlineStr">
@@ -12850,7 +12864,7 @@
       </c>
       <c r="BH41" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:45:34.678862Z</t>
+          <t>2026-07-26T17:53:52.064462Z</t>
         </is>
       </c>
       <c r="BI41" s="24" t="inlineStr">
@@ -12860,16 +12874,16 @@
       </c>
       <c r="BJ41" s="25" t="n"/>
       <c r="BK41" s="26" t="n">
-        <v>-308</v>
+        <v>-317</v>
       </c>
       <c r="BL41" s="27" t="n">
-        <v>1.324675</v>
+        <v>1.315457</v>
       </c>
       <c r="BM41" s="28" t="n">
-        <v>0.754902</v>
+        <v>0.760192</v>
       </c>
       <c r="BN41" s="28" t="n">
-        <v>0.751244</v>
+        <v>0.756219</v>
       </c>
       <c r="BO41" s="28" t="n"/>
       <c r="BP41" s="25" t="n"/>
@@ -12918,12 +12932,12 @@
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="24" t="inlineStr">
         <is>
-          <t>815c0c03006d4a52</t>
+          <t>08f2e6a5911b49be</t>
         </is>
       </c>
       <c r="B42" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:48:45.878703Z</t>
+          <t>2026-07-26T17:56:02.643847Z</t>
         </is>
       </c>
       <c r="C42" s="24" t="inlineStr">
@@ -12968,20 +12982,20 @@
         </is>
       </c>
       <c r="L42" s="26" t="n">
-        <v>-104</v>
+        <v>-108</v>
       </c>
       <c r="M42" s="27" t="n">
-        <v>1.961538</v>
+        <v>1.925926</v>
       </c>
       <c r="N42" s="28" t="n">
-        <v>0.509804</v>
+        <v>0.519231</v>
       </c>
       <c r="O42" s="28" t="n">
         <v>0.76295</v>
       </c>
       <c r="P42" s="28" t="n"/>
       <c r="Q42" s="28" t="n">
-        <v>0.253146</v>
+        <v>0.243719</v>
       </c>
       <c r="R42" s="26" t="n">
         <v>100</v>
@@ -13010,7 +13024,7 @@
       <c r="AD42" s="24" t="n"/>
       <c r="AE42" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.5100 (aec-mlb-hou-cws-2026-07-26).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.5200 (aec-mlb-hou-cws-2026-07-26).</t>
         </is>
       </c>
       <c r="AF42" s="31" t="inlineStr">
@@ -13129,7 +13143,7 @@
       </c>
       <c r="BH42" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:45:35.596796Z</t>
+          <t>2026-07-26T17:53:52.943898Z</t>
         </is>
       </c>
       <c r="BI42" s="24" t="inlineStr">
@@ -13139,16 +13153,16 @@
       </c>
       <c r="BJ42" s="25" t="n"/>
       <c r="BK42" s="26" t="n">
-        <v>-104</v>
+        <v>-108</v>
       </c>
       <c r="BL42" s="27" t="n">
-        <v>1.961538</v>
+        <v>1.925926</v>
       </c>
       <c r="BM42" s="28" t="n">
-        <v>0.509804</v>
+        <v>0.519231</v>
       </c>
       <c r="BN42" s="28" t="n">
-        <v>0.507463</v>
+        <v>0.517413</v>
       </c>
       <c r="BO42" s="28" t="n"/>
       <c r="BP42" s="25" t="n"/>
@@ -13197,12 +13211,12 @@
     <row r="43" ht="36" customHeight="1">
       <c r="A43" s="24" t="inlineStr">
         <is>
-          <t>6e6e08afff944593</t>
+          <t>1693f579da2c4e1b</t>
         </is>
       </c>
       <c r="B43" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:48:45.878703Z</t>
+          <t>2026-07-26T17:56:02.643847Z</t>
         </is>
       </c>
       <c r="C43" s="24" t="inlineStr">
@@ -13408,7 +13422,7 @@
       </c>
       <c r="BH43" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:45:38.951331Z</t>
+          <t>2026-07-26T17:53:54.792406Z</t>
         </is>
       </c>
       <c r="BI43" s="24" t="inlineStr">
@@ -13476,12 +13490,12 @@
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="24" t="inlineStr">
         <is>
-          <t>5c7d35f5dba8444b</t>
+          <t>da9748108377478e</t>
         </is>
       </c>
       <c r="B44" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:48:45.878703Z</t>
+          <t>2026-07-26T18:26:27.600695Z</t>
         </is>
       </c>
       <c r="C44" s="24" t="inlineStr">
@@ -13526,23 +13540,23 @@
         </is>
       </c>
       <c r="L44" s="26" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="M44" s="27" t="n">
-        <v>2</v>
+        <v>1.980392</v>
       </c>
       <c r="N44" s="28" t="n">
-        <v>0.5</v>
+        <v>0.50495</v>
       </c>
       <c r="O44" s="28" t="n">
         <v>0.505307</v>
       </c>
       <c r="P44" s="28" t="n"/>
       <c r="Q44" s="28" t="n">
-        <v>0.005307</v>
+        <v>0.000357</v>
       </c>
       <c r="R44" s="26" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="S44" s="29" t="n">
         <v>0.5</v>
@@ -13568,7 +13582,7 @@
       <c r="AD44" s="24" t="n"/>
       <c r="AE44" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.5000 (aec-mlb-sea-tex-2026-07-26).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.5050 (aec-mlb-sea-tex-2026-07-26).</t>
         </is>
       </c>
       <c r="AF44" s="31" t="inlineStr">
@@ -13687,7 +13701,7 @@
       </c>
       <c r="BH44" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:45:40.235394Z</t>
+          <t>2026-07-26T18:26:09.586089Z</t>
         </is>
       </c>
       <c r="BI44" s="24" t="inlineStr">
@@ -13697,16 +13711,16 @@
       </c>
       <c r="BJ44" s="25" t="n"/>
       <c r="BK44" s="26" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="BL44" s="27" t="n">
-        <v>2</v>
+        <v>1.980392</v>
       </c>
       <c r="BM44" s="28" t="n">
-        <v>0.5</v>
+        <v>0.50495</v>
       </c>
       <c r="BN44" s="28" t="n">
-        <v>0.497512</v>
+        <v>0.502488</v>
       </c>
       <c r="BO44" s="28" t="n"/>
       <c r="BP44" s="25" t="n"/>
@@ -13755,12 +13769,12 @@
     <row r="45" ht="36" customHeight="1">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t>0e819391f1ed4f06</t>
+          <t>4b45dbe897ac4fb8</t>
         </is>
       </c>
       <c r="B45" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:48:45.878703Z</t>
+          <t>2026-07-26T18:26:27.600695Z</t>
         </is>
       </c>
       <c r="C45" s="24" t="inlineStr">
@@ -13805,23 +13819,23 @@
         </is>
       </c>
       <c r="L45" s="26" t="n">
-        <v>-106</v>
+        <v>100</v>
       </c>
       <c r="M45" s="27" t="n">
-        <v>1.943396</v>
+        <v>2</v>
       </c>
       <c r="N45" s="28" t="n">
-        <v>0.514563</v>
+        <v>0.5</v>
       </c>
       <c r="O45" s="28" t="n">
         <v>0.525689</v>
       </c>
       <c r="P45" s="28" t="n"/>
       <c r="Q45" s="28" t="n">
-        <v>0.011126</v>
+        <v>0.025689</v>
       </c>
       <c r="R45" s="26" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="S45" s="29" t="n">
         <v>0.75</v>
@@ -13847,7 +13861,7 @@
       <c r="AD45" s="24" t="n"/>
       <c r="AE45" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.5150 (aec-mlb-laa-sf-2026-07-26).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.5000 (aec-mlb-laa-sf-2026-07-26).</t>
         </is>
       </c>
       <c r="AF45" s="31" t="inlineStr">
@@ -13966,7 +13980,7 @@
       </c>
       <c r="BH45" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:45:42.030821Z</t>
+          <t>2026-07-26T18:26:10.629070Z</t>
         </is>
       </c>
       <c r="BI45" s="24" t="inlineStr">
@@ -13976,16 +13990,16 @@
       </c>
       <c r="BJ45" s="25" t="n"/>
       <c r="BK45" s="26" t="n">
-        <v>-106</v>
+        <v>100</v>
       </c>
       <c r="BL45" s="27" t="n">
-        <v>1.943396</v>
+        <v>2</v>
       </c>
       <c r="BM45" s="28" t="n">
-        <v>0.514563</v>
+        <v>0.5</v>
       </c>
       <c r="BN45" s="28" t="n">
-        <v>0.5124379999999999</v>
+        <v>0.497512</v>
       </c>
       <c r="BO45" s="28" t="n"/>
       <c r="BP45" s="25" t="n"/>
@@ -14034,12 +14048,12 @@
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="24" t="inlineStr">
         <is>
-          <t>0578edfa7bf44616</t>
+          <t>c0753eb5dc654ac2</t>
         </is>
       </c>
       <c r="B46" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:48:45.878703Z</t>
+          <t>2026-07-26T18:26:27.600695Z</t>
         </is>
       </c>
       <c r="C46" s="24" t="inlineStr">
@@ -14084,23 +14098,23 @@
         </is>
       </c>
       <c r="L46" s="26" t="n">
-        <v>-167</v>
+        <v>-178</v>
       </c>
       <c r="M46" s="27" t="n">
-        <v>1.598802</v>
+        <v>1.561798</v>
       </c>
       <c r="N46" s="28" t="n">
-        <v>0.625468</v>
+        <v>0.640288</v>
       </c>
       <c r="O46" s="28" t="n">
         <v>0.613204</v>
       </c>
       <c r="P46" s="28" t="n"/>
       <c r="Q46" s="28" t="n">
-        <v>-0.012264</v>
+        <v>-0.027084</v>
       </c>
       <c r="R46" s="26" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="S46" s="29" t="n">
         <v>1.75</v>
@@ -14126,7 +14140,7 @@
       <c r="AD46" s="24" t="n"/>
       <c r="AE46" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.6250 (aec-mlb-nyy-phi-2026-07-26).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.6400 (aec-mlb-nyy-phi-2026-07-26).</t>
         </is>
       </c>
       <c r="AF46" s="31" t="inlineStr">
@@ -14245,7 +14259,7 @@
       </c>
       <c r="BH46" s="24" t="inlineStr">
         <is>
-          <t>2026-07-26T12:45:43.638425Z</t>
+          <t>2026-07-26T18:26:12.125118Z</t>
         </is>
       </c>
       <c r="BI46" s="24" t="inlineStr">
@@ -14255,16 +14269,16 @@
       </c>
       <c r="BJ46" s="25" t="n"/>
       <c r="BK46" s="26" t="n">
-        <v>-167</v>
+        <v>-178</v>
       </c>
       <c r="BL46" s="27" t="n">
-        <v>1.598802</v>
+        <v>1.561798</v>
       </c>
       <c r="BM46" s="28" t="n">
-        <v>0.625468</v>
+        <v>0.640288</v>
       </c>
       <c r="BN46" s="28" t="n">
-        <v>0.621891</v>
+        <v>0.636816</v>
       </c>
       <c r="BO46" s="28" t="n"/>
       <c r="BP46" s="25" t="n"/>

</xml_diff>

<commit_message>
Document ledger routing; real daily forecast run confirms gate removal works live
docs/LEDGER_ROUTING.md: fixed, verified-against-code reference for which
sport/market goes into which of the four ledgers (Main/Flat/Research/Gated
Research), including the real PRODUCTION_SPORTS=(mlb,wnba) restriction
(NBA/NFL never reach Main despite being strong), the 2026-07-30 gate
removal on Main, and the 2026-07-31 Gated Research tightening -- and why
those two are deliberately opposite philosophies, per explicit operator
direction.

Ran a real `daily` forecast end to end after this session's changes.
Confirmed live: several real Main-ledger picks logged with negative edge
(e.g. -0.055, -0.11, -0.045) still got real proportional position sizing
instead of being silently excluded -- the gate removal works exactly as
intended on a real run, not just in tests. Full test suite green (500),
verify-chain clean (0 breaks).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -26220,12 +26220,12 @@
     <row r="86" ht="36" customHeight="1">
       <c r="A86" s="24" t="inlineStr">
         <is>
-          <t>5c1de5107cbf415c</t>
+          <t>019af6336be54b97</t>
         </is>
       </c>
       <c r="B86" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C86" s="24" t="inlineStr">
@@ -26431,7 +26431,7 @@
       </c>
       <c r="BH86" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:43.582472Z</t>
+          <t>2026-07-30T16:50:41.017805Z</t>
         </is>
       </c>
       <c r="BI86" s="24" t="inlineStr">
@@ -26495,12 +26495,12 @@
     <row r="87" ht="36" customHeight="1">
       <c r="A87" s="24" t="inlineStr">
         <is>
-          <t>cb18883e5acd4fc1</t>
+          <t>93a9ab3e13ae46e2</t>
         </is>
       </c>
       <c r="B87" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C87" s="24" t="inlineStr">
@@ -26706,7 +26706,7 @@
       </c>
       <c r="BH87" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:34.820648Z</t>
+          <t>2026-07-30T16:50:32.510615Z</t>
         </is>
       </c>
       <c r="BI87" s="24" t="inlineStr">
@@ -26778,12 +26778,12 @@
     <row r="88" ht="36" customHeight="1">
       <c r="A88" s="24" t="inlineStr">
         <is>
-          <t>d0bb56bfca18452b</t>
+          <t>83b81452e0604a7c</t>
         </is>
       </c>
       <c r="B88" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C88" s="24" t="inlineStr">
@@ -26989,7 +26989,7 @@
       </c>
       <c r="BH88" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:45.164513Z</t>
+          <t>2026-07-30T16:50:42.752974Z</t>
         </is>
       </c>
       <c r="BI88" s="24" t="inlineStr">
@@ -27053,12 +27053,12 @@
     <row r="89" ht="36" customHeight="1">
       <c r="A89" s="24" t="inlineStr">
         <is>
-          <t>b06367ea423d4241</t>
+          <t>466fae75fb36488a</t>
         </is>
       </c>
       <c r="B89" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C89" s="24" t="inlineStr">
@@ -27264,7 +27264,7 @@
       </c>
       <c r="BH89" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:35.604645Z</t>
+          <t>2026-07-30T16:50:33.425473Z</t>
         </is>
       </c>
       <c r="BI89" s="24" t="inlineStr">
@@ -27336,12 +27336,12 @@
     <row r="90" ht="36" customHeight="1">
       <c r="A90" s="24" t="inlineStr">
         <is>
-          <t>f5d55d23710c48b1</t>
+          <t>ce01b24809104070</t>
         </is>
       </c>
       <c r="B90" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C90" s="24" t="inlineStr">
@@ -27547,7 +27547,7 @@
       </c>
       <c r="BH90" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:46.511732Z</t>
+          <t>2026-07-30T16:50:44.006664Z</t>
         </is>
       </c>
       <c r="BI90" s="24" t="inlineStr">
@@ -27611,12 +27611,12 @@
     <row r="91" ht="36" customHeight="1">
       <c r="A91" s="24" t="inlineStr">
         <is>
-          <t>38a2be17c0934566</t>
+          <t>31e1a36c5d1b480d</t>
         </is>
       </c>
       <c r="B91" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C91" s="24" t="inlineStr">
@@ -27822,7 +27822,7 @@
       </c>
       <c r="BH91" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:36.708512Z</t>
+          <t>2026-07-30T16:50:34.454991Z</t>
         </is>
       </c>
       <c r="BI91" s="24" t="inlineStr">
@@ -27894,12 +27894,12 @@
     <row r="92" ht="36" customHeight="1">
       <c r="A92" s="24" t="inlineStr">
         <is>
-          <t>f664b50718e4462c</t>
+          <t>88de73c1654d4b88</t>
         </is>
       </c>
       <c r="B92" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C92" s="24" t="inlineStr">
@@ -28105,7 +28105,7 @@
       </c>
       <c r="BH92" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:39.761352Z</t>
+          <t>2026-07-30T16:50:37.403008Z</t>
         </is>
       </c>
       <c r="BI92" s="24" t="inlineStr">
@@ -28177,12 +28177,12 @@
     <row r="93" ht="36" customHeight="1">
       <c r="A93" s="24" t="inlineStr">
         <is>
-          <t>5a3ad9e95cd24035</t>
+          <t>9bb3a1797655440d</t>
         </is>
       </c>
       <c r="B93" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C93" s="24" t="inlineStr">
@@ -28388,7 +28388,7 @@
       </c>
       <c r="BH93" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:37.629917Z</t>
+          <t>2026-07-30T16:50:35.368337Z</t>
         </is>
       </c>
       <c r="BI93" s="24" t="inlineStr">
@@ -28460,12 +28460,12 @@
     <row r="94" ht="36" customHeight="1">
       <c r="A94" s="24" t="inlineStr">
         <is>
-          <t>d2c5d2884cb647ac</t>
+          <t>49751596f9a84157</t>
         </is>
       </c>
       <c r="B94" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C94" s="24" t="inlineStr">
@@ -28671,7 +28671,7 @@
       </c>
       <c r="BH94" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:38.590618Z</t>
+          <t>2026-07-30T16:50:36.357745Z</t>
         </is>
       </c>
       <c r="BI94" s="24" t="inlineStr">
@@ -28743,12 +28743,12 @@
     <row r="95" ht="36" customHeight="1">
       <c r="A95" s="24" t="inlineStr">
         <is>
-          <t>7f0894fbf5bf4c8c</t>
+          <t>9b063c850b944639</t>
         </is>
       </c>
       <c r="B95" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C95" s="24" t="inlineStr">
@@ -28954,7 +28954,7 @@
       </c>
       <c r="BH95" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:40.455520Z</t>
+          <t>2026-07-30T16:50:38.047846Z</t>
         </is>
       </c>
       <c r="BI95" s="24" t="inlineStr">
@@ -29026,12 +29026,12 @@
     <row r="96" ht="36" customHeight="1">
       <c r="A96" s="24" t="inlineStr">
         <is>
-          <t>cfd8401df8914da9</t>
+          <t>04d7e7d8bdea4505</t>
         </is>
       </c>
       <c r="B96" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C96" s="24" t="inlineStr">
@@ -29237,7 +29237,7 @@
       </c>
       <c r="BH96" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:41.519056Z</t>
+          <t>2026-07-30T16:50:39.045444Z</t>
         </is>
       </c>
       <c r="BI96" s="24" t="inlineStr">
@@ -29309,12 +29309,12 @@
     <row r="97" ht="36" customHeight="1">
       <c r="A97" s="24" t="inlineStr">
         <is>
-          <t>8b32ef5fbd5c4c2b</t>
+          <t>ed0278c0f0514b1a</t>
         </is>
       </c>
       <c r="B97" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:38:27.505893Z</t>
+          <t>2026-07-30T16:51:23.201418Z</t>
         </is>
       </c>
       <c r="C97" s="24" t="inlineStr">
@@ -29520,7 +29520,7 @@
       </c>
       <c r="BH97" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:37:42.508466Z</t>
+          <t>2026-07-30T16:50:40.015891Z</t>
         </is>
       </c>
       <c r="BI97" s="24" t="inlineStr">
@@ -29592,12 +29592,12 @@
     <row r="98" ht="36" customHeight="1">
       <c r="A98" s="24" t="inlineStr">
         <is>
-          <t>fc494f5a7100452c</t>
+          <t>6cbc6a8d3c464fc6</t>
         </is>
       </c>
       <c r="B98" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C98" s="24" t="inlineStr">
@@ -29653,13 +29653,13 @@
         <v>0.609375</v>
       </c>
       <c r="O98" s="28" t="n">
-        <v>0.550185</v>
+        <v>0.549881</v>
       </c>
       <c r="P98" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q98" s="28" t="n">
-        <v>-0.05919</v>
+        <v>-0.059494</v>
       </c>
       <c r="R98" s="26" t="n">
         <v>0</v>
@@ -29688,7 +29688,7 @@
       <c r="AD98" s="24" t="n"/>
       <c r="AE98" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.80-5.00; raw selected-side p=0.6442, calibrated p=0.5502.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.80-5.00; raw selected-side p=0.6427, calibrated p=0.5499.</t>
         </is>
       </c>
       <c r="AF98" s="31" t="inlineStr">
@@ -29807,7 +29807,7 @@
       </c>
       <c r="BH98" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI98" s="24" t="inlineStr">
@@ -29861,12 +29861,12 @@
     <row r="99" ht="36" customHeight="1">
       <c r="A99" s="24" t="inlineStr">
         <is>
-          <t>2560d02329574041</t>
+          <t>9b78db020f014a09</t>
         </is>
       </c>
       <c r="B99" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C99" s="24" t="inlineStr">
@@ -29922,16 +29922,16 @@
         <v>0.45045</v>
       </c>
       <c r="O99" s="28" t="n">
-        <v>0.453167</v>
+        <v>0.457387</v>
       </c>
       <c r="P99" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q99" s="28" t="n">
-        <v>0.002717</v>
+        <v>0.006937</v>
       </c>
       <c r="R99" s="26" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="S99" s="29" t="n">
         <v>0</v>
@@ -29957,7 +29957,7 @@
       <c r="AD99" s="24" t="n"/>
       <c r="AE99" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.80-5.00; raw selected-side p=0.4677, calibrated p=0.4532.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.80-5.00; raw selected-side p=0.4720, calibrated p=0.4574.</t>
         </is>
       </c>
       <c r="AF99" s="31" t="inlineStr">
@@ -30076,7 +30076,7 @@
       </c>
       <c r="BH99" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI99" s="24" t="inlineStr">
@@ -30130,12 +30130,12 @@
     <row r="100" ht="36" customHeight="1">
       <c r="A100" s="24" t="inlineStr">
         <is>
-          <t>ec53cd7feac04594</t>
+          <t>323598db4a4f45c3</t>
         </is>
       </c>
       <c r="B100" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C100" s="24" t="inlineStr">
@@ -30191,13 +30191,13 @@
         <v>0.64539</v>
       </c>
       <c r="O100" s="28" t="n">
-        <v>0.567654</v>
+        <v>0.56786</v>
       </c>
       <c r="P100" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q100" s="28" t="n">
-        <v>-0.077736</v>
+        <v>-0.07753</v>
       </c>
       <c r="R100" s="26" t="n">
         <v>0</v>
@@ -30226,7 +30226,7 @@
       <c r="AD100" s="24" t="n"/>
       <c r="AE100" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.07-4.77; raw selected-side p=0.7331, calibrated p=0.5677.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.07-4.77; raw selected-side p=0.7341, calibrated p=0.5679.</t>
         </is>
       </c>
       <c r="AF100" s="31" t="inlineStr">
@@ -30345,7 +30345,7 @@
       </c>
       <c r="BH100" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI100" s="24" t="inlineStr">
@@ -30399,12 +30399,12 @@
     <row r="101" ht="36" customHeight="1">
       <c r="A101" s="24" t="inlineStr">
         <is>
-          <t>2376747d540f4e62</t>
+          <t>5b01d791c7e34ccd</t>
         </is>
       </c>
       <c r="B101" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C101" s="24" t="inlineStr">
@@ -30460,16 +30460,16 @@
         <v>0.485437</v>
       </c>
       <c r="O101" s="28" t="n">
-        <v>0.557647</v>
+        <v>0.562401</v>
       </c>
       <c r="P101" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q101" s="28" t="n">
-        <v>0.07221</v>
+        <v>0.076964</v>
       </c>
       <c r="R101" s="26" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="S101" s="29" t="n">
         <v>0</v>
@@ -30495,7 +30495,7 @@
       <c r="AD101" s="24" t="n"/>
       <c r="AE101" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.07-4.77; raw selected-side p=0.5754, calibrated p=0.5576.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.07-4.77; raw selected-side p=0.5803, calibrated p=0.5624.</t>
         </is>
       </c>
       <c r="AF101" s="31" t="inlineStr">
@@ -30614,7 +30614,7 @@
       </c>
       <c r="BH101" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI101" s="24" t="inlineStr">
@@ -30668,12 +30668,12 @@
     <row r="102" ht="36" customHeight="1">
       <c r="A102" s="24" t="inlineStr">
         <is>
-          <t>83babb2bfb9a495a</t>
+          <t>f8c95634d709437f</t>
         </is>
       </c>
       <c r="B102" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C102" s="24" t="inlineStr">
@@ -30729,13 +30729,13 @@
         <v>0.640288</v>
       </c>
       <c r="O102" s="28" t="n">
-        <v>0.5562279999999999</v>
+        <v>0.555422</v>
       </c>
       <c r="P102" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q102" s="28" t="n">
-        <v>-0.08406</v>
+        <v>-0.084866</v>
       </c>
       <c r="R102" s="26" t="n">
         <v>0</v>
@@ -30764,7 +30764,7 @@
       <c r="AD102" s="24" t="n"/>
       <c r="AE102" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.49-4.55; raw selected-side p=0.6750, calibrated p=0.5562.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.49-4.55; raw selected-side p=0.6708, calibrated p=0.5554.</t>
         </is>
       </c>
       <c r="AF102" s="31" t="inlineStr">
@@ -30883,7 +30883,7 @@
       </c>
       <c r="BH102" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI102" s="24" t="inlineStr">
@@ -30937,12 +30937,12 @@
     <row r="103" ht="36" customHeight="1">
       <c r="A103" s="24" t="inlineStr">
         <is>
-          <t>cb8a704f328b4eb8</t>
+          <t>11100a2d97ba4145</t>
         </is>
       </c>
       <c r="B103" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C103" s="24" t="inlineStr">
@@ -30989,25 +30989,25 @@
         </is>
       </c>
       <c r="L103" s="26" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="M103" s="27" t="n">
-        <v>2.15</v>
+        <v>2.13</v>
       </c>
       <c r="N103" s="28" t="n">
-        <v>0.465116</v>
+        <v>0.469484</v>
       </c>
       <c r="O103" s="28" t="n">
-        <v>0.500848</v>
+        <v>0.501333</v>
       </c>
       <c r="P103" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q103" s="28" t="n">
-        <v>0.035732</v>
+        <v>0.031849</v>
       </c>
       <c r="R103" s="26" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="S103" s="29" t="n">
         <v>0</v>
@@ -31033,7 +31033,7 @@
       <c r="AD103" s="24" t="n"/>
       <c r="AE103" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.49-4.55; raw selected-side p=0.5168, calibrated p=0.5008.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.49-4.55; raw selected-side p=0.5173, calibrated p=0.5013.</t>
         </is>
       </c>
       <c r="AF103" s="31" t="inlineStr">
@@ -31152,7 +31152,7 @@
       </c>
       <c r="BH103" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI103" s="24" t="inlineStr">
@@ -31164,16 +31164,16 @@
         <v>8.5</v>
       </c>
       <c r="BK103" s="26" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="BL103" s="27" t="n">
-        <v>2.15</v>
+        <v>2.13</v>
       </c>
       <c r="BM103" s="28" t="n">
-        <v>0.465116</v>
+        <v>0.469484</v>
       </c>
       <c r="BN103" s="28" t="n">
-        <v>0.462687</v>
+        <v>0.467662</v>
       </c>
       <c r="BO103" s="28" t="n"/>
       <c r="BP103" s="25" t="n"/>
@@ -31206,12 +31206,12 @@
     <row r="104" ht="36" customHeight="1">
       <c r="A104" s="24" t="inlineStr">
         <is>
-          <t>294f59ac18cc43e2</t>
+          <t>efd1c2ce32cf41d1</t>
         </is>
       </c>
       <c r="B104" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C104" s="24" t="inlineStr">
@@ -31267,16 +31267,16 @@
         <v>0.590164</v>
       </c>
       <c r="O104" s="28" t="n">
-        <v>0.5436029999999999</v>
+        <v>0.545322</v>
       </c>
       <c r="P104" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q104" s="28" t="n">
-        <v>-0.046561</v>
+        <v>-0.044842</v>
       </c>
       <c r="R104" s="26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S104" s="29" t="n">
         <v>0</v>
@@ -31302,7 +31302,7 @@
       <c r="AD104" s="24" t="n"/>
       <c r="AE104" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.30-4.84; raw selected-side p=0.6107, calibrated p=0.5436.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.30-4.84; raw selected-side p=0.6194, calibrated p=0.5453.</t>
         </is>
       </c>
       <c r="AF104" s="31" t="inlineStr">
@@ -31421,7 +31421,7 @@
       </c>
       <c r="BH104" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI104" s="24" t="inlineStr">
@@ -31475,12 +31475,12 @@
     <row r="105" ht="36" customHeight="1">
       <c r="A105" s="24" t="inlineStr">
         <is>
-          <t>ccc8e32211a0463b</t>
+          <t>61e5d86f074d4d19</t>
         </is>
       </c>
       <c r="B105" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C105" s="24" t="inlineStr">
@@ -31536,13 +31536,13 @@
         <v>0.480769</v>
       </c>
       <c r="O105" s="28" t="n">
-        <v>0.567203</v>
+        <v>0.567688</v>
       </c>
       <c r="P105" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q105" s="28" t="n">
-        <v>0.086434</v>
+        <v>0.086919</v>
       </c>
       <c r="R105" s="26" t="n">
         <v>68</v>
@@ -31571,7 +31571,7 @@
       <c r="AD105" s="24" t="n"/>
       <c r="AE105" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.30-4.84; raw selected-side p=0.5852, calibrated p=0.5672.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.30-4.84; raw selected-side p=0.5857, calibrated p=0.5677.</t>
         </is>
       </c>
       <c r="AF105" s="31" t="inlineStr">
@@ -31690,7 +31690,7 @@
       </c>
       <c r="BH105" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI105" s="24" t="inlineStr">
@@ -31744,12 +31744,12 @@
     <row r="106" ht="36" customHeight="1">
       <c r="A106" s="24" t="inlineStr">
         <is>
-          <t>5a15233209c74b50</t>
+          <t>38800a441fd34920</t>
         </is>
       </c>
       <c r="B106" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C106" s="24" t="inlineStr">
@@ -31805,13 +31805,13 @@
         <v>0.34965</v>
       </c>
       <c r="O106" s="28" t="n">
-        <v>0.492424</v>
+        <v>0.492778</v>
       </c>
       <c r="P106" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q106" s="28" t="n">
-        <v>0.142774</v>
+        <v>0.143128</v>
       </c>
       <c r="R106" s="26" t="n">
         <v>96</v>
@@ -31840,7 +31840,7 @@
       <c r="AD106" s="24" t="n"/>
       <c r="AE106" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.06-4.34; raw selected-side p=0.3503, calibrated p=0.4924.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.06-4.35; raw selected-side p=0.3520, calibrated p=0.4928.</t>
         </is>
       </c>
       <c r="AF106" s="31" t="inlineStr">
@@ -31959,7 +31959,7 @@
       </c>
       <c r="BH106" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI106" s="24" t="inlineStr">
@@ -32013,12 +32013,12 @@
     <row r="107" ht="36" customHeight="1">
       <c r="A107" s="24" t="inlineStr">
         <is>
-          <t>27ad9d992fb34c00</t>
+          <t>6d96e06825254f55</t>
         </is>
       </c>
       <c r="B107" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C107" s="24" t="inlineStr">
@@ -32074,13 +32074,13 @@
         <v>0.45045</v>
       </c>
       <c r="O107" s="28" t="n">
-        <v>0.518552</v>
+        <v>0.5180670000000001</v>
       </c>
       <c r="P107" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q107" s="28" t="n">
-        <v>0.068102</v>
+        <v>0.067617</v>
       </c>
       <c r="R107" s="26" t="n">
         <v>59</v>
@@ -32109,7 +32109,7 @@
       <c r="AD107" s="24" t="n"/>
       <c r="AE107" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.06-4.34; raw selected-side p=0.5351, calibrated p=0.5186.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.06-4.35; raw selected-side p=0.5345, calibrated p=0.5181.</t>
         </is>
       </c>
       <c r="AF107" s="31" t="inlineStr">
@@ -32228,7 +32228,7 @@
       </c>
       <c r="BH107" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI107" s="24" t="inlineStr">
@@ -32282,12 +32282,12 @@
     <row r="108" ht="36" customHeight="1">
       <c r="A108" s="24" t="inlineStr">
         <is>
-          <t>592a3274609a40d1</t>
+          <t>542874cd741e4c30</t>
         </is>
       </c>
       <c r="B108" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C108" s="24" t="inlineStr">
@@ -32343,16 +32343,16 @@
         <v>0.590164</v>
       </c>
       <c r="O108" s="28" t="n">
-        <v>0.549213</v>
+        <v>0.547424</v>
       </c>
       <c r="P108" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q108" s="28" t="n">
-        <v>-0.040951</v>
+        <v>-0.04274</v>
       </c>
       <c r="R108" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S108" s="29" t="n">
         <v>0</v>
@@ -32378,7 +32378,7 @@
       <c r="AD108" s="24" t="n"/>
       <c r="AE108" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.87-4.53; raw selected-side p=0.6392, calibrated p=0.5492.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.87-4.53; raw selected-side p=0.6301, calibrated p=0.5474.</t>
         </is>
       </c>
       <c r="AF108" s="31" t="inlineStr">
@@ -32497,7 +32497,7 @@
       </c>
       <c r="BH108" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI108" s="24" t="inlineStr">
@@ -32551,12 +32551,12 @@
     <row r="109" ht="36" customHeight="1">
       <c r="A109" s="24" t="inlineStr">
         <is>
-          <t>055ba7f1dc734ae1</t>
+          <t>0afc14c7a0ea4e1a</t>
         </is>
       </c>
       <c r="B109" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C109" s="24" t="inlineStr">
@@ -32612,13 +32612,13 @@
         <v>0.490196</v>
       </c>
       <c r="O109" s="28" t="n">
-        <v>0.544939</v>
+        <v>0.544648</v>
       </c>
       <c r="P109" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q109" s="28" t="n">
-        <v>0.054743</v>
+        <v>0.054452</v>
       </c>
       <c r="R109" s="26" t="n">
         <v>52</v>
@@ -32647,7 +32647,7 @@
       <c r="AD109" s="24" t="n"/>
       <c r="AE109" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.87-4.53; raw selected-side p=0.5623, calibrated p=0.5449.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.87-4.53; raw selected-side p=0.5619, calibrated p=0.5446.</t>
         </is>
       </c>
       <c r="AF109" s="31" t="inlineStr">
@@ -32766,7 +32766,7 @@
       </c>
       <c r="BH109" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI109" s="24" t="inlineStr">
@@ -32820,12 +32820,12 @@
     <row r="110" ht="36" customHeight="1">
       <c r="A110" s="24" t="inlineStr">
         <is>
-          <t>c1db02ed98c54843</t>
+          <t>5021001434414d0e</t>
         </is>
       </c>
       <c r="B110" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C110" s="24" t="inlineStr">
@@ -32881,13 +32881,13 @@
         <v>0.49505</v>
       </c>
       <c r="O110" s="28" t="n">
-        <v>0.544035</v>
+        <v>0.543779</v>
       </c>
       <c r="P110" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q110" s="28" t="n">
-        <v>0.048985</v>
+        <v>0.048729</v>
       </c>
       <c r="R110" s="26" t="n">
         <v>49</v>
@@ -32916,7 +32916,7 @@
       <c r="AD110" s="24" t="n"/>
       <c r="AE110" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 5.03-4.48; raw selected-side p=0.6129, calibrated p=0.5440.</t>
+          <t>Measured Edge Margin: Trend Engine projected 5.03-4.48; raw selected-side p=0.6116, calibrated p=0.5438.</t>
         </is>
       </c>
       <c r="AF110" s="31" t="inlineStr">
@@ -33035,7 +33035,7 @@
       </c>
       <c r="BH110" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI110" s="24" t="inlineStr">
@@ -33089,12 +33089,12 @@
     <row r="111" ht="36" customHeight="1">
       <c r="A111" s="24" t="inlineStr">
         <is>
-          <t>26679dde013e4286</t>
+          <t>c9fafefee3684c6d</t>
         </is>
       </c>
       <c r="B111" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C111" s="24" t="inlineStr">
@@ -33150,16 +33150,16 @@
         <v>0.534884</v>
       </c>
       <c r="O111" s="28" t="n">
-        <v>0.595772</v>
+        <v>0.603678</v>
       </c>
       <c r="P111" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q111" s="28" t="n">
-        <v>0.060888</v>
+        <v>0.06879399999999999</v>
       </c>
       <c r="R111" s="26" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="S111" s="29" t="n">
         <v>0</v>
@@ -33185,7 +33185,7 @@
       <c r="AD111" s="24" t="n"/>
       <c r="AE111" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 5.03-4.48; raw selected-side p=0.6147, calibrated p=0.5958.</t>
+          <t>Measured Edge Totals: Trend Engine projected 5.03-4.48; raw selected-side p=0.6228, calibrated p=0.6037.</t>
         </is>
       </c>
       <c r="AF111" s="31" t="inlineStr">
@@ -33304,7 +33304,7 @@
       </c>
       <c r="BH111" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI111" s="24" t="inlineStr">
@@ -33358,12 +33358,12 @@
     <row r="112" ht="36" customHeight="1">
       <c r="A112" s="24" t="inlineStr">
         <is>
-          <t>f49c58d2da02434d</t>
+          <t>95186e18c67a45f8</t>
         </is>
       </c>
       <c r="B112" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C112" s="24" t="inlineStr">
@@ -33419,13 +33419,13 @@
         <v>0.604743</v>
       </c>
       <c r="O112" s="28" t="n">
-        <v>0.559774</v>
+        <v>0.55947</v>
       </c>
       <c r="P112" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q112" s="28" t="n">
-        <v>-0.044969</v>
+        <v>-0.045273</v>
       </c>
       <c r="R112" s="26" t="n">
         <v>0</v>
@@ -33454,7 +33454,7 @@
       <c r="AD112" s="24" t="n"/>
       <c r="AE112" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.48-4.27; raw selected-side p=0.6930, calibrated p=0.5598.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.48-4.27; raw selected-side p=0.6915, calibrated p=0.5595.</t>
         </is>
       </c>
       <c r="AF112" s="31" t="inlineStr">
@@ -33573,7 +33573,7 @@
       </c>
       <c r="BH112" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI112" s="24" t="inlineStr">
@@ -33627,12 +33627,12 @@
     <row r="113" ht="36" customHeight="1">
       <c r="A113" s="24" t="inlineStr">
         <is>
-          <t>617450175dad44e3</t>
+          <t>e560b1bb79ae4f50</t>
         </is>
       </c>
       <c r="B113" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C113" s="24" t="inlineStr">
@@ -33688,16 +33688,16 @@
         <v>0.480769</v>
       </c>
       <c r="O113" s="28" t="n">
-        <v>0.479748</v>
+        <v>0.475237</v>
       </c>
       <c r="P113" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q113" s="28" t="n">
-        <v>-0.001021</v>
+        <v>-0.005532</v>
       </c>
       <c r="R113" s="26" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="S113" s="29" t="n">
         <v>0</v>
@@ -33723,7 +33723,7 @@
       <c r="AD113" s="24" t="n"/>
       <c r="AE113" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.48-4.27; raw selected-side p=0.4950, calibrated p=0.4797.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.48-4.27; raw selected-side p=0.4904, calibrated p=0.4752.</t>
         </is>
       </c>
       <c r="AF113" s="31" t="inlineStr">
@@ -33842,7 +33842,7 @@
       </c>
       <c r="BH113" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI113" s="24" t="inlineStr">
@@ -33896,12 +33896,12 @@
     <row r="114" ht="36" customHeight="1">
       <c r="A114" s="24" t="inlineStr">
         <is>
-          <t>b153c3cef0924c63</t>
+          <t>3659e0c9b5d14b9c</t>
         </is>
       </c>
       <c r="B114" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C114" s="24" t="inlineStr">
@@ -33957,13 +33957,13 @@
         <v>0.590164</v>
       </c>
       <c r="O114" s="28" t="n">
-        <v>0.5493209999999999</v>
+        <v>0.548682</v>
       </c>
       <c r="P114" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q114" s="28" t="n">
-        <v>-0.040843</v>
+        <v>-0.041482</v>
       </c>
       <c r="R114" s="26" t="n">
         <v>4</v>
@@ -33992,7 +33992,7 @@
       <c r="AD114" s="24" t="n"/>
       <c r="AE114" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.65-4.92; raw selected-side p=0.6398, calibrated p=0.5493.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.65-4.92; raw selected-side p=0.6365, calibrated p=0.5487.</t>
         </is>
       </c>
       <c r="AF114" s="31" t="inlineStr">
@@ -34111,7 +34111,7 @@
       </c>
       <c r="BH114" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI114" s="24" t="inlineStr">
@@ -34165,12 +34165,12 @@
     <row r="115" ht="36" customHeight="1">
       <c r="A115" s="24" t="inlineStr">
         <is>
-          <t>c9b8880ee8884f3e</t>
+          <t>3cc0f9e8e6b54d87</t>
         </is>
       </c>
       <c r="B115" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="C115" s="24" t="inlineStr">
@@ -34226,16 +34226,16 @@
         <v>0.530516</v>
       </c>
       <c r="O115" s="28" t="n">
-        <v>0.547995</v>
+        <v>0.544745</v>
       </c>
       <c r="P115" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q115" s="28" t="n">
-        <v>0.017479</v>
+        <v>0.014229</v>
       </c>
       <c r="R115" s="26" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="S115" s="29" t="n">
         <v>0</v>
@@ -34261,7 +34261,7 @@
       <c r="AD115" s="24" t="n"/>
       <c r="AE115" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.65-4.92; raw selected-side p=0.5654, calibrated p=0.5480.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.65-4.92; raw selected-side p=0.5621, calibrated p=0.5447.</t>
         </is>
       </c>
       <c r="AF115" s="31" t="inlineStr">
@@ -34380,7 +34380,7 @@
       </c>
       <c r="BH115" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:39:08.609380Z</t>
+          <t>2026-07-30T16:51:51.403706Z</t>
         </is>
       </c>
       <c r="BI115" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Real ledger state from second daily forecast + settlement run
Confirms the full pipeline (settle -> flat forecast -> main forecast)
runs cleanly end to end after this session's fixes: gate removal, Gated
Research tightening, dashboard/refresh_prices fix, archived retired-model
picks. Zero failures across every sport in the settlement report.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -26220,12 +26220,12 @@
     <row r="86" ht="36" customHeight="1">
       <c r="A86" s="24" t="inlineStr">
         <is>
-          <t>019af6336be54b97</t>
+          <t>90555303e32f47c0</t>
         </is>
       </c>
       <c r="B86" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C86" s="24" t="inlineStr">
@@ -26431,7 +26431,7 @@
       </c>
       <c r="BH86" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:41.017805Z</t>
+          <t>2026-07-30T17:17:41.975528Z</t>
         </is>
       </c>
       <c r="BI86" s="24" t="inlineStr">
@@ -26495,12 +26495,12 @@
     <row r="87" ht="36" customHeight="1">
       <c r="A87" s="24" t="inlineStr">
         <is>
-          <t>93a9ab3e13ae46e2</t>
+          <t>46446adc53524558</t>
         </is>
       </c>
       <c r="B87" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C87" s="24" t="inlineStr">
@@ -26706,7 +26706,7 @@
       </c>
       <c r="BH87" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:32.510615Z</t>
+          <t>2026-07-30T17:17:33.085623Z</t>
         </is>
       </c>
       <c r="BI87" s="24" t="inlineStr">
@@ -26778,12 +26778,12 @@
     <row r="88" ht="36" customHeight="1">
       <c r="A88" s="24" t="inlineStr">
         <is>
-          <t>83b81452e0604a7c</t>
+          <t>9ed711934b3742e5</t>
         </is>
       </c>
       <c r="B88" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C88" s="24" t="inlineStr">
@@ -26989,7 +26989,7 @@
       </c>
       <c r="BH88" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:42.752974Z</t>
+          <t>2026-07-30T17:17:43.676555Z</t>
         </is>
       </c>
       <c r="BI88" s="24" t="inlineStr">
@@ -27053,12 +27053,12 @@
     <row r="89" ht="36" customHeight="1">
       <c r="A89" s="24" t="inlineStr">
         <is>
-          <t>466fae75fb36488a</t>
+          <t>89d488b018874530</t>
         </is>
       </c>
       <c r="B89" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C89" s="24" t="inlineStr">
@@ -27264,7 +27264,7 @@
       </c>
       <c r="BH89" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:33.425473Z</t>
+          <t>2026-07-30T17:17:34.062012Z</t>
         </is>
       </c>
       <c r="BI89" s="24" t="inlineStr">
@@ -27336,12 +27336,12 @@
     <row r="90" ht="36" customHeight="1">
       <c r="A90" s="24" t="inlineStr">
         <is>
-          <t>ce01b24809104070</t>
+          <t>1315e1b8446b4cc6</t>
         </is>
       </c>
       <c r="B90" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C90" s="24" t="inlineStr">
@@ -27547,7 +27547,7 @@
       </c>
       <c r="BH90" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:44.006664Z</t>
+          <t>2026-07-30T17:17:44.949554Z</t>
         </is>
       </c>
       <c r="BI90" s="24" t="inlineStr">
@@ -27611,12 +27611,12 @@
     <row r="91" ht="36" customHeight="1">
       <c r="A91" s="24" t="inlineStr">
         <is>
-          <t>31e1a36c5d1b480d</t>
+          <t>5352883f901947bd</t>
         </is>
       </c>
       <c r="B91" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C91" s="24" t="inlineStr">
@@ -27822,7 +27822,7 @@
       </c>
       <c r="BH91" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:34.454991Z</t>
+          <t>2026-07-30T17:17:35.081580Z</t>
         </is>
       </c>
       <c r="BI91" s="24" t="inlineStr">
@@ -27894,12 +27894,12 @@
     <row r="92" ht="36" customHeight="1">
       <c r="A92" s="24" t="inlineStr">
         <is>
-          <t>88de73c1654d4b88</t>
+          <t>308e6d5daced4850</t>
         </is>
       </c>
       <c r="B92" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C92" s="24" t="inlineStr">
@@ -28105,7 +28105,7 @@
       </c>
       <c r="BH92" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:37.403008Z</t>
+          <t>2026-07-30T17:17:38.217983Z</t>
         </is>
       </c>
       <c r="BI92" s="24" t="inlineStr">
@@ -28177,12 +28177,12 @@
     <row r="93" ht="36" customHeight="1">
       <c r="A93" s="24" t="inlineStr">
         <is>
-          <t>9bb3a1797655440d</t>
+          <t>3637a4075d654228</t>
         </is>
       </c>
       <c r="B93" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C93" s="24" t="inlineStr">
@@ -28388,7 +28388,7 @@
       </c>
       <c r="BH93" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:35.368337Z</t>
+          <t>2026-07-30T17:17:36.074233Z</t>
         </is>
       </c>
       <c r="BI93" s="24" t="inlineStr">
@@ -28460,12 +28460,12 @@
     <row r="94" ht="36" customHeight="1">
       <c r="A94" s="24" t="inlineStr">
         <is>
-          <t>49751596f9a84157</t>
+          <t>3a3c0a538c744d8f</t>
         </is>
       </c>
       <c r="B94" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C94" s="24" t="inlineStr">
@@ -28671,7 +28671,7 @@
       </c>
       <c r="BH94" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:36.357745Z</t>
+          <t>2026-07-30T17:17:37.061484Z</t>
         </is>
       </c>
       <c r="BI94" s="24" t="inlineStr">
@@ -28743,12 +28743,12 @@
     <row r="95" ht="36" customHeight="1">
       <c r="A95" s="24" t="inlineStr">
         <is>
-          <t>9b063c850b944639</t>
+          <t>89188b6bddfa4e04</t>
         </is>
       </c>
       <c r="B95" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C95" s="24" t="inlineStr">
@@ -28954,7 +28954,7 @@
       </c>
       <c r="BH95" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:38.047846Z</t>
+          <t>2026-07-30T17:17:38.913634Z</t>
         </is>
       </c>
       <c r="BI95" s="24" t="inlineStr">
@@ -29026,12 +29026,12 @@
     <row r="96" ht="36" customHeight="1">
       <c r="A96" s="24" t="inlineStr">
         <is>
-          <t>04d7e7d8bdea4505</t>
+          <t>13b93429e47d4e18</t>
         </is>
       </c>
       <c r="B96" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C96" s="24" t="inlineStr">
@@ -29237,7 +29237,7 @@
       </c>
       <c r="BH96" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:39.045444Z</t>
+          <t>2026-07-30T17:17:40.032869Z</t>
         </is>
       </c>
       <c r="BI96" s="24" t="inlineStr">
@@ -29309,12 +29309,12 @@
     <row r="97" ht="36" customHeight="1">
       <c r="A97" s="24" t="inlineStr">
         <is>
-          <t>ed0278c0f0514b1a</t>
+          <t>075812f4dde4432b</t>
         </is>
       </c>
       <c r="B97" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:23.201418Z</t>
+          <t>2026-07-30T17:18:22.482445Z</t>
         </is>
       </c>
       <c r="C97" s="24" t="inlineStr">
@@ -29359,23 +29359,23 @@
         </is>
       </c>
       <c r="L97" s="26" t="n">
-        <v>-144</v>
+        <v>-147</v>
       </c>
       <c r="M97" s="27" t="n">
-        <v>1.694444</v>
+        <v>1.680272</v>
       </c>
       <c r="N97" s="28" t="n">
-        <v>0.590164</v>
+        <v>0.5951419999999999</v>
       </c>
       <c r="O97" s="28" t="n">
         <v>0.593883</v>
       </c>
       <c r="P97" s="28" t="n"/>
       <c r="Q97" s="28" t="n">
-        <v>0.003719</v>
+        <v>-0.001259</v>
       </c>
       <c r="R97" s="26" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="S97" s="29" t="n">
         <v>1.5</v>
@@ -29401,7 +29401,7 @@
       <c r="AD97" s="24" t="n"/>
       <c r="AE97" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.6242; executable ask 0.5900 (aec-mlb-sea-lad-2026-07-30); model edge vs ask +0.0039.</t>
+          <t>Learned LR call at threshold 0.6242; executable ask 0.5950 (aec-mlb-sea-lad-2026-07-30); model edge vs ask -0.0011.</t>
         </is>
       </c>
       <c r="AF97" s="31" t="inlineStr">
@@ -29520,7 +29520,7 @@
       </c>
       <c r="BH97" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:50:40.015891Z</t>
+          <t>2026-07-30T17:17:41.015176Z</t>
         </is>
       </c>
       <c r="BI97" s="24" t="inlineStr">
@@ -29530,16 +29530,16 @@
       </c>
       <c r="BJ97" s="25" t="n"/>
       <c r="BK97" s="26" t="n">
-        <v>-144</v>
+        <v>-147</v>
       </c>
       <c r="BL97" s="27" t="n">
-        <v>1.694444</v>
+        <v>1.680272</v>
       </c>
       <c r="BM97" s="28" t="n">
-        <v>0.590164</v>
+        <v>0.5951419999999999</v>
       </c>
       <c r="BN97" s="28" t="n">
-        <v>0.5870649999999999</v>
+        <v>0.59204</v>
       </c>
       <c r="BO97" s="28" t="n"/>
       <c r="BP97" s="25" t="n"/>
@@ -29592,12 +29592,12 @@
     <row r="98" ht="36" customHeight="1">
       <c r="A98" s="24" t="inlineStr">
         <is>
-          <t>6cbc6a8d3c464fc6</t>
+          <t>41c5bee3def94e38</t>
         </is>
       </c>
       <c r="B98" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C98" s="24" t="inlineStr">
@@ -29653,13 +29653,13 @@
         <v>0.609375</v>
       </c>
       <c r="O98" s="28" t="n">
-        <v>0.549881</v>
+        <v>0.551079</v>
       </c>
       <c r="P98" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q98" s="28" t="n">
-        <v>-0.059494</v>
+        <v>-0.058296</v>
       </c>
       <c r="R98" s="26" t="n">
         <v>0</v>
@@ -29688,7 +29688,7 @@
       <c r="AD98" s="24" t="n"/>
       <c r="AE98" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.80-5.00; raw selected-side p=0.6427, calibrated p=0.5499.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.80-5.00; raw selected-side p=0.6488, calibrated p=0.5511.</t>
         </is>
       </c>
       <c r="AF98" s="31" t="inlineStr">
@@ -29807,7 +29807,7 @@
       </c>
       <c r="BH98" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI98" s="24" t="inlineStr">
@@ -29861,12 +29861,12 @@
     <row r="99" ht="36" customHeight="1">
       <c r="A99" s="24" t="inlineStr">
         <is>
-          <t>9b78db020f014a09</t>
+          <t>c7d1c1ea6a644a75</t>
         </is>
       </c>
       <c r="B99" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C99" s="24" t="inlineStr">
@@ -29922,16 +29922,16 @@
         <v>0.45045</v>
       </c>
       <c r="O99" s="28" t="n">
-        <v>0.457387</v>
+        <v>0.465051</v>
       </c>
       <c r="P99" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q99" s="28" t="n">
-        <v>0.006937</v>
+        <v>0.014601</v>
       </c>
       <c r="R99" s="26" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="S99" s="29" t="n">
         <v>0</v>
@@ -29957,7 +29957,7 @@
       <c r="AD99" s="24" t="n"/>
       <c r="AE99" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.80-5.00; raw selected-side p=0.4720, calibrated p=0.4574.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.80-5.00; raw selected-side p=0.4799, calibrated p=0.4651.</t>
         </is>
       </c>
       <c r="AF99" s="31" t="inlineStr">
@@ -30076,7 +30076,7 @@
       </c>
       <c r="BH99" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI99" s="24" t="inlineStr">
@@ -30130,12 +30130,12 @@
     <row r="100" ht="36" customHeight="1">
       <c r="A100" s="24" t="inlineStr">
         <is>
-          <t>323598db4a4f45c3</t>
+          <t>aaa374fcf56346ca</t>
         </is>
       </c>
       <c r="B100" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C100" s="24" t="inlineStr">
@@ -30191,13 +30191,13 @@
         <v>0.64539</v>
       </c>
       <c r="O100" s="28" t="n">
-        <v>0.56786</v>
+        <v>0.5684399999999999</v>
       </c>
       <c r="P100" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q100" s="28" t="n">
-        <v>-0.07753</v>
+        <v>-0.07695</v>
       </c>
       <c r="R100" s="26" t="n">
         <v>0</v>
@@ -30226,7 +30226,7 @@
       <c r="AD100" s="24" t="n"/>
       <c r="AE100" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.07-4.77; raw selected-side p=0.7341, calibrated p=0.5679.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.07-4.77; raw selected-side p=0.7371, calibrated p=0.5684.</t>
         </is>
       </c>
       <c r="AF100" s="31" t="inlineStr">
@@ -30345,7 +30345,7 @@
       </c>
       <c r="BH100" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI100" s="24" t="inlineStr">
@@ -30399,12 +30399,12 @@
     <row r="101" ht="36" customHeight="1">
       <c r="A101" s="24" t="inlineStr">
         <is>
-          <t>5b01d791c7e34ccd</t>
+          <t>dc0ec81ac7a64b06</t>
         </is>
       </c>
       <c r="B101" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C101" s="24" t="inlineStr">
@@ -30460,16 +30460,16 @@
         <v>0.485437</v>
       </c>
       <c r="O101" s="28" t="n">
-        <v>0.562401</v>
+        <v>0.556337</v>
       </c>
       <c r="P101" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q101" s="28" t="n">
-        <v>0.076964</v>
+        <v>0.0709</v>
       </c>
       <c r="R101" s="26" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="S101" s="29" t="n">
         <v>0</v>
@@ -30495,7 +30495,7 @@
       <c r="AD101" s="24" t="n"/>
       <c r="AE101" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.07-4.77; raw selected-side p=0.5803, calibrated p=0.5624.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.07-4.77; raw selected-side p=0.5740, calibrated p=0.5563.</t>
         </is>
       </c>
       <c r="AF101" s="31" t="inlineStr">
@@ -30614,7 +30614,7 @@
       </c>
       <c r="BH101" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI101" s="24" t="inlineStr">
@@ -30668,12 +30668,12 @@
     <row r="102" ht="36" customHeight="1">
       <c r="A102" s="24" t="inlineStr">
         <is>
-          <t>f8c95634d709437f</t>
+          <t>a711dc733b2644a6</t>
         </is>
       </c>
       <c r="B102" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C102" s="24" t="inlineStr">
@@ -30720,22 +30720,22 @@
         </is>
       </c>
       <c r="L102" s="26" t="n">
-        <v>-178</v>
+        <v>-174</v>
       </c>
       <c r="M102" s="27" t="n">
-        <v>1.561798</v>
+        <v>1.574713</v>
       </c>
       <c r="N102" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.635036</v>
       </c>
       <c r="O102" s="28" t="n">
-        <v>0.555422</v>
+        <v>0.555677</v>
       </c>
       <c r="P102" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q102" s="28" t="n">
-        <v>-0.084866</v>
+        <v>-0.079359</v>
       </c>
       <c r="R102" s="26" t="n">
         <v>0</v>
@@ -30764,7 +30764,7 @@
       <c r="AD102" s="24" t="n"/>
       <c r="AE102" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.49-4.55; raw selected-side p=0.6708, calibrated p=0.5554.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.49-4.55; raw selected-side p=0.6722, calibrated p=0.5557.</t>
         </is>
       </c>
       <c r="AF102" s="31" t="inlineStr">
@@ -30883,7 +30883,7 @@
       </c>
       <c r="BH102" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI102" s="24" t="inlineStr">
@@ -30895,16 +30895,16 @@
         <v>1.5</v>
       </c>
       <c r="BK102" s="26" t="n">
-        <v>-178</v>
+        <v>-174</v>
       </c>
       <c r="BL102" s="27" t="n">
-        <v>1.561798</v>
+        <v>1.574713</v>
       </c>
       <c r="BM102" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.635036</v>
       </c>
       <c r="BN102" s="28" t="n">
-        <v>0.636816</v>
+        <v>0.631841</v>
       </c>
       <c r="BO102" s="28" t="n"/>
       <c r="BP102" s="25" t="n"/>
@@ -30937,12 +30937,12 @@
     <row r="103" ht="36" customHeight="1">
       <c r="A103" s="24" t="inlineStr">
         <is>
-          <t>11100a2d97ba4145</t>
+          <t>1772c061995f4a46</t>
         </is>
       </c>
       <c r="B103" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C103" s="24" t="inlineStr">
@@ -30998,13 +30998,13 @@
         <v>0.469484</v>
       </c>
       <c r="O103" s="28" t="n">
-        <v>0.501333</v>
+        <v>0.501139</v>
       </c>
       <c r="P103" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q103" s="28" t="n">
-        <v>0.031849</v>
+        <v>0.031655</v>
       </c>
       <c r="R103" s="26" t="n">
         <v>41</v>
@@ -31033,7 +31033,7 @@
       <c r="AD103" s="24" t="n"/>
       <c r="AE103" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.49-4.55; raw selected-side p=0.5173, calibrated p=0.5013.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.49-4.55; raw selected-side p=0.5171, calibrated p=0.5011.</t>
         </is>
       </c>
       <c r="AF103" s="31" t="inlineStr">
@@ -31152,7 +31152,7 @@
       </c>
       <c r="BH103" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI103" s="24" t="inlineStr">
@@ -31173,7 +31173,7 @@
         <v>0.469484</v>
       </c>
       <c r="BN103" s="28" t="n">
-        <v>0.467662</v>
+        <v>0.465347</v>
       </c>
       <c r="BO103" s="28" t="n"/>
       <c r="BP103" s="25" t="n"/>
@@ -31206,12 +31206,12 @@
     <row r="104" ht="36" customHeight="1">
       <c r="A104" s="24" t="inlineStr">
         <is>
-          <t>efd1c2ce32cf41d1</t>
+          <t>669fab5c44624df9</t>
         </is>
       </c>
       <c r="B104" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C104" s="24" t="inlineStr">
@@ -31267,13 +31267,13 @@
         <v>0.590164</v>
       </c>
       <c r="O104" s="28" t="n">
-        <v>0.545322</v>
+        <v>0.545381</v>
       </c>
       <c r="P104" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q104" s="28" t="n">
-        <v>-0.044842</v>
+        <v>-0.044783</v>
       </c>
       <c r="R104" s="26" t="n">
         <v>2</v>
@@ -31302,7 +31302,7 @@
       <c r="AD104" s="24" t="n"/>
       <c r="AE104" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.30-4.84; raw selected-side p=0.6194, calibrated p=0.5453.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.30-4.84; raw selected-side p=0.6198, calibrated p=0.5454.</t>
         </is>
       </c>
       <c r="AF104" s="31" t="inlineStr">
@@ -31421,7 +31421,7 @@
       </c>
       <c r="BH104" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI104" s="24" t="inlineStr">
@@ -31475,12 +31475,12 @@
     <row r="105" ht="36" customHeight="1">
       <c r="A105" s="24" t="inlineStr">
         <is>
-          <t>61e5d86f074d4d19</t>
+          <t>07ca08b26f114d8a</t>
         </is>
       </c>
       <c r="B105" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C105" s="24" t="inlineStr">
@@ -31536,16 +31536,16 @@
         <v>0.480769</v>
       </c>
       <c r="O105" s="28" t="n">
-        <v>0.567688</v>
+        <v>0.571665</v>
       </c>
       <c r="P105" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q105" s="28" t="n">
-        <v>0.086919</v>
+        <v>0.090896</v>
       </c>
       <c r="R105" s="26" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="S105" s="29" t="n">
         <v>0</v>
@@ -31571,7 +31571,7 @@
       <c r="AD105" s="24" t="n"/>
       <c r="AE105" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.30-4.84; raw selected-side p=0.5857, calibrated p=0.5677.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.30-4.84; raw selected-side p=0.5898, calibrated p=0.5717.</t>
         </is>
       </c>
       <c r="AF105" s="31" t="inlineStr">
@@ -31690,7 +31690,7 @@
       </c>
       <c r="BH105" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI105" s="24" t="inlineStr">
@@ -31744,12 +31744,12 @@
     <row r="106" ht="36" customHeight="1">
       <c r="A106" s="24" t="inlineStr">
         <is>
-          <t>38800a441fd34920</t>
+          <t>fbde174a130249fd</t>
         </is>
       </c>
       <c r="B106" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C106" s="24" t="inlineStr">
@@ -31805,16 +31805,16 @@
         <v>0.34965</v>
       </c>
       <c r="O106" s="28" t="n">
-        <v>0.492778</v>
+        <v>0.493426</v>
       </c>
       <c r="P106" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q106" s="28" t="n">
-        <v>0.143128</v>
+        <v>0.143776</v>
       </c>
       <c r="R106" s="26" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S106" s="29" t="n">
         <v>0</v>
@@ -31840,7 +31840,7 @@
       <c r="AD106" s="24" t="n"/>
       <c r="AE106" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.06-4.35; raw selected-side p=0.3520, calibrated p=0.4928.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.06-4.35; raw selected-side p=0.3553, calibrated p=0.4934.</t>
         </is>
       </c>
       <c r="AF106" s="31" t="inlineStr">
@@ -31959,7 +31959,7 @@
       </c>
       <c r="BH106" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI106" s="24" t="inlineStr">
@@ -32013,12 +32013,12 @@
     <row r="107" ht="36" customHeight="1">
       <c r="A107" s="24" t="inlineStr">
         <is>
-          <t>6d96e06825254f55</t>
+          <t>4b46515e5e434be0</t>
         </is>
       </c>
       <c r="B107" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C107" s="24" t="inlineStr">
@@ -32074,16 +32074,16 @@
         <v>0.45045</v>
       </c>
       <c r="O107" s="28" t="n">
-        <v>0.5180670000000001</v>
+        <v>0.523111</v>
       </c>
       <c r="P107" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q107" s="28" t="n">
-        <v>0.067617</v>
+        <v>0.072661</v>
       </c>
       <c r="R107" s="26" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="S107" s="29" t="n">
         <v>0</v>
@@ -32109,7 +32109,7 @@
       <c r="AD107" s="24" t="n"/>
       <c r="AE107" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.06-4.35; raw selected-side p=0.5345, calibrated p=0.5181.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.06-4.35; raw selected-side p=0.5397, calibrated p=0.5231.</t>
         </is>
       </c>
       <c r="AF107" s="31" t="inlineStr">
@@ -32228,7 +32228,7 @@
       </c>
       <c r="BH107" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI107" s="24" t="inlineStr">
@@ -32282,12 +32282,12 @@
     <row r="108" ht="36" customHeight="1">
       <c r="A108" s="24" t="inlineStr">
         <is>
-          <t>542874cd741e4c30</t>
+          <t>44c06d8e6f2e4571</t>
         </is>
       </c>
       <c r="B108" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C108" s="24" t="inlineStr">
@@ -32343,16 +32343,16 @@
         <v>0.590164</v>
       </c>
       <c r="O108" s="28" t="n">
-        <v>0.547424</v>
+        <v>0.548201</v>
       </c>
       <c r="P108" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q108" s="28" t="n">
-        <v>-0.04274</v>
+        <v>-0.041963</v>
       </c>
       <c r="R108" s="26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S108" s="29" t="n">
         <v>0</v>
@@ -32378,7 +32378,7 @@
       <c r="AD108" s="24" t="n"/>
       <c r="AE108" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.87-4.53; raw selected-side p=0.6301, calibrated p=0.5474.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.87-4.53; raw selected-side p=0.6341, calibrated p=0.5482.</t>
         </is>
       </c>
       <c r="AF108" s="31" t="inlineStr">
@@ -32497,7 +32497,7 @@
       </c>
       <c r="BH108" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI108" s="24" t="inlineStr">
@@ -32551,12 +32551,12 @@
     <row r="109" ht="36" customHeight="1">
       <c r="A109" s="24" t="inlineStr">
         <is>
-          <t>0afc14c7a0ea4e1a</t>
+          <t>3f4d266778b94a7a</t>
         </is>
       </c>
       <c r="B109" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C109" s="24" t="inlineStr">
@@ -32612,13 +32612,13 @@
         <v>0.490196</v>
       </c>
       <c r="O109" s="28" t="n">
-        <v>0.544648</v>
+        <v>0.544745</v>
       </c>
       <c r="P109" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q109" s="28" t="n">
-        <v>0.054452</v>
+        <v>0.054549</v>
       </c>
       <c r="R109" s="26" t="n">
         <v>52</v>
@@ -32647,7 +32647,7 @@
       <c r="AD109" s="24" t="n"/>
       <c r="AE109" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.87-4.53; raw selected-side p=0.5619, calibrated p=0.5446.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.87-4.53; raw selected-side p=0.5621, calibrated p=0.5447.</t>
         </is>
       </c>
       <c r="AF109" s="31" t="inlineStr">
@@ -32766,7 +32766,7 @@
       </c>
       <c r="BH109" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI109" s="24" t="inlineStr">
@@ -32820,12 +32820,12 @@
     <row r="110" ht="36" customHeight="1">
       <c r="A110" s="24" t="inlineStr">
         <is>
-          <t>5021001434414d0e</t>
+          <t>f1aaeac92c434837</t>
         </is>
       </c>
       <c r="B110" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C110" s="24" t="inlineStr">
@@ -32881,16 +32881,16 @@
         <v>0.49505</v>
       </c>
       <c r="O110" s="28" t="n">
-        <v>0.543779</v>
+        <v>0.545273</v>
       </c>
       <c r="P110" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q110" s="28" t="n">
-        <v>0.048729</v>
+        <v>0.050223</v>
       </c>
       <c r="R110" s="26" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="S110" s="29" t="n">
         <v>0</v>
@@ -32916,7 +32916,7 @@
       <c r="AD110" s="24" t="n"/>
       <c r="AE110" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 5.03-4.48; raw selected-side p=0.6116, calibrated p=0.5438.</t>
+          <t>Measured Edge Margin: Trend Engine projected 5.03-4.48; raw selected-side p=0.6192, calibrated p=0.5453.</t>
         </is>
       </c>
       <c r="AF110" s="31" t="inlineStr">
@@ -33035,7 +33035,7 @@
       </c>
       <c r="BH110" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI110" s="24" t="inlineStr">
@@ -33089,12 +33089,12 @@
     <row r="111" ht="36" customHeight="1">
       <c r="A111" s="24" t="inlineStr">
         <is>
-          <t>c9fafefee3684c6d</t>
+          <t>06fc768981f24774</t>
         </is>
       </c>
       <c r="B111" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C111" s="24" t="inlineStr">
@@ -33150,16 +33150,16 @@
         <v>0.534884</v>
       </c>
       <c r="O111" s="28" t="n">
-        <v>0.603678</v>
+        <v>0.606589</v>
       </c>
       <c r="P111" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q111" s="28" t="n">
-        <v>0.06879399999999999</v>
+        <v>0.071705</v>
       </c>
       <c r="R111" s="26" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="S111" s="29" t="n">
         <v>0</v>
@@ -33185,7 +33185,7 @@
       <c r="AD111" s="24" t="n"/>
       <c r="AE111" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 5.03-4.48; raw selected-side p=0.6228, calibrated p=0.6037.</t>
+          <t>Measured Edge Totals: Trend Engine projected 5.03-4.48; raw selected-side p=0.6258, calibrated p=0.6066.</t>
         </is>
       </c>
       <c r="AF111" s="31" t="inlineStr">
@@ -33304,7 +33304,7 @@
       </c>
       <c r="BH111" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI111" s="24" t="inlineStr">
@@ -33358,12 +33358,12 @@
     <row r="112" ht="36" customHeight="1">
       <c r="A112" s="24" t="inlineStr">
         <is>
-          <t>95186e18c67a45f8</t>
+          <t>8fcdf7b8d2a84fb0</t>
         </is>
       </c>
       <c r="B112" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C112" s="24" t="inlineStr">
@@ -33419,13 +33419,13 @@
         <v>0.604743</v>
       </c>
       <c r="O112" s="28" t="n">
-        <v>0.55947</v>
+        <v>0.559057</v>
       </c>
       <c r="P112" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q112" s="28" t="n">
-        <v>-0.045273</v>
+        <v>-0.045686</v>
       </c>
       <c r="R112" s="26" t="n">
         <v>0</v>
@@ -33454,7 +33454,7 @@
       <c r="AD112" s="24" t="n"/>
       <c r="AE112" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.48-4.27; raw selected-side p=0.6915, calibrated p=0.5595.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.48-4.27; raw selected-side p=0.6894, calibrated p=0.5591.</t>
         </is>
       </c>
       <c r="AF112" s="31" t="inlineStr">
@@ -33573,7 +33573,7 @@
       </c>
       <c r="BH112" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI112" s="24" t="inlineStr">
@@ -33627,12 +33627,12 @@
     <row r="113" ht="36" customHeight="1">
       <c r="A113" s="24" t="inlineStr">
         <is>
-          <t>e560b1bb79ae4f50</t>
+          <t>1fcd8188a5d744d5</t>
         </is>
       </c>
       <c r="B113" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C113" s="24" t="inlineStr">
@@ -33688,16 +33688,16 @@
         <v>0.480769</v>
       </c>
       <c r="O113" s="28" t="n">
-        <v>0.475237</v>
+        <v>0.475868</v>
       </c>
       <c r="P113" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q113" s="28" t="n">
-        <v>-0.005532</v>
+        <v>-0.004901</v>
       </c>
       <c r="R113" s="26" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S113" s="29" t="n">
         <v>0</v>
@@ -33723,7 +33723,7 @@
       <c r="AD113" s="24" t="n"/>
       <c r="AE113" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.48-4.27; raw selected-side p=0.4904, calibrated p=0.4752.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.48-4.27; raw selected-side p=0.4910, calibrated p=0.4759.</t>
         </is>
       </c>
       <c r="AF113" s="31" t="inlineStr">
@@ -33842,7 +33842,7 @@
       </c>
       <c r="BH113" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI113" s="24" t="inlineStr">
@@ -33896,12 +33896,12 @@
     <row r="114" ht="36" customHeight="1">
       <c r="A114" s="24" t="inlineStr">
         <is>
-          <t>3659e0c9b5d14b9c</t>
+          <t>406ef34d5a2c4b99</t>
         </is>
       </c>
       <c r="B114" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C114" s="24" t="inlineStr">
@@ -33948,25 +33948,25 @@
         </is>
       </c>
       <c r="L114" s="26" t="n">
-        <v>-144</v>
+        <v>-141</v>
       </c>
       <c r="M114" s="27" t="n">
-        <v>1.694444</v>
+        <v>1.70922</v>
       </c>
       <c r="N114" s="28" t="n">
-        <v>0.590164</v>
+        <v>0.585062</v>
       </c>
       <c r="O114" s="28" t="n">
-        <v>0.548682</v>
+        <v>0.549055</v>
       </c>
       <c r="P114" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q114" s="28" t="n">
-        <v>-0.041482</v>
+        <v>-0.036007</v>
       </c>
       <c r="R114" s="26" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S114" s="29" t="n">
         <v>0</v>
@@ -33992,7 +33992,7 @@
       <c r="AD114" s="24" t="n"/>
       <c r="AE114" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.65-4.92; raw selected-side p=0.6365, calibrated p=0.5487.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.65-4.92; raw selected-side p=0.6384, calibrated p=0.5491.</t>
         </is>
       </c>
       <c r="AF114" s="31" t="inlineStr">
@@ -34111,7 +34111,7 @@
       </c>
       <c r="BH114" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI114" s="24" t="inlineStr">
@@ -34123,16 +34123,16 @@
         <v>1.5</v>
       </c>
       <c r="BK114" s="26" t="n">
-        <v>-144</v>
+        <v>-141</v>
       </c>
       <c r="BL114" s="27" t="n">
-        <v>1.694444</v>
+        <v>1.70922</v>
       </c>
       <c r="BM114" s="28" t="n">
-        <v>0.590164</v>
+        <v>0.585062</v>
       </c>
       <c r="BN114" s="28" t="n">
-        <v>0.5870649999999999</v>
+        <v>0.58209</v>
       </c>
       <c r="BO114" s="28" t="n"/>
       <c r="BP114" s="25" t="n"/>
@@ -34165,12 +34165,12 @@
     <row r="115" ht="36" customHeight="1">
       <c r="A115" s="24" t="inlineStr">
         <is>
-          <t>3cc0f9e8e6b54d87</t>
+          <t>40f8491d5a594177</t>
         </is>
       </c>
       <c r="B115" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="C115" s="24" t="inlineStr">
@@ -34217,25 +34217,25 @@
         </is>
       </c>
       <c r="L115" s="26" t="n">
-        <v>-113</v>
+        <v>-115</v>
       </c>
       <c r="M115" s="27" t="n">
-        <v>1.884956</v>
+        <v>1.869565</v>
       </c>
       <c r="N115" s="28" t="n">
-        <v>0.530516</v>
+        <v>0.534884</v>
       </c>
       <c r="O115" s="28" t="n">
-        <v>0.544745</v>
+        <v>0.548092</v>
       </c>
       <c r="P115" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q115" s="28" t="n">
-        <v>0.014229</v>
+        <v>0.013208</v>
       </c>
       <c r="R115" s="26" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="S115" s="29" t="n">
         <v>0</v>
@@ -34261,7 +34261,7 @@
       <c r="AD115" s="24" t="n"/>
       <c r="AE115" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.65-4.92; raw selected-side p=0.5621, calibrated p=0.5447.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.65-4.92; raw selected-side p=0.5655, calibrated p=0.5481.</t>
         </is>
       </c>
       <c r="AF115" s="31" t="inlineStr">
@@ -34380,7 +34380,7 @@
       </c>
       <c r="BH115" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T16:51:51.403706Z</t>
+          <t>2026-07-30T17:18:50.985439Z</t>
         </is>
       </c>
       <c r="BI115" s="24" t="inlineStr">
@@ -34392,16 +34392,16 @@
         <v>8.5</v>
       </c>
       <c r="BK115" s="26" t="n">
-        <v>-113</v>
+        <v>-115</v>
       </c>
       <c r="BL115" s="27" t="n">
-        <v>1.884956</v>
+        <v>1.869565</v>
       </c>
       <c r="BM115" s="28" t="n">
-        <v>0.530516</v>
+        <v>0.534884</v>
       </c>
       <c r="BN115" s="28" t="n">
-        <v>0.527363</v>
+        <v>0.532338</v>
       </c>
       <c r="BO115" s="28" t="n"/>
       <c r="BP115" s="25" t="n"/>

</xml_diff>

<commit_message>
Real ledger state from final daily forecast + settlement run
Third and final daily run this session: zero failures across every sport.
Confirms the full pipeline is stable after all of today's changes (gate
removal, Gated Research tightening, retired-model/calibration archival,
dashboard fixes). Full test suite (501) passing, ruff at baseline (118),
verify-chain clean (0 breaks), dashboard healthy.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -4414,12 +4414,12 @@
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>90555303e32f47c0</t>
+          <t>fc8f7bc914e241ff</t>
         </is>
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C12" s="24" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="BH12" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:41.975528Z</t>
+          <t>2026-07-30T17:35:40.109396Z</t>
         </is>
       </c>
       <c r="BI12" s="24" t="inlineStr">
@@ -4689,12 +4689,12 @@
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>46446adc53524558</t>
+          <t>80054eebaf564b26</t>
         </is>
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C13" s="24" t="inlineStr">
@@ -4900,7 +4900,7 @@
       </c>
       <c r="BH13" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:33.085623Z</t>
+          <t>2026-07-30T17:35:31.601278Z</t>
         </is>
       </c>
       <c r="BI13" s="24" t="inlineStr">
@@ -4972,12 +4972,12 @@
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>9ed711934b3742e5</t>
+          <t>744dc55d146c49cf</t>
         </is>
       </c>
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C14" s="24" t="inlineStr">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="BH14" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:43.676555Z</t>
+          <t>2026-07-30T17:35:41.686769Z</t>
         </is>
       </c>
       <c r="BI14" s="24" t="inlineStr">
@@ -5247,12 +5247,12 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>89d488b018874530</t>
+          <t>560d43ddfce245d6</t>
         </is>
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C15" s="24" t="inlineStr">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="BH15" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:34.062012Z</t>
+          <t>2026-07-30T17:35:32.550865Z</t>
         </is>
       </c>
       <c r="BI15" s="24" t="inlineStr">
@@ -5530,12 +5530,12 @@
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>1315e1b8446b4cc6</t>
+          <t>35863d1c4eb643d3</t>
         </is>
       </c>
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C16" s="24" t="inlineStr">
@@ -5741,7 +5741,7 @@
       </c>
       <c r="BH16" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:44.949554Z</t>
+          <t>2026-07-30T17:35:42.962719Z</t>
         </is>
       </c>
       <c r="BI16" s="24" t="inlineStr">
@@ -5805,12 +5805,12 @@
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>5352883f901947bd</t>
+          <t>b912ee69b50f4e34</t>
         </is>
       </c>
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C17" s="24" t="inlineStr">
@@ -5855,23 +5855,23 @@
         </is>
       </c>
       <c r="L17" s="26" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="M17" s="27" t="n">
-        <v>2.06</v>
+        <v>2.02</v>
       </c>
       <c r="N17" s="28" t="n">
-        <v>0.485437</v>
+        <v>0.49505</v>
       </c>
       <c r="O17" s="28" t="n">
         <v>0.503115</v>
       </c>
       <c r="P17" s="28" t="n"/>
       <c r="Q17" s="28" t="n">
-        <v>0.017678</v>
+        <v>0.008064999999999999</v>
       </c>
       <c r="R17" s="26" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="S17" s="29" t="n">
         <v>0.5</v>
@@ -5897,7 +5897,7 @@
       <c r="AD17" s="24" t="n"/>
       <c r="AE17" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.6242; executable ask 0.4850 (aec-mlb-chc-stl-2026-07-30); model edge vs ask +0.0181.</t>
+          <t>Learned LR call at threshold 0.6242; executable ask 0.4950 (aec-mlb-chc-stl-2026-07-30); model edge vs ask +0.0081.</t>
         </is>
       </c>
       <c r="AF17" s="31" t="inlineStr">
@@ -6016,7 +6016,7 @@
       </c>
       <c r="BH17" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:35.081580Z</t>
+          <t>2026-07-30T17:35:33.545496Z</t>
         </is>
       </c>
       <c r="BI17" s="24" t="inlineStr">
@@ -6026,16 +6026,16 @@
       </c>
       <c r="BJ17" s="25" t="n"/>
       <c r="BK17" s="26" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="BL17" s="27" t="n">
-        <v>2.06</v>
+        <v>2.02</v>
       </c>
       <c r="BM17" s="28" t="n">
-        <v>0.485437</v>
+        <v>0.49505</v>
       </c>
       <c r="BN17" s="28" t="n">
-        <v>0.482587</v>
+        <v>0.492537</v>
       </c>
       <c r="BO17" s="28" t="n"/>
       <c r="BP17" s="25" t="n"/>
@@ -6088,12 +6088,12 @@
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>308e6d5daced4850</t>
+          <t>c9ac8606c6e2420d</t>
         </is>
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C18" s="24" t="inlineStr">
@@ -6299,7 +6299,7 @@
       </c>
       <c r="BH18" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:38.217983Z</t>
+          <t>2026-07-30T17:35:36.538063Z</t>
         </is>
       </c>
       <c r="BI18" s="24" t="inlineStr">
@@ -6371,12 +6371,12 @@
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>3637a4075d654228</t>
+          <t>c639d9950d1943cc</t>
         </is>
       </c>
       <c r="B19" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C19" s="24" t="inlineStr">
@@ -6582,7 +6582,7 @@
       </c>
       <c r="BH19" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:36.074233Z</t>
+          <t>2026-07-30T17:35:34.482178Z</t>
         </is>
       </c>
       <c r="BI19" s="24" t="inlineStr">
@@ -6654,12 +6654,12 @@
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>3a3c0a538c744d8f</t>
+          <t>bd1a3707dd5648f3</t>
         </is>
       </c>
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C20" s="24" t="inlineStr">
@@ -6865,7 +6865,7 @@
       </c>
       <c r="BH20" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:37.061484Z</t>
+          <t>2026-07-30T17:35:35.498307Z</t>
         </is>
       </c>
       <c r="BI20" s="24" t="inlineStr">
@@ -6937,12 +6937,12 @@
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>89188b6bddfa4e04</t>
+          <t>2d0fec361d884dcb</t>
         </is>
       </c>
       <c r="B21" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C21" s="24" t="inlineStr">
@@ -7148,7 +7148,7 @@
       </c>
       <c r="BH21" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:38.913634Z</t>
+          <t>2026-07-30T17:35:37.104809Z</t>
         </is>
       </c>
       <c r="BI21" s="24" t="inlineStr">
@@ -7220,12 +7220,12 @@
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>13b93429e47d4e18</t>
+          <t>12c2ee4e08e742ed</t>
         </is>
       </c>
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C22" s="24" t="inlineStr">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="BH22" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:40.032869Z</t>
+          <t>2026-07-30T17:35:38.204317Z</t>
         </is>
       </c>
       <c r="BI22" s="24" t="inlineStr">
@@ -7503,12 +7503,12 @@
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>075812f4dde4432b</t>
+          <t>6c2a35b7d0f845db</t>
         </is>
       </c>
       <c r="B23" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:22.482445Z</t>
+          <t>2026-07-30T17:36:17.628396Z</t>
         </is>
       </c>
       <c r="C23" s="24" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="BH23" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:17:41.015176Z</t>
+          <t>2026-07-30T17:35:39.188017Z</t>
         </is>
       </c>
       <c r="BI23" s="24" t="inlineStr">
@@ -7786,12 +7786,12 @@
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>41c5bee3def94e38</t>
+          <t>e204040905f94109</t>
         </is>
       </c>
       <c r="B24" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C24" s="24" t="inlineStr">
@@ -7838,22 +7838,22 @@
         </is>
       </c>
       <c r="L24" s="26" t="n">
-        <v>-156</v>
+        <v>-160</v>
       </c>
       <c r="M24" s="27" t="n">
-        <v>1.641026</v>
+        <v>1.625</v>
       </c>
       <c r="N24" s="28" t="n">
-        <v>0.609375</v>
+        <v>0.615385</v>
       </c>
       <c r="O24" s="28" t="n">
-        <v>0.551079</v>
+        <v>0.550293</v>
       </c>
       <c r="P24" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q24" s="28" t="n">
-        <v>-0.058296</v>
+        <v>-0.065092</v>
       </c>
       <c r="R24" s="26" t="n">
         <v>0</v>
@@ -7882,7 +7882,7 @@
       <c r="AD24" s="24" t="n"/>
       <c r="AE24" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.80-5.00; raw selected-side p=0.6488, calibrated p=0.5511.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.80-5.00; raw selected-side p=0.6448, calibrated p=0.5503.</t>
         </is>
       </c>
       <c r="AF24" s="31" t="inlineStr">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="BH24" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI24" s="24" t="inlineStr">
@@ -8013,16 +8013,16 @@
         <v>1.5</v>
       </c>
       <c r="BK24" s="26" t="n">
-        <v>-156</v>
+        <v>-160</v>
       </c>
       <c r="BL24" s="27" t="n">
-        <v>1.641026</v>
+        <v>1.625</v>
       </c>
       <c r="BM24" s="28" t="n">
-        <v>0.609375</v>
+        <v>0.615385</v>
       </c>
       <c r="BN24" s="28" t="n">
-        <v>0.606965</v>
+        <v>0.61194</v>
       </c>
       <c r="BO24" s="28" t="n"/>
       <c r="BP24" s="25" t="n"/>
@@ -8055,12 +8055,12 @@
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>c7d1c1ea6a644a75</t>
+          <t>605978e4b4f649e3</t>
         </is>
       </c>
       <c r="B25" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C25" s="24" t="inlineStr">
@@ -8116,16 +8116,16 @@
         <v>0.45045</v>
       </c>
       <c r="O25" s="28" t="n">
-        <v>0.465051</v>
+        <v>0.451615</v>
       </c>
       <c r="P25" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q25" s="28" t="n">
-        <v>0.014601</v>
+        <v>0.001165</v>
       </c>
       <c r="R25" s="26" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="S25" s="29" t="n">
         <v>0</v>
@@ -8151,7 +8151,7 @@
       <c r="AD25" s="24" t="n"/>
       <c r="AE25" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.80-5.00; raw selected-side p=0.4799, calibrated p=0.4651.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.80-5.00; raw selected-side p=0.4661, calibrated p=0.4516.</t>
         </is>
       </c>
       <c r="AF25" s="31" t="inlineStr">
@@ -8270,7 +8270,7 @@
       </c>
       <c r="BH25" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI25" s="24" t="inlineStr">
@@ -8324,12 +8324,12 @@
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>aaa374fcf56346ca</t>
+          <t>0058e2e4dee14815</t>
         </is>
       </c>
       <c r="B26" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C26" s="24" t="inlineStr">
@@ -8385,13 +8385,13 @@
         <v>0.64539</v>
       </c>
       <c r="O26" s="28" t="n">
-        <v>0.5684399999999999</v>
+        <v>0.56787</v>
       </c>
       <c r="P26" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q26" s="28" t="n">
-        <v>-0.07695</v>
+        <v>-0.07752000000000001</v>
       </c>
       <c r="R26" s="26" t="n">
         <v>0</v>
@@ -8420,7 +8420,7 @@
       <c r="AD26" s="24" t="n"/>
       <c r="AE26" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.07-4.77; raw selected-side p=0.7371, calibrated p=0.5684.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.07-4.77; raw selected-side p=0.7342, calibrated p=0.5679.</t>
         </is>
       </c>
       <c r="AF26" s="31" t="inlineStr">
@@ -8539,7 +8539,7 @@
       </c>
       <c r="BH26" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI26" s="24" t="inlineStr">
@@ -8593,12 +8593,12 @@
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>dc0ec81ac7a64b06</t>
+          <t>3fc8b2e5f3744a2c</t>
         </is>
       </c>
       <c r="B27" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C27" s="24" t="inlineStr">
@@ -8654,16 +8654,16 @@
         <v>0.485437</v>
       </c>
       <c r="O27" s="28" t="n">
-        <v>0.556337</v>
+        <v>0.562449</v>
       </c>
       <c r="P27" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q27" s="28" t="n">
-        <v>0.0709</v>
+        <v>0.077012</v>
       </c>
       <c r="R27" s="26" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="S27" s="29" t="n">
         <v>0</v>
@@ -8689,7 +8689,7 @@
       <c r="AD27" s="24" t="n"/>
       <c r="AE27" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.07-4.77; raw selected-side p=0.5740, calibrated p=0.5563.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.07-4.77; raw selected-side p=0.5803, calibrated p=0.5624.</t>
         </is>
       </c>
       <c r="AF27" s="31" t="inlineStr">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="BH27" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI27" s="24" t="inlineStr">
@@ -8862,12 +8862,12 @@
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>a711dc733b2644a6</t>
+          <t>dffb9fbd0449460f</t>
         </is>
       </c>
       <c r="B28" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C28" s="24" t="inlineStr">
@@ -8923,13 +8923,13 @@
         <v>0.635036</v>
       </c>
       <c r="O28" s="28" t="n">
-        <v>0.555677</v>
+        <v>0.556257</v>
       </c>
       <c r="P28" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q28" s="28" t="n">
-        <v>-0.079359</v>
+        <v>-0.078779</v>
       </c>
       <c r="R28" s="26" t="n">
         <v>0</v>
@@ -8958,7 +8958,7 @@
       <c r="AD28" s="24" t="n"/>
       <c r="AE28" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.49-4.55; raw selected-side p=0.6722, calibrated p=0.5557.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.49-4.55; raw selected-side p=0.6751, calibrated p=0.5563.</t>
         </is>
       </c>
       <c r="AF28" s="31" t="inlineStr">
@@ -9077,7 +9077,7 @@
       </c>
       <c r="BH28" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI28" s="24" t="inlineStr">
@@ -9131,12 +9131,12 @@
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>1772c061995f4a46</t>
+          <t>f51c71784cf44ec9</t>
         </is>
       </c>
       <c r="B29" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C29" s="24" t="inlineStr">
@@ -9192,16 +9192,16 @@
         <v>0.469484</v>
       </c>
       <c r="O29" s="28" t="n">
-        <v>0.501139</v>
+        <v>0.500169</v>
       </c>
       <c r="P29" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q29" s="28" t="n">
-        <v>0.031655</v>
+        <v>0.030685</v>
       </c>
       <c r="R29" s="26" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="S29" s="29" t="n">
         <v>0</v>
@@ -9227,7 +9227,7 @@
       <c r="AD29" s="24" t="n"/>
       <c r="AE29" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.49-4.55; raw selected-side p=0.5171, calibrated p=0.5011.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.49-4.55; raw selected-side p=0.5161, calibrated p=0.5002.</t>
         </is>
       </c>
       <c r="AF29" s="31" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="BH29" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI29" s="24" t="inlineStr">
@@ -9367,7 +9367,7 @@
         <v>0.469484</v>
       </c>
       <c r="BN29" s="28" t="n">
-        <v>0.465347</v>
+        <v>0.467662</v>
       </c>
       <c r="BO29" s="28" t="n"/>
       <c r="BP29" s="25" t="n"/>
@@ -9400,12 +9400,12 @@
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>669fab5c44624df9</t>
+          <t>634cf752e2a24e63</t>
         </is>
       </c>
       <c r="B30" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C30" s="24" t="inlineStr">
@@ -9461,13 +9461,13 @@
         <v>0.590164</v>
       </c>
       <c r="O30" s="28" t="n">
-        <v>0.545381</v>
+        <v>0.545558</v>
       </c>
       <c r="P30" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q30" s="28" t="n">
-        <v>-0.044783</v>
+        <v>-0.044606</v>
       </c>
       <c r="R30" s="26" t="n">
         <v>2</v>
@@ -9496,7 +9496,7 @@
       <c r="AD30" s="24" t="n"/>
       <c r="AE30" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.30-4.84; raw selected-side p=0.6198, calibrated p=0.5454.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.30-4.84; raw selected-side p=0.6207, calibrated p=0.5456.</t>
         </is>
       </c>
       <c r="AF30" s="31" t="inlineStr">
@@ -9615,7 +9615,7 @@
       </c>
       <c r="BH30" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI30" s="24" t="inlineStr">
@@ -9669,12 +9669,12 @@
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>07ca08b26f114d8a</t>
+          <t>e2588cf35ad940ba</t>
         </is>
       </c>
       <c r="B31" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C31" s="24" t="inlineStr">
@@ -9730,16 +9730,16 @@
         <v>0.480769</v>
       </c>
       <c r="O31" s="28" t="n">
-        <v>0.571665</v>
+        <v>0.565796</v>
       </c>
       <c r="P31" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q31" s="28" t="n">
-        <v>0.090896</v>
+        <v>0.08502700000000001</v>
       </c>
       <c r="R31" s="26" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="S31" s="29" t="n">
         <v>0</v>
@@ -9765,7 +9765,7 @@
       <c r="AD31" s="24" t="n"/>
       <c r="AE31" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.30-4.84; raw selected-side p=0.5898, calibrated p=0.5717.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.30-4.84; raw selected-side p=0.5837, calibrated p=0.5658.</t>
         </is>
       </c>
       <c r="AF31" s="31" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="BH31" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI31" s="24" t="inlineStr">
@@ -9938,12 +9938,12 @@
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>fbde174a130249fd</t>
+          <t>352566a371184051</t>
         </is>
       </c>
       <c r="B32" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C32" s="24" t="inlineStr">
@@ -9978,11 +9978,11 @@
       </c>
       <c r="I32" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J32" s="25" t="n">
-        <v>-1.5</v>
+        <v>1.5</v>
       </c>
       <c r="K32" s="24" t="inlineStr">
         <is>
@@ -9990,25 +9990,25 @@
         </is>
       </c>
       <c r="L32" s="26" t="n">
-        <v>186</v>
+        <v>-190</v>
       </c>
       <c r="M32" s="27" t="n">
-        <v>2.86</v>
+        <v>1.526316</v>
       </c>
       <c r="N32" s="28" t="n">
-        <v>0.34965</v>
+        <v>0.655172</v>
       </c>
       <c r="O32" s="28" t="n">
-        <v>0.493426</v>
+        <v>0.551885</v>
       </c>
       <c r="P32" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q32" s="28" t="n">
-        <v>0.143776</v>
+        <v>-0.103287</v>
       </c>
       <c r="R32" s="26" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="S32" s="29" t="n">
         <v>0</v>
@@ -10034,7 +10034,7 @@
       <c r="AD32" s="24" t="n"/>
       <c r="AE32" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.06-4.35; raw selected-side p=0.3553, calibrated p=0.4934.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.06-4.35; raw selected-side p=0.6529, calibrated p=0.5519.</t>
         </is>
       </c>
       <c r="AF32" s="31" t="inlineStr">
@@ -10153,7 +10153,7 @@
       </c>
       <c r="BH32" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI32" s="24" t="inlineStr">
@@ -10162,19 +10162,19 @@
         </is>
       </c>
       <c r="BJ32" s="25" t="n">
-        <v>-1.5</v>
+        <v>1.5</v>
       </c>
       <c r="BK32" s="26" t="n">
-        <v>186</v>
+        <v>-190</v>
       </c>
       <c r="BL32" s="27" t="n">
-        <v>2.86</v>
+        <v>1.526316</v>
       </c>
       <c r="BM32" s="28" t="n">
-        <v>0.34965</v>
+        <v>0.655172</v>
       </c>
       <c r="BN32" s="28" t="n">
-        <v>0.348259</v>
+        <v>0.651741</v>
       </c>
       <c r="BO32" s="28" t="n"/>
       <c r="BP32" s="25" t="n"/>
@@ -10207,12 +10207,12 @@
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>4b46515e5e434be0</t>
+          <t>a98d4331a06540a7</t>
         </is>
       </c>
       <c r="B33" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C33" s="24" t="inlineStr">
@@ -10268,16 +10268,16 @@
         <v>0.45045</v>
       </c>
       <c r="O33" s="28" t="n">
-        <v>0.523111</v>
+        <v>0.51797</v>
       </c>
       <c r="P33" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q33" s="28" t="n">
-        <v>0.072661</v>
+        <v>0.06752</v>
       </c>
       <c r="R33" s="26" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="S33" s="29" t="n">
         <v>0</v>
@@ -10303,7 +10303,7 @@
       <c r="AD33" s="24" t="n"/>
       <c r="AE33" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.06-4.35; raw selected-side p=0.5397, calibrated p=0.5231.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.06-4.35; raw selected-side p=0.5344, calibrated p=0.5180.</t>
         </is>
       </c>
       <c r="AF33" s="31" t="inlineStr">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="BH33" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI33" s="24" t="inlineStr">
@@ -10476,12 +10476,12 @@
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>44c06d8e6f2e4571</t>
+          <t>c2a31243c46a4c16</t>
         </is>
       </c>
       <c r="B34" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -10537,13 +10537,13 @@
         <v>0.590164</v>
       </c>
       <c r="O34" s="28" t="n">
-        <v>0.548201</v>
+        <v>0.548436</v>
       </c>
       <c r="P34" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q34" s="28" t="n">
-        <v>-0.041963</v>
+        <v>-0.041728</v>
       </c>
       <c r="R34" s="26" t="n">
         <v>4</v>
@@ -10572,7 +10572,7 @@
       <c r="AD34" s="24" t="n"/>
       <c r="AE34" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.87-4.53; raw selected-side p=0.6341, calibrated p=0.5482.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.87-4.53; raw selected-side p=0.6353, calibrated p=0.5484.</t>
         </is>
       </c>
       <c r="AF34" s="31" t="inlineStr">
@@ -10691,7 +10691,7 @@
       </c>
       <c r="BH34" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI34" s="24" t="inlineStr">
@@ -10745,12 +10745,12 @@
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>3f4d266778b94a7a</t>
+          <t>cfc66be27ba44376</t>
         </is>
       </c>
       <c r="B35" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
@@ -10806,16 +10806,16 @@
         <v>0.490196</v>
       </c>
       <c r="O35" s="28" t="n">
-        <v>0.544745</v>
+        <v>0.54683</v>
       </c>
       <c r="P35" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q35" s="28" t="n">
-        <v>0.054549</v>
+        <v>0.056634</v>
       </c>
       <c r="R35" s="26" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="S35" s="29" t="n">
         <v>0</v>
@@ -10841,7 +10841,7 @@
       <c r="AD35" s="24" t="n"/>
       <c r="AE35" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.87-4.53; raw selected-side p=0.5621, calibrated p=0.5447.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.87-4.53; raw selected-side p=0.5642, calibrated p=0.5468.</t>
         </is>
       </c>
       <c r="AF35" s="31" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="BH35" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI35" s="24" t="inlineStr">
@@ -11014,12 +11014,12 @@
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>f1aaeac92c434837</t>
+          <t>ce5a73aaf9164402</t>
         </is>
       </c>
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C36" s="24" t="inlineStr">
@@ -11075,13 +11075,13 @@
         <v>0.49505</v>
       </c>
       <c r="O36" s="28" t="n">
-        <v>0.545273</v>
+        <v>0.544801</v>
       </c>
       <c r="P36" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q36" s="28" t="n">
-        <v>0.050223</v>
+        <v>0.049751</v>
       </c>
       <c r="R36" s="26" t="n">
         <v>50</v>
@@ -11110,7 +11110,7 @@
       <c r="AD36" s="24" t="n"/>
       <c r="AE36" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 5.03-4.48; raw selected-side p=0.6192, calibrated p=0.5453.</t>
+          <t>Measured Edge Margin: Trend Engine projected 5.03-4.48; raw selected-side p=0.6168, calibrated p=0.5448.</t>
         </is>
       </c>
       <c r="AF36" s="31" t="inlineStr">
@@ -11229,7 +11229,7 @@
       </c>
       <c r="BH36" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI36" s="24" t="inlineStr">
@@ -11283,12 +11283,12 @@
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>06fc768981f24774</t>
+          <t>182dc01bc38040c2</t>
         </is>
       </c>
       <c r="B37" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C37" s="24" t="inlineStr">
@@ -11344,16 +11344,16 @@
         <v>0.534884</v>
       </c>
       <c r="O37" s="28" t="n">
-        <v>0.606589</v>
+        <v>0.60329</v>
       </c>
       <c r="P37" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q37" s="28" t="n">
-        <v>0.071705</v>
+        <v>0.06840599999999999</v>
       </c>
       <c r="R37" s="26" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="S37" s="29" t="n">
         <v>0</v>
@@ -11379,7 +11379,7 @@
       <c r="AD37" s="24" t="n"/>
       <c r="AE37" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 5.03-4.48; raw selected-side p=0.6258, calibrated p=0.6066.</t>
+          <t>Measured Edge Totals: Trend Engine projected 5.03-4.48; raw selected-side p=0.6224, calibrated p=0.6033.</t>
         </is>
       </c>
       <c r="AF37" s="31" t="inlineStr">
@@ -11498,7 +11498,7 @@
       </c>
       <c r="BH37" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI37" s="24" t="inlineStr">
@@ -11552,12 +11552,12 @@
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>8fcdf7b8d2a84fb0</t>
+          <t>9fee0946d450487e</t>
         </is>
       </c>
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C38" s="24" t="inlineStr">
@@ -11613,13 +11613,13 @@
         <v>0.604743</v>
       </c>
       <c r="O38" s="28" t="n">
-        <v>0.559057</v>
+        <v>0.55947</v>
       </c>
       <c r="P38" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q38" s="28" t="n">
-        <v>-0.045686</v>
+        <v>-0.045273</v>
       </c>
       <c r="R38" s="26" t="n">
         <v>0</v>
@@ -11648,7 +11648,7 @@
       <c r="AD38" s="24" t="n"/>
       <c r="AE38" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.48-4.27; raw selected-side p=0.6894, calibrated p=0.5591.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.48-4.27; raw selected-side p=0.6915, calibrated p=0.5595.</t>
         </is>
       </c>
       <c r="AF38" s="31" t="inlineStr">
@@ -11767,7 +11767,7 @@
       </c>
       <c r="BH38" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI38" s="24" t="inlineStr">
@@ -11821,12 +11821,12 @@
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>1fcd8188a5d744d5</t>
+          <t>bf3262fcec7d4e69</t>
         </is>
       </c>
       <c r="B39" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C39" s="24" t="inlineStr">
@@ -11882,16 +11882,16 @@
         <v>0.480769</v>
       </c>
       <c r="O39" s="28" t="n">
-        <v>0.475868</v>
+        <v>0.474412</v>
       </c>
       <c r="P39" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q39" s="28" t="n">
-        <v>-0.004901</v>
+        <v>-0.006357</v>
       </c>
       <c r="R39" s="26" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S39" s="29" t="n">
         <v>0</v>
@@ -11917,7 +11917,7 @@
       <c r="AD39" s="24" t="n"/>
       <c r="AE39" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.48-4.27; raw selected-side p=0.4910, calibrated p=0.4759.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.48-4.27; raw selected-side p=0.4895, calibrated p=0.4744.</t>
         </is>
       </c>
       <c r="AF39" s="31" t="inlineStr">
@@ -12036,7 +12036,7 @@
       </c>
       <c r="BH39" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI39" s="24" t="inlineStr">
@@ -12090,12 +12090,12 @@
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>406ef34d5a2c4b99</t>
+          <t>9f8d56c5e8a7470f</t>
         </is>
       </c>
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C40" s="24" t="inlineStr">
@@ -12151,13 +12151,13 @@
         <v>0.585062</v>
       </c>
       <c r="O40" s="28" t="n">
-        <v>0.549055</v>
+        <v>0.54937</v>
       </c>
       <c r="P40" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q40" s="28" t="n">
-        <v>-0.036007</v>
+        <v>-0.035692</v>
       </c>
       <c r="R40" s="26" t="n">
         <v>7</v>
@@ -12186,7 +12186,7 @@
       <c r="AD40" s="24" t="n"/>
       <c r="AE40" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.65-4.92; raw selected-side p=0.6384, calibrated p=0.5491.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.65-4.92; raw selected-side p=0.6401, calibrated p=0.5494.</t>
         </is>
       </c>
       <c r="AF40" s="31" t="inlineStr">
@@ -12305,7 +12305,7 @@
       </c>
       <c r="BH40" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI40" s="24" t="inlineStr">
@@ -12359,12 +12359,12 @@
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="24" t="inlineStr">
         <is>
-          <t>40f8491d5a594177</t>
+          <t>097c5c0ee3544fc6</t>
         </is>
       </c>
       <c r="B41" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="C41" s="24" t="inlineStr">
@@ -12420,16 +12420,16 @@
         <v>0.534884</v>
       </c>
       <c r="O41" s="28" t="n">
-        <v>0.548092</v>
+        <v>0.5411550000000001</v>
       </c>
       <c r="P41" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q41" s="28" t="n">
-        <v>0.013208</v>
+        <v>0.006271</v>
       </c>
       <c r="R41" s="26" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="S41" s="29" t="n">
         <v>0</v>
@@ -12455,7 +12455,7 @@
       <c r="AD41" s="24" t="n"/>
       <c r="AE41" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.65-4.92; raw selected-side p=0.5655, calibrated p=0.5481.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.65-4.92; raw selected-side p=0.5584, calibrated p=0.5412.</t>
         </is>
       </c>
       <c r="AF41" s="31" t="inlineStr">
@@ -12574,7 +12574,7 @@
       </c>
       <c r="BH41" s="24" t="inlineStr">
         <is>
-          <t>2026-07-30T17:18:50.985439Z</t>
+          <t>2026-07-30T17:36:41.418998Z</t>
         </is>
       </c>
       <c r="BI41" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Real ledger state from final daily verification run
Confirms end-to-end: MLB moneyline (15/15 logged), KBO (4/5), NPB (2/4),
soccer flat (19 logged, main correctly inert pending promotion), MLB
availability capture (30 teams, 3550 real transaction entries with
position_type now populated for the pitching-staff/position-player
features). 571 tests passing, ruff at baseline.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flat_picks.xlsx
+++ b/data/flat_picks.xlsx
@@ -40888,12 +40888,12 @@
     <row r="134" ht="36" customHeight="1">
       <c r="A134" s="24" t="inlineStr">
         <is>
-          <t>c5cc4fbf72d94454</t>
+          <t>90ed8dea529842b2</t>
         </is>
       </c>
       <c r="B134" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C134" s="24" t="inlineStr">
@@ -41099,7 +41099,7 @@
       </c>
       <c r="BH134" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:17.717034Z</t>
+          <t>2026-08-02T08:13:20.816313Z</t>
         </is>
       </c>
       <c r="BI134" s="24" t="inlineStr">
@@ -41163,12 +41163,12 @@
     <row r="135" ht="36" customHeight="1">
       <c r="A135" s="24" t="inlineStr">
         <is>
-          <t>5d4e31a9e08a43d0</t>
+          <t>42e2fc79ca9a4a9c</t>
         </is>
       </c>
       <c r="B135" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C135" s="24" t="inlineStr">
@@ -41222,11 +41222,11 @@
         <v>0.5594710000000001</v>
       </c>
       <c r="O135" s="28" t="n">
-        <v>0.510265</v>
+        <v>0.510238</v>
       </c>
       <c r="P135" s="28" t="n"/>
       <c r="Q135" s="28" t="n">
-        <v>-0.049206</v>
+        <v>-0.049233</v>
       </c>
       <c r="R135" s="26" t="n">
         <v>0</v>
@@ -41255,7 +41255,7 @@
       <c r="AD135" s="24" t="n"/>
       <c r="AE135" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.6242; executable ask 0.5600 (aec-mlb-phi-bal-2026-08-02); model edge vs ask -0.0497.</t>
+          <t>Learned LR call at threshold 0.6242; executable ask 0.5600 (aec-mlb-phi-bal-2026-08-02); model edge vs ask -0.0498.</t>
         </is>
       </c>
       <c r="AF135" s="31" t="inlineStr">
@@ -41359,7 +41359,7 @@
       </c>
       <c r="BE135" s="24" t="inlineStr">
         <is>
-          <t>ddb4f7d0b87c8828</t>
+          <t>1171153bd71f9707</t>
         </is>
       </c>
       <c r="BF135" s="24" t="inlineStr">
@@ -41374,7 +41374,7 @@
       </c>
       <c r="BH135" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:02.839017Z</t>
+          <t>2026-08-02T08:13:05.641697Z</t>
         </is>
       </c>
       <c r="BI135" s="24" t="inlineStr">
@@ -41426,7 +41426,7 @@
       </c>
       <c r="CF135" s="24" t="inlineStr">
         <is>
-          <t>1.021</t>
+          <t>1.0205</t>
         </is>
       </c>
       <c r="CG135" s="24" t="inlineStr">
@@ -41446,12 +41446,12 @@
     <row r="136" ht="36" customHeight="1">
       <c r="A136" s="24" t="inlineStr">
         <is>
-          <t>7a8f508157344849</t>
+          <t>749a82d5447e4505</t>
         </is>
       </c>
       <c r="B136" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C136" s="24" t="inlineStr">
@@ -41496,23 +41496,23 @@
         </is>
       </c>
       <c r="L136" s="26" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="M136" s="27" t="n">
-        <v>2</v>
+        <v>1.961538</v>
       </c>
       <c r="N136" s="28" t="n">
-        <v>0.5</v>
+        <v>0.509804</v>
       </c>
       <c r="O136" s="28" t="n">
         <v>0.57112</v>
       </c>
       <c r="P136" s="28" t="n"/>
       <c r="Q136" s="28" t="n">
-        <v>0.07112</v>
+        <v>0.061316</v>
       </c>
       <c r="R136" s="26" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="S136" s="29" t="n">
         <v>1.25</v>
@@ -41538,7 +41538,7 @@
       <c r="AD136" s="24" t="n"/>
       <c r="AE136" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5001; executable ask 0.5000 (aec-wnba-la-por-2026-08-02); model edge vs ask +0.0711.</t>
+          <t>Learned LR call at threshold 0.5001; executable ask 0.5100 (aec-wnba-la-por-2026-08-02); model edge vs ask +0.0611.</t>
         </is>
       </c>
       <c r="AF136" s="31" t="inlineStr">
@@ -41657,7 +41657,7 @@
       </c>
       <c r="BH136" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:18.670669Z</t>
+          <t>2026-08-02T08:13:21.684170Z</t>
         </is>
       </c>
       <c r="BI136" s="24" t="inlineStr">
@@ -41667,16 +41667,16 @@
       </c>
       <c r="BJ136" s="25" t="n"/>
       <c r="BK136" s="26" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="BL136" s="27" t="n">
-        <v>2</v>
+        <v>1.961538</v>
       </c>
       <c r="BM136" s="28" t="n">
-        <v>0.5</v>
+        <v>0.509804</v>
       </c>
       <c r="BN136" s="28" t="n">
-        <v>0.49505</v>
+        <v>0.50495</v>
       </c>
       <c r="BO136" s="28" t="n"/>
       <c r="BP136" s="25" t="n"/>
@@ -41717,12 +41717,12 @@
     <row r="137" ht="36" customHeight="1">
       <c r="A137" s="24" t="inlineStr">
         <is>
-          <t>79d6afc1fc4746e2</t>
+          <t>02c326da75c04def</t>
         </is>
       </c>
       <c r="B137" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C137" s="24" t="inlineStr">
@@ -41776,11 +41776,11 @@
         <v>0.539171</v>
       </c>
       <c r="O137" s="28" t="n">
-        <v>0.600347</v>
+        <v>0.600484</v>
       </c>
       <c r="P137" s="28" t="n"/>
       <c r="Q137" s="28" t="n">
-        <v>0.061176</v>
+        <v>0.061313</v>
       </c>
       <c r="R137" s="26" t="n">
         <v>52</v>
@@ -41809,7 +41809,7 @@
       <c r="AD137" s="24" t="n"/>
       <c r="AE137" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.6242; executable ask 0.5400 (aec-mlb-wsh-atl-2026-08-02); model edge vs ask +0.0603.</t>
+          <t>Learned LR call at threshold 0.6242; executable ask 0.5400 (aec-mlb-wsh-atl-2026-08-02); model edge vs ask +0.0605.</t>
         </is>
       </c>
       <c r="AF137" s="31" t="inlineStr">
@@ -41913,7 +41913,7 @@
       </c>
       <c r="BE137" s="24" t="inlineStr">
         <is>
-          <t>5a8b8f0237e0f7f7</t>
+          <t>33e4872540af0996</t>
         </is>
       </c>
       <c r="BF137" s="24" t="inlineStr">
@@ -41928,7 +41928,7 @@
       </c>
       <c r="BH137" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:03.921396Z</t>
+          <t>2026-08-02T08:13:06.812114Z</t>
         </is>
       </c>
       <c r="BI137" s="24" t="inlineStr">
@@ -41980,7 +41980,7 @@
       </c>
       <c r="CF137" s="24" t="inlineStr">
         <is>
-          <t>1.0206</t>
+          <t>1.0179</t>
         </is>
       </c>
       <c r="CG137" s="24" t="inlineStr">
@@ -42000,12 +42000,12 @@
     <row r="138" ht="36" customHeight="1">
       <c r="A138" s="24" t="inlineStr">
         <is>
-          <t>18adc888433f43af</t>
+          <t>1b0d58ea5ddf4585</t>
         </is>
       </c>
       <c r="B138" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C138" s="24" t="inlineStr">
@@ -42211,7 +42211,7 @@
       </c>
       <c r="BH138" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:20.306110Z</t>
+          <t>2026-08-02T08:13:23.088966Z</t>
         </is>
       </c>
       <c r="BI138" s="24" t="inlineStr">
@@ -42275,12 +42275,12 @@
     <row r="139" ht="36" customHeight="1">
       <c r="A139" s="24" t="inlineStr">
         <is>
-          <t>1a4d0e4b3c3b4548</t>
+          <t>9210eb4913ae42b7</t>
         </is>
       </c>
       <c r="B139" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C139" s="24" t="inlineStr">
@@ -42486,7 +42486,7 @@
       </c>
       <c r="BH139" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:04.884951Z</t>
+          <t>2026-08-02T08:13:07.749432Z</t>
         </is>
       </c>
       <c r="BI139" s="24" t="inlineStr">
@@ -42558,12 +42558,12 @@
     <row r="140" ht="36" customHeight="1">
       <c r="A140" s="24" t="inlineStr">
         <is>
-          <t>407bc99297bb4c5d</t>
+          <t>8e62edf21af4439d</t>
         </is>
       </c>
       <c r="B140" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C140" s="24" t="inlineStr">
@@ -42769,7 +42769,7 @@
       </c>
       <c r="BH140" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:21.289872Z</t>
+          <t>2026-08-02T08:13:24.146087Z</t>
         </is>
       </c>
       <c r="BI140" s="24" t="inlineStr">
@@ -42833,12 +42833,12 @@
     <row r="141" ht="36" customHeight="1">
       <c r="A141" s="24" t="inlineStr">
         <is>
-          <t>5abb308247ea4956</t>
+          <t>3ffd2767c126417b</t>
         </is>
       </c>
       <c r="B141" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C141" s="24" t="inlineStr">
@@ -42892,11 +42892,11 @@
         <v>0.574468</v>
       </c>
       <c r="O141" s="28" t="n">
-        <v>0.542333</v>
+        <v>0.542254</v>
       </c>
       <c r="P141" s="28" t="n"/>
       <c r="Q141" s="28" t="n">
-        <v>-0.032135</v>
+        <v>-0.032214</v>
       </c>
       <c r="R141" s="26" t="n">
         <v>5</v>
@@ -43029,7 +43029,7 @@
       </c>
       <c r="BE141" s="24" t="inlineStr">
         <is>
-          <t>8082ba852600e9f8</t>
+          <t>5595772130180b8e</t>
         </is>
       </c>
       <c r="BF141" s="24" t="inlineStr">
@@ -43044,7 +43044,7 @@
       </c>
       <c r="BH141" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:05.948352Z</t>
+          <t>2026-08-02T08:13:08.800726Z</t>
         </is>
       </c>
       <c r="BI141" s="24" t="inlineStr">
@@ -43096,7 +43096,7 @@
       </c>
       <c r="CF141" s="24" t="inlineStr">
         <is>
-          <t>1.0052</t>
+          <t>1.0067</t>
         </is>
       </c>
       <c r="CG141" s="24" t="inlineStr">
@@ -43116,12 +43116,12 @@
     <row r="142" ht="36" customHeight="1">
       <c r="A142" s="24" t="inlineStr">
         <is>
-          <t>2751717f31eb4059</t>
+          <t>8bc0d32ebf6d47c7</t>
         </is>
       </c>
       <c r="B142" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C142" s="24" t="inlineStr">
@@ -43327,7 +43327,7 @@
       </c>
       <c r="BH142" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:08.776580Z</t>
+          <t>2026-08-02T08:13:11.786575Z</t>
         </is>
       </c>
       <c r="BI142" s="24" t="inlineStr">
@@ -43399,12 +43399,12 @@
     <row r="143" ht="36" customHeight="1">
       <c r="A143" s="24" t="inlineStr">
         <is>
-          <t>a6f1e315fecb4898</t>
+          <t>b2f0dc2391bd4bec</t>
         </is>
       </c>
       <c r="B143" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C143" s="24" t="inlineStr">
@@ -43458,11 +43458,11 @@
         <v>0.480769</v>
       </c>
       <c r="O143" s="28" t="n">
-        <v>0.519194</v>
+        <v>0.51911</v>
       </c>
       <c r="P143" s="28" t="n"/>
       <c r="Q143" s="28" t="n">
-        <v>0.038425</v>
+        <v>0.038341</v>
       </c>
       <c r="R143" s="26" t="n">
         <v>41</v>
@@ -43491,7 +43491,7 @@
       <c r="AD143" s="24" t="n"/>
       <c r="AE143" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.6242; executable ask 0.4800 (aec-mlb-mia-nym-2026-08-02); model edge vs ask +0.0392.</t>
+          <t>Learned LR call at threshold 0.6242; executable ask 0.4800 (aec-mlb-mia-nym-2026-08-02); model edge vs ask +0.0391.</t>
         </is>
       </c>
       <c r="AF143" s="31" t="inlineStr">
@@ -43595,7 +43595,7 @@
       </c>
       <c r="BE143" s="24" t="inlineStr">
         <is>
-          <t>2d38d059d757eb9e</t>
+          <t>4b8fc292fe99e924</t>
         </is>
       </c>
       <c r="BF143" s="24" t="inlineStr">
@@ -43610,7 +43610,7 @@
       </c>
       <c r="BH143" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:07.556434Z</t>
+          <t>2026-08-02T08:13:10.416744Z</t>
         </is>
       </c>
       <c r="BI143" s="24" t="inlineStr">
@@ -43662,7 +43662,7 @@
       </c>
       <c r="CF143" s="24" t="inlineStr">
         <is>
-          <t>1.0227</t>
+          <t>1.0243</t>
         </is>
       </c>
       <c r="CG143" s="24" t="inlineStr">
@@ -43682,12 +43682,12 @@
     <row r="144" ht="36" customHeight="1">
       <c r="A144" s="24" t="inlineStr">
         <is>
-          <t>9cfe550b2b8d45f2</t>
+          <t>8b5ec6c1f1f44422</t>
         </is>
       </c>
       <c r="B144" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C144" s="24" t="inlineStr">
@@ -43741,11 +43741,11 @@
         <v>0.420168</v>
       </c>
       <c r="O144" s="28" t="n">
-        <v>0.51845</v>
+        <v>0.518281</v>
       </c>
       <c r="P144" s="28" t="n"/>
       <c r="Q144" s="28" t="n">
-        <v>0.09828199999999999</v>
+        <v>0.09811300000000001</v>
       </c>
       <c r="R144" s="26" t="n">
         <v>70</v>
@@ -43774,7 +43774,7 @@
       <c r="AD144" s="24" t="n"/>
       <c r="AE144" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.6242; executable ask 0.4200 (aec-mlb-pit-cin-2026-08-02); model edge vs ask +0.0984.</t>
+          <t>Learned LR call at threshold 0.6242; executable ask 0.4200 (aec-mlb-pit-cin-2026-08-02); model edge vs ask +0.0983.</t>
         </is>
       </c>
       <c r="AF144" s="31" t="inlineStr">
@@ -43878,7 +43878,7 @@
       </c>
       <c r="BE144" s="24" t="inlineStr">
         <is>
-          <t>ddeca2e105ed897c</t>
+          <t>e81c9e33420b63e5</t>
         </is>
       </c>
       <c r="BF144" s="24" t="inlineStr">
@@ -43893,7 +43893,7 @@
       </c>
       <c r="BH144" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:06.897751Z</t>
+          <t>2026-08-02T08:13:09.748235Z</t>
         </is>
       </c>
       <c r="BI144" s="24" t="inlineStr">
@@ -43945,7 +43945,7 @@
       </c>
       <c r="CF144" s="24" t="inlineStr">
         <is>
-          <t>1.003</t>
+          <t>0.9998</t>
         </is>
       </c>
       <c r="CG144" s="24" t="inlineStr">
@@ -43965,12 +43965,12 @@
     <row r="145" ht="36" customHeight="1">
       <c r="A145" s="24" t="inlineStr">
         <is>
-          <t>dbf17318f3b04172</t>
+          <t>0c2c7bd30be04cd8</t>
         </is>
       </c>
       <c r="B145" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C145" s="24" t="inlineStr">
@@ -44176,7 +44176,7 @@
       </c>
       <c r="BH145" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:09.528742Z</t>
+          <t>2026-08-02T08:13:12.455661Z</t>
         </is>
       </c>
       <c r="BI145" s="24" t="inlineStr">
@@ -44248,12 +44248,12 @@
     <row r="146" ht="36" customHeight="1">
       <c r="A146" s="24" t="inlineStr">
         <is>
-          <t>0e889584bda548c1</t>
+          <t>f9875c3874ed4fbd</t>
         </is>
       </c>
       <c r="B146" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C146" s="24" t="inlineStr">
@@ -44307,11 +44307,11 @@
         <v>0.465116</v>
       </c>
       <c r="O146" s="28" t="n">
-        <v>0.549412</v>
+        <v>0.549359</v>
       </c>
       <c r="P146" s="28" t="n"/>
       <c r="Q146" s="28" t="n">
-        <v>0.084296</v>
+        <v>0.084243</v>
       </c>
       <c r="R146" s="26" t="n">
         <v>63</v>
@@ -44444,7 +44444,7 @@
       </c>
       <c r="BE146" s="24" t="inlineStr">
         <is>
-          <t>a08edee3cd28001e</t>
+          <t>a1252a581a025628</t>
         </is>
       </c>
       <c r="BF146" s="24" t="inlineStr">
@@ -44459,7 +44459,7 @@
       </c>
       <c r="BH146" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:10.401780Z</t>
+          <t>2026-08-02T08:13:13.419852Z</t>
         </is>
       </c>
       <c r="BI146" s="24" t="inlineStr">
@@ -44511,7 +44511,7 @@
       </c>
       <c r="CF146" s="24" t="inlineStr">
         <is>
-          <t>1.0103</t>
+          <t>1.0113</t>
         </is>
       </c>
       <c r="CG146" s="24" t="inlineStr">
@@ -44531,12 +44531,12 @@
     <row r="147" ht="36" customHeight="1">
       <c r="A147" s="24" t="inlineStr">
         <is>
-          <t>d3cc2a684a754d13</t>
+          <t>ffef63b948424414</t>
         </is>
       </c>
       <c r="B147" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C147" s="24" t="inlineStr">
@@ -44590,11 +44590,11 @@
         <v>0.490196</v>
       </c>
       <c r="O147" s="28" t="n">
-        <v>0.5999989999999999</v>
+        <v>0.600004</v>
       </c>
       <c r="P147" s="28" t="n"/>
       <c r="Q147" s="28" t="n">
-        <v>0.109803</v>
+        <v>0.109808</v>
       </c>
       <c r="R147" s="26" t="n">
         <v>76</v>
@@ -44727,7 +44727,7 @@
       </c>
       <c r="BE147" s="24" t="inlineStr">
         <is>
-          <t>8a8f8b72edb34435</t>
+          <t>6c183dcf06abc223</t>
         </is>
       </c>
       <c r="BF147" s="24" t="inlineStr">
@@ -44742,7 +44742,7 @@
       </c>
       <c r="BH147" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:11.443231Z</t>
+          <t>2026-08-02T08:13:14.485980Z</t>
         </is>
       </c>
       <c r="BI147" s="24" t="inlineStr">
@@ -44794,7 +44794,7 @@
       </c>
       <c r="CF147" s="24" t="inlineStr">
         <is>
-          <t>1.0303</t>
+          <t>1.0304</t>
         </is>
       </c>
       <c r="CG147" s="24" t="inlineStr">
@@ -44814,12 +44814,12 @@
     <row r="148" ht="36" customHeight="1">
       <c r="A148" s="24" t="inlineStr">
         <is>
-          <t>4c2b96cd3d92494b</t>
+          <t>17809722892c48e2</t>
         </is>
       </c>
       <c r="B148" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C148" s="24" t="inlineStr">
@@ -44873,11 +44873,11 @@
         <v>0.684543</v>
       </c>
       <c r="O148" s="28" t="n">
-        <v>0.625617</v>
+        <v>0.625671</v>
       </c>
       <c r="P148" s="28" t="n"/>
       <c r="Q148" s="28" t="n">
-        <v>-0.058926</v>
+        <v>-0.058872</v>
       </c>
       <c r="R148" s="26" t="n">
         <v>0</v>
@@ -44906,7 +44906,7 @@
       <c r="AD148" s="24" t="n"/>
       <c r="AE148" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.6242; executable ask 0.6850 (aec-mlb-mil-laa-2026-08-02); model edge vs ask -0.0594.</t>
+          <t>Learned LR call at threshold 0.6242; executable ask 0.6850 (aec-mlb-mil-laa-2026-08-02); model edge vs ask -0.0593.</t>
         </is>
       </c>
       <c r="AF148" s="31" t="inlineStr">
@@ -45010,7 +45010,7 @@
       </c>
       <c r="BE148" s="24" t="inlineStr">
         <is>
-          <t>b4ef4d89871f7ba6</t>
+          <t>f8a2203f6c655d56</t>
         </is>
       </c>
       <c r="BF148" s="24" t="inlineStr">
@@ -45025,7 +45025,7 @@
       </c>
       <c r="BH148" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:12.131172Z</t>
+          <t>2026-08-02T08:13:15.230743Z</t>
         </is>
       </c>
       <c r="BI148" s="24" t="inlineStr">
@@ -45077,7 +45077,7 @@
       </c>
       <c r="CF148" s="24" t="inlineStr">
         <is>
-          <t>1.0177</t>
+          <t>1.0188</t>
         </is>
       </c>
       <c r="CG148" s="24" t="inlineStr">
@@ -45097,12 +45097,12 @@
     <row r="149" ht="36" customHeight="1">
       <c r="A149" s="24" t="inlineStr">
         <is>
-          <t>d24cc6fafa2f4671</t>
+          <t>c446ab1817c94fd9</t>
         </is>
       </c>
       <c r="B149" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C149" s="24" t="inlineStr">
@@ -45308,7 +45308,7 @@
       </c>
       <c r="BH149" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:13.443758Z</t>
+          <t>2026-08-02T08:13:16.521010Z</t>
         </is>
       </c>
       <c r="BI149" s="24" t="inlineStr">
@@ -45380,12 +45380,12 @@
     <row r="150" ht="36" customHeight="1">
       <c r="A150" s="24" t="inlineStr">
         <is>
-          <t>2cb74c9d3fd64bcf</t>
+          <t>caff83a7aa4b4ac4</t>
         </is>
       </c>
       <c r="B150" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C150" s="24" t="inlineStr">
@@ -45591,7 +45591,7 @@
       </c>
       <c r="BH150" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:15.238873Z</t>
+          <t>2026-08-02T08:13:18.297617Z</t>
         </is>
       </c>
       <c r="BI150" s="24" t="inlineStr">
@@ -45663,12 +45663,12 @@
     <row r="151" ht="36" customHeight="1">
       <c r="A151" s="24" t="inlineStr">
         <is>
-          <t>62f4495bc07841de</t>
+          <t>976b298ef7914583</t>
         </is>
       </c>
       <c r="B151" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C151" s="24" t="inlineStr">
@@ -45722,11 +45722,11 @@
         <v>0.579832</v>
       </c>
       <c r="O151" s="28" t="n">
-        <v>0.589015</v>
+        <v>0.589077</v>
       </c>
       <c r="P151" s="28" t="n"/>
       <c r="Q151" s="28" t="n">
-        <v>0.009183</v>
+        <v>0.009245</v>
       </c>
       <c r="R151" s="26" t="n">
         <v>26</v>
@@ -45755,7 +45755,7 @@
       <c r="AD151" s="24" t="n"/>
       <c r="AE151" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.6242; executable ask 0.5800 (aec-mlb-sf-sd-2026-08-02); model edge vs ask +0.0090.</t>
+          <t>Learned LR call at threshold 0.6242; executable ask 0.5800 (aec-mlb-sf-sd-2026-08-02); model edge vs ask +0.0091.</t>
         </is>
       </c>
       <c r="AF151" s="31" t="inlineStr">
@@ -45859,7 +45859,7 @@
       </c>
       <c r="BE151" s="24" t="inlineStr">
         <is>
-          <t>c332f3cd0c06de36</t>
+          <t>ba92c3edd0b161e2</t>
         </is>
       </c>
       <c r="BF151" s="24" t="inlineStr">
@@ -45874,7 +45874,7 @@
       </c>
       <c r="BH151" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:14.354504Z</t>
+          <t>2026-08-02T08:13:17.365911Z</t>
         </is>
       </c>
       <c r="BI151" s="24" t="inlineStr">
@@ -45926,7 +45926,7 @@
       </c>
       <c r="CF151" s="24" t="inlineStr">
         <is>
-          <t>1.0122</t>
+          <t>1.011</t>
         </is>
       </c>
       <c r="CG151" s="24" t="inlineStr">
@@ -45946,12 +45946,12 @@
     <row r="152" ht="36" customHeight="1">
       <c r="A152" s="24" t="inlineStr">
         <is>
-          <t>9b1bd9a3e7c64463</t>
+          <t>bebfa96d9cd7493d</t>
         </is>
       </c>
       <c r="B152" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:10.920987Z</t>
+          <t>2026-08-02T08:14:17.540470Z</t>
         </is>
       </c>
       <c r="C152" s="24" t="inlineStr">
@@ -46005,11 +46005,11 @@
         <v>0.6</v>
       </c>
       <c r="O152" s="28" t="n">
-        <v>0.559402</v>
+        <v>0.559386</v>
       </c>
       <c r="P152" s="28" t="n"/>
       <c r="Q152" s="28" t="n">
-        <v>-0.040598</v>
+        <v>-0.040614</v>
       </c>
       <c r="R152" s="26" t="n">
         <v>1</v>
@@ -46142,7 +46142,7 @@
       </c>
       <c r="BE152" s="24" t="inlineStr">
         <is>
-          <t>eb0d325be4c32457</t>
+          <t>9c6127bfe5faaf19</t>
         </is>
       </c>
       <c r="BF152" s="24" t="inlineStr">
@@ -46157,7 +46157,7 @@
       </c>
       <c r="BH152" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:16.250112Z</t>
+          <t>2026-08-02T08:13:19.268959Z</t>
         </is>
       </c>
       <c r="BI152" s="24" t="inlineStr">
@@ -46209,7 +46209,7 @@
       </c>
       <c r="CF152" s="24" t="inlineStr">
         <is>
-          <t>1.0168</t>
+          <t>1.0171</t>
         </is>
       </c>
       <c r="CG152" s="24" t="inlineStr">
@@ -46229,12 +46229,12 @@
     <row r="153" ht="36" customHeight="1">
       <c r="A153" s="24" t="inlineStr">
         <is>
-          <t>078aa36bb2ab4520</t>
+          <t>369b161bac2147f6</t>
         </is>
       </c>
       <c r="B153" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C153" s="24" t="inlineStr">
@@ -46290,13 +46290,13 @@
         <v>0.579832</v>
       </c>
       <c r="O153" s="28" t="n">
-        <v>0.613785</v>
+        <v>0.613621</v>
       </c>
       <c r="P153" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q153" s="28" t="n">
-        <v>0.033953</v>
+        <v>0.033789</v>
       </c>
       <c r="R153" s="26" t="n">
         <v>42</v>
@@ -46325,7 +46325,7 @@
       <c r="AD153" s="24" t="n"/>
       <c r="AE153" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.52-4.52; raw selected-side p=0.6734, calibrated p=0.6138.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.52-4.52; raw selected-side p=0.6731, calibrated p=0.6136.</t>
         </is>
       </c>
       <c r="AF153" s="31" t="inlineStr">
@@ -46444,7 +46444,7 @@
       </c>
       <c r="BH153" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI153" s="24" t="inlineStr">
@@ -46498,12 +46498,12 @@
     <row r="154" ht="36" customHeight="1">
       <c r="A154" s="24" t="inlineStr">
         <is>
-          <t>01da5bdcf3d84064</t>
+          <t>fd682a75c55f4436</t>
         </is>
       </c>
       <c r="B154" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C154" s="24" t="inlineStr">
@@ -46559,13 +46559,13 @@
         <v>0.526066</v>
       </c>
       <c r="O154" s="28" t="n">
-        <v>0.537985</v>
+        <v>0.538976</v>
       </c>
       <c r="P154" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q154" s="28" t="n">
-        <v>0.011919</v>
+        <v>0.01291</v>
       </c>
       <c r="R154" s="26" t="n">
         <v>31</v>
@@ -46594,7 +46594,7 @@
       <c r="AD154" s="24" t="n"/>
       <c r="AE154" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.52-4.52; raw selected-side p=0.5879, calibrated p=0.5380.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.52-4.52; raw selected-side p=0.5908, calibrated p=0.5390.</t>
         </is>
       </c>
       <c r="AF154" s="31" t="inlineStr">
@@ -46713,7 +46713,7 @@
       </c>
       <c r="BH154" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI154" s="24" t="inlineStr">
@@ -46767,12 +46767,12 @@
     <row r="155" ht="36" customHeight="1">
       <c r="A155" s="24" t="inlineStr">
         <is>
-          <t>4496f2eb6d614af5</t>
+          <t>3c66c2c35ec54eb4</t>
         </is>
       </c>
       <c r="B155" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C155" s="24" t="inlineStr">
@@ -46828,13 +46828,13 @@
         <v>0.62963</v>
       </c>
       <c r="O155" s="28" t="n">
-        <v>0.572549</v>
+        <v>0.57268</v>
       </c>
       <c r="P155" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q155" s="28" t="n">
-        <v>-0.057081</v>
+        <v>-0.05695</v>
       </c>
       <c r="R155" s="26" t="n">
         <v>0</v>
@@ -46863,7 +46863,7 @@
       <c r="AD155" s="24" t="n"/>
       <c r="AE155" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 5.24-4.76; raw selected-side p=0.6105, calibrated p=0.5725.</t>
+          <t>Measured Edge Margin: Trend Engine projected 5.24-4.76; raw selected-side p=0.6107, calibrated p=0.5727.</t>
         </is>
       </c>
       <c r="AF155" s="31" t="inlineStr">
@@ -46982,7 +46982,7 @@
       </c>
       <c r="BH155" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI155" s="24" t="inlineStr">
@@ -47036,12 +47036,12 @@
     <row r="156" ht="36" customHeight="1">
       <c r="A156" s="24" t="inlineStr">
         <is>
-          <t>5ddf3d557d4f4574</t>
+          <t>d9c9964ad56f4f3e</t>
         </is>
       </c>
       <c r="B156" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C156" s="24" t="inlineStr">
@@ -47088,22 +47088,22 @@
         </is>
       </c>
       <c r="L156" s="26" t="n">
-        <v>-125</v>
+        <v>-122</v>
       </c>
       <c r="M156" s="27" t="n">
-        <v>1.8</v>
+        <v>1.819672</v>
       </c>
       <c r="N156" s="28" t="n">
-        <v>0.555556</v>
+        <v>0.54955</v>
       </c>
       <c r="O156" s="28" t="n">
-        <v>0.510034</v>
+        <v>0.510837</v>
       </c>
       <c r="P156" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q156" s="28" t="n">
-        <v>-0.045522</v>
+        <v>-0.038713</v>
       </c>
       <c r="R156" s="26" t="n">
         <v>0</v>
@@ -47132,7 +47132,7 @@
       <c r="AD156" s="24" t="n"/>
       <c r="AE156" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 5.24-4.76; raw selected-side p=0.5061, calibrated p=0.5100.</t>
+          <t>Measured Edge Totals: Trend Engine projected 5.24-4.76; raw selected-side p=0.5084, calibrated p=0.5108.</t>
         </is>
       </c>
       <c r="AF156" s="31" t="inlineStr">
@@ -47251,7 +47251,7 @@
       </c>
       <c r="BH156" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI156" s="24" t="inlineStr">
@@ -47263,16 +47263,16 @@
         <v>9.5</v>
       </c>
       <c r="BK156" s="26" t="n">
-        <v>-125</v>
+        <v>-122</v>
       </c>
       <c r="BL156" s="27" t="n">
-        <v>1.8</v>
+        <v>1.819672</v>
       </c>
       <c r="BM156" s="28" t="n">
-        <v>0.555556</v>
+        <v>0.54955</v>
       </c>
       <c r="BN156" s="28" t="n">
-        <v>0.552239</v>
+        <v>0.547264</v>
       </c>
       <c r="BO156" s="28" t="n"/>
       <c r="BP156" s="25" t="n"/>
@@ -47305,12 +47305,12 @@
     <row r="157" ht="36" customHeight="1">
       <c r="A157" s="24" t="inlineStr">
         <is>
-          <t>a59b10ac192d4010</t>
+          <t>dc37e3573aff4532</t>
         </is>
       </c>
       <c r="B157" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C157" s="24" t="inlineStr">
@@ -47366,16 +47366,16 @@
         <v>0.615385</v>
       </c>
       <c r="O157" s="28" t="n">
-        <v>0.604928</v>
+        <v>0.6049600000000001</v>
       </c>
       <c r="P157" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q157" s="28" t="n">
-        <v>-0.010457</v>
+        <v>-0.010425</v>
       </c>
       <c r="R157" s="26" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S157" s="29" t="n">
         <v>1.5</v>
@@ -47401,7 +47401,7 @@
       <c r="AD157" s="24" t="n"/>
       <c r="AE157" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.39-4.52; raw selected-side p=0.6599, calibrated p=0.6049.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.39-4.52; raw selected-side p=0.6599, calibrated p=0.6050.</t>
         </is>
       </c>
       <c r="AF157" s="31" t="inlineStr">
@@ -47520,7 +47520,7 @@
       </c>
       <c r="BH157" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI157" s="24" t="inlineStr">
@@ -47574,12 +47574,12 @@
     <row r="158" ht="36" customHeight="1">
       <c r="A158" s="24" t="inlineStr">
         <is>
-          <t>ec055a248c144078</t>
+          <t>54bbdea2b4a7473d</t>
         </is>
       </c>
       <c r="B158" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C158" s="24" t="inlineStr">
@@ -47635,16 +47635,16 @@
         <v>0.539171</v>
       </c>
       <c r="O158" s="28" t="n">
-        <v>0.537268</v>
+        <v>0.535628</v>
       </c>
       <c r="P158" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q158" s="28" t="n">
-        <v>-0.001903</v>
+        <v>-0.003543</v>
       </c>
       <c r="R158" s="26" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="S158" s="29" t="n">
         <v>1</v>
@@ -47670,7 +47670,7 @@
       <c r="AD158" s="24" t="n"/>
       <c r="AE158" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.39-4.52; raw selected-side p=0.5858, calibrated p=0.5373.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.39-4.52; raw selected-side p=0.5810, calibrated p=0.5356.</t>
         </is>
       </c>
       <c r="AF158" s="31" t="inlineStr">
@@ -47789,7 +47789,7 @@
       </c>
       <c r="BH158" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI158" s="24" t="inlineStr">
@@ -47843,12 +47843,12 @@
     <row r="159" ht="36" customHeight="1">
       <c r="A159" s="24" t="inlineStr">
         <is>
-          <t>cca6c9c74ca340b5</t>
+          <t>f58f51b49eb0439e</t>
         </is>
       </c>
       <c r="B159" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C159" s="24" t="inlineStr">
@@ -47904,13 +47904,13 @@
         <v>0.615385</v>
       </c>
       <c r="O159" s="28" t="n">
-        <v>0.602074</v>
+        <v>0.601483</v>
       </c>
       <c r="P159" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q159" s="28" t="n">
-        <v>-0.013311</v>
+        <v>-0.013902</v>
       </c>
       <c r="R159" s="26" t="n">
         <v>18</v>
@@ -47939,7 +47939,7 @@
       <c r="AD159" s="24" t="n"/>
       <c r="AE159" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.47-4.63; raw selected-side p=0.6555, calibrated p=0.6021.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.47-4.63; raw selected-side p=0.6546, calibrated p=0.6015.</t>
         </is>
       </c>
       <c r="AF159" s="31" t="inlineStr">
@@ -48058,7 +48058,7 @@
       </c>
       <c r="BH159" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI159" s="24" t="inlineStr">
@@ -48112,12 +48112,12 @@
     <row r="160" ht="36" customHeight="1">
       <c r="A160" s="24" t="inlineStr">
         <is>
-          <t>f10621d536a646e7</t>
+          <t>21f34d3890d94e90</t>
         </is>
       </c>
       <c r="B160" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C160" s="24" t="inlineStr">
@@ -48173,16 +48173,16 @@
         <v>0.514563</v>
       </c>
       <c r="O160" s="28" t="n">
-        <v>0.539233</v>
+        <v>0.541044</v>
       </c>
       <c r="P160" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q160" s="28" t="n">
-        <v>0.02467</v>
+        <v>0.026481</v>
       </c>
       <c r="R160" s="26" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="S160" s="29" t="n">
         <v>1</v>
@@ -48208,7 +48208,7 @@
       <c r="AD160" s="24" t="n"/>
       <c r="AE160" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.47-4.63; raw selected-side p=0.5916, calibrated p=0.5392.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.47-4.63; raw selected-side p=0.5968, calibrated p=0.5410.</t>
         </is>
       </c>
       <c r="AF160" s="31" t="inlineStr">
@@ -48327,7 +48327,7 @@
       </c>
       <c r="BH160" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI160" s="24" t="inlineStr">
@@ -48381,12 +48381,12 @@
     <row r="161" ht="36" customHeight="1">
       <c r="A161" s="24" t="inlineStr">
         <is>
-          <t>6c28ba57551a4fd0</t>
+          <t>eaf1e26bf8444035</t>
         </is>
       </c>
       <c r="B161" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C161" s="24" t="inlineStr">
@@ -48442,19 +48442,19 @@
         <v>0.6</v>
       </c>
       <c r="O161" s="28" t="n">
-        <v>0.611325</v>
+        <v>0.605288</v>
       </c>
       <c r="P161" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q161" s="28" t="n">
-        <v>0.011325</v>
+        <v>0.005288</v>
       </c>
       <c r="R161" s="26" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="S161" s="29" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="T161" s="24" t="inlineStr">
         <is>
@@ -48477,7 +48477,7 @@
       <c r="AD161" s="24" t="n"/>
       <c r="AE161" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.52-4.47; raw selected-side p=0.6696, calibrated p=0.6113.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.52-4.47; raw selected-side p=0.6604, calibrated p=0.6053.</t>
         </is>
       </c>
       <c r="AF161" s="31" t="inlineStr">
@@ -48596,7 +48596,7 @@
       </c>
       <c r="BH161" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI161" s="24" t="inlineStr">
@@ -48650,12 +48650,12 @@
     <row r="162" ht="36" customHeight="1">
       <c r="A162" s="24" t="inlineStr">
         <is>
-          <t>7806dcc79f0e44d9</t>
+          <t>16d99165e5eb4502</t>
         </is>
       </c>
       <c r="B162" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C162" s="24" t="inlineStr">
@@ -48711,13 +48711,13 @@
         <v>0.526066</v>
       </c>
       <c r="O162" s="28" t="n">
-        <v>0.51287</v>
+        <v>0.512136</v>
       </c>
       <c r="P162" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q162" s="28" t="n">
-        <v>-0.013196</v>
+        <v>-0.01393</v>
       </c>
       <c r="R162" s="26" t="n">
         <v>12</v>
@@ -48746,7 +48746,7 @@
       <c r="AD162" s="24" t="n"/>
       <c r="AE162" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.52-4.47; raw selected-side p=0.5144, calibrated p=0.5129.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.52-4.47; raw selected-side p=0.5122, calibrated p=0.5121.</t>
         </is>
       </c>
       <c r="AF162" s="31" t="inlineStr">
@@ -48865,7 +48865,7 @@
       </c>
       <c r="BH162" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI162" s="24" t="inlineStr">
@@ -48919,12 +48919,12 @@
     <row r="163" ht="36" customHeight="1">
       <c r="A163" s="24" t="inlineStr">
         <is>
-          <t>a362b4c4fdc84417</t>
+          <t>17e0b52acb514401</t>
         </is>
       </c>
       <c r="B163" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C163" s="24" t="inlineStr">
@@ -48980,16 +48980,16 @@
         <v>0.6</v>
       </c>
       <c r="O163" s="28" t="n">
-        <v>0.57537</v>
+        <v>0.579077</v>
       </c>
       <c r="P163" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q163" s="28" t="n">
-        <v>-0.02463</v>
+        <v>-0.020923</v>
       </c>
       <c r="R163" s="26" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="S163" s="29" t="n">
         <v>1.25</v>
@@ -49015,7 +49015,7 @@
       <c r="AD163" s="24" t="n"/>
       <c r="AE163" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.31-4.86; raw selected-side p=0.6148, calibrated p=0.5754.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.31-4.85; raw selected-side p=0.6204, calibrated p=0.5791.</t>
         </is>
       </c>
       <c r="AF163" s="31" t="inlineStr">
@@ -49134,7 +49134,7 @@
       </c>
       <c r="BH163" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI163" s="24" t="inlineStr">
@@ -49188,12 +49188,12 @@
     <row r="164" ht="36" customHeight="1">
       <c r="A164" s="24" t="inlineStr">
         <is>
-          <t>d9b01478f9a84f75</t>
+          <t>09d0628db5ea4403</t>
         </is>
       </c>
       <c r="B164" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C164" s="24" t="inlineStr">
@@ -49249,13 +49249,13 @@
         <v>0.485437</v>
       </c>
       <c r="O164" s="28" t="n">
-        <v>0.519021</v>
+        <v>0.519517</v>
       </c>
       <c r="P164" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q164" s="28" t="n">
-        <v>0.033584</v>
+        <v>0.03408</v>
       </c>
       <c r="R164" s="26" t="n">
         <v>42</v>
@@ -49284,7 +49284,7 @@
       <c r="AD164" s="24" t="n"/>
       <c r="AE164" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.31-4.86; raw selected-side p=0.5324, calibrated p=0.5190.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.31-4.85; raw selected-side p=0.5339, calibrated p=0.5195.</t>
         </is>
       </c>
       <c r="AF164" s="31" t="inlineStr">
@@ -49403,7 +49403,7 @@
       </c>
       <c r="BH164" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI164" s="24" t="inlineStr">
@@ -49457,12 +49457,12 @@
     <row r="165" ht="36" customHeight="1">
       <c r="A165" s="24" t="inlineStr">
         <is>
-          <t>f5a51297d21a4272</t>
+          <t>d8ba96ac30194d6f</t>
         </is>
       </c>
       <c r="B165" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C165" s="24" t="inlineStr">
@@ -49518,13 +49518,13 @@
         <v>0.640288</v>
       </c>
       <c r="O165" s="28" t="n">
-        <v>0.580521</v>
+        <v>0.582391</v>
       </c>
       <c r="P165" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q165" s="28" t="n">
-        <v>-0.059767</v>
+        <v>-0.057897</v>
       </c>
       <c r="R165" s="26" t="n">
         <v>0</v>
@@ -49553,7 +49553,7 @@
       <c r="AD165" s="24" t="n"/>
       <c r="AE165" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.10-4.64; raw selected-side p=0.6227, calibrated p=0.5805.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.10-4.64; raw selected-side p=0.6255, calibrated p=0.5824.</t>
         </is>
       </c>
       <c r="AF165" s="31" t="inlineStr">
@@ -49672,7 +49672,7 @@
       </c>
       <c r="BH165" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI165" s="24" t="inlineStr">
@@ -49726,12 +49726,12 @@
     <row r="166" ht="36" customHeight="1">
       <c r="A166" s="24" t="inlineStr">
         <is>
-          <t>8cb7ff179f6342c7</t>
+          <t>3da034338735473e</t>
         </is>
       </c>
       <c r="B166" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C166" s="24" t="inlineStr">
@@ -49778,25 +49778,25 @@
         </is>
       </c>
       <c r="L166" s="26" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="M166" s="27" t="n">
-        <v>2.11</v>
+        <v>2.08</v>
       </c>
       <c r="N166" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.480769</v>
       </c>
       <c r="O166" s="28" t="n">
-        <v>0.509419</v>
+        <v>0.511145</v>
       </c>
       <c r="P166" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q166" s="28" t="n">
-        <v>0.035485</v>
+        <v>0.030376</v>
       </c>
       <c r="R166" s="26" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="S166" s="29" t="n">
         <v>1</v>
@@ -49822,7 +49822,7 @@
       <c r="AD166" s="24" t="n"/>
       <c r="AE166" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.10-4.64; raw selected-side p=0.5043, calibrated p=0.5094.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.10-4.64; raw selected-side p=0.5093, calibrated p=0.5111.</t>
         </is>
       </c>
       <c r="AF166" s="31" t="inlineStr">
@@ -49941,7 +49941,7 @@
       </c>
       <c r="BH166" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI166" s="24" t="inlineStr">
@@ -49953,16 +49953,16 @@
         <v>8.5</v>
       </c>
       <c r="BK166" s="26" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="BL166" s="27" t="n">
-        <v>2.11</v>
+        <v>2.08</v>
       </c>
       <c r="BM166" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.480769</v>
       </c>
       <c r="BN166" s="28" t="n">
-        <v>0.472637</v>
+        <v>0.477612</v>
       </c>
       <c r="BO166" s="28" t="n"/>
       <c r="BP166" s="25" t="n"/>
@@ -49995,12 +49995,12 @@
     <row r="167" ht="36" customHeight="1">
       <c r="A167" s="24" t="inlineStr">
         <is>
-          <t>36f82871b4654938</t>
+          <t>99288d8a84204483</t>
         </is>
       </c>
       <c r="B167" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C167" s="24" t="inlineStr">
@@ -50056,13 +50056,13 @@
         <v>0.609375</v>
       </c>
       <c r="O167" s="28" t="n">
-        <v>0.608864</v>
+        <v>0.608241</v>
       </c>
       <c r="P167" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q167" s="28" t="n">
-        <v>-0.000511</v>
+        <v>-0.001134</v>
       </c>
       <c r="R167" s="26" t="n">
         <v>24</v>
@@ -50091,7 +50091,7 @@
       <c r="AD167" s="24" t="n"/>
       <c r="AE167" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.57-4.52; raw selected-side p=0.6659, calibrated p=0.6089.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.57-4.52; raw selected-side p=0.6649, calibrated p=0.6082.</t>
         </is>
       </c>
       <c r="AF167" s="31" t="inlineStr">
@@ -50210,7 +50210,7 @@
       </c>
       <c r="BH167" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI167" s="24" t="inlineStr">
@@ -50264,12 +50264,12 @@
     <row r="168" ht="36" customHeight="1">
       <c r="A168" s="24" t="inlineStr">
         <is>
-          <t>1ada589f9f0e41a0</t>
+          <t>3cdc25ad8f074bf1</t>
         </is>
       </c>
       <c r="B168" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C168" s="24" t="inlineStr">
@@ -50325,16 +50325,16 @@
         <v>0.514563</v>
       </c>
       <c r="O168" s="28" t="n">
-        <v>0.582372</v>
+        <v>0.584935</v>
       </c>
       <c r="P168" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q168" s="28" t="n">
-        <v>0.06780899999999999</v>
+        <v>0.070372</v>
       </c>
       <c r="R168" s="26" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="S168" s="29" t="n">
         <v>1.25</v>
@@ -50360,7 +50360,7 @@
       <c r="AD168" s="24" t="n"/>
       <c r="AE168" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.57-4.52; raw selected-side p=0.7178, calibrated p=0.5824.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.57-4.52; raw selected-side p=0.7253, calibrated p=0.5849.</t>
         </is>
       </c>
       <c r="AF168" s="31" t="inlineStr">
@@ -50479,7 +50479,7 @@
       </c>
       <c r="BH168" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI168" s="24" t="inlineStr">
@@ -50533,12 +50533,12 @@
     <row r="169" ht="36" customHeight="1">
       <c r="A169" s="24" t="inlineStr">
         <is>
-          <t>03e1fbb5a19d452f</t>
+          <t>162a409666464718</t>
         </is>
       </c>
       <c r="B169" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C169" s="24" t="inlineStr">
@@ -50594,16 +50594,16 @@
         <v>0.609375</v>
       </c>
       <c r="O169" s="28" t="n">
-        <v>0.586983</v>
+        <v>0.590625</v>
       </c>
       <c r="P169" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q169" s="28" t="n">
-        <v>-0.022392</v>
+        <v>-0.01875</v>
       </c>
       <c r="R169" s="26" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S169" s="29" t="n">
         <v>1.25</v>
@@ -50629,7 +50629,7 @@
       <c r="AD169" s="24" t="n"/>
       <c r="AE169" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 5.19-4.94; raw selected-side p=0.6325, calibrated p=0.5870.</t>
+          <t>Measured Edge Margin: Trend Engine projected 5.19-4.94; raw selected-side p=0.6381, calibrated p=0.5906.</t>
         </is>
       </c>
       <c r="AF169" s="31" t="inlineStr">
@@ -50748,7 +50748,7 @@
       </c>
       <c r="BH169" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI169" s="24" t="inlineStr">
@@ -50802,12 +50802,12 @@
     <row r="170" ht="36" customHeight="1">
       <c r="A170" s="24" t="inlineStr">
         <is>
-          <t>783371d561c04b99</t>
+          <t>ec3154b3f008419a</t>
         </is>
       </c>
       <c r="B170" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C170" s="24" t="inlineStr">
@@ -50863,13 +50863,13 @@
         <v>0.514563</v>
       </c>
       <c r="O170" s="28" t="n">
-        <v>0.581381</v>
+        <v>0.58133</v>
       </c>
       <c r="P170" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q170" s="28" t="n">
-        <v>0.066818</v>
+        <v>0.06676700000000001</v>
       </c>
       <c r="R170" s="26" t="n">
         <v>58</v>
@@ -50898,7 +50898,7 @@
       <c r="AD170" s="24" t="n"/>
       <c r="AE170" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 5.19-4.94; raw selected-side p=0.7149, calibrated p=0.5814.</t>
+          <t>Measured Edge Totals: Trend Engine projected 5.19-4.94; raw selected-side p=0.7147, calibrated p=0.5813.</t>
         </is>
       </c>
       <c r="AF170" s="31" t="inlineStr">
@@ -51017,7 +51017,7 @@
       </c>
       <c r="BH170" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI170" s="24" t="inlineStr">
@@ -51071,12 +51071,12 @@
     <row r="171" ht="36" customHeight="1">
       <c r="A171" s="24" t="inlineStr">
         <is>
-          <t>b7549529bf0d4e26</t>
+          <t>815a00f76da542fe</t>
         </is>
       </c>
       <c r="B171" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C171" s="24" t="inlineStr">
@@ -51132,19 +51132,19 @@
         <v>0.45045</v>
       </c>
       <c r="O171" s="28" t="n">
-        <v>0.599613</v>
+        <v>0.597842</v>
       </c>
       <c r="P171" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q171" s="28" t="n">
-        <v>0.149163</v>
+        <v>0.147392</v>
       </c>
       <c r="R171" s="26" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="S171" s="29" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="T171" s="24" t="inlineStr">
         <is>
@@ -51167,7 +51167,7 @@
       <c r="AD171" s="24" t="n"/>
       <c r="AE171" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.33-4.07; raw selected-side p=0.6518, calibrated p=0.5996.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.33-4.07; raw selected-side p=0.6491, calibrated p=0.5978.</t>
         </is>
       </c>
       <c r="AF171" s="31" t="inlineStr">
@@ -51286,7 +51286,7 @@
       </c>
       <c r="BH171" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI171" s="24" t="inlineStr">
@@ -51340,12 +51340,12 @@
     <row r="172" ht="36" customHeight="1">
       <c r="A172" s="24" t="inlineStr">
         <is>
-          <t>d7286d0a4a5447d7</t>
+          <t>46713fab65434a63</t>
         </is>
       </c>
       <c r="B172" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C172" s="24" t="inlineStr">
@@ -51401,13 +51401,13 @@
         <v>0.519231</v>
       </c>
       <c r="O172" s="28" t="n">
-        <v>0.520268</v>
+        <v>0.520183</v>
       </c>
       <c r="P172" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q172" s="28" t="n">
-        <v>0.001037</v>
+        <v>0.000952</v>
       </c>
       <c r="R172" s="26" t="n">
         <v>25</v>
@@ -51436,7 +51436,7 @@
       <c r="AD172" s="24" t="n"/>
       <c r="AE172" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.33-4.07; raw selected-side p=0.5361, calibrated p=0.5203.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.33-4.07; raw selected-side p=0.5358, calibrated p=0.5202.</t>
         </is>
       </c>
       <c r="AF172" s="31" t="inlineStr">
@@ -51555,7 +51555,7 @@
       </c>
       <c r="BH172" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI172" s="24" t="inlineStr">
@@ -51609,12 +51609,12 @@
     <row r="173" ht="36" customHeight="1">
       <c r="A173" s="24" t="inlineStr">
         <is>
-          <t>fa32400389b34365</t>
+          <t>48edf9807b6f4b8c</t>
         </is>
       </c>
       <c r="B173" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C173" s="24" t="inlineStr">
@@ -51661,25 +51661,25 @@
         </is>
       </c>
       <c r="L173" s="26" t="n">
-        <v>-147</v>
+        <v>-144</v>
       </c>
       <c r="M173" s="27" t="n">
-        <v>1.680272</v>
+        <v>1.694444</v>
       </c>
       <c r="N173" s="28" t="n">
-        <v>0.5951419999999999</v>
+        <v>0.590164</v>
       </c>
       <c r="O173" s="28" t="n">
-        <v>0.598859</v>
+        <v>0.603484</v>
       </c>
       <c r="P173" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q173" s="28" t="n">
-        <v>0.003717</v>
+        <v>0.01332</v>
       </c>
       <c r="R173" s="26" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="S173" s="29" t="n">
         <v>1.5</v>
@@ -51705,7 +51705,7 @@
       <c r="AD173" s="24" t="n"/>
       <c r="AE173" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.86-4.74; raw selected-side p=0.6506, calibrated p=0.5989.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.86-4.74; raw selected-side p=0.6576, calibrated p=0.6035.</t>
         </is>
       </c>
       <c r="AF173" s="31" t="inlineStr">
@@ -51824,7 +51824,7 @@
       </c>
       <c r="BH173" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI173" s="24" t="inlineStr">
@@ -51836,16 +51836,16 @@
         <v>1.5</v>
       </c>
       <c r="BK173" s="26" t="n">
-        <v>-147</v>
+        <v>-144</v>
       </c>
       <c r="BL173" s="27" t="n">
-        <v>1.680272</v>
+        <v>1.694444</v>
       </c>
       <c r="BM173" s="28" t="n">
-        <v>0.5951419999999999</v>
+        <v>0.590164</v>
       </c>
       <c r="BN173" s="28" t="n">
-        <v>0.59204</v>
+        <v>0.5870649999999999</v>
       </c>
       <c r="BO173" s="28" t="n"/>
       <c r="BP173" s="25" t="n"/>
@@ -51878,12 +51878,12 @@
     <row r="174" ht="36" customHeight="1">
       <c r="A174" s="24" t="inlineStr">
         <is>
-          <t>d0d74634187e4468</t>
+          <t>ceb05fd83303498e</t>
         </is>
       </c>
       <c r="B174" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C174" s="24" t="inlineStr">
@@ -51939,13 +51939,13 @@
         <v>0.539171</v>
       </c>
       <c r="O174" s="28" t="n">
-        <v>0.5763239999999999</v>
+        <v>0.576119</v>
       </c>
       <c r="P174" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q174" s="28" t="n">
-        <v>0.037153</v>
+        <v>0.036948</v>
       </c>
       <c r="R174" s="26" t="n">
         <v>43</v>
@@ -51974,7 +51974,7 @@
       <c r="AD174" s="24" t="n"/>
       <c r="AE174" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.86-4.74; raw selected-side p=0.7001, calibrated p=0.5763.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.86-4.74; raw selected-side p=0.6995, calibrated p=0.5761.</t>
         </is>
       </c>
       <c r="AF174" s="31" t="inlineStr">
@@ -52093,7 +52093,7 @@
       </c>
       <c r="BH174" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI174" s="24" t="inlineStr">
@@ -52147,12 +52147,12 @@
     <row r="175" ht="36" customHeight="1">
       <c r="A175" s="24" t="inlineStr">
         <is>
-          <t>938a2a4b8e0948e7</t>
+          <t>5cc69ac6020448c4</t>
         </is>
       </c>
       <c r="B175" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C175" s="24" t="inlineStr">
@@ -52208,16 +52208,16 @@
         <v>0.625468</v>
       </c>
       <c r="O175" s="28" t="n">
-        <v>0.607814</v>
+        <v>0.609159</v>
       </c>
       <c r="P175" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q175" s="28" t="n">
-        <v>-0.017654</v>
+        <v>-0.016309</v>
       </c>
       <c r="R175" s="26" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S175" s="29" t="n">
         <v>1.5</v>
@@ -52243,7 +52243,7 @@
       <c r="AD175" s="24" t="n"/>
       <c r="AE175" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.39-4.46; raw selected-side p=0.6643, calibrated p=0.6078.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.39-4.46; raw selected-side p=0.6663, calibrated p=0.6092.</t>
         </is>
       </c>
       <c r="AF175" s="31" t="inlineStr">
@@ -52362,7 +52362,7 @@
       </c>
       <c r="BH175" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI175" s="24" t="inlineStr">
@@ -52416,12 +52416,12 @@
     <row r="176" ht="36" customHeight="1">
       <c r="A176" s="24" t="inlineStr">
         <is>
-          <t>c23696d38c114e3f</t>
+          <t>db7dd970bc2d441a</t>
         </is>
       </c>
       <c r="B176" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C176" s="24" t="inlineStr">
@@ -52477,16 +52477,16 @@
         <v>0.465116</v>
       </c>
       <c r="O176" s="28" t="n">
-        <v>0.532757</v>
+        <v>0.5347730000000001</v>
       </c>
       <c r="P176" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q176" s="28" t="n">
-        <v>0.06764100000000001</v>
+        <v>0.069657</v>
       </c>
       <c r="R176" s="26" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="S176" s="29" t="n">
         <v>1</v>
@@ -52512,7 +52512,7 @@
       <c r="AD176" s="24" t="n"/>
       <c r="AE176" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.39-4.46; raw selected-side p=0.5726, calibrated p=0.5328.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.39-4.46; raw selected-side p=0.5785, calibrated p=0.5348.</t>
         </is>
       </c>
       <c r="AF176" s="31" t="inlineStr">
@@ -52631,7 +52631,7 @@
       </c>
       <c r="BH176" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI176" s="24" t="inlineStr">
@@ -52685,12 +52685,12 @@
     <row r="177" ht="36" customHeight="1">
       <c r="A177" s="24" t="inlineStr">
         <is>
-          <t>f6ffe1e44fcf4e12</t>
+          <t>0bcb6def44ac4301</t>
         </is>
       </c>
       <c r="B177" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C177" s="24" t="inlineStr">
@@ -52746,16 +52746,16 @@
         <v>0.615385</v>
       </c>
       <c r="O177" s="28" t="n">
-        <v>0.580783</v>
+        <v>0.583342</v>
       </c>
       <c r="P177" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q177" s="28" t="n">
-        <v>-0.034602</v>
+        <v>-0.032043</v>
       </c>
       <c r="R177" s="26" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S177" s="29" t="n">
         <v>1.25</v>
@@ -52781,7 +52781,7 @@
       <c r="AD177" s="24" t="n"/>
       <c r="AE177" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.27-4.69; raw selected-side p=0.6230, calibrated p=0.5808.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.27-4.69; raw selected-side p=0.6270, calibrated p=0.5833.</t>
         </is>
       </c>
       <c r="AF177" s="31" t="inlineStr">
@@ -52900,7 +52900,7 @@
       </c>
       <c r="BH177" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI177" s="24" t="inlineStr">
@@ -52954,12 +52954,12 @@
     <row r="178" ht="36" customHeight="1">
       <c r="A178" s="24" t="inlineStr">
         <is>
-          <t>7b5670abdd724134</t>
+          <t>1b350ff7843a4b2b</t>
         </is>
       </c>
       <c r="B178" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C178" s="24" t="inlineStr">
@@ -53015,13 +53015,13 @@
         <v>0.469484</v>
       </c>
       <c r="O178" s="28" t="n">
-        <v>0.5126309999999999</v>
+        <v>0.5111790000000001</v>
       </c>
       <c r="P178" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q178" s="28" t="n">
-        <v>0.043147</v>
+        <v>0.041695</v>
       </c>
       <c r="R178" s="26" t="n">
         <v>46</v>
@@ -53050,7 +53050,7 @@
       <c r="AD178" s="24" t="n"/>
       <c r="AE178" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.27-4.69; raw selected-side p=0.5137, calibrated p=0.5126.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.27-4.69; raw selected-side p=0.5094, calibrated p=0.5112.</t>
         </is>
       </c>
       <c r="AF178" s="31" t="inlineStr">
@@ -53169,7 +53169,7 @@
       </c>
       <c r="BH178" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI178" s="24" t="inlineStr">
@@ -53223,12 +53223,12 @@
     <row r="179" ht="36" customHeight="1">
       <c r="A179" s="24" t="inlineStr">
         <is>
-          <t>38d74e93696841b9</t>
+          <t>ae7fce6ee07a4a79</t>
         </is>
       </c>
       <c r="B179" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C179" s="24" t="inlineStr">
@@ -53284,16 +53284,16 @@
         <v>0.574468</v>
       </c>
       <c r="O179" s="28" t="n">
-        <v>0.627268</v>
+        <v>0.629958</v>
       </c>
       <c r="P179" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q179" s="28" t="n">
-        <v>0.0528</v>
+        <v>0.05549</v>
       </c>
       <c r="R179" s="26" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S179" s="29" t="n">
         <v>1.5</v>
@@ -53319,7 +53319,7 @@
       <c r="AD179" s="24" t="n"/>
       <c r="AE179" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.62-4.38; raw selected-side p=0.6939, calibrated p=0.6273.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.62-4.38; raw selected-side p=0.6980, calibrated p=0.6300.</t>
         </is>
       </c>
       <c r="AF179" s="31" t="inlineStr">
@@ -53438,7 +53438,7 @@
       </c>
       <c r="BH179" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI179" s="24" t="inlineStr">
@@ -53492,12 +53492,12 @@
     <row r="180" ht="36" customHeight="1">
       <c r="A180" s="24" t="inlineStr">
         <is>
-          <t>9ccb474a854942ff</t>
+          <t>7e400b8c271b4bdb</t>
         </is>
       </c>
       <c r="B180" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="C180" s="24" t="inlineStr">
@@ -53553,13 +53553,13 @@
         <v>0.54955</v>
       </c>
       <c r="O180" s="28" t="n">
-        <v>0.51246</v>
+        <v>0.512614</v>
       </c>
       <c r="P180" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q180" s="28" t="n">
-        <v>-0.03709</v>
+        <v>-0.036936</v>
       </c>
       <c r="R180" s="26" t="n">
         <v>6</v>
@@ -53588,7 +53588,7 @@
       <c r="AD180" s="24" t="n"/>
       <c r="AE180" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.62-4.38; raw selected-side p=0.5132, calibrated p=0.5125.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.62-4.38; raw selected-side p=0.5137, calibrated p=0.5126.</t>
         </is>
       </c>
       <c r="AF180" s="31" t="inlineStr">
@@ -53707,7 +53707,7 @@
       </c>
       <c r="BH180" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:12:44.561466Z</t>
+          <t>2026-08-02T08:15:06.961660Z</t>
         </is>
       </c>
       <c r="BI180" s="24" t="inlineStr">
@@ -53761,12 +53761,12 @@
     <row r="181" ht="36" customHeight="1">
       <c r="A181" s="24" t="inlineStr">
         <is>
-          <t>657b410054e34a2a</t>
+          <t>8895b43c04ca4e60</t>
         </is>
       </c>
       <c r="B181" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C181" s="24" t="inlineStr">
@@ -53811,13 +53811,13 @@
         </is>
       </c>
       <c r="L181" s="26" t="n">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="M181" s="27" t="n">
-        <v>3.23</v>
+        <v>3.33</v>
       </c>
       <c r="N181" s="28" t="n">
-        <v>0.309598</v>
+        <v>0.3003</v>
       </c>
       <c r="O181" s="28" t="n">
         <v>0.456135</v>
@@ -53826,10 +53826,10 @@
         <v>0.2</v>
       </c>
       <c r="Q181" s="28" t="n">
-        <v>0.146537</v>
+        <v>0.155835</v>
       </c>
       <c r="R181" s="26" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="S181" s="29" t="n">
         <v>1</v>
@@ -53855,7 +53855,7 @@
       <c r="AD181" s="24" t="n"/>
       <c r="AE181" s="31" t="inlineStr">
         <is>
-          <t>Poisson-DC rates 1.64 (home) / 1.24 (away) from EWMA attack/defense strengths. Executable ask 0.3100 (atc-lpa-ald-gim-2026-08-02-ald).</t>
+          <t>Poisson-DC rates 1.64 (home) / 1.24 (away) from EWMA attack/defense strengths. Executable ask 0.3000 (atc-lpa-ald-gim-2026-08-02-ald).</t>
         </is>
       </c>
       <c r="AF181" s="31" t="inlineStr">
@@ -53974,7 +53974,7 @@
       </c>
       <c r="BH181" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:22.045184Z</t>
+          <t>2026-08-02T08:13:25.124724Z</t>
         </is>
       </c>
       <c r="BI181" s="24" t="inlineStr">
@@ -53984,13 +53984,13 @@
       </c>
       <c r="BJ181" s="25" t="n"/>
       <c r="BK181" s="26" t="n">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="BL181" s="27" t="n">
-        <v>3.23</v>
+        <v>3.33</v>
       </c>
       <c r="BM181" s="28" t="n">
-        <v>0.309598</v>
+        <v>0.3003</v>
       </c>
       <c r="BN181" s="28" t="n"/>
       <c r="BO181" s="28" t="n"/>
@@ -54024,12 +54024,12 @@
     <row r="182" ht="36" customHeight="1">
       <c r="A182" s="24" t="inlineStr">
         <is>
-          <t>6e6a3d07fd53427a</t>
+          <t>68921d6049b14dc0</t>
         </is>
       </c>
       <c r="B182" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C182" s="24" t="inlineStr">
@@ -54237,7 +54237,7 @@
       </c>
       <c r="BH182" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:22.065186Z</t>
+          <t>2026-08-02T08:13:25.131583Z</t>
         </is>
       </c>
       <c r="BI182" s="24" t="inlineStr">
@@ -54287,12 +54287,12 @@
     <row r="183" ht="36" customHeight="1">
       <c r="A183" s="24" t="inlineStr">
         <is>
-          <t>de3f150652ef466b</t>
+          <t>6d04be7a00184ee7</t>
         </is>
       </c>
       <c r="B183" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C183" s="24" t="inlineStr">
@@ -54500,7 +54500,7 @@
       </c>
       <c r="BH183" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:22.485293Z</t>
+          <t>2026-08-02T08:13:25.638678Z</t>
         </is>
       </c>
       <c r="BI183" s="24" t="inlineStr">
@@ -54550,12 +54550,12 @@
     <row r="184" ht="36" customHeight="1">
       <c r="A184" s="24" t="inlineStr">
         <is>
-          <t>4e0dc7c6fdc24b58</t>
+          <t>1c1a8c5c85614630</t>
         </is>
       </c>
       <c r="B184" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C184" s="24" t="inlineStr">
@@ -54763,7 +54763,7 @@
       </c>
       <c r="BH184" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:23.168431Z</t>
+          <t>2026-08-02T08:13:26.192927Z</t>
         </is>
       </c>
       <c r="BI184" s="24" t="inlineStr">
@@ -54813,12 +54813,12 @@
     <row r="185" ht="36" customHeight="1">
       <c r="A185" s="24" t="inlineStr">
         <is>
-          <t>f3e3be0dcf8a420b</t>
+          <t>0b4878d459e146f4</t>
         </is>
       </c>
       <c r="B185" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C185" s="24" t="inlineStr">
@@ -55026,7 +55026,7 @@
       </c>
       <c r="BH185" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:23.717602Z</t>
+          <t>2026-08-02T08:13:26.834968Z</t>
         </is>
       </c>
       <c r="BI185" s="24" t="inlineStr">
@@ -55076,12 +55076,12 @@
     <row r="186" ht="36" customHeight="1">
       <c r="A186" s="24" t="inlineStr">
         <is>
-          <t>4ddd29c26709402b</t>
+          <t>c744f8ab62ba4957</t>
         </is>
       </c>
       <c r="B186" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C186" s="24" t="inlineStr">
@@ -55289,7 +55289,7 @@
       </c>
       <c r="BH186" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:23.676456Z</t>
+          <t>2026-08-02T08:13:26.808979Z</t>
         </is>
       </c>
       <c r="BI186" s="24" t="inlineStr">
@@ -55339,12 +55339,12 @@
     <row r="187" ht="36" customHeight="1">
       <c r="A187" s="24" t="inlineStr">
         <is>
-          <t>20b8b805540145f3</t>
+          <t>73d4e6e35b2b448b</t>
         </is>
       </c>
       <c r="B187" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C187" s="24" t="inlineStr">
@@ -55552,7 +55552,7 @@
       </c>
       <c r="BH187" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:24.238512Z</t>
+          <t>2026-08-02T08:13:27.355220Z</t>
         </is>
       </c>
       <c r="BI187" s="24" t="inlineStr">
@@ -55602,12 +55602,12 @@
     <row r="188" ht="36" customHeight="1">
       <c r="A188" s="24" t="inlineStr">
         <is>
-          <t>0dc79436f18d40c0</t>
+          <t>eb5f7ec32e1c421a</t>
         </is>
       </c>
       <c r="B188" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C188" s="24" t="inlineStr">
@@ -55652,13 +55652,13 @@
         </is>
       </c>
       <c r="L188" s="26" t="n">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="M188" s="27" t="n">
-        <v>2.78</v>
+        <v>2.7</v>
       </c>
       <c r="N188" s="28" t="n">
-        <v>0.359712</v>
+        <v>0.37037</v>
       </c>
       <c r="O188" s="28" t="n">
         <v>0.456135</v>
@@ -55667,7 +55667,7 @@
         <v>0.2</v>
       </c>
       <c r="Q188" s="28" t="n">
-        <v>0.09642299999999999</v>
+        <v>0.08576499999999999</v>
       </c>
       <c r="R188" s="26" t="n">
         <v>0</v>
@@ -55696,7 +55696,7 @@
       <c r="AD188" s="24" t="n"/>
       <c r="AE188" s="31" t="inlineStr">
         <is>
-          <t>Poisson-DC rates 1.64 (home) / 1.24 (away) from EWMA attack/defense strengths. Executable ask 0.3600 (atc-arg2-ccns-ala-2026-08-02-ccns).</t>
+          <t>Poisson-DC rates 1.64 (home) / 1.24 (away) from EWMA attack/defense strengths. Executable ask 0.3700 (atc-arg2-ccns-ala-2026-08-02-ccns).</t>
         </is>
       </c>
       <c r="AF188" s="31" t="inlineStr">
@@ -55815,7 +55815,7 @@
       </c>
       <c r="BH188" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:24.757447Z</t>
+          <t>2026-08-02T08:13:27.689892Z</t>
         </is>
       </c>
       <c r="BI188" s="24" t="inlineStr">
@@ -55825,13 +55825,13 @@
       </c>
       <c r="BJ188" s="25" t="n"/>
       <c r="BK188" s="26" t="n">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="BL188" s="27" t="n">
-        <v>2.78</v>
+        <v>2.7</v>
       </c>
       <c r="BM188" s="28" t="n">
-        <v>0.359712</v>
+        <v>0.37037</v>
       </c>
       <c r="BN188" s="28" t="n"/>
       <c r="BO188" s="28" t="n"/>
@@ -55865,12 +55865,12 @@
     <row r="189" ht="36" customHeight="1">
       <c r="A189" s="24" t="inlineStr">
         <is>
-          <t>090a09d5fd4d406d</t>
+          <t>fe7efae2999247f8</t>
         </is>
       </c>
       <c r="B189" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C189" s="24" t="inlineStr">
@@ -56078,7 +56078,7 @@
       </c>
       <c r="BH189" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:25.306877Z</t>
+          <t>2026-08-02T08:13:28.471107Z</t>
         </is>
       </c>
       <c r="BI189" s="24" t="inlineStr">
@@ -56128,12 +56128,12 @@
     <row r="190" ht="36" customHeight="1">
       <c r="A190" s="24" t="inlineStr">
         <is>
-          <t>db361424be8b4858</t>
+          <t>c2bed9f78628467d</t>
         </is>
       </c>
       <c r="B190" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C190" s="24" t="inlineStr">
@@ -56178,13 +56178,13 @@
         </is>
       </c>
       <c r="L190" s="26" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="M190" s="27" t="n">
-        <v>2.44</v>
+        <v>2.5</v>
       </c>
       <c r="N190" s="28" t="n">
-        <v>0.409836</v>
+        <v>0.4</v>
       </c>
       <c r="O190" s="28" t="n">
         <v>0.5359159999999999</v>
@@ -56193,7 +56193,7 @@
         <v>0.2</v>
       </c>
       <c r="Q190" s="28" t="n">
-        <v>0.12608</v>
+        <v>0.135916</v>
       </c>
       <c r="R190" s="26" t="n">
         <v>0</v>
@@ -56222,7 +56222,7 @@
       <c r="AD190" s="24" t="n"/>
       <c r="AE190" s="31" t="inlineStr">
         <is>
-          <t>Poisson-DC rates 1.84 (home) / 1.10 (away) from EWMA attack/defense strengths. Executable ask 0.4100 (atc-pdc-ser-ohi-2026-08-02-ser).</t>
+          <t>Poisson-DC rates 1.84 (home) / 1.10 (away) from EWMA attack/defense strengths. Executable ask 0.4000 (atc-pdc-ser-ohi-2026-08-02-ser).</t>
         </is>
       </c>
       <c r="AF190" s="31" t="inlineStr">
@@ -56341,7 +56341,7 @@
       </c>
       <c r="BH190" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:26.361618Z</t>
+          <t>2026-08-02T08:13:29.617042Z</t>
         </is>
       </c>
       <c r="BI190" s="24" t="inlineStr">
@@ -56351,13 +56351,13 @@
       </c>
       <c r="BJ190" s="25" t="n"/>
       <c r="BK190" s="26" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="BL190" s="27" t="n">
-        <v>2.44</v>
+        <v>2.5</v>
       </c>
       <c r="BM190" s="28" t="n">
-        <v>0.409836</v>
+        <v>0.4</v>
       </c>
       <c r="BN190" s="28" t="n"/>
       <c r="BO190" s="28" t="n"/>
@@ -56391,12 +56391,12 @@
     <row r="191" ht="36" customHeight="1">
       <c r="A191" s="24" t="inlineStr">
         <is>
-          <t>04c349013aee44d2</t>
+          <t>1625b968d3704de2</t>
         </is>
       </c>
       <c r="B191" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C191" s="24" t="inlineStr">
@@ -56441,13 +56441,13 @@
         </is>
       </c>
       <c r="L191" s="26" t="n">
-        <v>-163</v>
+        <v>-170</v>
       </c>
       <c r="M191" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.588235</v>
       </c>
       <c r="N191" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.62963</v>
       </c>
       <c r="O191" s="28" t="n">
         <v>0.414794</v>
@@ -56456,7 +56456,7 @@
         <v>0.19</v>
       </c>
       <c r="Q191" s="28" t="n">
-        <v>-0.204978</v>
+        <v>-0.214836</v>
       </c>
       <c r="R191" s="26" t="n">
         <v>0</v>
@@ -56485,7 +56485,7 @@
       <c r="AD191" s="24" t="n"/>
       <c r="AE191" s="31" t="inlineStr">
         <is>
-          <t>Poisson-DC rates 1.41 (home) / 1.16 (away) from EWMA attack/defense strengths. Executable ask 0.6200 (atc-pdc-unc-hua-2026-08-02-unc).</t>
+          <t>Poisson-DC rates 1.41 (home) / 1.16 (away) from EWMA attack/defense strengths. Executable ask 0.6300 (atc-pdc-unc-hua-2026-08-02-unc).</t>
         </is>
       </c>
       <c r="AF191" s="31" t="inlineStr">
@@ -56604,7 +56604,7 @@
       </c>
       <c r="BH191" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:26.390990Z</t>
+          <t>2026-08-02T08:13:29.597576Z</t>
         </is>
       </c>
       <c r="BI191" s="24" t="inlineStr">
@@ -56614,13 +56614,13 @@
       </c>
       <c r="BJ191" s="25" t="n"/>
       <c r="BK191" s="26" t="n">
-        <v>-163</v>
+        <v>-170</v>
       </c>
       <c r="BL191" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.588235</v>
       </c>
       <c r="BM191" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.62963</v>
       </c>
       <c r="BN191" s="28" t="n"/>
       <c r="BO191" s="28" t="n"/>
@@ -56654,12 +56654,12 @@
     <row r="192" ht="36" customHeight="1">
       <c r="A192" s="24" t="inlineStr">
         <is>
-          <t>febf181e3cf644fb</t>
+          <t>a04b66b6c1b34776</t>
         </is>
       </c>
       <c r="B192" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C192" s="24" t="inlineStr">
@@ -56867,7 +56867,7 @@
       </c>
       <c r="BH192" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:27.403873Z</t>
+          <t>2026-08-02T08:13:30.643343Z</t>
         </is>
       </c>
       <c r="BI192" s="24" t="inlineStr">
@@ -56917,12 +56917,12 @@
     <row r="193" ht="36" customHeight="1">
       <c r="A193" s="24" t="inlineStr">
         <is>
-          <t>e8120f658b9f43f0</t>
+          <t>51d8c1e5ebd04dda</t>
         </is>
       </c>
       <c r="B193" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C193" s="24" t="inlineStr">
@@ -57130,7 +57130,7 @@
       </c>
       <c r="BH193" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:27.951055Z</t>
+          <t>2026-08-02T08:13:31.136989Z</t>
         </is>
       </c>
       <c r="BI193" s="24" t="inlineStr">
@@ -57180,12 +57180,12 @@
     <row r="194" ht="36" customHeight="1">
       <c r="A194" s="24" t="inlineStr">
         <is>
-          <t>fe7aa333f3cf4748</t>
+          <t>02705219e5ed4075</t>
         </is>
       </c>
       <c r="B194" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C194" s="24" t="inlineStr">
@@ -57230,13 +57230,13 @@
         </is>
       </c>
       <c r="L194" s="26" t="n">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="M194" s="27" t="n">
-        <v>2.86</v>
+        <v>2.94</v>
       </c>
       <c r="N194" s="28" t="n">
-        <v>0.34965</v>
+        <v>0.340136</v>
       </c>
       <c r="O194" s="28" t="n">
         <v>0.406677</v>
@@ -57245,7 +57245,7 @@
         <v>0.19</v>
       </c>
       <c r="Q194" s="28" t="n">
-        <v>0.057027</v>
+        <v>0.066541</v>
       </c>
       <c r="R194" s="26" t="n">
         <v>0</v>
@@ -57274,7 +57274,7 @@
       <c r="AD194" s="24" t="n"/>
       <c r="AE194" s="31" t="inlineStr">
         <is>
-          <t>Poisson-DC rates 1.38 (home) / 1.56 (away) from EWMA attack/defense strengths. Executable ask 0.3500 (atc-ecu1-leo-bsc-2026-08-02-bsc).</t>
+          <t>Poisson-DC rates 1.38 (home) / 1.56 (away) from EWMA attack/defense strengths. Executable ask 0.3400 (atc-ecu1-leo-bsc-2026-08-02-bsc).</t>
         </is>
       </c>
       <c r="AF194" s="31" t="inlineStr">
@@ -57393,7 +57393,7 @@
       </c>
       <c r="BH194" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:28.476441Z</t>
+          <t>2026-08-02T08:13:31.689990Z</t>
         </is>
       </c>
       <c r="BI194" s="24" t="inlineStr">
@@ -57403,13 +57403,13 @@
       </c>
       <c r="BJ194" s="25" t="n"/>
       <c r="BK194" s="26" t="n">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="BL194" s="27" t="n">
-        <v>2.86</v>
+        <v>2.94</v>
       </c>
       <c r="BM194" s="28" t="n">
-        <v>0.34965</v>
+        <v>0.340136</v>
       </c>
       <c r="BN194" s="28" t="n"/>
       <c r="BO194" s="28" t="n"/>
@@ -57443,12 +57443,12 @@
     <row r="195" ht="36" customHeight="1">
       <c r="A195" s="24" t="inlineStr">
         <is>
-          <t>eaf56d55f08b405f</t>
+          <t>9aad1ad1093340c8</t>
         </is>
       </c>
       <c r="B195" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C195" s="24" t="inlineStr">
@@ -57493,13 +57493,13 @@
         </is>
       </c>
       <c r="L195" s="26" t="n">
-        <v>-223</v>
+        <v>-233</v>
       </c>
       <c r="M195" s="27" t="n">
-        <v>1.44843</v>
+        <v>1.429185</v>
       </c>
       <c r="N195" s="28" t="n">
-        <v>0.690402</v>
+        <v>0.6997</v>
       </c>
       <c r="O195" s="28" t="n">
         <v>0.515227</v>
@@ -57508,7 +57508,7 @@
         <v>0.04</v>
       </c>
       <c r="Q195" s="28" t="n">
-        <v>-0.175175</v>
+        <v>-0.184473</v>
       </c>
       <c r="R195" s="26" t="n">
         <v>0</v>
@@ -57537,7 +57537,7 @@
       <c r="AD195" s="24" t="n"/>
       <c r="AE195" s="31" t="inlineStr">
         <is>
-          <t>Poisson-DC rates 0.88 (home) / 1.54 (away) from EWMA attack/defense strengths. Executable ask 0.6900 (atc-clbf-fvco-aja-2026-08-02-aja).</t>
+          <t>Poisson-DC rates 0.88 (home) / 1.54 (away) from EWMA attack/defense strengths. Executable ask 0.7000 (atc-clbf-fvco-aja-2026-08-02-aja).</t>
         </is>
       </c>
       <c r="AF195" s="31" t="inlineStr">
@@ -57656,7 +57656,7 @@
       </c>
       <c r="BH195" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:30.155770Z</t>
+          <t>2026-08-02T08:13:33.477773Z</t>
         </is>
       </c>
       <c r="BI195" s="24" t="inlineStr">
@@ -57666,13 +57666,13 @@
       </c>
       <c r="BJ195" s="25" t="n"/>
       <c r="BK195" s="26" t="n">
-        <v>-223</v>
+        <v>-233</v>
       </c>
       <c r="BL195" s="27" t="n">
-        <v>1.44843</v>
+        <v>1.429185</v>
       </c>
       <c r="BM195" s="28" t="n">
-        <v>0.690402</v>
+        <v>0.6997</v>
       </c>
       <c r="BN195" s="28" t="n"/>
       <c r="BO195" s="28" t="n"/>
@@ -57706,12 +57706,12 @@
     <row r="196" ht="36" customHeight="1">
       <c r="A196" s="24" t="inlineStr">
         <is>
-          <t>2e984910a37c454e</t>
+          <t>6d3bef7531ca4fda</t>
         </is>
       </c>
       <c r="B196" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C196" s="24" t="inlineStr">
@@ -57756,13 +57756,13 @@
         </is>
       </c>
       <c r="L196" s="26" t="n">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="M196" s="27" t="n">
-        <v>2.78</v>
+        <v>2.86</v>
       </c>
       <c r="N196" s="28" t="n">
-        <v>0.359712</v>
+        <v>0.34965</v>
       </c>
       <c r="O196" s="28" t="n">
         <v>0.575359</v>
@@ -57771,7 +57771,7 @@
         <v>0.04</v>
       </c>
       <c r="Q196" s="28" t="n">
-        <v>0.215647</v>
+        <v>0.225709</v>
       </c>
       <c r="R196" s="26" t="n">
         <v>100</v>
@@ -57800,7 +57800,7 @@
       <c r="AD196" s="24" t="n"/>
       <c r="AE196" s="31" t="inlineStr">
         <is>
-          <t>Poisson-DC rates 1.92 (home) / 1.01 (away) from EWMA attack/defense strengths. Executable ask 0.3600 (atc-clbf-fey-ata-2026-08-02-fey).</t>
+          <t>Poisson-DC rates 1.92 (home) / 1.01 (away) from EWMA attack/defense strengths. Executable ask 0.3500 (atc-clbf-fey-ata-2026-08-02-fey).</t>
         </is>
       </c>
       <c r="AF196" s="31" t="inlineStr">
@@ -57919,7 +57919,7 @@
       </c>
       <c r="BH196" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:30.185486Z</t>
+          <t>2026-08-02T08:13:33.464341Z</t>
         </is>
       </c>
       <c r="BI196" s="24" t="inlineStr">
@@ -57929,13 +57929,13 @@
       </c>
       <c r="BJ196" s="25" t="n"/>
       <c r="BK196" s="26" t="n">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="BL196" s="27" t="n">
-        <v>2.78</v>
+        <v>2.86</v>
       </c>
       <c r="BM196" s="28" t="n">
-        <v>0.359712</v>
+        <v>0.34965</v>
       </c>
       <c r="BN196" s="28" t="n"/>
       <c r="BO196" s="28" t="n"/>
@@ -57969,12 +57969,12 @@
     <row r="197" ht="36" customHeight="1">
       <c r="A197" s="24" t="inlineStr">
         <is>
-          <t>b75303f0a3574809</t>
+          <t>9e6c25b2c8f14a9f</t>
         </is>
       </c>
       <c r="B197" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C197" s="24" t="inlineStr">
@@ -58182,7 +58182,7 @@
       </c>
       <c r="BH197" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:30.672870Z</t>
+          <t>2026-08-02T08:13:33.982808Z</t>
         </is>
       </c>
       <c r="BI197" s="24" t="inlineStr">
@@ -58232,12 +58232,12 @@
     <row r="198" ht="36" customHeight="1">
       <c r="A198" s="24" t="inlineStr">
         <is>
-          <t>fc6eab56fbaa4ac6</t>
+          <t>0d1ed220585e4d89</t>
         </is>
       </c>
       <c r="B198" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C198" s="24" t="inlineStr">
@@ -58445,7 +58445,7 @@
       </c>
       <c r="BH198" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:30.781687Z</t>
+          <t>2026-08-02T08:13:34.058807Z</t>
         </is>
       </c>
       <c r="BI198" s="24" t="inlineStr">
@@ -58495,12 +58495,12 @@
     <row r="199" ht="36" customHeight="1">
       <c r="A199" s="24" t="inlineStr">
         <is>
-          <t>cc94b2f1ebbc4630</t>
+          <t>a91697472841420d</t>
         </is>
       </c>
       <c r="B199" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:14:17.312478Z</t>
+          <t>2026-08-02T08:16:59.190075Z</t>
         </is>
       </c>
       <c r="C199" s="24" t="inlineStr">
@@ -58545,13 +58545,13 @@
         </is>
       </c>
       <c r="L199" s="26" t="n">
-        <v>-127</v>
+        <v>-133</v>
       </c>
       <c r="M199" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.75188</v>
       </c>
       <c r="N199" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.570815</v>
       </c>
       <c r="O199" s="28" t="n">
         <v>0.482992</v>
@@ -58560,7 +58560,7 @@
         <v>0.04</v>
       </c>
       <c r="Q199" s="28" t="n">
-        <v>-0.07647900000000001</v>
+        <v>-0.087823</v>
       </c>
       <c r="R199" s="26" t="n">
         <v>0</v>
@@ -58589,7 +58589,7 @@
       <c r="AD199" s="24" t="n"/>
       <c r="AE199" s="31" t="inlineStr">
         <is>
-          <t>Poisson-DC rates 1.69 (home) / 1.17 (away) from EWMA attack/defense strengths. Executable ask 0.5600 (atc-clbf-lfc-lee-2026-08-02-lfc).</t>
+          <t>Poisson-DC rates 1.69 (home) / 1.17 (away) from EWMA attack/defense strengths. Executable ask 0.5700 (atc-clbf-lfc-lee-2026-08-02-lfc).</t>
         </is>
       </c>
       <c r="AF199" s="31" t="inlineStr">
@@ -58708,7 +58708,7 @@
       </c>
       <c r="BH199" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T07:11:31.252931Z</t>
+          <t>2026-08-02T08:13:34.558949Z</t>
         </is>
       </c>
       <c r="BI199" s="24" t="inlineStr">
@@ -58718,13 +58718,13 @@
       </c>
       <c r="BJ199" s="25" t="n"/>
       <c r="BK199" s="26" t="n">
-        <v>-127</v>
+        <v>-133</v>
       </c>
       <c r="BL199" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.75188</v>
       </c>
       <c r="BM199" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.570815</v>
       </c>
       <c r="BN199" s="28" t="n"/>
       <c r="BO199" s="28" t="n"/>

</xml_diff>